<commit_message>
Update participant OI report - 2026-09-07
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -193,14 +193,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>3846</v>
+        <v>9068</v>
       </c>
     </row>
     <row r="3">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>82</v>
+        <v>8095</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-3764</v>
+        <v>-973</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>3846</v>
+        <v>9068</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,28 +729,28 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>218910</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>209842</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>205996</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>200070</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>187130</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>178219</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="14" t="n">
-        <v>-156667</v>
+      <c r="S3" s="11" t="n">
+        <v>141650</v>
       </c>
     </row>
     <row r="4">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>282</v>
+        <v>48</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>2200</v>
+        <v>364</v>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="G4" s="14" t="n">
-        <v>-1918</v>
+        <v>-316</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,28 +798,28 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>11053</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>11369</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>13287</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>13267</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>20477</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>20288</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -827,8 +827,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>85563</v>
+      <c r="S4" s="11" t="n">
+        <v>-173050</v>
       </c>
     </row>
     <row r="5">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>187</v>
+        <v>1298</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>923</v>
+        <v>15553</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-736</v>
+        <v>-14255</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -867,20 +867,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-250093</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-235838</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-235102</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-229163</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-222032</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-209315</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>8511</v>
+        <v>33056</v>
       </c>
     </row>
     <row r="6">
@@ -906,13 +906,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>-1920</v>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>4051</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -920,15 +920,15 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-728</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>-1192</v>
+        <v>-1452</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>5503</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,20 +936,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>20130</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>14627</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>15819</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>15826</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>14425</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>10808</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>34022</v>
+        <v>118543</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-1369</v>
+        <v>13492</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-1369</v>
+        <v>13492</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="14" t="n">
-        <v>3924</v>
+      <c r="S7" s="11" t="n">
+        <v>-26059</v>
       </c>
     </row>
     <row r="8">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="14" t="n">
-        <v>-1918</v>
+        <v>-316</v>
       </c>
     </row>
     <row r="9">
@@ -1091,13 +1091,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>-82103</v>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>1160811</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
@@ -1105,53 +1105,53 @@
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>74564</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+        <v>1019161</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>141650</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>367520</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>225870</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>382537</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>273067</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>261983</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>-156667</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>225870</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>382537</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>273067</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>261983</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>195682</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S9" s="14" t="n">
-        <v>-215</v>
+        <v>-245</v>
       </c>
     </row>
     <row r="10">
@@ -1160,21 +1160,21 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>215</v>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>-275</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>-30</v>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-215</v>
+        <v>-245</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,28 +1190,28 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>3650</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>3895</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>4110</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>4260</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>4835</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>4310</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>68</v>
+      <c r="S10" s="11" t="n">
+        <v>-1013</v>
       </c>
     </row>
     <row r="11">
@@ -1235,15 +1235,15 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>6433</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>-2320</v>
+        <v>237122</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>231770</v>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="G11" s="11" t="n">
-        <v>8753</v>
+        <v>5352</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,20 +1259,20 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-298102</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-303454</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-312207</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-299253</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-248061</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-225462</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="S11" s="14" t="n">
-        <v>-38077</v>
+        <v>-20951</v>
       </c>
     </row>
     <row r="12">
@@ -1304,23 +1304,23 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>30446</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>-117684</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>148130</v>
+        <v>339165</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>485922</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>-146757</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,20 +1328,20 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>-73068</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>73689</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>-74441</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>21925</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>-18758</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>25471</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-10130</v>
+        <v>-25366</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-45224</v>
+        <v>1736823</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-45225</v>
+        <v>1736823</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-358</v>
+        <v>-155</v>
       </c>
     </row>
     <row r="14">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-736</v>
+        <v>-14255</v>
       </c>
     </row>
     <row r="15">
@@ -1483,13 +1483,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="n">
-        <v>441611</v>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>-30631</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,53 +1497,53 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>356048</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
+        <v>142419</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>-173050</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>-889308</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>-716258</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>-801821</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>-712140</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>-756948</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q15" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="14" t="n">
-        <v>85563</v>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>-716258</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>-801821</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>-712140</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>-756948</v>
-      </c>
-      <c r="N15" s="12" t="n">
-        <v>-686046</v>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q15" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S15" s="11" t="n">
-        <v>8753</v>
+        <v>5352</v>
       </c>
     </row>
     <row r="16">
@@ -1552,13 +1552,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>68</v>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>-1013</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1568,51 +1568,51 @@
       <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>-1013</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>31094</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>32107</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>32039</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>30008</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>31923</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>68</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>32107</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>32039</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>30008</v>
-      </c>
-      <c r="M16" s="12" t="n">
-        <v>31923</v>
-      </c>
-      <c r="N16" s="12" t="n">
-        <v>31784</v>
-      </c>
-      <c r="P16" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q16" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R16" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>-69138</v>
+      <c r="S16" s="14" t="n">
+        <v>50236</v>
       </c>
     </row>
     <row r="17">
@@ -1627,61 +1627,61 @@
         </is>
       </c>
       <c r="C17" s="14" t="n">
-        <v>18950</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="n">
-        <v>88088</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+        <v>34247</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>-15989</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>50236</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>631147</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>580911</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>650049</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>593223</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>632465</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>-69138</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>580911</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>650049</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>593223</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>632465</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>551407</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>20246</v>
+      <c r="S17" s="14" t="n">
+        <v>-28550</v>
       </c>
     </row>
     <row r="18">
@@ -1696,61 +1696,61 @@
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>113196</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>129689</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+        <v>72419</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>-51408</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>123827</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>227067</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>103240</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>119733</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>88909</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>92559</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>-16493</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>103240</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>119733</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>88909</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>92559</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>102855</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="11" t="n">
-        <v>2747</v>
+      <c r="S18" s="14" t="n">
+        <v>-12351</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>573825</v>
+        <v>75022</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>573825</v>
+        <v>75022</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="11" t="n">
-        <v>-85</v>
+      <c r="S19" s="14" t="n">
+        <v>19283</v>
       </c>
     </row>
     <row r="20">
@@ -1855,9 +1855,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>-1192</v>
+      <c r="S20" s="11" t="n">
+        <v>5503</v>
       </c>
     </row>
     <row r="21">
@@ -1881,15 +1881,15 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>10221</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="n">
-        <v>1710</v>
+        <v>31280</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>-1776</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>8511</v>
+        <v>33056</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,28 +1905,28 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3218140</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3185084</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3176573</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3173496</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>3185328</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3192623</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>148130</v>
+      <c r="S21" s="14" t="n">
+        <v>-146757</v>
       </c>
     </row>
     <row r="22">
@@ -1944,13 +1944,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="n">
-        <v>3508</v>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>-71</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>41585</v>
+        <v>20880</v>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-38077</v>
+        <v>-20951</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,28 +1974,28 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4296590</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4275639</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4237562</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4234485</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4195881</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4220839</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>-16493</v>
+      <c r="S22" s="14" t="n">
+        <v>123827</v>
       </c>
     </row>
     <row r="23">
@@ -2019,61 +2019,61 @@
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>-5212</v>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E23" s="11" t="n">
-        <v>-25458</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+        <v>-18402</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>10148</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>-28550</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>601593</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>630143</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>609897</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>593002</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>551323</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>20246</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>630143</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>609897</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>593002</v>
-      </c>
-      <c r="M23" s="12" t="n">
-        <v>551323</v>
-      </c>
-      <c r="N23" s="12" t="n">
-        <v>563880</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>9320</v>
+        <v>16445</v>
       </c>
     </row>
     <row r="24">
@@ -2088,7 +2088,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>14708</v>
+        <v>17271</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
@@ -2096,7 +2096,7 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>5388</v>
+        <v>826</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>9320</v>
+        <v>16445</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,20 +2112,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>476857</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>460412</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>451092</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>467987</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>459230</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>464336</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-26639</v>
+        <v>-80826</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>23225</v>
+        <v>30078</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>23225</v>
+        <v>30078</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="11" t="n">
-        <v>-3481</v>
+      <c r="S25" s="14" t="n">
+        <v>6931</v>
       </c>
     </row>
     <row r="26">
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>87376</v>
+        <v>156865</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>53354</v>
+        <v>38322</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>34022</v>
+        <v>118543</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1094613</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>976070</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>942048</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>903152</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>823961</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>708815</v>
       </c>
     </row>
     <row r="28">
@@ -2306,7 +2306,7 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>218</v>
+        <v>0</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>10348</v>
+        <v>25366</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-10130</v>
+        <v>-25366</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-334069</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-308703</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-298573</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-291576</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-251520</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-232982</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>13556</v>
+        <v>7569</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2373,15 +2373,15 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>10809</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G29" s="11" t="n">
-        <v>2747</v>
+        <v>19920</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>-12351</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-184197</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-171846</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-174593</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-169158</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-150845</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-139051</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 04-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 07-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>26838</v>
+        <v>390</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>53477</v>
+        <v>81216</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-26639</v>
+        <v>-80826</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-576347</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-495521</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-468882</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-442418</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-421596</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-336782</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23910.9</v>
+        <v>23883.15</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24005.75</v>
+        <v>23890</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>127988</v>
+        <v>164824</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>127988</v>
+        <v>164824</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23895.85</v>
+        <v>23737.9</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23897.7</v>
+        <v>23779.15</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24080.25000000001</v>
+        <v>24018.9</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23915.40000000001</v>
+        <v>23790.75</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2597,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="14" t="n">
-        <v>34606</v>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>-4049</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,15 +2611,15 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>30682</v>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="n">
-        <v>3924</v>
+        <v>22010</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>-26059</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-418487</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-392428</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-396352</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-383834</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-396117</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-361418</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24043</v>
+        <v>23954.45</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23933.1</v>
+        <v>23802.35</v>
       </c>
     </row>
     <row r="34">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>1058</v>
+        <v>155</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-358</v>
+        <v>-155</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>26446</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>26601</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>26959</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>28547</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>28940</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>29511</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23970.35000000001</v>
+        <v>23866.8</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23950.8</v>
+        <v>23813.95</v>
       </c>
     </row>
     <row r="35">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>11007</v>
+        <v>22653</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,15 +2745,15 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>11092</v>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G35" s="11" t="n">
-        <v>-85</v>
+        <v>3370</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>19283</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>137452</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>118169</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>118254</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>108203</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>100354</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>92473</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23933.1</v>
+        <v>23802.35</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>19733</v>
+        <v>16911</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,15 +2806,15 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>23214</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="n">
-        <v>-3481</v>
+        <v>9980</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>6931</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>254589</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>247658</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>251139</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>247084</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>266823</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>239434</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23860.45</v>
+        <v>23714.7</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>66046</v>
+        <v>35515</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>66046</v>
+        <v>35515</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23823.2</v>
+        <v>23650.25</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23750.55</v>
+        <v>23562.60000000001</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>10.68</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.34</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.59</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.49</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.19</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.994992330910013</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9997263611508541</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9984194572259013</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9999294072299643</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>1.005517111378178</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>1.006164539061341</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,898    PCR(OI) 0.84    Max Pain 24,000</t>
+          <t>Spot 23,779    PCR(OI) 0.56    Max Pain 23,800</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23898.82741935484</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23904.24112903226</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23911.24274193549</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23916.13830645161</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23923.80967741935</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23932.86491935484</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23779.15</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23897.7</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23873.45</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23914.45</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>24055.8</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>24080.4</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>24000</v>
+        <v>23800</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>233506</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>-49467</v>
+        <v>269738</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>239010</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>7532383</v>
+        <v>7544220</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,35 +3158,35 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
+        <v>0.976081019024068</v>
+      </c>
+      <c r="K46" s="25" t="n">
         <v>0.9813887944889631</v>
       </c>
-      <c r="K46" s="25" t="n">
+      <c r="L46" s="25" t="n">
         <v>0.9933791141865997</v>
       </c>
-      <c r="L46" s="25" t="n">
+      <c r="M46" s="25" t="n">
         <v>0.9970635633790684</v>
       </c>
-      <c r="M46" s="25" t="n">
+      <c r="N46" s="25" t="n">
         <v>1.002328084679025</v>
       </c>
-      <c r="N46" s="25" t="n">
-        <v>1.011430829957649</v>
-      </c>
       <c r="P46" s="28" t="n">
-        <v>24200</v>
+        <v>23900</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>180285</v>
-      </c>
-      <c r="R46" s="14" t="n">
-        <v>-1055</v>
+        <v>273322</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>195972</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>2877335</v>
-      </c>
-      <c r="T46" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>5736012</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3197,35 +3197,35 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
+        <v>24361.86088709677</v>
+      </c>
+      <c r="K47" s="18" t="n">
         <v>24350.89959677419</v>
       </c>
-      <c r="K47" s="18" t="n">
+      <c r="L47" s="18" t="n">
         <v>24336.7810483871</v>
       </c>
-      <c r="L47" s="18" t="n">
+      <c r="M47" s="18" t="n">
         <v>24323.42419354839</v>
       </c>
-      <c r="M47" s="18" t="n">
+      <c r="N47" s="18" t="n">
         <v>24309.40564516129</v>
       </c>
-      <c r="N47" s="18" t="n">
-        <v>24292.96129032258</v>
-      </c>
       <c r="P47" s="28" t="n">
-        <v>25000</v>
+        <v>24000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>218310</v>
-      </c>
-      <c r="R47" s="14" t="n">
-        <v>-38492</v>
+        <v>331482</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>97976</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>752670</v>
-      </c>
-      <c r="T47" s="31" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>4402666</v>
+      </c>
+      <c r="T47" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3236,21 +3236,21 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
+        <v>23779.15</v>
+      </c>
+      <c r="K48" s="18" t="n">
         <v>23897.7</v>
       </c>
-      <c r="K48" s="18" t="n">
+      <c r="L48" s="18" t="n">
         <v>24175.65</v>
       </c>
-      <c r="L48" s="18" t="n">
+      <c r="M48" s="18" t="n">
         <v>24252</v>
       </c>
-      <c r="M48" s="18" t="n">
+      <c r="N48" s="18" t="n">
         <v>24366</v>
       </c>
-      <c r="N48" s="18" t="n">
-        <v>24570.65</v>
-      </c>
-      <c r="P48" s="32" t="inlineStr">
+      <c r="P48" s="31" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3268,29 +3268,29 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
+          <t>07-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="30" t="inlineStr">
+        <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="K49" s="30" t="inlineStr">
+      <c r="L49" s="30" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="L49" s="30" t="inlineStr">
+      <c r="M49" s="30" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="30" t="inlineStr">
+      <c r="N49" s="30" t="inlineStr">
         <is>
           <t>14-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="30" t="inlineStr">
-        <is>
-          <t>07-Aug-2026</t>
-        </is>
-      </c>
       <c r="P49" s="27" t="inlineStr">
         <is>
           <t>Strike</t>
@@ -3318,17 +3318,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
-        <v>23900</v>
+      <c r="P50" s="32" t="n">
+        <v>23700</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>171059</v>
+        <v>162831</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>64327</v>
+        <v>43718</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>7170241</v>
+        <v>6432837</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3337,17 +3337,17 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="33" t="n">
-        <v>23800</v>
+      <c r="P51" s="32" t="n">
+        <v>23600</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>169564</v>
+        <v>155723</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>59469</v>
+        <v>28431</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>3578353</v>
+        <v>3798587</v>
       </c>
       <c r="T51" s="30" t="inlineStr">
         <is>
@@ -3356,19 +3356,19 @@
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="33" t="n">
-        <v>23000</v>
+      <c r="P52" s="32" t="n">
+        <v>23500</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>181983</v>
+        <v>172885</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>17908</v>
+        <v>12949</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>771093</v>
-      </c>
-      <c r="T52" s="31" t="inlineStr">
+        <v>2308377</v>
+      </c>
+      <c r="T52" s="33" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 04-Sep-2026    1 DAY AGO = 03-Sep-2026    2 DAYS AGO = 02-Sep-2026    3 DAYS AGO = 01-Sep-2026    4 DAYS AGO = 31-Aug-2026    (generated 04-Sep-2026 20:50 IST)</t>
+          <t>TODAY = 07-Sep-2026    1 DAY AGO = 04-Sep-2026    2 DAYS AGO = 03-Sep-2026    3 DAYS AGO = 02-Sep-2026    4 DAYS AGO = 01-Sep-2026    (generated 07-Sep-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-08
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -190,17 +190,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>9068</v>
+        <v>6728</v>
       </c>
     </row>
     <row r="3">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>8095</v>
+        <v>6698</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-973</v>
+        <v>-30</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>9068</v>
+        <v>6728</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,28 +729,28 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>225638</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>218910</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>209842</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>205996</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>200070</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>187130</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>141650</v>
+      <c r="S3" s="14" t="n">
+        <v>-23881</v>
       </c>
     </row>
     <row r="4">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>48</v>
+        <v>954</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
@@ -782,15 +782,15 @@
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>364</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="n">
-        <v>-316</v>
+        <v>735</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>219</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,28 +798,28 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>11272</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>11053</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>11369</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>13287</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>13267</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>20477</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -827,8 +827,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>-173050</v>
+      <c r="S4" s="14" t="n">
+        <v>145688</v>
       </c>
     </row>
     <row r="5">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>1298</v>
+        <v>2196</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>15553</v>
+        <v>13660</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-14255</v>
+        <v>-11464</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -867,28 +867,28 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-261557</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-250093</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-235838</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-235102</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-229163</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-222032</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -896,8 +896,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>33056</v>
+      <c r="S5" s="14" t="n">
+        <v>-5154</v>
       </c>
     </row>
     <row r="6">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>4051</v>
+        <v>3895</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-1452</v>
+        <v>-622</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>5503</v>
+        <v>4517</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,20 +936,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>24647</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>20130</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>14627</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>15819</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>15826</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>14425</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>118543</v>
+        <v>20802</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>13492</v>
+        <v>13743</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>13492</v>
+        <v>13743</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>-26059</v>
+      <c r="S7" s="14" t="n">
+        <v>15273</v>
       </c>
     </row>
     <row r="8">
@@ -1071,9 +1071,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>-316</v>
+      <c r="S8" s="11" t="n">
+        <v>219</v>
       </c>
     </row>
     <row r="9">
@@ -1091,29 +1091,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>1160811</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>1019161</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>141650</v>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>-2106587</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>-2082706</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>-23881</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,20 +1121,20 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>343639</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>367520</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>225870</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>382537</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>273067</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>261983</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="14" t="n">
-        <v>-245</v>
+        <v>-217</v>
       </c>
     </row>
     <row r="10">
@@ -1160,21 +1160,21 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="n">
-        <v>-275</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>-30</v>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>517</v>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-245</v>
+        <v>-217</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,20 +1190,20 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>3433</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>3650</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>3895</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>4110</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>4260</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>4835</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>-1013</v>
+        <v>-261</v>
       </c>
     </row>
     <row r="11">
@@ -1229,29 +1229,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="n">
-        <v>237122</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>231770</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G11" s="11" t="n">
-        <v>5352</v>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>-336207</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>-332227</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>-3980</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,20 +1259,20 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-302082</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-298102</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-303454</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-312207</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-299253</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-248061</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="S11" s="14" t="n">
-        <v>-20951</v>
+        <v>-4234</v>
       </c>
     </row>
     <row r="12">
@@ -1298,67 +1298,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>339165</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>485922</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>-609489</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>-637567</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>28078</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>-44990</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>-73068</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>73689</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>-74441</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>21925</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-146757</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>-73068</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>73689</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>-74441</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>21925</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>-18758</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-25366</v>
+        <v>-17000</v>
       </c>
     </row>
     <row r="13">
@@ -1369,11 +1369,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1736823</v>
+        <v>-3051983</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1736823</v>
+        <v>-3051983</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-155</v>
+        <v>-1519</v>
       </c>
     </row>
     <row r="14">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-14255</v>
+        <v>-11464</v>
       </c>
     </row>
     <row r="15">
@@ -1489,61 +1489,61 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>-30631</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="n">
-        <v>142419</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+        <v>-1048833</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>-1194521</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>145688</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>-743620</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>-889308</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>-716258</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>-801821</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>-712140</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>-173050</v>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>-889308</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>-716258</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>-801821</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>-712140</v>
-      </c>
-      <c r="N15" s="12" t="n">
-        <v>-756948</v>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q15" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="11" t="n">
-        <v>5352</v>
+      <c r="S15" s="14" t="n">
+        <v>-3980</v>
       </c>
     </row>
     <row r="16">
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>-1013</v>
+        <v>-261</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="G16" s="11" t="n">
-        <v>-1013</v>
+        <v>-261</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>30833</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>31094</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>32107</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>32039</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>30008</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>31923</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>50236</v>
+        <v>19498</v>
       </c>
     </row>
     <row r="17">
@@ -1621,13 +1621,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="n">
-        <v>34247</v>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>-132520</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="E17" s="14" t="n">
-        <v>-15989</v>
+        <v>-152018</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>50236</v>
+        <v>19498</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,20 +1651,20 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>650645</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>631147</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>580911</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>650049</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>593223</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>632465</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="14" t="n">
-        <v>-28550</v>
+        <v>-9721</v>
       </c>
     </row>
     <row r="18">
@@ -1690,13 +1690,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="n">
-        <v>72419</v>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>-481258</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
@@ -1704,15 +1704,15 @@
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>-51408</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="n">
-        <v>123827</v>
+        <v>-316333</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>-164925</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,20 +1720,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>62142</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>227067</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>103240</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>119733</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>88909</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>92559</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-12351</v>
+        <v>-9871</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>75022</v>
+        <v>-1662872</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>75022</v>
+        <v>-1662872</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>19283</v>
+        <v>10625</v>
       </c>
     </row>
     <row r="20">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>5503</v>
+        <v>4517</v>
       </c>
     </row>
     <row r="21">
@@ -1881,61 +1881,61 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>31280</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="11" t="n">
-        <v>-1776</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
+        <v>2548</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>7702</v>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>-5154</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3212986</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3218140</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3185084</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3176573</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3173496</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>33056</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>3218140</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>3185084</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>3176573</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>3173496</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>3185328</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-146757</v>
+      <c r="S21" s="11" t="n">
+        <v>28078</v>
       </c>
     </row>
     <row r="22">
@@ -1944,13 +1944,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="n">
-        <v>-71</v>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>1086</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>20880</v>
+        <v>5320</v>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-20951</v>
+        <v>-4234</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,28 +1974,28 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4300824</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4296590</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4275639</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4237562</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4234485</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4195881</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>123827</v>
+      <c r="S22" s="11" t="n">
+        <v>-164925</v>
       </c>
     </row>
     <row r="23">
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>-18402</v>
+        <v>-1093</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>10148</v>
+        <v>8628</v>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-28550</v>
+        <v>-9721</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,20 +2043,20 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>591872</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>601593</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>630143</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>609897</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>593002</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>551323</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>16445</v>
+        <v>19109</v>
       </c>
     </row>
     <row r="24">
@@ -2088,15 +2088,15 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>17271</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="n">
-        <v>826</v>
+        <v>15994</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>-3115</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>16445</v>
+        <v>19109</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,28 +2112,28 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>495966</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>476857</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>460412</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>451092</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>467987</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>459230</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>-80826</v>
+      <c r="S24" s="11" t="n">
+        <v>6069</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>30078</v>
+        <v>18535</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>30078</v>
+        <v>18535</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>6931</v>
+      <c r="S25" s="11" t="n">
+        <v>-24379</v>
       </c>
     </row>
     <row r="26">
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>156865</v>
+        <v>67919</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>38322</v>
+        <v>47117</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>118543</v>
+        <v>20802</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1115415</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1094613</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>976070</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>942048</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>903152</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>823961</v>
       </c>
     </row>
     <row r="28">
@@ -2300,13 +2300,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="n">
-        <v>0</v>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>-15</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>25366</v>
+        <v>16985</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-25366</v>
+        <v>-17000</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-351069</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-334069</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-308703</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-298573</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-291576</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-251520</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>7569</v>
+        <v>7176</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>19920</v>
+        <v>17047</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-12351</v>
+        <v>-9871</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-194068</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-184197</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-171846</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-174593</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-169158</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-150845</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 07-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 08-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>390</v>
+        <v>26569</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2432,15 +2432,15 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>81216</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G30" s="14" t="n">
-        <v>-80826</v>
+        <v>20500</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="n">
+        <v>6069</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-570278</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-576347</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-495521</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-468882</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-442418</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-421596</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23883.15</v>
+        <v>23743.1</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23890</v>
+        <v>23758.95</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>164824</v>
+        <v>101649</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>164824</v>
+        <v>101649</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23737.9</v>
+        <v>23623.1</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23779.15</v>
+        <v>23635.1</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24018.9</v>
+        <v>23857.51666666667</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23790.75</v>
+        <v>23653.74166666666</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2597,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="n">
-        <v>-4049</v>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>23189</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,15 +2611,15 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>22010</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G33" s="11" t="n">
-        <v>-26059</v>
+        <v>7916</v>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>15273</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-403214</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-418487</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-392428</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-396352</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-383834</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-396117</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23954.45</v>
+        <v>23808.23333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23802.35</v>
+        <v>23672.38333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>155</v>
+        <v>1585</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-155</v>
+        <v>-1519</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>24927</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>26446</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>26601</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>26959</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>28547</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>28940</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23866.8</v>
+        <v>23721.66666666666</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23813.95</v>
+        <v>23691.025</v>
       </c>
     </row>
     <row r="35">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>22653</v>
+        <v>17107</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>3370</v>
+        <v>6482</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>19283</v>
+        <v>10625</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>148077</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>137452</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>118169</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>118254</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>108203</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>100354</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23802.35</v>
+        <v>23672.38333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>16911</v>
+        <v>13779</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,15 +2806,15 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>9980</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>6931</v>
+        <v>38158</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>-24379</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>230210</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>254589</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>247658</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>251139</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>247084</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>266823</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23714.7</v>
+        <v>23585.81666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>35515</v>
+        <v>54141</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>35515</v>
+        <v>54141</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23650.25</v>
+        <v>23536.53333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23562.60000000001</v>
+        <v>23449.96666666666</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.23</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.16</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>10.68</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.34</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.59</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.49</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9890959913034546</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.994992330910013</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9997263611508541</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9984194572259013</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9999294072299643</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>1.005517111378178</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,779    PCR(OI) 0.56    Max Pain 23,800</t>
+          <t>Spot 23,635    PCR(OI) 0.61    Max Pain 23,650</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23895.65846774193</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23898.82741935484</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23904.24112903226</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23911.24274193549</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23916.13830645161</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23923.80967741935</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23635.1</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23779.15</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23897.7</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23873.45</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23914.45</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>24055.8</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23800</v>
+        <v>23650</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>269738</v>
+        <v>448385</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>239010</v>
+        <v>436889</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>7544220</v>
+        <v>18633376</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.976081019024068</v>
+        <v>0.9702143527251239</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9813887944889631</v>
@@ -3173,16 +3173,16 @@
         <v>1.002328084679025</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23900</v>
+        <v>23700</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>273322</v>
+        <v>304146</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>195972</v>
+        <v>258905</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>5736012</v>
+        <v>26512058</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24361.86088709677</v>
+        <v>24360.69919354839</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24350.89959677419</v>
@@ -3215,17 +3215,17 @@
         <v>24000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>331482</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>97976</v>
+        <v>200822</v>
+      </c>
+      <c r="R47" s="14" t="n">
+        <v>-124534</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>4402666</v>
+        <v>4782742</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23779.15</v>
+        <v>23635.1</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23897.7</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="30" t="inlineStr">
-        <is>
-          <t>07-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="30" t="inlineStr">
+      <c r="J49" s="32" t="inlineStr">
+        <is>
+          <t>08-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="32" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="30" t="inlineStr">
+      <c r="L49" s="32" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="30" t="inlineStr">
+      <c r="M49" s="32" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="30" t="inlineStr">
+      <c r="N49" s="32" t="inlineStr">
         <is>
           <t>14-Aug-2026</t>
         </is>
@@ -3318,17 +3318,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
-        <v>23700</v>
+      <c r="P50" s="33" t="n">
+        <v>23600</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>162831</v>
+        <v>310517</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>43718</v>
+        <v>156530</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>6432837</v>
+        <v>27367299</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3337,47 +3337,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="32" t="n">
-        <v>23600</v>
+      <c r="P51" s="33" t="n">
+        <v>23550</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>155723</v>
+        <v>163536</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>28431</v>
+        <v>92287</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>3798587</v>
-      </c>
-      <c r="T51" s="30" t="inlineStr">
+        <v>15564615</v>
+      </c>
+      <c r="T51" s="32" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
+      <c r="P52" s="33" t="n">
         <v>23500</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>172885</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>12949</v>
+        <v>145280</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>-24898</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>2308377</v>
-      </c>
-      <c r="T52" s="33" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>10475788</v>
+      </c>
+      <c r="T52" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 07-Sep-2026    1 DAY AGO = 04-Sep-2026    2 DAYS AGO = 03-Sep-2026    3 DAYS AGO = 02-Sep-2026    4 DAYS AGO = 01-Sep-2026    (generated 07-Sep-2026 20:31 IST)</t>
+          <t>TODAY = 08-Sep-2026    1 DAY AGO = 07-Sep-2026    2 DAYS AGO = 04-Sep-2026    3 DAYS AGO = 03-Sep-2026    4 DAYS AGO = 02-Sep-2026    (generated 08-Sep-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-09
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -190,17 +190,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>6728</v>
+        <v>4842</v>
       </c>
     </row>
     <row r="3">
@@ -705,15 +705,15 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>6698</v>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="n">
-        <v>-30</v>
+        <v>6950</v>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>2108</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,34 +721,34 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>6728</v>
+        <v>4842</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="14" t="n">
+        <v>230480</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>225638</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="14" t="n">
         <v>218910</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="14" t="n">
         <v>209842</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>205996</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>200070</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
+      <c r="Q3" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="14" t="n">
-        <v>-23881</v>
+      <c r="S3" s="13" t="n">
+        <v>-16983</v>
       </c>
     </row>
     <row r="4">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>954</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="n">
-        <v>735</v>
+        <v>291</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>-3048</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -790,36 +790,36 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>219</v>
+        <v>3339</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="14" t="n">
+        <v>14611</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>11272</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="14" t="n">
         <v>11053</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="14" t="n">
         <v>11369</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="14" t="n">
         <v>13287</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>13267</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -827,8 +827,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>145688</v>
+      <c r="S4" s="11" t="n">
+        <v>-88058</v>
       </c>
     </row>
     <row r="5">
@@ -843,52 +843,52 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>2196</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+        <v>1844</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n">
-        <v>13660</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="E5" s="13" t="n">
+        <v>16537</v>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-11464</v>
+      <c r="G5" s="13" t="n">
+        <v>-14693</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="14" t="n">
+        <v>-276250</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-261557</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="14" t="n">
         <v>-250093</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="14" t="n">
         <v>-235838</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="14" t="n">
         <v>-235102</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-229163</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -896,8 +896,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="14" t="n">
-        <v>-5154</v>
+      <c r="S5" s="11" t="n">
+        <v>26996</v>
       </c>
     </row>
     <row r="6">
@@ -912,15 +912,15 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>3895</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>-622</v>
+        <v>9087</v>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>2575</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -928,28 +928,28 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>4517</v>
+        <v>6512</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
+        <v>31159</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>24647</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>20130</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="14" t="n">
         <v>14627</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="14" t="n">
         <v>15819</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>15826</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>20802</v>
+        <v>69230</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>13743</v>
+        <v>18172</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>13743</v>
+        <v>18172</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="14" t="n">
-        <v>15273</v>
+      <c r="S7" s="11" t="n">
+        <v>-1994</v>
       </c>
     </row>
     <row r="8">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>219</v>
+        <v>3339</v>
       </c>
     </row>
     <row r="9">
@@ -1091,56 +1091,56 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>-2106587</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>-2082706</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>741965</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>758948</v>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>-23881</v>
+      <c r="G9" s="13" t="n">
+        <v>-16983</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="14" t="n">
+        <v>326656</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>343639</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="14" t="n">
         <v>367520</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="14" t="n">
         <v>225870</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="14" t="n">
         <v>382537</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>273067</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
+      <c r="Q9" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>-217</v>
+      <c r="S9" s="13" t="n">
+        <v>-1999</v>
       </c>
     </row>
     <row r="10">
@@ -1166,52 +1166,52 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>300</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="14" t="n">
-        <v>517</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="E10" s="13" t="n">
+        <v>1999</v>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>-217</v>
+      <c r="G10" s="13" t="n">
+        <v>-1999</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
+        <v>1434</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>3433</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>3650</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="14" t="n">
         <v>3895</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="14" t="n">
         <v>4110</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>4260</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q10" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>-261</v>
+      <c r="S10" s="13" t="n">
+        <v>18840</v>
       </c>
     </row>
     <row r="11">
@@ -1229,56 +1229,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="n">
-        <v>-336207</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>-332227</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>101528</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>142089</v>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-3980</v>
+      <c r="G11" s="13" t="n">
+        <v>-40561</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="14" t="n">
+        <v>-342643</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-302082</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="14" t="n">
         <v>-298102</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="14" t="n">
         <v>-303454</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="14" t="n">
         <v>-312207</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-299253</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="13" t="inlineStr">
+      <c r="Q11" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>-4234</v>
+      <c r="S11" s="13" t="n">
+        <v>-4405</v>
       </c>
     </row>
     <row r="12">
@@ -1298,21 +1298,21 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>-609489</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>-637567</v>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>249758</v>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>190216</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
@@ -1320,34 +1320,34 @@
         </is>
       </c>
       <c r="G12" s="11" t="n">
-        <v>28078</v>
+        <v>59542</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="14" t="n">
+        <v>14552</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>-44990</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <v>-73068</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="14" t="n">
         <v>73689</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="14" t="n">
         <v>-74441</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>21925</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="13" t="inlineStr">
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>-17000</v>
+      <c r="S12" s="13" t="n">
+        <v>-7909</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-3051983</v>
+        <v>1093251</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-3051983</v>
+        <v>1093252</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-1519</v>
+        <v>-806</v>
       </c>
     </row>
     <row r="14">
@@ -1463,7 +1463,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
+      <c r="Q14" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>-11464</v>
+      <c r="S14" s="13" t="n">
+        <v>-14693</v>
       </c>
     </row>
     <row r="15">
@@ -1483,56 +1483,56 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="n">
-        <v>-1048833</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>-1194521</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G15" s="14" t="n">
-        <v>145688</v>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>285475</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>373533</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>-88058</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-831678</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-743620</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-889308</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>-716258</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>-801821</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-712140</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
+      <c r="Q15" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>-3980</v>
+      <c r="S15" s="13" t="n">
+        <v>-40561</v>
       </c>
     </row>
     <row r="16">
@@ -1552,56 +1552,56 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>-261</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="n">
-        <v>-261</v>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>18800</v>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>-40</v>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>18840</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="14" t="n">
+        <v>49673</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>30833</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <v>31094</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="14" t="n">
         <v>32107</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="14" t="n">
         <v>32039</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>30008</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
+      <c r="Q16" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>19498</v>
+      <c r="S16" s="13" t="n">
+        <v>9607</v>
       </c>
     </row>
     <row r="17">
@@ -1621,56 +1621,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="n">
-        <v>-132520</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>-152018</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>98581</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>88974</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>19498</v>
+      <c r="G17" s="13" t="n">
+        <v>9607</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="12" t="n">
+      <c r="J17" s="14" t="n">
+        <v>660252</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <v>650645</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="14" t="n">
         <v>631147</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="14" t="n">
         <v>580911</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="14" t="n">
         <v>650049</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>593223</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
+      <c r="Q17" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1680,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>-9721</v>
+      <c r="S17" s="13" t="n">
+        <v>-27404</v>
       </c>
     </row>
     <row r="18">
@@ -1690,67 +1690,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="n">
-        <v>-481258</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>-316333</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="n">
+        <v>127590</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>67979</v>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>59611</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="n">
+        <v>121753</v>
+      </c>
+      <c r="K18" s="14" t="n">
+        <v>62142</v>
+      </c>
+      <c r="L18" s="14" t="n">
+        <v>227067</v>
+      </c>
+      <c r="M18" s="14" t="n">
+        <v>103240</v>
+      </c>
+      <c r="N18" s="14" t="n">
+        <v>119733</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>-164925</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>62142</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>227067</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>103240</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>119733</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>88909</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>-9871</v>
+      <c r="S18" s="13" t="n">
+        <v>-13223</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-1662872</v>
+        <v>530446</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-1662872</v>
+        <v>530446</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1786,7 +1786,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
+      <c r="Q19" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>10625</v>
+      <c r="S19" s="13" t="n">
+        <v>18254</v>
       </c>
     </row>
     <row r="20">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>4517</v>
+        <v>6512</v>
       </c>
     </row>
     <row r="21">
@@ -1881,44 +1881,44 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>2548</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+        <v>27436</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
-        <v>7702</v>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G21" s="14" t="n">
-        <v>-5154</v>
+      <c r="E21" s="13" t="n">
+        <v>440</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>26996</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="14" t="n">
+        <v>3239982</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3212986</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <v>3218140</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="14" t="n">
         <v>3185084</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="14" t="n">
         <v>3176573</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3173496</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="S21" s="11" t="n">
-        <v>28078</v>
+        <v>59542</v>
       </c>
     </row>
     <row r="22">
@@ -1950,52 +1950,52 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>1086</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
+        <v>16687</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
-        <v>5320</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="E22" s="13" t="n">
+        <v>21092</v>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>-4234</v>
+      <c r="G22" s="13" t="n">
+        <v>-4405</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J22" s="14" t="n">
+        <v>-4305229</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-4300824</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="14" t="n">
         <v>-4296590</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="14" t="n">
         <v>-4275639</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="14" t="n">
         <v>-4237562</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4234485</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q22" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>-164925</v>
+      <c r="S22" s="13" t="n">
+        <v>59611</v>
       </c>
     </row>
     <row r="23">
@@ -2013,50 +2013,50 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="n">
-        <v>-1093</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>11241</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n">
-        <v>8628</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
+      <c r="E23" s="13" t="n">
+        <v>38645</v>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>-9721</v>
+      <c r="G23" s="13" t="n">
+        <v>-27404</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="J23" s="14" t="n">
+        <v>564468</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>591872</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <v>601593</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="14" t="n">
         <v>630143</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="14" t="n">
         <v>609897</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>593002</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>19109</v>
+        <v>4813</v>
       </c>
     </row>
     <row r="24">
@@ -2088,15 +2088,15 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>15994</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="n">
-        <v>-3115</v>
+        <v>18605</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>13792</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2104,36 +2104,36 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>19109</v>
+        <v>4813</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J24" s="14" t="n">
+        <v>500779</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>495966</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="14" t="n">
         <v>476857</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="14" t="n">
         <v>460412</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="14" t="n">
         <v>451092</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>467987</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q24" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="11" t="n">
-        <v>6069</v>
+      <c r="S24" s="13" t="n">
+        <v>-48098</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>18535</v>
+        <v>73969</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>18535</v>
+        <v>73969</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="11" t="n">
-        <v>-24379</v>
+        <v>-15454</v>
       </c>
     </row>
     <row r="26">
@@ -2255,15 +2255,15 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>67919</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+        <v>103254</v>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
-        <v>47117</v>
+      <c r="E27" s="13" t="n">
+        <v>34024</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,27 +2271,27 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>20802</v>
+        <v>69230</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>1184645</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>1115415</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>1094613</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="14" t="n">
         <v>976070</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>942048</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>903152</v>
       </c>
     </row>
     <row r="28">
@@ -2300,49 +2300,49 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="14" t="n">
-        <v>-15</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="14" t="n">
-        <v>16985</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="E28" s="13" t="n">
+        <v>7909</v>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>-17000</v>
+      <c r="G28" s="13" t="n">
+        <v>-7909</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-358978</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-351069</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-334069</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="14" t="n">
         <v>-308703</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>-298573</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-291576</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,47 +2365,47 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>7176</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+        <v>20089</v>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>17047</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
+      <c r="E29" s="13" t="n">
+        <v>33312</v>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>-9871</v>
+      <c r="G29" s="13" t="n">
+        <v>-13223</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-207291</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-194068</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-184197</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="14" t="n">
         <v>-171846</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>-174593</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-169158</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 08-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 09-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,51 +2424,51 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>26569</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
+        <v>28796</v>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>20500</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G30" s="11" t="n">
-        <v>6069</v>
+      <c r="E30" s="13" t="n">
+        <v>76894</v>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>-48098</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-618376</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-570278</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-576347</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="14" t="n">
         <v>-495521</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="14" t="n">
         <v>-468882</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-442418</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23743.1</v>
+        <v>23522.05</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23758.95</v>
+        <v>23571.55</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>101649</v>
+        <v>152139</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>101649</v>
+        <v>152139</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23623.1</v>
+        <v>23431.5</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23635.1</v>
+        <v>23431.5</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23857.51666666667</v>
+        <v>23664.91666666667</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23653.74166666666</v>
+        <v>23454.84166666667</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2597,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
-        <v>23189</v>
+      <c r="C33" s="13" t="n">
+        <v>19615</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,43 +2611,43 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>7916</v>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="n">
-        <v>15273</v>
+        <v>21609</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>-1994</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-405208</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-403214</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-418487</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="14" t="n">
         <v>-392428</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="14" t="n">
         <v>-396352</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-383834</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23808.23333333333</v>
+        <v>23618.23333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23672.38333333333</v>
+        <v>23478.18333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2664,13 +2664,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="14" t="n">
-        <v>66</v>
+      <c r="C34" s="13" t="n">
+        <v>23</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>1585</v>
+        <v>829</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,35 +2686,35 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-1519</v>
+        <v>-806</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>24121</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>24927</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>26446</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="14" t="n">
         <v>26601</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="14" t="n">
         <v>26959</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>28547</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23721.66666666666</v>
+        <v>23524.86666666667</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23691.025</v>
+        <v>23501.525</v>
       </c>
     </row>
     <row r="35">
@@ -2731,13 +2731,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>17107</v>
+      <c r="C35" s="13" t="n">
+        <v>32067</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,43 +2745,43 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>6482</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
+        <v>13813</v>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>10625</v>
+      <c r="G35" s="13" t="n">
+        <v>18254</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>166331</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>148077</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>137452</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="14" t="n">
         <v>118169</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="14" t="n">
         <v>118254</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>108203</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23672.38333333333</v>
+        <v>23478.18333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,13 +2792,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>13779</v>
+      <c r="C36" s="13" t="n">
+        <v>26117</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>38158</v>
+        <v>41571</v>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
@@ -2814,35 +2814,35 @@
         </is>
       </c>
       <c r="G36" s="11" t="n">
-        <v>-24379</v>
+        <v>-15454</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>214756</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>230210</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>254589</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="14" t="n">
         <v>247658</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="14" t="n">
         <v>251139</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>247084</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23585.81666666666</v>
+        <v>23384.81666666667</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>54141</v>
+        <v>77822</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>54141</v>
+        <v>77822</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23536.53333333333</v>
+        <v>23338.13333333334</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23449.96666666666</v>
+        <v>23244.76666666667</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.23</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.16</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>10.68</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.34</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.59</v>
       </c>
     </row>
     <row r="41">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 08-Sep-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 15-Sep-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9808503997602754</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9890959913034546</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.994992330910013</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9997263611508541</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9984194572259013</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9999294072299643</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,635    PCR(OI) 0.61    Max Pain 23,650</t>
+          <t>Spot 23,432    PCR(OI) 0.59    Max Pain 23,600</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23888.96411290322</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23895.65846774193</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23898.82741935484</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23904.24112903226</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23911.24274193549</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23916.13830645161</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23431.5</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23635.1</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23779.15</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23897.7</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23873.45</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23914.45</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23650</v>
-      </c>
-      <c r="Q45" s="12" t="n">
-        <v>448385</v>
+        <v>23700</v>
+      </c>
+      <c r="Q45" s="14" t="n">
+        <v>161846</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>436889</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>18633376</v>
+        <v>87098</v>
+      </c>
+      <c r="S45" s="14" t="n">
+        <v>1928737</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9702143527251239</v>
+        <v>0.9619214632061579</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9813887944889631</v>
@@ -3173,16 +3173,16 @@
         <v>1.002328084679025</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23700</v>
-      </c>
-      <c r="Q46" s="12" t="n">
-        <v>304146</v>
+        <v>23800</v>
+      </c>
+      <c r="Q46" s="14" t="n">
+        <v>137629</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>258905</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>26512058</v>
+        <v>47825</v>
+      </c>
+      <c r="S46" s="14" t="n">
+        <v>1645701</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24360.69919354839</v>
+        <v>24359.05725806452</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24350.89959677419</v>
@@ -3214,18 +3214,18 @@
       <c r="P47" s="28" t="n">
         <v>24000</v>
       </c>
-      <c r="Q47" s="12" t="n">
-        <v>200822</v>
-      </c>
-      <c r="R47" s="14" t="n">
-        <v>-124534</v>
-      </c>
-      <c r="S47" s="12" t="n">
-        <v>4782742</v>
+      <c r="Q47" s="14" t="n">
+        <v>181017</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>53815</v>
+      </c>
+      <c r="S47" s="14" t="n">
+        <v>1328506</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23635.1</v>
+        <v>23431.5</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23897.7</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="32" t="inlineStr">
-        <is>
-          <t>08-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="32" t="inlineStr">
+      <c r="J49" s="30" t="inlineStr">
+        <is>
+          <t>09-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="30" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="32" t="inlineStr">
+      <c r="L49" s="30" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="32" t="inlineStr">
+      <c r="M49" s="30" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="32" t="inlineStr">
+      <c r="N49" s="30" t="inlineStr">
         <is>
           <t>14-Aug-2026</t>
         </is>
@@ -3318,17 +3318,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
-        <v>23600</v>
-      </c>
-      <c r="Q50" s="12" t="n">
-        <v>310517</v>
+      <c r="P50" s="32" t="n">
+        <v>23400</v>
+      </c>
+      <c r="Q50" s="14" t="n">
+        <v>80282</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>156530</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>27367299</v>
+        <v>26876</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>2075393</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3337,47 +3337,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="33" t="n">
-        <v>23550</v>
-      </c>
-      <c r="Q51" s="12" t="n">
-        <v>163536</v>
+      <c r="P51" s="32" t="n">
+        <v>23000</v>
+      </c>
+      <c r="Q51" s="14" t="n">
+        <v>140559</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>92287</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>15564615</v>
-      </c>
-      <c r="T51" s="32" t="inlineStr">
+        <v>45711</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>1010918</v>
+      </c>
+      <c r="T51" s="30" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="33" t="n">
-        <v>23500</v>
-      </c>
-      <c r="Q52" s="12" t="n">
-        <v>145280</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>-24898</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>10475788</v>
-      </c>
-      <c r="T52" s="32" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="P52" s="32" t="n">
+        <v>22100</v>
+      </c>
+      <c r="Q52" s="14" t="n">
+        <v>78679</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>6022</v>
+      </c>
+      <c r="S52" s="14" t="n">
+        <v>200332</v>
+      </c>
+      <c r="T52" s="33" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 08-Sep-2026    1 DAY AGO = 07-Sep-2026    2 DAYS AGO = 04-Sep-2026    3 DAYS AGO = 03-Sep-2026    4 DAYS AGO = 02-Sep-2026    (generated 08-Sep-2026 20:32 IST)</t>
+          <t>TODAY = 09-Sep-2026    1 DAY AGO = 08-Sep-2026    2 DAYS AGO = 07-Sep-2026    3 DAYS AGO = 04-Sep-2026    4 DAYS AGO = 03-Sep-2026    (generated 09-Sep-2026 21:25 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-10
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -190,17 +190,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>4842</v>
+        <v>491</v>
       </c>
     </row>
     <row r="3">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>6950</v>
+        <v>3385</v>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="13" t="n">
-        <v>2108</v>
+        <v>2894</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>4842</v>
+        <v>491</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,28 +729,28 @@
         </is>
       </c>
       <c r="J3" s="14" t="n">
+        <v>230971</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>230480</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="14" t="n">
         <v>225638</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="14" t="n">
         <v>218910</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="14" t="n">
         <v>209842</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>205996</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="13" t="n">
-        <v>-16983</v>
+      <c r="S3" s="11" t="n">
+        <v>53504</v>
       </c>
     </row>
     <row r="4">
@@ -768,13 +768,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>291</v>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>-454</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>-3048</v>
+        <v>-735</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>3339</v>
+        <v>281</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,28 +798,28 @@
         </is>
       </c>
       <c r="J4" s="14" t="n">
+        <v>14892</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>14611</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="14" t="n">
         <v>11272</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="14" t="n">
         <v>11053</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="14" t="n">
         <v>11369</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>13287</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q4" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -827,8 +827,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>-88058</v>
+      <c r="S4" s="13" t="n">
+        <v>17176</v>
       </c>
     </row>
     <row r="5">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>1844</v>
+        <v>667</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E5" s="13" t="n">
-        <v>16537</v>
+        <v>6261</v>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-14693</v>
+        <v>-5594</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -867,20 +867,20 @@
         </is>
       </c>
       <c r="J5" s="14" t="n">
+        <v>-281844</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-276250</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="14" t="n">
         <v>-261557</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="14" t="n">
         <v>-250093</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="N5" s="14" t="n">
         <v>-235838</v>
       </c>
-      <c r="N5" s="14" t="n">
-        <v>-235102</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>26996</v>
+        <v>5829</v>
       </c>
     </row>
     <row r="6">
@@ -912,15 +912,15 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>9087</v>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="n">
-        <v>2575</v>
+        <v>3435</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>-1387</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>6512</v>
+        <v>4822</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,20 +936,20 @@
         </is>
       </c>
       <c r="J6" s="14" t="n">
+        <v>35981</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>31159</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="14" t="n">
         <v>24647</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="14" t="n">
         <v>20130</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="14" t="n">
         <v>14627</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>15819</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>69230</v>
+        <v>83287</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>18172</v>
+        <v>7033</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>18172</v>
+        <v>7033</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-1994</v>
+        <v>-3189</v>
       </c>
     </row>
     <row r="8">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>3339</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>741965</v>
+        <v>480054</v>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
@@ -1105,15 +1105,15 @@
         </is>
       </c>
       <c r="E9" s="13" t="n">
-        <v>758948</v>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G9" s="13" t="n">
-        <v>-16983</v>
+        <v>426550</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>53504</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,28 +1121,28 @@
         </is>
       </c>
       <c r="J9" s="14" t="n">
+        <v>380160</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>326656</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="L9" s="14" t="n">
         <v>343639</v>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="M9" s="14" t="n">
         <v>367520</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="N9" s="14" t="n">
         <v>225870</v>
       </c>
-      <c r="N9" s="14" t="n">
-        <v>382537</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="13" t="n">
-        <v>-1999</v>
+      <c r="S9" s="11" t="n">
+        <v>66</v>
       </c>
     </row>
     <row r="10">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
@@ -1174,15 +1174,15 @@
         </is>
       </c>
       <c r="E10" s="13" t="n">
-        <v>1999</v>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="n">
-        <v>-1999</v>
+        <v>134</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>66</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,20 +1190,20 @@
         </is>
       </c>
       <c r="J10" s="14" t="n">
+        <v>1500</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>1434</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="14" t="n">
         <v>3433</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="14" t="n">
         <v>3650</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="14" t="n">
         <v>3895</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>4110</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="S10" s="13" t="n">
-        <v>18840</v>
+        <v>865</v>
       </c>
     </row>
     <row r="11">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>101528</v>
+        <v>65051</v>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
@@ -1243,15 +1243,15 @@
         </is>
       </c>
       <c r="E11" s="13" t="n">
-        <v>142089</v>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="n">
-        <v>-40561</v>
+        <v>41279</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>23772</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,28 +1259,28 @@
         </is>
       </c>
       <c r="J11" s="14" t="n">
+        <v>-318871</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-342643</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="14" t="n">
         <v>-302082</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="M11" s="14" t="n">
         <v>-298102</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="14" t="n">
         <v>-303454</v>
       </c>
-      <c r="N11" s="14" t="n">
-        <v>-312207</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="13" t="n">
-        <v>-4405</v>
+      <c r="S11" s="11" t="n">
+        <v>23764</v>
       </c>
     </row>
     <row r="12">
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>249758</v>
+        <v>35719</v>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
@@ -1312,15 +1312,15 @@
         </is>
       </c>
       <c r="E12" s="13" t="n">
-        <v>190216</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>59542</v>
+        <v>113061</v>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="n">
+        <v>-77342</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,20 +1328,20 @@
         </is>
       </c>
       <c r="J12" s="14" t="n">
+        <v>-62790</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>14552</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="14" t="n">
         <v>-44990</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="M12" s="14" t="n">
         <v>-73068</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="14" t="n">
         <v>73689</v>
       </c>
-      <c r="N12" s="14" t="n">
-        <v>-74441</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="S12" s="13" t="n">
-        <v>-7909</v>
+        <v>-12783</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1093251</v>
+        <v>581024</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1093252</v>
+        <v>581024</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-806</v>
+        <v>-426</v>
       </c>
     </row>
     <row r="14">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="13" t="n">
-        <v>-14693</v>
+        <v>-5594</v>
       </c>
     </row>
     <row r="15">
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="C15" s="13" t="n">
-        <v>285475</v>
+        <v>340509</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,15 +1497,15 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>373533</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="n">
-        <v>-88058</v>
+        <v>323333</v>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>17176</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,28 +1513,28 @@
         </is>
       </c>
       <c r="J15" s="14" t="n">
+        <v>-814502</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-831678</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="14" t="n">
         <v>-743620</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="14" t="n">
         <v>-889308</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="14" t="n">
         <v>-716258</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-801821</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="13" t="n">
-        <v>-40561</v>
+      <c r="S15" s="11" t="n">
+        <v>23772</v>
       </c>
     </row>
     <row r="16">
@@ -1558,15 +1558,15 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>18800</v>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="n">
-        <v>-40</v>
+        <v>865</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="G16" s="13" t="n">
-        <v>18840</v>
+        <v>865</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="14" t="n">
+        <v>50538</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>49673</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="14" t="n">
         <v>30833</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="14" t="n">
         <v>31094</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="14" t="n">
         <v>32107</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>32039</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="13" t="n">
-        <v>9607</v>
+        <v>2512</v>
       </c>
     </row>
     <row r="17">
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="C17" s="13" t="n">
-        <v>98581</v>
+        <v>54168</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>88974</v>
+        <v>51656</v>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="G17" s="13" t="n">
-        <v>9607</v>
+        <v>2512</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,20 +1651,20 @@
         </is>
       </c>
       <c r="J17" s="14" t="n">
+        <v>662764</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <v>660252</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="L17" s="14" t="n">
         <v>650645</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="M17" s="14" t="n">
         <v>631147</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="N17" s="14" t="n">
         <v>580911</v>
       </c>
-      <c r="N17" s="14" t="n">
-        <v>650049</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="13" t="n">
-        <v>-27404</v>
+        <v>-22548</v>
       </c>
     </row>
     <row r="18">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>127590</v>
+        <v>120344</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1704,15 +1704,15 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>67979</v>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G18" s="13" t="n">
-        <v>59611</v>
+        <v>140897</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>-20553</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,20 +1720,20 @@
         </is>
       </c>
       <c r="J18" s="14" t="n">
+        <v>101200</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>121753</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="14" t="n">
         <v>62142</v>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="M18" s="14" t="n">
         <v>227067</v>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="N18" s="14" t="n">
         <v>103240</v>
       </c>
-      <c r="N18" s="14" t="n">
-        <v>119733</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="S18" s="13" t="n">
-        <v>-13223</v>
+        <v>-11868</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>530446</v>
+        <v>515886</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>530446</v>
+        <v>515886</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="13" t="n">
-        <v>18254</v>
+        <v>14651</v>
       </c>
     </row>
     <row r="20">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>6512</v>
+        <v>4822</v>
       </c>
     </row>
     <row r="21">
@@ -1881,15 +1881,15 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>27436</v>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="n">
-        <v>440</v>
+        <v>3382</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>-2447</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>26996</v>
+        <v>5829</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,28 +1905,28 @@
         </is>
       </c>
       <c r="J21" s="14" t="n">
+        <v>3245811</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3239982</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="14" t="n">
         <v>3212986</v>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="M21" s="14" t="n">
         <v>3218140</v>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="N21" s="14" t="n">
         <v>3185084</v>
       </c>
-      <c r="N21" s="14" t="n">
-        <v>3176573</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q21" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>59542</v>
+      <c r="S21" s="13" t="n">
+        <v>-77342</v>
       </c>
     </row>
     <row r="22">
@@ -1950,61 +1950,61 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>16687</v>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="n">
-        <v>21092</v>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
+        <v>11692</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>-12072</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="n">
+        <v>23764</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>-4281465</v>
+      </c>
+      <c r="K22" s="14" t="n">
+        <v>-4305229</v>
+      </c>
+      <c r="L22" s="14" t="n">
+        <v>-4300824</v>
+      </c>
+      <c r="M22" s="14" t="n">
+        <v>-4296590</v>
+      </c>
+      <c r="N22" s="14" t="n">
+        <v>-4275639</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="13" t="n">
-        <v>-4405</v>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J22" s="14" t="n">
-        <v>-4305229</v>
-      </c>
-      <c r="K22" s="14" t="n">
-        <v>-4300824</v>
-      </c>
-      <c r="L22" s="14" t="n">
-        <v>-4296590</v>
-      </c>
-      <c r="M22" s="14" t="n">
-        <v>-4275639</v>
-      </c>
-      <c r="N22" s="14" t="n">
-        <v>-4237562</v>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q22" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="13" t="n">
-        <v>59611</v>
+      <c r="S22" s="11" t="n">
+        <v>-20553</v>
       </c>
     </row>
     <row r="23">
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>11241</v>
+        <v>1639</v>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="E23" s="13" t="n">
-        <v>38645</v>
+        <v>24187</v>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-27404</v>
+        <v>-22548</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,28 +2043,28 @@
         </is>
       </c>
       <c r="J23" s="14" t="n">
+        <v>541920</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>564468</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="L23" s="14" t="n">
         <v>591872</v>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="M23" s="14" t="n">
         <v>601593</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="N23" s="14" t="n">
         <v>630143</v>
       </c>
-      <c r="N23" s="14" t="n">
-        <v>609897</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q23" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>4813</v>
+      <c r="S23" s="13" t="n">
+        <v>-7045</v>
       </c>
     </row>
     <row r="24">
@@ -2082,13 +2082,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="n">
-        <v>18605</v>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="n">
+        <v>-2514</v>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
@@ -2096,15 +2096,15 @@
         </is>
       </c>
       <c r="E24" s="13" t="n">
-        <v>13792</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="n">
-        <v>4813</v>
+        <v>4531</v>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>-7045</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,20 +2112,20 @@
         </is>
       </c>
       <c r="J24" s="14" t="n">
+        <v>493734</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>500779</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="14" t="n">
         <v>495966</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="14" t="n">
         <v>476857</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="14" t="n">
         <v>460412</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>451092</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="13" t="n">
-        <v>-48098</v>
+        <v>-58636</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>73969</v>
+        <v>14199</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>73969</v>
+        <v>14199</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="11" t="n">
-        <v>-15454</v>
+        <v>-11036</v>
       </c>
     </row>
     <row r="26">
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>103254</v>
+        <v>108053</v>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="E27" s="13" t="n">
-        <v>34024</v>
+        <v>24766</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>69230</v>
+        <v>83287</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="14" t="n">
+        <v>1267932</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>1184645</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="14" t="n">
         <v>1115415</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="14" t="n">
         <v>1094613</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="14" t="n">
         <v>976070</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>942048</v>
       </c>
     </row>
     <row r="28">
@@ -2300,13 +2300,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="n">
-        <v>0</v>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="n">
+        <v>-5</v>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="E28" s="13" t="n">
-        <v>7909</v>
+        <v>12778</v>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="G28" s="13" t="n">
-        <v>-7909</v>
+        <v>-12783</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="14" t="n">
+        <v>-371761</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-358978</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="14" t="n">
         <v>-351069</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="14" t="n">
         <v>-334069</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="14" t="n">
         <v>-308703</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-298573</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>20089</v>
+        <v>6508</v>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="E29" s="13" t="n">
-        <v>33312</v>
+        <v>18376</v>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="G29" s="13" t="n">
-        <v>-13223</v>
+        <v>-11868</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="14" t="n">
+        <v>-219159</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-207291</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="14" t="n">
         <v>-194068</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="14" t="n">
         <v>-184197</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="14" t="n">
         <v>-171846</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-174593</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 09-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 10-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>28796</v>
+        <v>12586</v>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="E30" s="13" t="n">
-        <v>76894</v>
+        <v>71222</v>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-48098</v>
+        <v>-58636</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="14" t="n">
+        <v>-677012</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-618376</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="14" t="n">
         <v>-570278</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="14" t="n">
         <v>-576347</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="14" t="n">
         <v>-495521</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-468882</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23522.05</v>
+        <v>23446.6</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23571.55</v>
+        <v>23494.95</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>152139</v>
+        <v>127142</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>152139</v>
+        <v>127142</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23431.5</v>
+        <v>23380.1</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23431.5</v>
+        <v>23477.8</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23664.91666666667</v>
+        <v>23636.65000000001</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23454.84166666667</v>
+        <v>23464.375</v>
       </c>
     </row>
     <row r="33">
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="C33" s="13" t="n">
-        <v>19615</v>
+        <v>5395</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>21609</v>
+        <v>8584</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-1994</v>
+        <v>-3189</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="14" t="n">
+        <v>-408397</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-405208</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="14" t="n">
         <v>-403214</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="14" t="n">
         <v>-418487</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="14" t="n">
         <v>-392428</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-396352</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23618.23333333333</v>
+        <v>23565.8</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23478.18333333333</v>
+        <v>23450.95</v>
       </c>
     </row>
     <row r="34">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="C34" s="13" t="n">
-        <v>23</v>
+        <v>113</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>829</v>
+        <v>539</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-806</v>
+        <v>-426</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="14" t="n">
+        <v>23695</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>24121</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="14" t="n">
         <v>24927</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="14" t="n">
         <v>26446</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="14" t="n">
         <v>26601</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>26959</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23524.86666666667</v>
+        <v>23521.8</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23501.525</v>
+        <v>23437.525</v>
       </c>
     </row>
     <row r="35">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="C35" s="13" t="n">
-        <v>32067</v>
+        <v>17675</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>13813</v>
+        <v>3024</v>
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
         </is>
       </c>
       <c r="G35" s="13" t="n">
-        <v>18254</v>
+        <v>14651</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="14" t="n">
+        <v>180982</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>166331</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="14" t="n">
         <v>148077</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="14" t="n">
         <v>137452</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="14" t="n">
         <v>118169</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>118254</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23478.18333333333</v>
+        <v>23450.95</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="C36" s="13" t="n">
-        <v>26117</v>
+        <v>16376</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>41571</v>
+        <v>27412</v>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
@@ -2814,7 +2814,7 @@
         </is>
       </c>
       <c r="G36" s="11" t="n">
-        <v>-15454</v>
+        <v>-11036</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="14" t="n">
+        <v>203720</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>214756</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="14" t="n">
         <v>230210</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="14" t="n">
         <v>254589</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="14" t="n">
         <v>247658</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>251139</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23384.81666666667</v>
+        <v>23406.95</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>77822</v>
+        <v>39559</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>77822</v>
+        <v>39559</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23338.13333333334</v>
+        <v>23336.1</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23244.76666666667</v>
+        <v>23292.1</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.92</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.23</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.16</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>10.68</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.34</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9829176264436748</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9808503997602754</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9890959913034546</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.994992330910013</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9997263611508541</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9984194572259013</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,432    PCR(OI) 0.59    Max Pain 23,600</t>
+          <t>Spot 23,478    PCR(OI) 0.64    Max Pain 23,500</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23885.82661290323</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23888.96411290322</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23895.65846774193</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23898.82741935484</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23904.24112903226</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23911.24274193549</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23477.8</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23431.5</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23635.1</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23779.15</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23897.7</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23873.45</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23700</v>
+        <v>23500</v>
       </c>
       <c r="Q45" s="14" t="n">
-        <v>161846</v>
+        <v>180147</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>87098</v>
+        <v>56011</v>
       </c>
       <c r="S45" s="14" t="n">
-        <v>1928737</v>
+        <v>2977798</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9619214632061579</v>
+        <v>0.9638074198858003</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9813887944889631</v>
@@ -3173,20 +3173,20 @@
         <v>1.002328084679025</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23800</v>
+        <v>24000</v>
       </c>
       <c r="Q46" s="14" t="n">
-        <v>137629</v>
+        <v>214443</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>47825</v>
+        <v>33426</v>
       </c>
       <c r="S46" s="14" t="n">
-        <v>1645701</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>896853</v>
+      </c>
+      <c r="T46" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24359.05725806452</v>
+        <v>24359.43064516129</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24350.89959677419</v>
@@ -3212,20 +3212,20 @@
         <v>24309.40564516129</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>24000</v>
+        <v>24500</v>
       </c>
       <c r="Q47" s="14" t="n">
-        <v>181017</v>
+        <v>171767</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>53815</v>
+        <v>55571</v>
       </c>
       <c r="S47" s="14" t="n">
-        <v>1328506</v>
+        <v>848564</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23431.5</v>
+        <v>23477.8</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23897.7</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="30" t="inlineStr">
-        <is>
-          <t>09-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="30" t="inlineStr">
+      <c r="J49" s="32" t="inlineStr">
+        <is>
+          <t>10-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="32" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="30" t="inlineStr">
+      <c r="L49" s="32" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="30" t="inlineStr">
+      <c r="M49" s="32" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="30" t="inlineStr">
+      <c r="N49" s="32" t="inlineStr">
         <is>
           <t>14-Aug-2026</t>
         </is>
@@ -3318,17 +3318,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
+      <c r="P50" s="33" t="n">
         <v>23400</v>
       </c>
       <c r="Q50" s="14" t="n">
-        <v>80282</v>
+        <v>122869</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>26876</v>
+        <v>42587</v>
       </c>
       <c r="S50" s="14" t="n">
-        <v>2075393</v>
+        <v>3765046</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3337,38 +3337,38 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="32" t="n">
+      <c r="P51" s="33" t="n">
         <v>23000</v>
       </c>
       <c r="Q51" s="14" t="n">
-        <v>140559</v>
+        <v>163298</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>45711</v>
+        <v>22739</v>
       </c>
       <c r="S51" s="14" t="n">
-        <v>1010918</v>
+        <v>914254</v>
       </c>
       <c r="T51" s="30" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>22100</v>
+      <c r="P52" s="33" t="n">
+        <v>22500</v>
       </c>
       <c r="Q52" s="14" t="n">
-        <v>78679</v>
+        <v>124737</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>6022</v>
+        <v>52744</v>
       </c>
       <c r="S52" s="14" t="n">
-        <v>200332</v>
-      </c>
-      <c r="T52" s="33" t="inlineStr">
+        <v>411516</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 09-Sep-2026    1 DAY AGO = 08-Sep-2026    2 DAYS AGO = 07-Sep-2026    3 DAYS AGO = 04-Sep-2026    4 DAYS AGO = 03-Sep-2026    (generated 09-Sep-2026 21:25 IST)</t>
+          <t>TODAY = 10-Sep-2026    1 DAY AGO = 09-Sep-2026    2 DAYS AGO = 08-Sep-2026    3 DAYS AGO = 07-Sep-2026    4 DAYS AGO = 04-Sep-2026    (generated 10-Sep-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-11
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -129,19 +129,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,7 +187,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,11 +196,11 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>491</v>
+        <v>517</v>
       </c>
     </row>
     <row r="3">
@@ -699,21 +699,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="n">
-        <v>3385</v>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>2894</v>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>-476</v>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>-993</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>491</v>
+        <v>517</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,28 +729,28 @@
         </is>
       </c>
       <c r="J3" s="14" t="n">
+        <v>231488</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>230971</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="14" t="n">
         <v>230480</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="14" t="n">
         <v>225638</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="14" t="n">
         <v>218910</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>209842</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q3" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>53504</v>
+      <c r="S3" s="13" t="n">
+        <v>-150498</v>
       </c>
     </row>
     <row r="4">
@@ -768,67 +768,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>-454</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>-735</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>459</v>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>1003</v>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="n">
+        <v>-544</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>14348</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>14892</v>
+      </c>
+      <c r="L4" s="14" t="n">
+        <v>14611</v>
+      </c>
+      <c r="M4" s="14" t="n">
+        <v>11272</v>
+      </c>
+      <c r="N4" s="14" t="n">
+        <v>11053</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>281</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="14" t="n">
-        <v>14892</v>
-      </c>
-      <c r="K4" s="14" t="n">
-        <v>14611</v>
-      </c>
-      <c r="L4" s="14" t="n">
-        <v>11272</v>
-      </c>
-      <c r="M4" s="14" t="n">
-        <v>11053</v>
-      </c>
-      <c r="N4" s="14" t="n">
-        <v>11369</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
       <c r="S4" s="13" t="n">
-        <v>17176</v>
+        <v>61381</v>
       </c>
     </row>
     <row r="5">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>667</v>
+        <v>1558</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E5" s="13" t="n">
-        <v>6261</v>
+        <v>4596</v>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-5594</v>
+        <v>-3038</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -867,20 +867,20 @@
         </is>
       </c>
       <c r="J5" s="14" t="n">
+        <v>-284882</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-281844</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="14" t="n">
         <v>-276250</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="14" t="n">
         <v>-261557</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="N5" s="14" t="n">
         <v>-250093</v>
       </c>
-      <c r="N5" s="14" t="n">
-        <v>-235838</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>5829</v>
+        <v>19515</v>
       </c>
     </row>
     <row r="6">
@@ -906,13 +906,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>3435</v>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>-128</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-1387</v>
+        <v>-3193</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>4822</v>
+        <v>3065</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,20 +936,20 @@
         </is>
       </c>
       <c r="J6" s="14" t="n">
+        <v>39046</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>35981</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="14" t="n">
         <v>31159</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="14" t="n">
         <v>24647</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="14" t="n">
         <v>20130</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>14627</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>83287</v>
+        <v>21452</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>7033</v>
+        <v>1413</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>7033</v>
+        <v>1413</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q7" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>-3189</v>
+      <c r="S7" s="13" t="n">
+        <v>2226</v>
       </c>
     </row>
     <row r="8">
@@ -1071,9 +1071,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q8" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>281</v>
+      <c r="S8" s="13" t="n">
+        <v>-544</v>
       </c>
     </row>
     <row r="9">
@@ -1091,13 +1091,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>480054</v>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>-97628</v>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
@@ -1105,53 +1105,53 @@
         </is>
       </c>
       <c r="E9" s="13" t="n">
-        <v>426550</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
+        <v>52870</v>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>-150498</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>229662</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>380160</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>326656</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <v>343639</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <v>367520</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>53504</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>380160</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>326656</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>343639</v>
-      </c>
-      <c r="M9" s="14" t="n">
-        <v>367520</v>
-      </c>
-      <c r="N9" s="14" t="n">
-        <v>225870</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>66</v>
+        <v>551</v>
       </c>
     </row>
     <row r="10">
@@ -1166,15 +1166,15 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>200</v>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="n">
-        <v>134</v>
+        <v>0</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>-551</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>66</v>
+        <v>551</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,20 +1190,20 @@
         </is>
       </c>
       <c r="J10" s="14" t="n">
+        <v>2051</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="14" t="n">
         <v>1434</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="14" t="n">
         <v>3433</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="14" t="n">
         <v>3650</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>3895</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="S10" s="13" t="n">
-        <v>865</v>
+        <v>6286</v>
       </c>
     </row>
     <row r="11">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>65051</v>
+        <v>46982</v>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="E11" s="13" t="n">
-        <v>41279</v>
+        <v>15209</v>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="G11" s="11" t="n">
-        <v>23772</v>
+        <v>31773</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,28 +1259,28 @@
         </is>
       </c>
       <c r="J11" s="14" t="n">
+        <v>-287098</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-318871</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="14" t="n">
         <v>-342643</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="M11" s="14" t="n">
         <v>-302082</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="14" t="n">
         <v>-298102</v>
       </c>
-      <c r="N11" s="14" t="n">
-        <v>-303454</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q11" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>23764</v>
+      <c r="S11" s="13" t="n">
+        <v>-10083</v>
       </c>
     </row>
     <row r="12">
@@ -1304,61 +1304,61 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>35719</v>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>113061</v>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
+        <v>50474</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>-67702</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>118176</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="n">
+        <v>55386</v>
+      </c>
+      <c r="K12" s="14" t="n">
+        <v>-62790</v>
+      </c>
+      <c r="L12" s="14" t="n">
+        <v>14552</v>
+      </c>
+      <c r="M12" s="14" t="n">
+        <v>-44990</v>
+      </c>
+      <c r="N12" s="14" t="n">
+        <v>-73068</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="13" t="n">
-        <v>-77342</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="n">
-        <v>-62790</v>
-      </c>
-      <c r="K12" s="14" t="n">
-        <v>14552</v>
-      </c>
-      <c r="L12" s="14" t="n">
-        <v>-44990</v>
-      </c>
-      <c r="M12" s="14" t="n">
-        <v>-73068</v>
-      </c>
-      <c r="N12" s="14" t="n">
-        <v>73689</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S12" s="13" t="n">
-        <v>-12783</v>
+        <v>-7745</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>581024</v>
+        <v>-172</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>581024</v>
+        <v>-174</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-426</v>
+        <v>-1771</v>
       </c>
     </row>
     <row r="14">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="13" t="n">
-        <v>-5594</v>
+        <v>-3038</v>
       </c>
     </row>
     <row r="15">
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="C15" s="13" t="n">
-        <v>340509</v>
+        <v>770521</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>323333</v>
+        <v>709140</v>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="G15" s="13" t="n">
-        <v>17176</v>
+        <v>61381</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="14" t="n">
+        <v>-753121</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-814502</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="14" t="n">
         <v>-831678</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="14" t="n">
         <v>-743620</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="14" t="n">
         <v>-889308</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-716258</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="11" t="n">
-        <v>23772</v>
+        <v>31773</v>
       </c>
     </row>
     <row r="16">
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>865</v>
+        <v>6286</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="G16" s="13" t="n">
-        <v>865</v>
+        <v>6286</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="14" t="n">
+        <v>56824</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>50538</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="14" t="n">
         <v>49673</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="14" t="n">
         <v>30833</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="14" t="n">
         <v>31094</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>32107</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="13" t="n">
-        <v>2512</v>
+        <v>6947</v>
       </c>
     </row>
     <row r="17">
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="C17" s="13" t="n">
-        <v>54168</v>
+        <v>206875</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>51656</v>
+        <v>199928</v>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="G17" s="13" t="n">
-        <v>2512</v>
+        <v>6947</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,20 +1651,20 @@
         </is>
       </c>
       <c r="J17" s="14" t="n">
+        <v>669711</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <v>662764</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="L17" s="14" t="n">
         <v>660252</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="M17" s="14" t="n">
         <v>650645</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="N17" s="14" t="n">
         <v>631147</v>
       </c>
-      <c r="N17" s="14" t="n">
-        <v>580911</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="13" t="n">
-        <v>-22548</v>
+        <v>-22318</v>
       </c>
     </row>
     <row r="18">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>120344</v>
+        <v>263134</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>140897</v>
+        <v>337749</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="G18" s="11" t="n">
-        <v>-20553</v>
+        <v>-74615</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,20 +1720,20 @@
         </is>
       </c>
       <c r="J18" s="14" t="n">
+        <v>26585</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>101200</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="14" t="n">
         <v>121753</v>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="M18" s="14" t="n">
         <v>62142</v>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="N18" s="14" t="n">
         <v>227067</v>
       </c>
-      <c r="N18" s="14" t="n">
-        <v>103240</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="S18" s="13" t="n">
-        <v>-11868</v>
+        <v>-13748</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>515886</v>
+        <v>1246816</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>515886</v>
+        <v>1246817</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="13" t="n">
-        <v>14651</v>
+        <v>16366</v>
       </c>
     </row>
     <row r="20">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>4822</v>
+        <v>3065</v>
       </c>
     </row>
     <row r="21">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>3382</v>
+        <v>18358</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>-2447</v>
+        <v>-1157</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>5829</v>
+        <v>19515</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,28 +1905,28 @@
         </is>
       </c>
       <c r="J21" s="14" t="n">
+        <v>3265326</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3245811</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="14" t="n">
         <v>3239982</v>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="M21" s="14" t="n">
         <v>3212986</v>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="N21" s="14" t="n">
         <v>3218140</v>
       </c>
-      <c r="N21" s="14" t="n">
-        <v>3185084</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="13" t="n">
-        <v>-77342</v>
+      <c r="S21" s="11" t="n">
+        <v>118176</v>
       </c>
     </row>
     <row r="22">
@@ -1944,29 +1944,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="n">
-        <v>11692</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>-12072</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G22" s="11" t="n">
-        <v>23764</v>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="n">
+        <v>-2285</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>7798</v>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>-10083</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="14" t="n">
+        <v>-4291548</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-4281465</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="14" t="n">
         <v>-4305229</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="14" t="n">
         <v>-4300824</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="14" t="n">
         <v>-4296590</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-4275639</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="11" t="n">
-        <v>-20553</v>
+        <v>-74615</v>
       </c>
     </row>
     <row r="23">
@@ -2013,13 +2013,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="n">
-        <v>1639</v>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="n">
+        <v>-1298</v>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="E23" s="13" t="n">
-        <v>24187</v>
+        <v>21020</v>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-22548</v>
+        <v>-22318</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,28 +2043,28 @@
         </is>
       </c>
       <c r="J23" s="14" t="n">
+        <v>519602</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>541920</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="L23" s="14" t="n">
         <v>564468</v>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="M23" s="14" t="n">
         <v>591872</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="N23" s="14" t="n">
         <v>601593</v>
       </c>
-      <c r="N23" s="14" t="n">
-        <v>630143</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="13" t="n">
-        <v>-7045</v>
+      <c r="S23" s="11" t="n">
+        <v>12886</v>
       </c>
     </row>
     <row r="24">
@@ -2082,13 +2082,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="n">
-        <v>-2514</v>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>19077</v>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
@@ -2096,15 +2096,15 @@
         </is>
       </c>
       <c r="E24" s="13" t="n">
-        <v>4531</v>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="n">
-        <v>-7045</v>
+        <v>6191</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>12886</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,28 +2112,28 @@
         </is>
       </c>
       <c r="J24" s="14" t="n">
+        <v>506620</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>493734</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="14" t="n">
         <v>500779</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="14" t="n">
         <v>495966</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="14" t="n">
         <v>476857</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>460412</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="13" t="n">
-        <v>-58636</v>
+      <c r="S24" s="11" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>14199</v>
+        <v>33852</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>14199</v>
+        <v>33852</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="11" t="n">
-        <v>-11036</v>
+        <v>-16821</v>
       </c>
     </row>
     <row r="26">
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>108053</v>
+        <v>48581</v>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="E27" s="13" t="n">
-        <v>24766</v>
+        <v>27129</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>83287</v>
+        <v>21452</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="14" t="n">
+        <v>1289384</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>1267932</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="14" t="n">
         <v>1184645</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="14" t="n">
         <v>1115415</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="14" t="n">
         <v>1094613</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>976070</v>
       </c>
     </row>
     <row r="28">
@@ -2300,13 +2300,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="n">
-        <v>-5</v>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="E28" s="13" t="n">
-        <v>12778</v>
+        <v>7745</v>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="G28" s="13" t="n">
-        <v>-12783</v>
+        <v>-7745</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="14" t="n">
+        <v>-379506</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-371761</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="14" t="n">
         <v>-358978</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="14" t="n">
         <v>-351069</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="14" t="n">
         <v>-334069</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-308703</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>6508</v>
+        <v>12924</v>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="E29" s="13" t="n">
-        <v>18376</v>
+        <v>26672</v>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="G29" s="13" t="n">
-        <v>-11868</v>
+        <v>-13748</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="14" t="n">
+        <v>-232907</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-219159</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="14" t="n">
         <v>-207291</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="14" t="n">
         <v>-194068</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="14" t="n">
         <v>-184197</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-171846</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 10-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 11-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>12586</v>
+        <v>52125</v>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
@@ -2432,15 +2432,15 @@
         </is>
       </c>
       <c r="E30" s="13" t="n">
-        <v>71222</v>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="n">
-        <v>-58636</v>
+        <v>52084</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="n">
+        <v>41</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="14" t="n">
+        <v>-676971</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-677012</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="14" t="n">
         <v>-618376</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="14" t="n">
         <v>-570278</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="14" t="n">
         <v>-576347</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-495521</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23446.6</v>
+        <v>23270.3</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23494.95</v>
+        <v>23448.1</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>127142</v>
+        <v>113630</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>127142</v>
+        <v>113630</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23380.1</v>
+        <v>23231.4</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23477.8</v>
+        <v>23398.1</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23636.65000000001</v>
+        <v>23703.7</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23464.375</v>
+        <v>23378.65</v>
       </c>
     </row>
     <row r="33">
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="C33" s="13" t="n">
-        <v>5395</v>
+        <v>9147</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,15 +2611,15 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>8584</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G33" s="11" t="n">
-        <v>-3189</v>
+        <v>6921</v>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="n">
+        <v>2226</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="14" t="n">
+        <v>-406171</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-408397</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="14" t="n">
         <v>-405208</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="14" t="n">
         <v>-403214</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="14" t="n">
         <v>-418487</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-392428</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23565.8</v>
+        <v>23575.9</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23450.95</v>
+        <v>23359.2</v>
       </c>
     </row>
     <row r="34">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="C34" s="13" t="n">
-        <v>113</v>
+        <v>0</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>539</v>
+        <v>1771</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-426</v>
+        <v>-1771</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="14" t="n">
+        <v>21924</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>23695</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="14" t="n">
         <v>24121</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="14" t="n">
         <v>24927</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="14" t="n">
         <v>26446</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>26601</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23521.8</v>
+        <v>23487</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23437.525</v>
+        <v>23339.75</v>
       </c>
     </row>
     <row r="35">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="C35" s="13" t="n">
-        <v>17675</v>
+        <v>22837</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>3024</v>
+        <v>6471</v>
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
         </is>
       </c>
       <c r="G35" s="13" t="n">
-        <v>14651</v>
+        <v>16366</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="14" t="n">
+        <v>197348</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>180982</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="14" t="n">
         <v>166331</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="14" t="n">
         <v>148077</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="14" t="n">
         <v>137452</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>118169</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23450.95</v>
+        <v>23359.2</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="C36" s="13" t="n">
-        <v>16376</v>
+        <v>33112</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>27412</v>
+        <v>49933</v>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
@@ -2814,7 +2814,7 @@
         </is>
       </c>
       <c r="G36" s="11" t="n">
-        <v>-11036</v>
+        <v>-16821</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="14" t="n">
+        <v>186899</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>203720</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="14" t="n">
         <v>214756</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="14" t="n">
         <v>230210</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="14" t="n">
         <v>254589</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>247658</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23406.95</v>
+        <v>23270.3</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>39559</v>
+        <v>65096</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>39559</v>
+        <v>65096</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23336.1</v>
+        <v>23142.5</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23292.1</v>
+        <v>23053.60000000001</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.8</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.92</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.23</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.16</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>10.68</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9796606494773291</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9829176264436748</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9808503997602754</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9890959913034546</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.994992330910013</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9997263611508541</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,478    PCR(OI) 0.64    Max Pain 23,500</t>
+          <t>Spot 23,398    PCR(OI) 1.06    Max Pain 23,450</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23883.88266129032</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23885.82661290323</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23888.96411290322</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23895.65846774193</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23898.82741935484</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23904.24112903226</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23398.1</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23477.8</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23431.5</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23635.1</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23779.15</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23897.7</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23500</v>
+        <v>23800</v>
       </c>
       <c r="Q45" s="14" t="n">
-        <v>180147</v>
+        <v>178369</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>56011</v>
+        <v>31720</v>
       </c>
       <c r="S45" s="14" t="n">
-        <v>2977798</v>
+        <v>2525667</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9638074198858003</v>
+        <v>0.9605609315602034</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9813887944889631</v>
@@ -3176,13 +3176,13 @@
         <v>24000</v>
       </c>
       <c r="Q46" s="14" t="n">
-        <v>214443</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>33426</v>
+        <v>210284</v>
+      </c>
+      <c r="R46" s="13" t="n">
+        <v>-4159</v>
       </c>
       <c r="S46" s="14" t="n">
-        <v>896853</v>
+        <v>2344476</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24359.43064516129</v>
+        <v>24358.78790322581</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24350.89959677419</v>
@@ -3215,13 +3215,13 @@
         <v>24500</v>
       </c>
       <c r="Q47" s="14" t="n">
-        <v>171767</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>55571</v>
+        <v>155594</v>
+      </c>
+      <c r="R47" s="13" t="n">
+        <v>-16173</v>
       </c>
       <c r="S47" s="14" t="n">
-        <v>848564</v>
+        <v>928032</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23477.8</v>
+        <v>23398.1</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23897.7</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="32" t="inlineStr">
-        <is>
-          <t>10-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="32" t="inlineStr">
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>11-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="32" t="inlineStr">
+      <c r="L49" s="29" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="32" t="inlineStr">
+      <c r="M49" s="29" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="32" t="inlineStr">
+      <c r="N49" s="29" t="inlineStr">
         <is>
           <t>14-Aug-2026</t>
         </is>
@@ -3318,66 +3318,66 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
-        <v>23400</v>
+      <c r="P50" s="32" t="n">
+        <v>23300</v>
       </c>
       <c r="Q50" s="14" t="n">
-        <v>122869</v>
+        <v>212343</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>42587</v>
+        <v>116304</v>
       </c>
       <c r="S50" s="14" t="n">
-        <v>3765046</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
+        <v>7105072</v>
+      </c>
+      <c r="T50" s="33" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="33" t="n">
+      <c r="P51" s="32" t="n">
+        <v>23200</v>
+      </c>
+      <c r="Q51" s="14" t="n">
+        <v>169816</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>56084</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>4813332</v>
+      </c>
+      <c r="T51" s="33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="P52" s="32" t="n">
         <v>23000</v>
       </c>
-      <c r="Q51" s="14" t="n">
-        <v>163298</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>22739</v>
-      </c>
-      <c r="S51" s="14" t="n">
-        <v>914254</v>
-      </c>
-      <c r="T51" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="P52" s="33" t="n">
-        <v>22500</v>
-      </c>
       <c r="Q52" s="14" t="n">
-        <v>124737</v>
+        <v>190141</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>52744</v>
+        <v>26843</v>
       </c>
       <c r="S52" s="14" t="n">
-        <v>411516</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>2775462</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 10-Sep-2026    1 DAY AGO = 09-Sep-2026    2 DAYS AGO = 08-Sep-2026    3 DAYS AGO = 07-Sep-2026    4 DAYS AGO = 04-Sep-2026    (generated 10-Sep-2026 20:31 IST)</t>
+          <t>TODAY = 11-Sep-2026    1 DAY AGO = 10-Sep-2026    2 DAYS AGO = 09-Sep-2026    3 DAYS AGO = 08-Sep-2026    4 DAYS AGO = 07-Sep-2026    (generated 11-Sep-2026 20:41 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-15
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -129,22 +129,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,20 +187,20 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>517</v>
+        <v>7975</v>
       </c>
     </row>
     <row r="3">
@@ -699,13 +699,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="n">
-        <v>-476</v>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>6296</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-993</v>
+        <v>-1679</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,36 +721,36 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>517</v>
+        <v>7975</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>239463</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>231488</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>230971</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>230480</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="12" t="n">
         <v>225638</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>218910</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="13" t="n">
-        <v>-150498</v>
+      <c r="S3" s="11" t="n">
+        <v>205106</v>
       </c>
     </row>
     <row r="4">
@@ -768,58 +768,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>459</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>-503</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="13" t="n">
-        <v>1003</v>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
+      <c r="E4" s="14" t="n">
+        <v>123</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="13" t="n">
-        <v>-544</v>
+      <c r="G4" s="14" t="n">
+        <v>-626</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="12" t="n">
+        <v>13722</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>14348</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="12" t="n">
         <v>14892</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="12" t="n">
         <v>14611</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="12" t="n">
         <v>11272</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>11053</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -827,8 +827,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="13" t="n">
-        <v>61381</v>
+      <c r="S4" s="11" t="n">
+        <v>-34360</v>
       </c>
     </row>
     <row r="5">
@@ -843,52 +843,52 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>1558</v>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
+        <v>5006</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
-        <v>4596</v>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="E5" s="14" t="n">
+        <v>11176</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n">
-        <v>-3038</v>
+      <c r="G5" s="14" t="n">
+        <v>-6170</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="14" t="n">
+      <c r="J5" s="12" t="n">
+        <v>-291052</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-284882</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="12" t="n">
         <v>-281844</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="12" t="n">
         <v>-276250</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="N5" s="12" t="n">
         <v>-261557</v>
       </c>
-      <c r="N5" s="14" t="n">
-        <v>-250093</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -896,8 +896,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>19515</v>
+      <c r="S5" s="14" t="n">
+        <v>-23761</v>
       </c>
     </row>
     <row r="6">
@@ -906,67 +906,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>-128</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>-3193</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>2125</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>3304</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>-1179</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>37867</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>39046</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>35981</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>31159</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>24647</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>3065</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="n">
-        <v>39046</v>
-      </c>
-      <c r="K6" s="14" t="n">
-        <v>35981</v>
-      </c>
-      <c r="L6" s="14" t="n">
-        <v>31159</v>
-      </c>
-      <c r="M6" s="14" t="n">
-        <v>24647</v>
-      </c>
-      <c r="N6" s="14" t="n">
-        <v>20130</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>21452</v>
+        <v>143400</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>1413</v>
+        <v>12924</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>1413</v>
+        <v>12924</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="13" t="n">
-        <v>2226</v>
+      <c r="S7" s="11" t="n">
+        <v>-41310</v>
       </c>
     </row>
     <row r="8">
@@ -1071,7 +1071,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="12" t="inlineStr">
+      <c r="Q8" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="13" t="n">
-        <v>-544</v>
+      <c r="S8" s="14" t="n">
+        <v>-626</v>
       </c>
     </row>
     <row r="9">
@@ -1091,50 +1091,50 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
-        <v>-97628</v>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>52870</v>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G9" s="13" t="n">
-        <v>-150498</v>
+      <c r="C9" s="14" t="n">
+        <v>-1015988</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>-1221094</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>205106</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="14" t="n">
+      <c r="J9" s="12" t="n">
+        <v>434768</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>229662</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="L9" s="12" t="n">
         <v>380160</v>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="M9" s="12" t="n">
         <v>326656</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="N9" s="12" t="n">
         <v>343639</v>
       </c>
-      <c r="N9" s="14" t="n">
-        <v>367520</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>551</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="10">
@@ -1160,13 +1160,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>0</v>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>-300</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>-551</v>
+        <v>-1640</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -1182,36 +1182,36 @@
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>551</v>
+        <v>1340</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="12" t="n">
+        <v>3391</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>2051</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="12" t="n">
         <v>1500</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="12" t="n">
         <v>1434</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="12" t="n">
         <v>3433</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>3650</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="13" t="n">
-        <v>6286</v>
+      <c r="S10" s="11" t="n">
+        <v>-3354</v>
       </c>
     </row>
     <row r="11">
@@ -1229,67 +1229,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="n">
-        <v>46982</v>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>15209</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>-147453</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>-121510</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>-25943</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-313041</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-287098</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-318871</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-342643</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-302082</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>31773</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="14" t="n">
-        <v>-287098</v>
-      </c>
-      <c r="K11" s="14" t="n">
-        <v>-318871</v>
-      </c>
-      <c r="L11" s="14" t="n">
-        <v>-342643</v>
-      </c>
-      <c r="M11" s="14" t="n">
-        <v>-302082</v>
-      </c>
-      <c r="N11" s="14" t="n">
-        <v>-298102</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="13" t="n">
-        <v>-10083</v>
+      <c r="S11" s="11" t="n">
+        <v>42432</v>
       </c>
     </row>
     <row r="12">
@@ -1298,13 +1298,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>50474</v>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>-341182</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
@@ -1312,42 +1312,42 @@
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>-67702</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>118176</v>
+        <v>-160678</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>-180504</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="14" t="n">
+      <c r="J12" s="12" t="n">
+        <v>-125118</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>55386</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="12" t="n">
         <v>-62790</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="M12" s="12" t="n">
         <v>14552</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="12" t="n">
         <v>-44990</v>
       </c>
-      <c r="N12" s="14" t="n">
-        <v>-73068</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="12" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="13" t="n">
-        <v>-7745</v>
+      <c r="S12" s="14" t="n">
+        <v>-9383</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-172</v>
+        <v>-1504923</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-174</v>
+        <v>-1504922</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-1771</v>
+        <v>-766</v>
       </c>
     </row>
     <row r="14">
@@ -1463,7 +1463,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="12" t="inlineStr">
+      <c r="Q14" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="13" t="n">
-        <v>-3038</v>
+      <c r="S14" s="14" t="n">
+        <v>-6170</v>
       </c>
     </row>
     <row r="15">
@@ -1483,58 +1483,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="n">
-        <v>770521</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="n">
-        <v>709140</v>
-      </c>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G15" s="13" t="n">
-        <v>61381</v>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>-1476128</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>-1441768</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>-34360</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="12" t="n">
+        <v>-787481</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-753121</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="12" t="n">
         <v>-814502</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="12" t="n">
         <v>-831678</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="12" t="n">
         <v>-743620</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-889308</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="11" t="n">
-        <v>31773</v>
+      <c r="S15" s="14" t="n">
+        <v>-25943</v>
       </c>
     </row>
     <row r="16">
@@ -1552,13 +1552,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>6286</v>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>-3354</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1568,51 +1568,51 @@
       <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>-3354</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>53470</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>56824</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>50538</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>49673</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>30833</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="13" t="n">
-        <v>6286</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J16" s="14" t="n">
-        <v>56824</v>
-      </c>
-      <c r="K16" s="14" t="n">
-        <v>50538</v>
-      </c>
-      <c r="L16" s="14" t="n">
-        <v>49673</v>
-      </c>
-      <c r="M16" s="14" t="n">
-        <v>30833</v>
-      </c>
-      <c r="N16" s="14" t="n">
-        <v>31094</v>
-      </c>
-      <c r="P16" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q16" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R16" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="13" t="n">
-        <v>6947</v>
+      <c r="S16" s="14" t="n">
+        <v>8809</v>
       </c>
     </row>
     <row r="17">
@@ -1621,56 +1621,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>206875</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="n">
-        <v>199928</v>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>-273239</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>-282048</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
-        <v>6947</v>
+      <c r="G17" s="14" t="n">
+        <v>8809</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="14" t="n">
+      <c r="J17" s="12" t="n">
+        <v>678520</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>669711</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="L17" s="12" t="n">
         <v>662764</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="M17" s="12" t="n">
         <v>660252</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="N17" s="12" t="n">
         <v>650645</v>
       </c>
-      <c r="N17" s="14" t="n">
-        <v>631147</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="12" t="inlineStr">
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1680,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="13" t="n">
-        <v>-22318</v>
+      <c r="S17" s="14" t="n">
+        <v>-19589</v>
       </c>
     </row>
     <row r="18">
@@ -1690,67 +1690,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="n">
-        <v>263134</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>337749</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>-455221</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>-484127</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>28906</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>55491</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>26585</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>101200</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>121753</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>62142</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>-74615</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="14" t="n">
-        <v>26585</v>
-      </c>
-      <c r="K18" s="14" t="n">
-        <v>101200</v>
-      </c>
-      <c r="L18" s="14" t="n">
-        <v>121753</v>
-      </c>
-      <c r="M18" s="14" t="n">
-        <v>62142</v>
-      </c>
-      <c r="N18" s="14" t="n">
-        <v>227067</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="13" t="n">
-        <v>-13748</v>
+      <c r="S18" s="14" t="n">
+        <v>-11127</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>1246816</v>
+        <v>-2207942</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>1246817</v>
+        <v>-2207943</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q19" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="13" t="n">
-        <v>16366</v>
+      <c r="S19" s="11" t="n">
+        <v>-131</v>
       </c>
     </row>
     <row r="20">
@@ -1855,9 +1855,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q20" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>3065</v>
+      <c r="S20" s="14" t="n">
+        <v>-1179</v>
       </c>
     </row>
     <row r="21">
@@ -1875,58 +1875,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="n">
-        <v>18358</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="11" t="n">
-        <v>-1157</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G21" s="11" t="n">
-        <v>19515</v>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>-14100</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>9661</v>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>-23761</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="14" t="n">
+      <c r="J21" s="12" t="n">
+        <v>3241565</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3265326</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="12" t="n">
         <v>3245811</v>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="M21" s="12" t="n">
         <v>3239982</v>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="N21" s="12" t="n">
         <v>3212986</v>
       </c>
-      <c r="N21" s="14" t="n">
-        <v>3218140</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>118176</v>
+      <c r="S21" s="14" t="n">
+        <v>-180504</v>
       </c>
     </row>
     <row r="22">
@@ -1944,58 +1944,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="13" t="n">
-        <v>-2285</v>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="n">
-        <v>7798</v>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G22" s="13" t="n">
-        <v>-10083</v>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>1674</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>-40758</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="n">
+        <v>42432</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="14" t="n">
+      <c r="J22" s="12" t="n">
+        <v>-4249116</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4291548</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4281465</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4305229</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4300824</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-4296590</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>-74615</v>
+      <c r="S22" s="14" t="n">
+        <v>28906</v>
       </c>
     </row>
     <row r="23">
@@ -2013,50 +2013,50 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C23" s="13" t="n">
-        <v>-1298</v>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="n">
-        <v>21020</v>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="C23" s="14" t="n">
+        <v>-22668</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>-3079</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="13" t="n">
-        <v>-22318</v>
+      <c r="G23" s="14" t="n">
+        <v>-19589</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="14" t="n">
+      <c r="J23" s="12" t="n">
+        <v>500013</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>519602</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="L23" s="12" t="n">
         <v>541920</v>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="M23" s="12" t="n">
         <v>564468</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="N23" s="12" t="n">
         <v>591872</v>
       </c>
-      <c r="N23" s="14" t="n">
-        <v>601593</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>12886</v>
+        <v>918</v>
       </c>
     </row>
     <row r="24">
@@ -2088,15 +2088,15 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>19077</v>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
+        <v>3606</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="13" t="n">
-        <v>6191</v>
+      <c r="E24" s="14" t="n">
+        <v>2688</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2104,36 +2104,36 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>12886</v>
+        <v>918</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="14" t="n">
+      <c r="J24" s="12" t="n">
+        <v>507538</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>506620</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="12" t="n">
         <v>493734</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="12" t="n">
         <v>500779</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="12" t="n">
         <v>495966</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>476857</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q24" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="11" t="n">
-        <v>41</v>
+      <c r="S24" s="14" t="n">
+        <v>-122890</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>33852</v>
+        <v>-31488</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>33852</v>
+        <v>-31488</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="11" t="n">
-        <v>-16821</v>
+      <c r="S25" s="14" t="n">
+        <v>42207</v>
       </c>
     </row>
     <row r="26">
@@ -2255,15 +2255,15 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>48581</v>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="n">
-        <v>27129</v>
+        <v>142131</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>-1269</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,27 +2271,27 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>21452</v>
+        <v>143400</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>1432784</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1289384</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>1267932</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>1184645</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="12" t="n">
         <v>1115415</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>1094613</v>
       </c>
     </row>
     <row r="28">
@@ -2306,43 +2306,43 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
+        <v>84</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="13" t="n">
-        <v>7745</v>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>9467</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="13" t="n">
-        <v>-7745</v>
+      <c r="G28" s="14" t="n">
+        <v>-9383</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-388889</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-379506</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-371761</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-358978</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="12" t="n">
         <v>-351069</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-334069</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,47 +2365,47 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>12924</v>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
+        <v>16116</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="13" t="n">
-        <v>26672</v>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
+      <c r="E29" s="14" t="n">
+        <v>27243</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="13" t="n">
-        <v>-13748</v>
+      <c r="G29" s="14" t="n">
+        <v>-11127</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-244034</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-232907</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-219159</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-207291</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="12" t="n">
         <v>-194068</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-184197</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 11-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 15-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,51 +2424,51 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>52125</v>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
+        <v>11787</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="13" t="n">
-        <v>52084</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G30" s="11" t="n">
-        <v>41</v>
+      <c r="E30" s="14" t="n">
+        <v>134677</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>-122890</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-799861</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-676971</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-677012</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-618376</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="12" t="n">
         <v>-570278</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-576347</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23270.3</v>
+        <v>23576.15</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23448.1</v>
+        <v>23592.85</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>113630</v>
+        <v>170118</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>113630</v>
+        <v>170118</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23231.4</v>
+        <v>23118.6</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23398.1</v>
+        <v>23118.6</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23703.7</v>
+        <v>23909.01666666666</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23378.65</v>
+        <v>23197.64166666666</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2597,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v>9147</v>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>-37953</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,43 +2611,43 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>6921</v>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G33" s="13" t="n">
-        <v>2226</v>
+        <v>3357</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>-41310</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="14" t="n">
+      <c r="J33" s="12" t="n">
+        <v>-447481</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-406171</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="12" t="n">
         <v>-408397</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="12" t="n">
         <v>-405208</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="12" t="n">
         <v>-403214</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-418487</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23575.9</v>
+        <v>23750.93333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23359.2</v>
+        <v>23276.68333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2664,13 +2664,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C34" s="13" t="n">
-        <v>0</v>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>-98</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>1771</v>
+        <v>668</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,35 +2686,35 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-1771</v>
+        <v>-766</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="14" t="n">
+      <c r="J34" s="12" t="n">
+        <v>21158</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>21924</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="12" t="n">
         <v>23695</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="12" t="n">
         <v>24121</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="12" t="n">
         <v>24927</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>26446</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23487</v>
+        <v>23434.76666666666</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23339.75</v>
+        <v>23355.725</v>
       </c>
     </row>
     <row r="35">
@@ -2731,13 +2731,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="13" t="n">
-        <v>22837</v>
+      <c r="C35" s="14" t="n">
+        <v>16003</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,43 +2745,43 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>6471</v>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G35" s="13" t="n">
-        <v>16366</v>
+        <v>16134</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="n">
+        <v>-131</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="14" t="n">
+      <c r="J35" s="12" t="n">
+        <v>197217</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>197348</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="12" t="n">
         <v>180982</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="12" t="n">
         <v>166331</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="12" t="n">
         <v>148077</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>137452</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23359.2</v>
+        <v>23276.68333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,57 +2792,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="13" t="n">
-        <v>33112</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E36" s="11" t="n">
-        <v>49933</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="n">
-        <v>-16821</v>
+      <c r="C36" s="14" t="n">
+        <v>38739</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>-3468</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>42207</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="14" t="n">
+      <c r="J36" s="12" t="n">
+        <v>229106</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>186899</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="12" t="n">
         <v>203720</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="12" t="n">
         <v>214756</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="12" t="n">
         <v>230210</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>254589</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23270.3</v>
+        <v>22960.51666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>65096</v>
+        <v>16691</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>65096</v>
+        <v>16691</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23142.5</v>
+        <v>22802.43333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23053.60000000001</v>
+        <v>22486.26666666666</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>13.43</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>12.29</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.8</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.92</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.23</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.16</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9679688193651542</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9796606494773291</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9829176264436748</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9808503997602754</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9890959913034546</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.994992330910013</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,398    PCR(OI) 1.06    Max Pain 23,450</t>
+          <t>Spot 23,119    PCR(OI) 0.53    Max Pain 23,150</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23883.62056451613</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23883.88266129032</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23885.82661290323</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23888.96411290322</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23895.65846774193</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23898.82741935484</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23118.6</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23398.1</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23477.8</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23431.5</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23635.1</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23779.15</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23800</v>
-      </c>
-      <c r="Q45" s="14" t="n">
-        <v>178369</v>
+        <v>23150</v>
+      </c>
+      <c r="Q45" s="12" t="n">
+        <v>274958</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>31720</v>
-      </c>
-      <c r="S45" s="14" t="n">
-        <v>2525667</v>
+        <v>270833</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>4555174</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3158,35 +3158,35 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
+        <v>0.9488847137436824</v>
+      </c>
+      <c r="K46" s="25" t="n">
         <v>0.9605609315602034</v>
       </c>
-      <c r="K46" s="25" t="n">
+      <c r="L46" s="25" t="n">
         <v>0.9813887944889631</v>
       </c>
-      <c r="L46" s="25" t="n">
+      <c r="M46" s="25" t="n">
         <v>0.9933791141865997</v>
       </c>
-      <c r="M46" s="25" t="n">
+      <c r="N46" s="25" t="n">
         <v>0.9970635633790684</v>
       </c>
-      <c r="N46" s="25" t="n">
-        <v>1.002328084679025</v>
-      </c>
       <c r="P46" s="28" t="n">
-        <v>24000</v>
-      </c>
-      <c r="Q46" s="14" t="n">
-        <v>210284</v>
-      </c>
-      <c r="R46" s="13" t="n">
-        <v>-4159</v>
-      </c>
-      <c r="S46" s="14" t="n">
-        <v>2344476</v>
+        <v>23200</v>
+      </c>
+      <c r="Q46" s="12" t="n">
+        <v>254941</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>237074</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>10750950</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3197,35 +3197,35 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
+        <v>24363.97137096774</v>
+      </c>
+      <c r="K47" s="18" t="n">
         <v>24358.78790322581</v>
       </c>
-      <c r="K47" s="18" t="n">
+      <c r="L47" s="18" t="n">
         <v>24350.89959677419</v>
       </c>
-      <c r="L47" s="18" t="n">
+      <c r="M47" s="18" t="n">
         <v>24336.7810483871</v>
       </c>
-      <c r="M47" s="18" t="n">
+      <c r="N47" s="18" t="n">
         <v>24323.42419354839</v>
       </c>
-      <c r="N47" s="18" t="n">
-        <v>24309.40564516129</v>
-      </c>
       <c r="P47" s="28" t="n">
-        <v>24500</v>
-      </c>
-      <c r="Q47" s="14" t="n">
-        <v>155594</v>
-      </c>
-      <c r="R47" s="13" t="n">
-        <v>-16173</v>
-      </c>
-      <c r="S47" s="14" t="n">
-        <v>928032</v>
+        <v>23300</v>
+      </c>
+      <c r="Q47" s="12" t="n">
+        <v>292877</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>250153</v>
+      </c>
+      <c r="S47" s="12" t="n">
+        <v>15330890</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3236,19 +3236,19 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
+        <v>23118.6</v>
+      </c>
+      <c r="K48" s="18" t="n">
         <v>23398.1</v>
       </c>
-      <c r="K48" s="18" t="n">
+      <c r="L48" s="18" t="n">
         <v>23897.7</v>
       </c>
-      <c r="L48" s="18" t="n">
+      <c r="M48" s="18" t="n">
         <v>24175.65</v>
       </c>
-      <c r="M48" s="18" t="n">
+      <c r="N48" s="18" t="n">
         <v>24252</v>
-      </c>
-      <c r="N48" s="18" t="n">
-        <v>24366</v>
       </c>
       <c r="P48" s="31" t="inlineStr">
         <is>
@@ -3266,31 +3266,31 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="29" t="inlineStr">
+      <c r="J49" s="32" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="32" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="K49" s="29" t="inlineStr">
+      <c r="L49" s="32" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="29" t="inlineStr">
+      <c r="M49" s="32" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="29" t="inlineStr">
+      <c r="N49" s="32" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="29" t="inlineStr">
-        <is>
-          <t>14-Aug-2026</t>
-        </is>
-      </c>
       <c r="P49" s="27" t="inlineStr">
         <is>
           <t>Strike</t>
@@ -3318,57 +3318,57 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
-        <v>23300</v>
-      </c>
-      <c r="Q50" s="14" t="n">
-        <v>212343</v>
+      <c r="P50" s="33" t="n">
+        <v>23100</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>309516</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>116304</v>
-      </c>
-      <c r="S50" s="14" t="n">
-        <v>7105072</v>
-      </c>
-      <c r="T50" s="33" t="inlineStr">
+        <v>188011</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>15388724</v>
+      </c>
+      <c r="T50" s="30" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="32" t="n">
-        <v>23200</v>
-      </c>
-      <c r="Q51" s="14" t="n">
-        <v>169816</v>
+      <c r="P51" s="33" t="n">
+        <v>23050</v>
+      </c>
+      <c r="Q51" s="12" t="n">
+        <v>143060</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>56084</v>
-      </c>
-      <c r="S51" s="14" t="n">
-        <v>4813332</v>
-      </c>
-      <c r="T51" s="33" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>93626</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>8190938</v>
+      </c>
+      <c r="T51" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
+      <c r="P52" s="33" t="n">
         <v>23000</v>
       </c>
-      <c r="Q52" s="14" t="n">
-        <v>190141</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>26843</v>
-      </c>
-      <c r="S52" s="14" t="n">
-        <v>2775462</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
+      <c r="Q52" s="12" t="n">
+        <v>162136</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>-28005</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>8672206</v>
+      </c>
+      <c r="T52" s="32" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 11-Sep-2026    1 DAY AGO = 10-Sep-2026    2 DAYS AGO = 09-Sep-2026    3 DAYS AGO = 08-Sep-2026    4 DAYS AGO = 07-Sep-2026    (generated 11-Sep-2026 20:41 IST)</t>
+          <t>TODAY = 15-Sep-2026    1 DAY AGO = 11-Sep-2026    2 DAYS AGO = 10-Sep-2026    3 DAYS AGO = 09-Sep-2026    4 DAYS AGO = 08-Sep-2026    (generated 15-Sep-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-16
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -187,20 +187,20 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>7975</v>
+        <v>-6161</v>
       </c>
     </row>
     <row r="3">
@@ -701,27 +701,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>6296</v>
+        <v>-2713</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-1679</v>
+        <v>3448</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>7975</v>
+        <v>-6161</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>233302</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>239463</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>231488</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>230971</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>230480</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>225638</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>205106</v>
+        <v>-136438</v>
       </c>
     </row>
     <row r="4">
@@ -768,29 +768,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
-        <v>-503</v>
+      <c r="C4" s="11" t="n">
+        <v>-2683</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>123</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+        <v>-1507</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>-626</v>
+      <c r="G4" s="11" t="n">
+        <v>-1176</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,20 +798,20 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>12546</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>13722</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>14348</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>14892</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>14611</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>11272</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -819,7 +819,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-34360</v>
+        <v>176847</v>
       </c>
     </row>
     <row r="5">
@@ -837,67 +837,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="11" t="n">
-        <v>5006</v>
+      <c r="C5" s="14" t="n">
+        <v>1188</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>11176</v>
+        <v>-1761</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>2949</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-288103</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-291052</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-284882</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-281844</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-276250</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-6170</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-291052</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-284882</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-281844</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-276250</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-261557</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="14" t="n">
-        <v>-23761</v>
+      <c r="S5" s="11" t="n">
+        <v>-24561</v>
       </c>
     </row>
     <row r="6">
@@ -906,67 +906,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>2125</v>
+      <c r="C6" s="14" t="n">
+        <v>3464</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>3304</v>
+        <v>-924</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>4388</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>42255</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>37867</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>39046</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>35981</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>31159</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>-1179</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>37867</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>39046</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>35981</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>31159</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>24647</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>143400</v>
+        <v>-9669</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>12924</v>
+        <v>-744</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>12924</v>
+        <v>-744</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-41310</v>
+        <v>52106</v>
       </c>
     </row>
     <row r="8">
@@ -1071,7 +1071,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
+      <c r="Q8" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>-626</v>
+      <c r="S8" s="11" t="n">
+        <v>-1176</v>
       </c>
     </row>
     <row r="9">
@@ -1093,65 +1093,65 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>-1015988</v>
+        <v>179500</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>-1221094</v>
+        <v>315938</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>-136438</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>298330</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>434768</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>229662</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>380160</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>326656</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>205106</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>434768</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>229662</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>380160</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>326656</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>343639</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>1340</v>
+      <c r="S9" s="14" t="n">
+        <v>185</v>
       </c>
     </row>
     <row r="10">
@@ -1162,27 +1162,27 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>-300</v>
+        <v>438</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>-1640</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+        <v>253</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>1340</v>
+      <c r="G10" s="14" t="n">
+        <v>185</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,26 +1190,26 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>3576</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>3391</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>2051</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>1500</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>1434</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>3433</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>-3354</v>
+      <c r="S10" s="14" t="n">
+        <v>-3145</v>
       </c>
     </row>
     <row r="11">
@@ -1231,65 +1231,65 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>-147453</v>
+        <v>70614</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>-121510</v>
+        <v>45779</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>24835</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-288206</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-313041</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-287098</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-318871</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-342643</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-25943</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-313041</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-287098</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-318871</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-342643</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-302082</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S11" s="11" t="n">
-        <v>42432</v>
+        <v>-3488</v>
       </c>
     </row>
     <row r="12">
@@ -1300,65 +1300,65 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>-341182</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
+        <v>90302</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E12" s="11" t="n">
-        <v>-160678</v>
+      <c r="E12" s="14" t="n">
+        <v>-21115</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>111417</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>-13701</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>-125118</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>55386</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>-62790</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>14552</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-180504</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>-125118</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>55386</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>-62790</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>14552</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>-44990</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>-9383</v>
+      <c r="S12" s="11" t="n">
+        <v>-7951</v>
       </c>
     </row>
     <row r="13">
@@ -1369,11 +1369,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-1504923</v>
+        <v>340854</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-1504922</v>
+        <v>340855</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>-766</v>
+      <c r="S13" s="14" t="n">
+        <v>-151</v>
       </c>
     </row>
     <row r="14">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-6170</v>
+        <v>2949</v>
       </c>
     </row>
     <row r="15">
@@ -1485,27 +1485,27 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>-1476128</v>
+        <v>609670</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E15" s="14" t="n">
-        <v>-1441768</v>
+        <v>432823</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-34360</v>
+        <v>176847</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-610634</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-787481</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-753121</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-814502</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-831678</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-743620</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>-25943</v>
+        <v>24835</v>
       </c>
     </row>
     <row r="16">
@@ -1552,29 +1552,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>-3354</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="C16" s="14" t="n">
+        <v>-3145</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>-3354</v>
+      <c r="G16" s="14" t="n">
+        <v>-3145</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>50325</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>53470</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>56824</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>50538</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>49673</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>30833</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>8809</v>
+        <v>-98358</v>
       </c>
     </row>
     <row r="17">
@@ -1623,65 +1623,65 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>-273239</v>
+        <v>78162</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E17" s="14" t="n">
-        <v>-282048</v>
+        <v>176520</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>-98358</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>580162</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>678520</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>669711</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>662764</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>660252</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>8809</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>678520</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>669711</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>662764</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>660252</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>650645</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S17" s="14" t="n">
-        <v>-19589</v>
+        <v>36064</v>
       </c>
     </row>
     <row r="18">
@@ -1692,27 +1692,27 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>-455221</v>
+        <v>133723</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>-484127</v>
+        <v>209068</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G18" s="14" t="n">
-        <v>28906</v>
+        <v>-75345</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,26 +1720,26 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>-19854</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>55491</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>26585</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>101200</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>121753</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>62142</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="13" t="inlineStr">
+      <c r="Q18" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>-11127</v>
+      <c r="S18" s="11" t="n">
+        <v>-11003</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-2207942</v>
+        <v>818410</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-2207943</v>
+        <v>818411</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Q19" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="11" t="n">
-        <v>-131</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="20">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="14" t="n">
-        <v>-1179</v>
+        <v>4388</v>
       </c>
     </row>
     <row r="21">
@@ -1875,29 +1875,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n">
-        <v>-14100</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="C21" s="11" t="n">
+        <v>-19563</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
-        <v>9661</v>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
+      <c r="E21" s="11" t="n">
+        <v>4998</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="14" t="n">
-        <v>-23761</v>
+      <c r="G21" s="11" t="n">
+        <v>-24561</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,20 +1905,20 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3217004</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3241565</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3265326</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3245811</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>3239982</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3212986</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="Q21" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>-180504</v>
+        <v>111417</v>
       </c>
     </row>
     <row r="22">
@@ -1944,29 +1944,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
-        <v>1674</v>
+      <c r="C22" s="14" t="n">
+        <v>6646</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>-40758</v>
+        <v>10134</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G22" s="11" t="n">
-        <v>42432</v>
+        <v>-3488</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4252604</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4249116</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4291548</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4281465</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4305229</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4300824</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>28906</v>
+        <v>-75345</v>
       </c>
     </row>
     <row r="23">
@@ -2015,65 +2015,65 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>-22668</v>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+        <v>22564</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E23" s="11" t="n">
-        <v>-3079</v>
+      <c r="E23" s="14" t="n">
+        <v>-13500</v>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>36064</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>536077</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>500013</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>519602</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>541920</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>564468</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>-19589</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>500013</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>519602</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>541920</v>
-      </c>
-      <c r="M23" s="12" t="n">
-        <v>564468</v>
-      </c>
-      <c r="N23" s="12" t="n">
-        <v>591872</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>918</v>
+        <v>-8015</v>
       </c>
     </row>
     <row r="24">
@@ -2084,65 +2084,65 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>3606</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+        <v>-1232</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>2688</v>
+      <c r="E24" s="11" t="n">
+        <v>6783</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>-8015</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="n">
+        <v>499523</v>
+      </c>
+      <c r="K24" s="12" t="n">
+        <v>507538</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>506620</v>
+      </c>
+      <c r="M24" s="12" t="n">
+        <v>493734</v>
+      </c>
+      <c r="N24" s="12" t="n">
+        <v>500779</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q24" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>918</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="12" t="n">
-        <v>507538</v>
-      </c>
-      <c r="K24" s="12" t="n">
-        <v>506620</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>493734</v>
-      </c>
-      <c r="M24" s="12" t="n">
-        <v>500779</v>
-      </c>
-      <c r="N24" s="12" t="n">
-        <v>495966</v>
-      </c>
-      <c r="P24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-122890</v>
+        <v>28623</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-31488</v>
+        <v>8415</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-31488</v>
+        <v>8415</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>42207</v>
+        <v>-54193</v>
       </c>
     </row>
     <row r="26">
@@ -2249,29 +2249,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C27" s="11" t="n">
-        <v>142131</v>
+      <c r="C27" s="14" t="n">
+        <v>18426</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E27" s="11" t="n">
-        <v>-1269</v>
+        <v>28095</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>143400</v>
+        <v>-9669</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1423115</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1432784</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1289384</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1267932</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1184645</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1115415</v>
       </c>
     </row>
     <row r="28">
@@ -2302,27 +2302,27 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>84</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+        <v>-4</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="14" t="n">
-        <v>9467</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="E28" s="11" t="n">
+        <v>7947</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>-9383</v>
+      <c r="G28" s="11" t="n">
+        <v>-7951</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-396840</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-388889</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-379506</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-371761</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-358978</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-351069</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
-        <v>16116</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="n">
+        <v>10105</v>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>27243</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
+      <c r="E29" s="11" t="n">
+        <v>21108</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>-11127</v>
+      <c r="G29" s="11" t="n">
+        <v>-11003</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-255037</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-244034</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-232907</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-219159</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-207291</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-194068</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 15-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 16-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,29 +2418,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
-        <v>11787</v>
+      <c r="C30" s="14" t="n">
+        <v>28408</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>134677</v>
+        <v>-215</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-122890</v>
+        <v>28623</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-771238</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-799861</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-676971</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-677012</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-618376</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-570278</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23576.15</v>
+        <v>23201.6</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23592.85</v>
+        <v>23284.75</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>170118</v>
+        <v>56935</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>170118</v>
+        <v>56935</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23118.6</v>
+        <v>23116.1</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23118.6</v>
+        <v>23217.6</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23909.01666666666</v>
+        <v>23464.85</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23197.64166666666</v>
+        <v>23211.875</v>
       </c>
     </row>
     <row r="33">
@@ -2599,27 +2599,27 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>-37953</v>
+        <v>50458</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>3357</v>
+        <v>-1648</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-41310</v>
+        <v>52106</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-395375</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-447481</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-406171</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-408397</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-405208</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-403214</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23750.93333333333</v>
+        <v>23374.8</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23276.68333333333</v>
+        <v>23206.15</v>
       </c>
     </row>
     <row r="34">
@@ -2666,27 +2666,27 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>-98</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
+        <v>734</v>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="11" t="n">
-        <v>668</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="E34" s="14" t="n">
+        <v>885</v>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="11" t="n">
-        <v>-766</v>
+      <c r="G34" s="14" t="n">
+        <v>-151</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>21007</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>21158</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>21924</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>23695</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>24121</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>24927</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23434.76666666666</v>
+        <v>23296.2</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23355.725</v>
+        <v>23200.425</v>
       </c>
     </row>
     <row r="35">
@@ -2731,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>16003</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="C35" s="11" t="n">
+        <v>14031</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="11" t="n">
-        <v>16134</v>
+      <c r="E35" s="14" t="n">
+        <v>11793</v>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G35" s="11" t="n">
-        <v>-131</v>
+        <v>2238</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>199455</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>197217</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>197348</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>180982</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>166331</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>148077</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23276.68333333333</v>
+        <v>23206.15</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,27 +2794,27 @@
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>38739</v>
+        <v>-2852</v>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E36" s="14" t="n">
-        <v>-3468</v>
+        <v>51341</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>42207</v>
+        <v>-54193</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>174913</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>229106</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>186899</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>203720</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>214756</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>230210</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22960.51666666666</v>
+        <v>23127.55</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>16691</v>
+        <v>62371</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>16691</v>
+        <v>62371</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22802.43333333333</v>
+        <v>23037.5</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22486.26666666666</v>
+        <v>22958.89999999999</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>13.17</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>13.43</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>12.29</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.8</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.92</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.23</v>
       </c>
     </row>
     <row r="41">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 15-Sep-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 22-Sep-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9721766836399037</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9679688193651542</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9796606494773291</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9829176264436748</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9808503997602754</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9890959913034546</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,119    PCR(OI) 0.53    Max Pain 23,150</t>
+          <t>Spot 23,218    PCR(OI) 0.94    Max Pain 23,300</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23882.07862903226</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23883.62056451613</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23883.88266129032</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23885.82661290323</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23888.96411290322</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23895.65846774193</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23217.6</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23118.6</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23398.1</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23477.8</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23431.5</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23635.1</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23150</v>
+        <v>23500</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>274958</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>270833</v>
+        <v>115909</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>25954</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>4555174</v>
+        <v>1720743</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9488847137436824</v>
+        <v>0.9529168644130193</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9605609315602034</v>
@@ -3173,20 +3173,20 @@
         <v>0.9970635633790684</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23200</v>
+        <v>23800</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>254941</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>237074</v>
+        <v>96789</v>
+      </c>
+      <c r="R46" s="14" t="n">
+        <v>32700</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>10750950</v>
+        <v>787772</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24363.97137096774</v>
+        <v>24364.76975806452</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24358.78790322581</v>
@@ -3212,20 +3212,20 @@
         <v>24323.42419354839</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>23300</v>
+        <v>24000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>292877</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>250153</v>
+        <v>133191</v>
+      </c>
+      <c r="R47" s="14" t="n">
+        <v>27501</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>15330890</v>
+        <v>694739</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23118.6</v>
+        <v>23217.6</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23398.1</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="32" t="inlineStr">
-        <is>
-          <t>15-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="32" t="inlineStr">
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="32" t="inlineStr">
+      <c r="L49" s="29" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="32" t="inlineStr">
+      <c r="M49" s="29" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="32" t="inlineStr">
+      <c r="N49" s="29" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
@@ -3318,66 +3318,66 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
-        <v>23100</v>
+      <c r="P50" s="32" t="n">
+        <v>23200</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>309516</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>188011</v>
+        <v>114879</v>
+      </c>
+      <c r="R50" s="14" t="n">
+        <v>44834</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>15388724</v>
-      </c>
-      <c r="T50" s="30" t="inlineStr">
+        <v>3561470</v>
+      </c>
+      <c r="T50" s="33" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="33" t="n">
-        <v>23050</v>
+      <c r="P51" s="32" t="n">
+        <v>23000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>143060</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>93626</v>
+        <v>125115</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>52075</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>8190938</v>
-      </c>
-      <c r="T51" s="32" t="inlineStr">
+        <v>1943321</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="33" t="n">
-        <v>23000</v>
+      <c r="P52" s="32" t="n">
+        <v>22500</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>162136</v>
+        <v>102560</v>
       </c>
       <c r="R52" s="14" t="n">
-        <v>-28005</v>
+        <v>32165</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>8672206</v>
-      </c>
-      <c r="T52" s="32" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>649345</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 15-Sep-2026    1 DAY AGO = 11-Sep-2026    2 DAYS AGO = 10-Sep-2026    3 DAYS AGO = 09-Sep-2026    4 DAYS AGO = 08-Sep-2026    (generated 15-Sep-2026 20:32 IST)</t>
+          <t>TODAY = 16-Sep-2026    1 DAY AGO = 15-Sep-2026    2 DAYS AGO = 11-Sep-2026    3 DAYS AGO = 10-Sep-2026    4 DAYS AGO = 09-Sep-2026    (generated 16-Sep-2026 20:40 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-17
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -187,7 +187,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,11 +196,11 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-6161</v>
+        <v>5646</v>
       </c>
     </row>
     <row r="3">
@@ -701,65 +701,65 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-2713</v>
+        <v>5180</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>3448</v>
+        <v>-466</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>5646</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J3" s="12" t="n">
+        <v>238948</v>
+      </c>
+      <c r="K3" s="12" t="n">
+        <v>233302</v>
+      </c>
+      <c r="L3" s="12" t="n">
+        <v>239463</v>
+      </c>
+      <c r="M3" s="12" t="n">
+        <v>231488</v>
+      </c>
+      <c r="N3" s="12" t="n">
+        <v>230971</v>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G3" s="11" t="n">
-        <v>-6161</v>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n">
-        <v>233302</v>
-      </c>
-      <c r="K3" s="12" t="n">
-        <v>239463</v>
-      </c>
-      <c r="L3" s="12" t="n">
-        <v>231488</v>
-      </c>
-      <c r="M3" s="12" t="n">
-        <v>230971</v>
-      </c>
-      <c r="N3" s="12" t="n">
-        <v>230480</v>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>-136438</v>
+      <c r="S3" s="14" t="n">
+        <v>-7932</v>
       </c>
     </row>
     <row r="4">
@@ -770,65 +770,65 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>-2683</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+        <v>65</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E4" s="14" t="n">
-        <v>-1507</v>
+      <c r="E4" s="11" t="n">
+        <v>-247</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>312</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>12858</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>12546</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>13722</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>14348</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>14892</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>-1176</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>12546</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>13722</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>14348</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>14892</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>14611</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>176847</v>
+        <v>-101544</v>
       </c>
     </row>
     <row r="5">
@@ -837,67 +837,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
-        <v>1188</v>
+      <c r="C5" s="11" t="n">
+        <v>102</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>-1761</v>
+        <v>2040</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>-1938</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-290041</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-288103</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-291052</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-284882</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-281844</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>2949</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-288103</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-291052</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-284882</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-281844</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-276250</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>-24561</v>
+        <v>11278</v>
       </c>
     </row>
     <row r="6">
@@ -908,27 +908,27 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>3464</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
+        <v>-4025</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E6" s="14" t="n">
-        <v>-924</v>
+      <c r="E6" s="11" t="n">
+        <v>-5</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G6" s="14" t="n">
-        <v>4388</v>
+        <v>-4020</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,26 +936,26 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>38235</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>42255</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>37867</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>39046</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>35981</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>31159</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="9" t="inlineStr">
+      <c r="Q6" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -965,8 +965,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="11" t="n">
-        <v>-9669</v>
+      <c r="S6" s="14" t="n">
+        <v>-53770</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-744</v>
+        <v>1322</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-744</v>
+        <v>1322</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,7 +1002,7 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
+      <c r="Q7" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>52106</v>
+      <c r="S7" s="14" t="n">
+        <v>2734</v>
       </c>
     </row>
     <row r="8">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>-1176</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9">
@@ -1091,29 +1091,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
-        <v>179500</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="C9" s="11" t="n">
+        <v>382191</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="11" t="n">
-        <v>315938</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="E9" s="14" t="n">
+        <v>390123</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>-136438</v>
+      <c r="G9" s="14" t="n">
+        <v>-7932</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,26 +1121,26 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>290398</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>298330</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>434768</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>229662</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>380160</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>326656</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>185</v>
+      <c r="S9" s="11" t="n">
+        <v>673</v>
       </c>
     </row>
     <row r="10">
@@ -1160,29 +1160,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>438</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="C10" s="11" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n">
-        <v>253</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="E10" s="14" t="n">
+        <v>727</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>185</v>
+      <c r="G10" s="11" t="n">
+        <v>673</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,20 +1190,20 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>4249</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>3576</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>3391</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>2051</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>1500</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>1434</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="S10" s="14" t="n">
-        <v>-3145</v>
+        <v>4510</v>
       </c>
     </row>
     <row r="11">
@@ -1229,29 +1229,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
-        <v>70614</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="C11" s="11" t="n">
+        <v>46872</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E11" s="11" t="n">
-        <v>45779</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="E11" s="14" t="n">
+        <v>41558</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>24835</v>
+      <c r="G11" s="11" t="n">
+        <v>5314</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,26 +1259,26 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-282892</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-288206</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-313041</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-287098</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-318871</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-342643</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>-3488</v>
+      <c r="S11" s="14" t="n">
+        <v>-764</v>
       </c>
     </row>
     <row r="12">
@@ -1298,29 +1298,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n">
-        <v>90302</v>
+      <c r="C12" s="11" t="n">
+        <v>138191</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>-21115</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+        <v>136245</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>111417</v>
+      <c r="G12" s="11" t="n">
+        <v>1946</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,26 +1328,26 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>-11755</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>-13701</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>-125118</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>55386</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>-62790</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>14552</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>-7951</v>
+      <c r="S12" s="14" t="n">
+        <v>-2622</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>340854</v>
+        <v>568654</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>340855</v>
+        <v>568653</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="14" t="n">
-        <v>-151</v>
+        <v>424</v>
       </c>
     </row>
     <row r="14">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>2949</v>
+        <v>-1938</v>
       </c>
     </row>
     <row r="15">
@@ -1483,67 +1483,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
-        <v>609670</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="C15" s="14" t="n">
+        <v>417682</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="14" t="n">
-        <v>432823</v>
+      <c r="E15" s="11" t="n">
+        <v>519226</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>-101544</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>-712178</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>-610634</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>-787481</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>-753121</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>-814502</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>176847</v>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>-610634</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>-787481</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>-753121</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>-814502</v>
-      </c>
-      <c r="N15" s="12" t="n">
-        <v>-831678</v>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>24835</v>
+      <c r="S15" s="11" t="n">
+        <v>5314</v>
       </c>
     </row>
     <row r="16">
@@ -1554,27 +1554,27 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>-3145</v>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
+        <v>4560</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="14" t="n">
-        <v>0</v>
+      <c r="E16" s="11" t="n">
+        <v>50</v>
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-3145</v>
+        <v>4510</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>54835</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>50325</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>53470</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>56824</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>50538</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>49673</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>-98358</v>
+        <v>32548</v>
       </c>
     </row>
     <row r="17">
@@ -1621,29 +1621,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
-        <v>78162</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="C17" s="14" t="n">
+        <v>50103</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="14" t="n">
-        <v>176520</v>
+      <c r="E17" s="11" t="n">
+        <v>17555</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-98358</v>
+        <v>32548</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,26 +1651,26 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>612710</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>580162</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>678520</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>669711</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>662764</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>660252</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1680,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>36064</v>
+      <c r="S17" s="11" t="n">
+        <v>3488</v>
       </c>
     </row>
     <row r="18">
@@ -1690,67 +1690,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n">
-        <v>133723</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="C18" s="14" t="n">
+        <v>163101</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="14" t="n">
-        <v>209068</v>
+      <c r="E18" s="11" t="n">
+        <v>98614</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>64487</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>44633</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>-19854</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>55491</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>26585</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>101200</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>-75345</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>-19854</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>55491</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>26585</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>101200</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>121753</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="11" t="n">
-        <v>-11003</v>
+      <c r="S18" s="14" t="n">
+        <v>-8071</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>818410</v>
+        <v>635446</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>818411</v>
+        <v>635445</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Q19" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="11" t="n">
-        <v>2238</v>
+        <v>-4581</v>
       </c>
     </row>
     <row r="20">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="14" t="n">
-        <v>4388</v>
+        <v>-4020</v>
       </c>
     </row>
     <row r="21">
@@ -1877,27 +1877,27 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-19563</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
+        <v>11293</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>4998</v>
+      <c r="E21" s="14" t="n">
+        <v>15</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>-24561</v>
+        <v>11278</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,26 +1905,26 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3228282</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3217004</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3241565</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3265326</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>3245811</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3239982</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
+      <c r="Q21" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>111417</v>
+      <c r="S21" s="11" t="n">
+        <v>1946</v>
       </c>
     </row>
     <row r="22">
@@ -1944,29 +1944,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n">
-        <v>6646</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="C22" s="11" t="n">
+        <v>4012</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="11" t="n">
-        <v>10134</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="E22" s="14" t="n">
+        <v>4776</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>-3488</v>
+      <c r="G22" s="14" t="n">
+        <v>-764</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4253368</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4252604</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4249116</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4291548</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4281465</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4305229</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>-75345</v>
+        <v>64487</v>
       </c>
     </row>
     <row r="23">
@@ -2013,29 +2013,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n">
-        <v>22564</v>
+      <c r="C23" s="11" t="n">
+        <v>14534</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>-13500</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
+        <v>11046</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>36064</v>
+      <c r="G23" s="11" t="n">
+        <v>3488</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,26 +2043,26 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>539565</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>536077</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>500013</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>519602</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>541920</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>564468</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>-8015</v>
+      <c r="S23" s="14" t="n">
+        <v>-14002</v>
       </c>
     </row>
     <row r="24">
@@ -2082,29 +2082,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C24" s="11" t="n">
-        <v>-1232</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="C24" s="14" t="n">
+        <v>-3876</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>6783</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="E24" s="14" t="n">
+        <v>10126</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>-8015</v>
+      <c r="G24" s="14" t="n">
+        <v>-14002</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,26 +2112,26 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>485521</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>499523</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>507538</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>506620</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>493734</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>500779</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
+      <c r="Q24" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>28623</v>
+      <c r="S24" s="11" t="n">
+        <v>64463</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>8415</v>
+        <v>25963</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>8415</v>
+        <v>25963</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>-54193</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="26">
@@ -2251,27 +2251,27 @@
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C27" s="14" t="n">
-        <v>18426</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+        <v>-10131</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>28095</v>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="E27" s="14" t="n">
+        <v>43639</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G27" s="11" t="n">
-        <v>-9669</v>
+      <c r="G27" s="14" t="n">
+        <v>-53770</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1369345</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1423115</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1432784</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1289384</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1267932</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1184645</v>
       </c>
     </row>
     <row r="28">
@@ -2302,27 +2302,27 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>-4</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>7947</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>2622</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>-7951</v>
+      <c r="G28" s="14" t="n">
+        <v>-2622</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-399462</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-396840</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-388889</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-379506</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-371761</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-358978</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>10105</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>7943</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
-        <v>21108</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="E29" s="14" t="n">
+        <v>16014</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="11" t="n">
-        <v>-11003</v>
+      <c r="G29" s="14" t="n">
+        <v>-8071</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-263108</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-255037</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-244034</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-232907</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-219159</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-207291</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 16-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 17-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,29 +2418,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
-        <v>28408</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="C30" s="11" t="n">
+        <v>38197</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>-215</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
+      <c r="E30" s="11" t="n">
+        <v>-26266</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>28623</v>
+      <c r="G30" s="11" t="n">
+        <v>64463</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-706775</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-771238</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-799861</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-676971</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-677012</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-618376</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23201.6</v>
+        <v>23195.25</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23284.75</v>
+        <v>23363.55</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>56935</v>
+        <v>36009</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>56935</v>
+        <v>36009</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23116.1</v>
+        <v>23193.65</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23217.6</v>
+        <v>23270.6</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23464.85</v>
+        <v>23528.11666666666</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23211.875</v>
+        <v>23273.26666666666</v>
       </c>
     </row>
     <row r="33">
@@ -2597,29 +2597,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>50458</v>
+      <c r="C33" s="14" t="n">
+        <v>23278</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>-1648</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
+        <v>20544</v>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G33" s="11" t="n">
-        <v>52106</v>
+      <c r="G33" s="14" t="n">
+        <v>2734</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-392641</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-395375</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-447481</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-406171</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-408397</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-405208</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23374.8</v>
+        <v>23445.83333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23206.15</v>
+        <v>23275.93333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2664,29 +2664,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>734</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="C34" s="14" t="n">
+        <v>495</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>885</v>
+      <c r="E34" s="11" t="n">
+        <v>71</v>
       </c>
       <c r="F34" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-151</v>
+        <v>424</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>21431</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>21007</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>21158</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>21924</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>23695</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>24121</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23296.2</v>
+        <v>23358.21666666666</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23200.425</v>
+        <v>23278.6</v>
       </c>
     </row>
     <row r="35">
@@ -2731,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>14031</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="n">
+        <v>6990</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>11793</v>
+      <c r="E35" s="11" t="n">
+        <v>11571</v>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G35" s="11" t="n">
-        <v>2238</v>
+        <v>-4581</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>194874</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>199455</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>197217</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>197348</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>180982</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>166331</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23206.15</v>
+        <v>23275.93333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,27 +2794,27 @@
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>-2852</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+        <v>7167</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>51341</v>
+      <c r="E36" s="11" t="n">
+        <v>5744</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-54193</v>
+        <v>1423</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>176336</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>174913</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>229106</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>186899</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>203720</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>214756</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23127.55</v>
+        <v>23188.31666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>62371</v>
+        <v>37930</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>62371</v>
+        <v>37930</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23037.5</v>
+        <v>23106.03333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22958.89999999999</v>
+        <v>23018.41666666666</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>13.17</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>13.43</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>12.29</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.8</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.92</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9744981133829045</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9721766836399037</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9679688193651542</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9796606494773291</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9829176264436748</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9808503997602754</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,218    PCR(OI) 0.94    Max Pain 23,300</t>
+          <t>Spot 23,271    PCR(OI) 1.00    Max Pain 23,300</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23879.57419354839</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23882.07862903226</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23883.62056451613</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23883.88266129032</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23885.82661290323</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23888.96411290322</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23270.6</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23217.6</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23118.6</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23398.1</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23477.8</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23431.5</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3137,17 +3137,17 @@
         <v>23500</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>115909</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>25954</v>
+        <v>138215</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>22306</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>1720743</v>
+        <v>2090353</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9529168644130193</v>
+        <v>0.9550753819290334</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9605609315602034</v>
@@ -3173,16 +3173,16 @@
         <v>0.9970635633790684</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23800</v>
+        <v>24000</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>96789</v>
-      </c>
-      <c r="R46" s="14" t="n">
-        <v>32700</v>
+        <v>158613</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>25422</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>787772</v>
+        <v>917800</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24364.76975806452</v>
+        <v>24365.19717741936</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24358.78790322581</v>
@@ -3212,16 +3212,16 @@
         <v>24323.42419354839</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>24000</v>
+        <v>24500</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>133191</v>
-      </c>
-      <c r="R47" s="14" t="n">
-        <v>27501</v>
+        <v>160769</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>70039</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>694739</v>
+        <v>541187</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23217.6</v>
+        <v>23270.6</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23398.1</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="29" t="inlineStr">
-        <is>
-          <t>16-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="29" t="inlineStr">
+      <c r="J49" s="32" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="32" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="29" t="inlineStr">
+      <c r="L49" s="32" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="29" t="inlineStr">
+      <c r="M49" s="32" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="29" t="inlineStr">
+      <c r="N49" s="32" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
@@ -3318,55 +3318,55 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
+      <c r="P50" s="33" t="n">
         <v>23200</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>114879</v>
-      </c>
-      <c r="R50" s="14" t="n">
-        <v>44834</v>
+        <v>133831</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>18952</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>3561470</v>
-      </c>
-      <c r="T50" s="33" t="inlineStr">
+        <v>2923802</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="32" t="n">
+      <c r="P51" s="33" t="n">
         <v>23000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>125115</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>52075</v>
+        <v>148503</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>23388</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>1943321</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
+        <v>1748328</v>
+      </c>
+      <c r="T51" s="32" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>22500</v>
+      <c r="P52" s="33" t="n">
+        <v>22000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>102560</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>32165</v>
+        <v>167961</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>68828</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>649345</v>
+        <v>725341</v>
       </c>
       <c r="T52" s="30" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 16-Sep-2026    1 DAY AGO = 15-Sep-2026    2 DAYS AGO = 11-Sep-2026    3 DAYS AGO = 10-Sep-2026    4 DAYS AGO = 09-Sep-2026    (generated 16-Sep-2026 20:40 IST)</t>
+          <t>TODAY = 17-Sep-2026    1 DAY AGO = 16-Sep-2026    2 DAYS AGO = 15-Sep-2026    3 DAYS AGO = 11-Sep-2026    4 DAYS AGO = 10-Sep-2026    (generated 17-Sep-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-18
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,9 +187,6 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -201,6 +198,9 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>5646</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="3">
@@ -705,15 +705,15 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>5180</v>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="n">
-        <v>-466</v>
+        <v>2865</v>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>393</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,34 +721,34 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>5646</v>
+        <v>2472</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="14" t="n">
+        <v>241420</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>238948</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="14" t="n">
         <v>233302</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="14" t="n">
         <v>239463</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>231488</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>230971</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
+      <c r="Q3" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="14" t="n">
-        <v>-7932</v>
+      <c r="S3" s="13" t="n">
+        <v>-57383</v>
       </c>
     </row>
     <row r="4">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>65</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>-247</v>
+        <v>119</v>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>10</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -790,28 +790,28 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>312</v>
+        <v>109</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="14" t="n">
+        <v>12967</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>12858</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="14" t="n">
         <v>12546</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="14" t="n">
         <v>13722</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="14" t="n">
         <v>14348</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>14892</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-101544</v>
+        <v>-84419</v>
       </c>
     </row>
     <row r="5">
@@ -843,44 +843,44 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>102</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>2040</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G5" s="14" t="n">
-        <v>-1938</v>
+        <v>858</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>-755</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>1613</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="14" t="n">
+        <v>-288428</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-290041</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="14" t="n">
         <v>-288103</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="14" t="n">
         <v>-291052</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="14" t="n">
         <v>-284882</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-281844</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>11278</v>
+        <v>11435</v>
       </c>
     </row>
     <row r="6">
@@ -906,56 +906,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
-        <v>-4025</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>-5</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="C6" s="13" t="n">
+        <v>-3576</v>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>618</v>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>-4020</v>
+      <c r="G6" s="13" t="n">
+        <v>-4194</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
+        <v>34041</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>38235</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>42255</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="14" t="n">
         <v>37867</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="14" t="n">
         <v>39046</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>35981</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="13" t="inlineStr">
+      <c r="Q6" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -965,8 +965,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="14" t="n">
-        <v>-53770</v>
+      <c r="S6" s="13" t="n">
+        <v>-12095</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>1322</v>
+        <v>266</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>1322</v>
+        <v>266</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="14" t="n">
-        <v>2734</v>
+      <c r="S7" s="11" t="n">
+        <v>-7003</v>
       </c>
     </row>
     <row r="8">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>312</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9">
@@ -1097,44 +1097,44 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>382191</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
+        <v>211134</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="14" t="n">
-        <v>390123</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="E9" s="13" t="n">
+        <v>268517</v>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>-7932</v>
+      <c r="G9" s="13" t="n">
+        <v>-57383</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="14" t="n">
+        <v>233015</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>290398</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="14" t="n">
         <v>298330</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="14" t="n">
         <v>434768</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="14" t="n">
         <v>229662</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>380160</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>673</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="10">
@@ -1166,15 +1166,15 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>1400</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>727</v>
+        <v>1070</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>-300</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -1182,34 +1182,34 @@
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>673</v>
+        <v>1370</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
+        <v>5619</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>4249</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>3576</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="14" t="n">
         <v>3391</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="14" t="n">
         <v>2051</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>1500</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
+      <c r="Q10" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>4510</v>
+      <c r="S10" s="13" t="n">
+        <v>2450</v>
       </c>
     </row>
     <row r="11">
@@ -1235,15 +1235,15 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>46872</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
+        <v>45152</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E11" s="14" t="n">
-        <v>41558</v>
+      <c r="E11" s="13" t="n">
+        <v>30662</v>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
@@ -1251,36 +1251,36 @@
         </is>
       </c>
       <c r="G11" s="11" t="n">
-        <v>5314</v>
+        <v>14490</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="14" t="n">
+        <v>-268402</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-282892</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="14" t="n">
         <v>-288206</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="14" t="n">
         <v>-313041</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="14" t="n">
         <v>-287098</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-318871</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>-764</v>
+      <c r="S11" s="11" t="n">
+        <v>19777</v>
       </c>
     </row>
     <row r="12">
@@ -1304,15 +1304,15 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>138191</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
+        <v>49185</v>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E12" s="14" t="n">
-        <v>136245</v>
+      <c r="E12" s="13" t="n">
+        <v>7663</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
@@ -1320,36 +1320,36 @@
         </is>
       </c>
       <c r="G12" s="11" t="n">
-        <v>1946</v>
+        <v>41522</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="14" t="n">
+        <v>29767</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>-11755</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <v>-13701</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="14" t="n">
         <v>-125118</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="14" t="n">
         <v>55386</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>-62790</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R12" s="10" t="inlineStr">
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>-2622</v>
+      <c r="S12" s="11" t="n">
+        <v>1267</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>568654</v>
+        <v>306541</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>568653</v>
+        <v>306542</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,9 +1394,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="14" t="n">
-        <v>424</v>
+      <c r="S13" s="11" t="n">
+        <v>-645</v>
       </c>
     </row>
     <row r="14">
@@ -1463,9 +1463,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q14" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>-1938</v>
+      <c r="S14" s="11" t="n">
+        <v>1613</v>
       </c>
     </row>
     <row r="15">
@@ -1483,13 +1483,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
-        <v>417682</v>
+      <c r="C15" s="13" t="n">
+        <v>416987</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>519226</v>
+        <v>501406</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1505,28 +1505,28 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-101544</v>
+        <v>-84419</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-796597</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-712178</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-610634</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>-787481</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>-753121</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-814502</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="11" t="n">
-        <v>5314</v>
+        <v>14490</v>
       </c>
     </row>
     <row r="16">
@@ -1552,13 +1552,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
-        <v>4560</v>
+      <c r="C16" s="13" t="n">
+        <v>2600</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1566,42 +1566,42 @@
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>50</v>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
+        <v>150</v>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>4510</v>
+      <c r="G16" s="13" t="n">
+        <v>2450</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="14" t="n">
+        <v>57285</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>54835</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <v>50325</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="14" t="n">
         <v>53470</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="14" t="n">
         <v>56824</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>50538</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
+      <c r="Q16" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>32548</v>
+      <c r="S16" s="13" t="n">
+        <v>17743</v>
       </c>
     </row>
     <row r="17">
@@ -1621,13 +1621,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n">
-        <v>50103</v>
+      <c r="C17" s="13" t="n">
+        <v>112453</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1635,44 +1635,44 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>17555</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+        <v>94710</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>32548</v>
+      <c r="G17" s="13" t="n">
+        <v>17743</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="12" t="n">
+      <c r="J17" s="14" t="n">
+        <v>630453</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <v>612710</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="14" t="n">
         <v>580162</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="14" t="n">
         <v>678520</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="14" t="n">
         <v>669711</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>662764</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q17" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1680,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>3488</v>
+      <c r="S17" s="13" t="n">
+        <v>-38770</v>
       </c>
     </row>
     <row r="18">
@@ -1690,13 +1690,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
-        <v>163101</v>
+      <c r="C18" s="13" t="n">
+        <v>170153</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1704,42 +1704,42 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>98614</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
+        <v>105928</v>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>64487</v>
+      <c r="G18" s="13" t="n">
+        <v>64225</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="12" t="n">
+      <c r="J18" s="14" t="n">
+        <v>108858</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>44633</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="14" t="n">
         <v>-19854</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="14" t="n">
         <v>55491</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="14" t="n">
         <v>26585</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>101200</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="13" t="inlineStr">
+      <c r="Q18" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>-8071</v>
+      <c r="S18" s="13" t="n">
+        <v>-6680</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>635446</v>
+        <v>702193</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>635445</v>
+        <v>702194</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q19" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="11" t="n">
-        <v>-4581</v>
+      <c r="S19" s="13" t="n">
+        <v>14531</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
+      <c r="Q20" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>-4020</v>
+      <c r="S20" s="13" t="n">
+        <v>-4194</v>
       </c>
     </row>
     <row r="21">
@@ -1881,15 +1881,15 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>11293</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+        <v>13471</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
-        <v>15</v>
+      <c r="E21" s="13" t="n">
+        <v>2036</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1897,28 +1897,28 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>11278</v>
+        <v>11435</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="14" t="n">
+        <v>3239717</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3228282</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <v>3217004</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="14" t="n">
         <v>3241565</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="14" t="n">
         <v>3265326</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3245811</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="S21" s="11" t="n">
-        <v>1946</v>
+        <v>41522</v>
       </c>
     </row>
     <row r="22">
@@ -1950,50 +1950,50 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>4012</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="n">
-        <v>4776</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G22" s="14" t="n">
-        <v>-764</v>
+        <v>1329</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>-18448</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="n">
+        <v>19777</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J22" s="14" t="n">
+        <v>-4233591</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-4253368</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="14" t="n">
         <v>-4252604</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="14" t="n">
         <v>-4249116</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="14" t="n">
         <v>-4291548</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4281465</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
+      <c r="Q22" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>64487</v>
+      <c r="S22" s="13" t="n">
+        <v>64225</v>
       </c>
     </row>
     <row r="23">
@@ -2013,67 +2013,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="n">
-        <v>14534</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="n">
+        <v>-20510</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n">
-        <v>11046</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="E23" s="13" t="n">
+        <v>18260</v>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="n">
+        <v>-38770</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="n">
+        <v>500795</v>
+      </c>
+      <c r="K23" s="14" t="n">
+        <v>539565</v>
+      </c>
+      <c r="L23" s="14" t="n">
+        <v>536077</v>
+      </c>
+      <c r="M23" s="14" t="n">
+        <v>500013</v>
+      </c>
+      <c r="N23" s="14" t="n">
+        <v>519602</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>3488</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>539565</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>536077</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>500013</v>
-      </c>
-      <c r="M23" s="12" t="n">
-        <v>519602</v>
-      </c>
-      <c r="N23" s="12" t="n">
-        <v>541920</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-14002</v>
+      <c r="S23" s="11" t="n">
+        <v>7558</v>
       </c>
     </row>
     <row r="24">
@@ -2082,50 +2082,50 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="n">
-        <v>-3876</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>10874</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>10126</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G24" s="14" t="n">
-        <v>-14002</v>
+      <c r="E24" s="13" t="n">
+        <v>3316</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>7558</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J24" s="14" t="n">
+        <v>493079</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>485521</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="14" t="n">
         <v>499523</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="14" t="n">
         <v>507538</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="14" t="n">
         <v>506620</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>493734</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="11" t="n">
-        <v>64463</v>
+        <v>17508</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>25963</v>
+        <v>5164</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>25963</v>
+        <v>5164</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>1423</v>
+      <c r="S25" s="11" t="n">
+        <v>-6883</v>
       </c>
     </row>
     <row r="26">
@@ -2249,49 +2249,49 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="n">
-        <v>-10131</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>18839</v>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
-        <v>43639</v>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="E27" s="13" t="n">
+        <v>30934</v>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n">
-        <v>-53770</v>
+      <c r="G27" s="13" t="n">
+        <v>-12095</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>1357250</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>1369345</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>1423115</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="14" t="n">
         <v>1432784</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>1289384</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1267932</v>
       </c>
     </row>
     <row r="28">
@@ -2306,43 +2306,43 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E28" s="14" t="n">
-        <v>2622</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G28" s="14" t="n">
-        <v>-2622</v>
+        <v>70</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>-1197</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="n">
+        <v>1267</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-398195</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-399462</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-396840</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="14" t="n">
         <v>-388889</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>-379506</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-371761</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,47 +2365,47 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>7943</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+        <v>15088</v>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>16014</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
+      <c r="E29" s="13" t="n">
+        <v>21768</v>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>-8071</v>
+      <c r="G29" s="13" t="n">
+        <v>-6680</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-269788</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-263108</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-255037</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="14" t="n">
         <v>-244034</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>-232907</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-219159</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 17-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 18-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,15 +2424,15 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>38197</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E30" s="11" t="n">
-        <v>-26266</v>
+        <v>20207</v>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>2699</v>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
@@ -2440,35 +2440,35 @@
         </is>
       </c>
       <c r="G30" s="11" t="n">
-        <v>64463</v>
+        <v>17508</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-689267</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-706775</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-771238</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="14" t="n">
         <v>-799861</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="14" t="n">
         <v>-676971</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-677012</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23195.25</v>
+        <v>23334.7</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23363.55</v>
+        <v>23389.15</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>36009</v>
+        <v>54204</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>36009</v>
+        <v>54204</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23193.65</v>
+        <v>23286.6</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23270.6</v>
+        <v>23346.4</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23528.11666666666</v>
+        <v>23497.38333333333</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23273.26666666666</v>
+        <v>23343.55833333333</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2597,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
-        <v>23278</v>
+      <c r="C33" s="13" t="n">
+        <v>23486</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,43 +2611,43 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>20544</v>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="n">
-        <v>2734</v>
+        <v>30489</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>-7003</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-399644</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-392641</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-395375</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="14" t="n">
         <v>-447481</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="14" t="n">
         <v>-406171</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-408397</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23445.83333333333</v>
+        <v>23443.26666666667</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23275.93333333333</v>
+        <v>23340.71666666666</v>
       </c>
     </row>
     <row r="34">
@@ -2664,13 +2664,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="n">
-        <v>495</v>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>-9</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,43 +2678,43 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>71</v>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G34" s="14" t="n">
-        <v>424</v>
+        <v>636</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="n">
+        <v>-645</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>20786</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>21431</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>21007</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="14" t="n">
         <v>21158</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="14" t="n">
         <v>21924</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>23695</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23358.21666666666</v>
+        <v>23394.83333333333</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23278.6</v>
+        <v>23337.875</v>
       </c>
     </row>
     <row r="35">
@@ -2731,13 +2731,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>6990</v>
+      <c r="C35" s="13" t="n">
+        <v>23008</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,43 +2745,43 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>11571</v>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G35" s="11" t="n">
-        <v>-4581</v>
+        <v>8477</v>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="n">
+        <v>14531</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>209405</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>194874</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>199455</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="14" t="n">
         <v>197217</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="14" t="n">
         <v>197348</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>180982</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23275.93333333333</v>
+        <v>23340.71666666666</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,13 +2792,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>7167</v>
+      <c r="C36" s="13" t="n">
+        <v>9501</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,43 +2806,43 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>5744</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>1423</v>
+        <v>16384</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>-6883</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>169453</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>176336</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>174913</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="14" t="n">
         <v>229106</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="14" t="n">
         <v>186899</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>203720</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23188.31666666666</v>
+        <v>23292.28333333333</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>37930</v>
+        <v>55986</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>37930</v>
+        <v>55986</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23106.03333333333</v>
+        <v>23238.16666666666</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23018.41666666666</v>
+        <v>23189.73333333332</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>12.29</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>13.17</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>13.43</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>12.29</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.8</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9778148328815047</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9744981133829045</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9721766836399037</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9679688193651542</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9796606494773291</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9829176264436748</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,271    PCR(OI) 1.00    Max Pain 23,300</t>
+          <t>Spot 23,346    PCR(OI) 1.12    Max Pain 23,350</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23876.09516129032</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23879.57419354839</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23882.07862903226</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23883.62056451613</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23883.88266129032</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23885.82661290323</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23346.4</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23270.6</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23217.6</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23118.6</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23398.1</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23477.8</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23500</v>
-      </c>
-      <c r="Q45" s="12" t="n">
-        <v>138215</v>
+        <v>23700</v>
+      </c>
+      <c r="Q45" s="14" t="n">
+        <v>146088</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>22306</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>2090353</v>
+        <v>29761</v>
+      </c>
+      <c r="S45" s="14" t="n">
+        <v>1311724</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9550753819290334</v>
+        <v>0.9581623376424576</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9605609315602034</v>
@@ -3175,16 +3175,16 @@
       <c r="P46" s="28" t="n">
         <v>24000</v>
       </c>
-      <c r="Q46" s="12" t="n">
-        <v>158613</v>
+      <c r="Q46" s="14" t="n">
+        <v>177824</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>25422</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>917800</v>
-      </c>
-      <c r="T46" s="30" t="inlineStr">
+        <v>19211</v>
+      </c>
+      <c r="S46" s="14" t="n">
+        <v>913736</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24365.19717741936</v>
+        <v>24365.80846774194</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24358.78790322581</v>
@@ -3214,16 +3214,16 @@
       <c r="P47" s="28" t="n">
         <v>24500</v>
       </c>
-      <c r="Q47" s="12" t="n">
-        <v>160769</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>70039</v>
-      </c>
-      <c r="S47" s="12" t="n">
-        <v>541187</v>
-      </c>
-      <c r="T47" s="30" t="inlineStr">
+      <c r="Q47" s="14" t="n">
+        <v>154620</v>
+      </c>
+      <c r="R47" s="13" t="n">
+        <v>-6149</v>
+      </c>
+      <c r="S47" s="14" t="n">
+        <v>500022</v>
+      </c>
+      <c r="T47" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23270.6</v>
+        <v>23346.4</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23398.1</v>
@@ -3250,7 +3250,7 @@
       <c r="N48" s="18" t="n">
         <v>24252</v>
       </c>
-      <c r="P48" s="31" t="inlineStr">
+      <c r="P48" s="30" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="32" t="inlineStr">
-        <is>
-          <t>17-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="32" t="inlineStr">
+      <c r="J49" s="31" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="31" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="32" t="inlineStr">
+      <c r="L49" s="31" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="32" t="inlineStr">
+      <c r="M49" s="31" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="32" t="inlineStr">
+      <c r="N49" s="31" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
@@ -3318,57 +3318,57 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
-        <v>23200</v>
-      </c>
-      <c r="Q50" s="12" t="n">
-        <v>133831</v>
+      <c r="P50" s="32" t="n">
+        <v>23300</v>
+      </c>
+      <c r="Q50" s="14" t="n">
+        <v>195178</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>18952</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>2923802</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
+        <v>90670</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>7089453</v>
+      </c>
+      <c r="T50" s="33" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="33" t="n">
+      <c r="P51" s="32" t="n">
         <v>23000</v>
       </c>
-      <c r="Q51" s="12" t="n">
-        <v>148503</v>
+      <c r="Q51" s="14" t="n">
+        <v>169141</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>23388</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>1748328</v>
-      </c>
-      <c r="T51" s="32" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>20638</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>1959567</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="33" t="n">
+      <c r="P52" s="32" t="n">
         <v>22000</v>
       </c>
-      <c r="Q52" s="12" t="n">
-        <v>167961</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>68828</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>725341</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
+      <c r="Q52" s="14" t="n">
+        <v>165254</v>
+      </c>
+      <c r="R52" s="13" t="n">
+        <v>-2707</v>
+      </c>
+      <c r="S52" s="14" t="n">
+        <v>680980</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 17-Sep-2026    1 DAY AGO = 16-Sep-2026    2 DAYS AGO = 15-Sep-2026    3 DAYS AGO = 11-Sep-2026    4 DAYS AGO = 10-Sep-2026    (generated 17-Sep-2026 20:32 IST)</t>
+          <t>TODAY = 18-Sep-2026    1 DAY AGO = 17-Sep-2026    2 DAYS AGO = 16-Sep-2026    3 DAYS AGO = 15-Sep-2026    4 DAYS AGO = 11-Sep-2026    (generated 18-Sep-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-21
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -129,19 +129,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,20 +187,20 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>2472</v>
+        <v>299</v>
       </c>
     </row>
     <row r="3">
@@ -699,21 +699,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="n">
-        <v>2865</v>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>393</v>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>-917</v>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>-1216</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>2472</v>
+        <v>299</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="14" t="n">
+        <v>241719</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>241420</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="14" t="n">
         <v>238948</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="14" t="n">
         <v>233302</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="14" t="n">
         <v>239463</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>231488</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="13" t="n">
-        <v>-57383</v>
+        <v>-50388</v>
       </c>
     </row>
     <row r="4">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>119</v>
+        <v>213</v>
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E4" s="13" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>109</v>
+        <v>213</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,20 +798,20 @@
         </is>
       </c>
       <c r="J4" s="14" t="n">
+        <v>13180</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>12967</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="14" t="n">
         <v>12858</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="14" t="n">
         <v>12546</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="14" t="n">
         <v>13722</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>14348</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-84419</v>
+        <v>-31144</v>
       </c>
     </row>
     <row r="5">
@@ -837,29 +837,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>858</v>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>-755</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G5" s="11" t="n">
-        <v>1613</v>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>-675</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>1443</v>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>-2118</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -867,28 +867,28 @@
         </is>
       </c>
       <c r="J5" s="14" t="n">
+        <v>-290546</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-288428</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="14" t="n">
         <v>-290041</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="14" t="n">
         <v>-288103</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="N5" s="14" t="n">
         <v>-291052</v>
       </c>
-      <c r="N5" s="14" t="n">
-        <v>-284882</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q5" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -896,8 +896,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>11435</v>
+      <c r="S5" s="13" t="n">
+        <v>-8199</v>
       </c>
     </row>
     <row r="6">
@@ -912,23 +912,23 @@
         </is>
       </c>
       <c r="C6" s="13" t="n">
-        <v>-3576</v>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="n">
-        <v>618</v>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="n">
-        <v>-4194</v>
+        <v>-502</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>-2108</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>1606</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,28 +936,28 @@
         </is>
       </c>
       <c r="J6" s="14" t="n">
+        <v>35647</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>34041</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="14" t="n">
         <v>38235</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="14" t="n">
         <v>42255</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="14" t="n">
         <v>37867</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>39046</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R6" s="10" t="inlineStr">
@@ -965,8 +965,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="13" t="n">
-        <v>-12095</v>
+      <c r="S6" s="11" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>266</v>
+        <v>-1881</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>266</v>
+        <v>-1881</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q7" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>-7003</v>
+      <c r="S7" s="13" t="n">
+        <v>39124</v>
       </c>
     </row>
     <row r="8">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>109</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>211134</v>
+        <v>196373</v>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="E9" s="13" t="n">
-        <v>268517</v>
+        <v>246761</v>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
@@ -1113,7 +1113,7 @@
         </is>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-57383</v>
+        <v>-50388</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,20 +1121,20 @@
         </is>
       </c>
       <c r="J9" s="14" t="n">
+        <v>182627</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>233015</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="L9" s="14" t="n">
         <v>290398</v>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="M9" s="14" t="n">
         <v>298330</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="N9" s="14" t="n">
         <v>434768</v>
       </c>
-      <c r="N9" s="14" t="n">
-        <v>229662</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>1370</v>
+        <v>498</v>
       </c>
     </row>
     <row r="10">
@@ -1166,15 +1166,15 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>1070</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>-300</v>
+        <v>698</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>200</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>1370</v>
+        <v>498</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,20 +1190,20 @@
         </is>
       </c>
       <c r="J10" s="14" t="n">
+        <v>6117</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>5619</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="14" t="n">
         <v>4249</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="14" t="n">
         <v>3576</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="14" t="n">
         <v>3391</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>2051</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="S10" s="13" t="n">
-        <v>2450</v>
+        <v>12275</v>
       </c>
     </row>
     <row r="11">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>45152</v>
+        <v>33571</v>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="E11" s="13" t="n">
-        <v>30662</v>
+        <v>21525</v>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="G11" s="11" t="n">
-        <v>14490</v>
+        <v>12046</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,20 +1259,20 @@
         </is>
       </c>
       <c r="J11" s="14" t="n">
+        <v>-256356</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-268402</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="14" t="n">
         <v>-282892</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="M11" s="14" t="n">
         <v>-288206</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="14" t="n">
         <v>-313041</v>
       </c>
-      <c r="N11" s="14" t="n">
-        <v>-287098</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="S11" s="11" t="n">
-        <v>19777</v>
+        <v>22098</v>
       </c>
     </row>
     <row r="12">
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>49185</v>
+        <v>45834</v>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="E12" s="13" t="n">
-        <v>7663</v>
+        <v>7989</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
@@ -1320,7 +1320,7 @@
         </is>
       </c>
       <c r="G12" s="11" t="n">
-        <v>41522</v>
+        <v>37845</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,28 +1328,28 @@
         </is>
       </c>
       <c r="J12" s="14" t="n">
+        <v>67612</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>29767</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="14" t="n">
         <v>-11755</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="M12" s="14" t="n">
         <v>-13701</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="14" t="n">
         <v>-125118</v>
       </c>
-      <c r="N12" s="14" t="n">
-        <v>55386</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q12" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R12" s="10" t="inlineStr">
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>1267</v>
+      <c r="S12" s="13" t="n">
+        <v>-15554</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>306541</v>
+        <v>276476</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>306542</v>
+        <v>276475</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-645</v>
+        <v>-467</v>
       </c>
     </row>
     <row r="14">
@@ -1463,9 +1463,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q14" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="11" t="n">
-        <v>1613</v>
+      <c r="S14" s="13" t="n">
+        <v>-2118</v>
       </c>
     </row>
     <row r="15">
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="C15" s="13" t="n">
-        <v>416987</v>
+        <v>664875</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>501406</v>
+        <v>696019</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-84419</v>
+        <v>-31144</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="14" t="n">
+        <v>-827741</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-796597</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="14" t="n">
         <v>-712178</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="14" t="n">
         <v>-610634</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="14" t="n">
         <v>-787481</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-753121</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="11" t="n">
-        <v>14490</v>
+        <v>12046</v>
       </c>
     </row>
     <row r="16">
@@ -1558,15 +1558,15 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>2600</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="n">
-        <v>150</v>
+        <v>12075</v>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>-200</v>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="G16" s="13" t="n">
-        <v>2450</v>
+        <v>12275</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="14" t="n">
+        <v>69560</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>57285</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="14" t="n">
         <v>54835</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="14" t="n">
         <v>50325</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="14" t="n">
         <v>53470</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>56824</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="13" t="n">
-        <v>17743</v>
+        <v>7977</v>
       </c>
     </row>
     <row r="17">
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="C17" s="13" t="n">
-        <v>112453</v>
+        <v>94585</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>94710</v>
+        <v>86608</v>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="G17" s="13" t="n">
-        <v>17743</v>
+        <v>7977</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,28 +1651,28 @@
         </is>
       </c>
       <c r="J17" s="14" t="n">
+        <v>638430</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <v>630453</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="L17" s="14" t="n">
         <v>612710</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="M17" s="14" t="n">
         <v>580162</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="N17" s="14" t="n">
         <v>678520</v>
       </c>
-      <c r="N17" s="14" t="n">
-        <v>669711</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1680,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="13" t="n">
-        <v>-38770</v>
+      <c r="S17" s="11" t="n">
+        <v>3923</v>
       </c>
     </row>
     <row r="18">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>170153</v>
+        <v>224718</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>105928</v>
+        <v>213825</v>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="G18" s="13" t="n">
-        <v>64225</v>
+        <v>10893</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,28 +1720,28 @@
         </is>
       </c>
       <c r="J18" s="14" t="n">
+        <v>119751</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>108858</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="14" t="n">
         <v>44633</v>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="M18" s="14" t="n">
         <v>-19854</v>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="N18" s="14" t="n">
         <v>55491</v>
       </c>
-      <c r="N18" s="14" t="n">
-        <v>26585</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q18" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R18" s="10" t="inlineStr">
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="13" t="n">
-        <v>-6680</v>
+      <c r="S18" s="11" t="n">
+        <v>3444</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>702193</v>
+        <v>996253</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>702194</v>
+        <v>996252</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q19" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="13" t="n">
-        <v>14531</v>
+      <c r="S19" s="11" t="n">
+        <v>-5130</v>
       </c>
     </row>
     <row r="20">
@@ -1855,9 +1855,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="13" t="n">
-        <v>-4194</v>
+      <c r="S20" s="11" t="n">
+        <v>1606</v>
       </c>
     </row>
     <row r="21">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>13471</v>
+        <v>9600</v>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
@@ -1889,53 +1889,53 @@
         </is>
       </c>
       <c r="E21" s="13" t="n">
-        <v>2036</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
+        <v>17799</v>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>-8199</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="n">
+        <v>3231518</v>
+      </c>
+      <c r="K21" s="14" t="n">
+        <v>3239717</v>
+      </c>
+      <c r="L21" s="14" t="n">
+        <v>3228282</v>
+      </c>
+      <c r="M21" s="14" t="n">
+        <v>3217004</v>
+      </c>
+      <c r="N21" s="14" t="n">
+        <v>3241565</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>11435</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="14" t="n">
-        <v>3239717</v>
-      </c>
-      <c r="K21" s="14" t="n">
-        <v>3228282</v>
-      </c>
-      <c r="L21" s="14" t="n">
-        <v>3217004</v>
-      </c>
-      <c r="M21" s="14" t="n">
-        <v>3241565</v>
-      </c>
-      <c r="N21" s="14" t="n">
-        <v>3265326</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S21" s="11" t="n">
-        <v>41522</v>
+        <v>37845</v>
       </c>
     </row>
     <row r="22">
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>1329</v>
+        <v>6188</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>-18448</v>
+        <v>-15910</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="G22" s="11" t="n">
-        <v>19777</v>
+        <v>22098</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="14" t="n">
+        <v>-4211493</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-4233591</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="14" t="n">
         <v>-4253368</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="14" t="n">
         <v>-4252604</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="14" t="n">
         <v>-4249116</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-4291548</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="13" t="n">
-        <v>64225</v>
+        <v>10893</v>
       </c>
     </row>
     <row r="23">
@@ -2013,13 +2013,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="13" t="n">
-        <v>-20510</v>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>9676</v>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
@@ -2027,53 +2027,53 @@
         </is>
       </c>
       <c r="E23" s="13" t="n">
-        <v>18260</v>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
+        <v>5753</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>3923</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="n">
+        <v>504718</v>
+      </c>
+      <c r="K23" s="14" t="n">
+        <v>500795</v>
+      </c>
+      <c r="L23" s="14" t="n">
+        <v>539565</v>
+      </c>
+      <c r="M23" s="14" t="n">
+        <v>536077</v>
+      </c>
+      <c r="N23" s="14" t="n">
+        <v>500013</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="13" t="n">
-        <v>-38770</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="14" t="n">
-        <v>500795</v>
-      </c>
-      <c r="K23" s="14" t="n">
-        <v>539565</v>
-      </c>
-      <c r="L23" s="14" t="n">
-        <v>536077</v>
-      </c>
-      <c r="M23" s="14" t="n">
-        <v>500013</v>
-      </c>
-      <c r="N23" s="14" t="n">
-        <v>519602</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>7558</v>
+      <c r="S23" s="13" t="n">
+        <v>-17822</v>
       </c>
     </row>
     <row r="24">
@@ -2088,7 +2088,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>10874</v>
+        <v>9223</v>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
@@ -2096,53 +2096,53 @@
         </is>
       </c>
       <c r="E24" s="13" t="n">
-        <v>3316</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
+        <v>27045</v>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>-17822</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="n">
+        <v>475257</v>
+      </c>
+      <c r="K24" s="14" t="n">
+        <v>493079</v>
+      </c>
+      <c r="L24" s="14" t="n">
+        <v>485521</v>
+      </c>
+      <c r="M24" s="14" t="n">
+        <v>499523</v>
+      </c>
+      <c r="N24" s="14" t="n">
+        <v>507538</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q24" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>7558</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="14" t="n">
-        <v>493079</v>
-      </c>
-      <c r="K24" s="14" t="n">
-        <v>485521</v>
-      </c>
-      <c r="L24" s="14" t="n">
-        <v>499523</v>
-      </c>
-      <c r="M24" s="14" t="n">
-        <v>507538</v>
-      </c>
-      <c r="N24" s="14" t="n">
-        <v>506620</v>
-      </c>
-      <c r="P24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q24" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S24" s="11" t="n">
-        <v>17508</v>
+        <v>12103</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>5164</v>
+        <v>34687</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>5164</v>
+        <v>34687</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="11" t="n">
-        <v>-6883</v>
+        <v>-33527</v>
       </c>
     </row>
     <row r="26">
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>18839</v>
+        <v>19378</v>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
@@ -2263,15 +2263,15 @@
         </is>
       </c>
       <c r="E27" s="13" t="n">
-        <v>30934</v>
-      </c>
-      <c r="F27" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G27" s="13" t="n">
-        <v>-12095</v>
+        <v>19371</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="n">
+        <v>7</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="14" t="n">
+        <v>1357257</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>1357250</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="14" t="n">
         <v>1369345</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="14" t="n">
         <v>1423115</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="14" t="n">
         <v>1432784</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>1289384</v>
       </c>
     </row>
     <row r="28">
@@ -2300,29 +2300,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="n">
-        <v>70</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E28" s="11" t="n">
-        <v>-1197</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G28" s="11" t="n">
-        <v>1267</v>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="n">
+        <v>-830</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="n">
+        <v>14724</v>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G28" s="13" t="n">
+        <v>-15554</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="14" t="n">
+        <v>-413749</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-398195</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="14" t="n">
         <v>-399462</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="14" t="n">
         <v>-396840</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="14" t="n">
         <v>-388889</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-379506</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>15088</v>
+        <v>16334</v>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
@@ -2373,15 +2373,15 @@
         </is>
       </c>
       <c r="E29" s="13" t="n">
-        <v>21768</v>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G29" s="13" t="n">
-        <v>-6680</v>
+        <v>12890</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="n">
+        <v>3444</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="14" t="n">
+        <v>-266344</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-269788</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="14" t="n">
         <v>-263108</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="14" t="n">
         <v>-255037</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="14" t="n">
         <v>-244034</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-232907</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 18-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 21-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>20207</v>
+        <v>26867</v>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="E30" s="13" t="n">
-        <v>2699</v>
+        <v>14764</v>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="G30" s="11" t="n">
-        <v>17508</v>
+        <v>12103</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="14" t="n">
+        <v>-677164</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-689267</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="14" t="n">
         <v>-706775</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="14" t="n">
         <v>-771238</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="14" t="n">
         <v>-799861</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-676971</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23334.7</v>
+        <v>23330.2</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23389.15</v>
+        <v>23466.8</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>54204</v>
+        <v>61749</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>54204</v>
+        <v>61749</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23286.6</v>
+        <v>23314.8</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23346.4</v>
+        <v>23414.3</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23497.38333333333</v>
+        <v>23634.46666666666</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23343.55833333333</v>
+        <v>23406.46666666666</v>
       </c>
     </row>
     <row r="33">
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="C33" s="13" t="n">
-        <v>23486</v>
+        <v>53154</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,15 +2611,15 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>30489</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G33" s="11" t="n">
-        <v>-7003</v>
+        <v>14030</v>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="n">
+        <v>39124</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="14" t="n">
+        <v>-360520</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-399644</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="14" t="n">
         <v>-392641</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="14" t="n">
         <v>-395375</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="14" t="n">
         <v>-447481</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-406171</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23443.26666666667</v>
+        <v>23550.63333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23340.71666666666</v>
+        <v>23398.63333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>-9</v>
+        <v>-66</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>636</v>
+        <v>401</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-645</v>
+        <v>-467</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="14" t="n">
+        <v>20319</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>20786</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="14" t="n">
         <v>21431</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="14" t="n">
         <v>21007</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="14" t="n">
         <v>21158</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>21924</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23394.83333333333</v>
+        <v>23482.46666666666</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23337.875</v>
+        <v>23390.8</v>
       </c>
     </row>
     <row r="35">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="C35" s="13" t="n">
-        <v>23008</v>
+        <v>7148</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,15 +2745,15 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>8477</v>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G35" s="13" t="n">
-        <v>14531</v>
+        <v>12278</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="n">
+        <v>-5130</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="14" t="n">
+        <v>204275</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>209405</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="14" t="n">
         <v>194874</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="14" t="n">
         <v>199455</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="14" t="n">
         <v>197217</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>197348</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23340.71666666666</v>
+        <v>23398.63333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="C36" s="13" t="n">
-        <v>9501</v>
+        <v>8273</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>16384</v>
+        <v>41800</v>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
@@ -2814,7 +2814,7 @@
         </is>
       </c>
       <c r="G36" s="11" t="n">
-        <v>-6883</v>
+        <v>-33527</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="14" t="n">
+        <v>135926</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>169453</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="14" t="n">
         <v>176336</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="14" t="n">
         <v>174913</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="14" t="n">
         <v>229106</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>186899</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23292.28333333333</v>
+        <v>23330.46666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>55986</v>
+        <v>68509</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>55986</v>
+        <v>68509</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23238.16666666666</v>
+        <v>23246.63333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23189.73333333332</v>
+        <v>23178.46666666666</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.39</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>12.29</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>13.17</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>13.43</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>12.29</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9805221830332062</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9778148328815047</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9744981133829045</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9721766836399037</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9679688193651542</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9796606494773291</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,346    PCR(OI) 1.12    Max Pain 23,350</t>
+          <t>Spot 23,414    PCR(OI) 1.46    Max Pain 23,400</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23879.4189516129</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23876.09516129032</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23879.57419354839</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23882.07862903226</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23883.62056451613</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23883.88266129032</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23414.3</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23346.4</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23270.6</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23217.6</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23118.6</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23398.1</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23700</v>
+        <v>23500</v>
       </c>
       <c r="Q45" s="14" t="n">
-        <v>146088</v>
+        <v>178853</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>29761</v>
+        <v>36912</v>
       </c>
       <c r="S45" s="14" t="n">
-        <v>1311724</v>
+        <v>7146984</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3158,35 +3158,35 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
+        <v>0.960516959670768</v>
+      </c>
+      <c r="K46" s="25" t="n">
         <v>0.9581623376424576</v>
       </c>
-      <c r="K46" s="25" t="n">
+      <c r="L46" s="25" t="n">
         <v>0.9605609315602034</v>
       </c>
-      <c r="L46" s="25" t="n">
+      <c r="M46" s="25" t="n">
         <v>0.9813887944889631</v>
       </c>
-      <c r="M46" s="25" t="n">
+      <c r="N46" s="25" t="n">
         <v>0.9933791141865997</v>
       </c>
-      <c r="N46" s="25" t="n">
-        <v>0.9970635633790684</v>
-      </c>
       <c r="P46" s="28" t="n">
-        <v>24000</v>
+        <v>23600</v>
       </c>
       <c r="Q46" s="14" t="n">
-        <v>177824</v>
+        <v>164756</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>19211</v>
+        <v>43079</v>
       </c>
       <c r="S46" s="14" t="n">
-        <v>913736</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>3860663</v>
+      </c>
+      <c r="T46" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3197,33 +3197,33 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
+        <v>24376.7689516129</v>
+      </c>
+      <c r="K47" s="18" t="n">
         <v>24365.80846774194</v>
       </c>
-      <c r="K47" s="18" t="n">
+      <c r="L47" s="18" t="n">
         <v>24358.78790322581</v>
       </c>
-      <c r="L47" s="18" t="n">
+      <c r="M47" s="18" t="n">
         <v>24350.89959677419</v>
       </c>
-      <c r="M47" s="18" t="n">
+      <c r="N47" s="18" t="n">
         <v>24336.7810483871</v>
       </c>
-      <c r="N47" s="18" t="n">
-        <v>24323.42419354839</v>
-      </c>
       <c r="P47" s="28" t="n">
-        <v>24500</v>
+        <v>23700</v>
       </c>
       <c r="Q47" s="14" t="n">
-        <v>154620</v>
+        <v>145155</v>
       </c>
       <c r="R47" s="13" t="n">
-        <v>-6149</v>
+        <v>-933</v>
       </c>
       <c r="S47" s="14" t="n">
-        <v>500022</v>
-      </c>
-      <c r="T47" s="29" t="inlineStr">
+        <v>2459258</v>
+      </c>
+      <c r="T47" s="31" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3236,21 +3236,21 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
+        <v>23414.3</v>
+      </c>
+      <c r="K48" s="18" t="n">
         <v>23346.4</v>
       </c>
-      <c r="K48" s="18" t="n">
+      <c r="L48" s="18" t="n">
         <v>23398.1</v>
       </c>
-      <c r="L48" s="18" t="n">
+      <c r="M48" s="18" t="n">
         <v>23897.7</v>
       </c>
-      <c r="M48" s="18" t="n">
+      <c r="N48" s="18" t="n">
         <v>24175.65</v>
       </c>
-      <c r="N48" s="18" t="n">
-        <v>24252</v>
-      </c>
-      <c r="P48" s="30" t="inlineStr">
+      <c r="P48" s="32" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3266,31 +3266,31 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="31" t="inlineStr">
+      <c r="J49" s="30" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="30" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="K49" s="31" t="inlineStr">
+      <c r="L49" s="30" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="31" t="inlineStr">
+      <c r="M49" s="30" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="31" t="inlineStr">
+      <c r="N49" s="30" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="31" t="inlineStr">
-        <is>
-          <t>21-Aug-2026</t>
-        </is>
-      </c>
       <c r="P49" s="27" t="inlineStr">
         <is>
           <t>Strike</t>
@@ -3318,57 +3318,57 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
+      <c r="P50" s="33" t="n">
+        <v>23400</v>
+      </c>
+      <c r="Q50" s="14" t="n">
+        <v>247382</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>173731</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>8115411</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="P51" s="33" t="n">
         <v>23300</v>
       </c>
-      <c r="Q50" s="14" t="n">
-        <v>195178</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>90670</v>
-      </c>
-      <c r="S50" s="14" t="n">
-        <v>7089453</v>
-      </c>
-      <c r="T50" s="33" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="P51" s="32" t="n">
-        <v>23000</v>
-      </c>
       <c r="Q51" s="14" t="n">
-        <v>169141</v>
+        <v>243496</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>20638</v>
+        <v>48318</v>
       </c>
       <c r="S51" s="14" t="n">
-        <v>1959567</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>5246181</v>
+      </c>
+      <c r="T51" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>22000</v>
+      <c r="P52" s="33" t="n">
+        <v>22500</v>
       </c>
       <c r="Q52" s="14" t="n">
-        <v>165254</v>
-      </c>
-      <c r="R52" s="13" t="n">
-        <v>-2707</v>
+        <v>191934</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>53126</v>
       </c>
       <c r="S52" s="14" t="n">
-        <v>680980</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
+        <v>1363091</v>
+      </c>
+      <c r="T52" s="31" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 18-Sep-2026    1 DAY AGO = 17-Sep-2026    2 DAYS AGO = 16-Sep-2026    3 DAYS AGO = 15-Sep-2026    4 DAYS AGO = 11-Sep-2026    (generated 18-Sep-2026 20:32 IST)</t>
+          <t>TODAY = 21-Sep-2026    1 DAY AGO = 18-Sep-2026    2 DAYS AGO = 17-Sep-2026    3 DAYS AGO = 16-Sep-2026    4 DAYS AGO = 15-Sep-2026    (generated 21-Sep-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-22
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -129,22 +129,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -190,17 +190,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>299</v>
+        <v>3992</v>
       </c>
     </row>
     <row r="3">
@@ -699,13 +699,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="n">
-        <v>-917</v>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>3787</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-1216</v>
+        <v>-205</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,36 +721,36 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>299</v>
+        <v>3992</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>245711</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>241719</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>241420</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>238948</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="12" t="n">
         <v>233302</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>239463</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="13" t="n">
-        <v>-50388</v>
+      <c r="S3" s="11" t="n">
+        <v>123294</v>
       </c>
     </row>
     <row r="4">
@@ -774,14 +774,14 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>213</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="E4" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
@@ -790,36 +790,36 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>213</v>
+        <v>1</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="12" t="n">
+        <v>13181</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>13180</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="12" t="n">
         <v>12967</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="12" t="n">
         <v>12858</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="12" t="n">
         <v>12546</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>13722</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -827,8 +827,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>-31144</v>
+      <c r="S4" s="14" t="n">
+        <v>100686</v>
       </c>
     </row>
     <row r="5">
@@ -837,58 +837,58 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
-        <v>-675</v>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="C5" s="14" t="n">
+        <v>-7474</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
-        <v>1443</v>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="E5" s="14" t="n">
+        <v>4888</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n">
-        <v>-2118</v>
+      <c r="G5" s="14" t="n">
+        <v>-12362</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="14" t="n">
+      <c r="J5" s="12" t="n">
+        <v>-302908</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-290546</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="12" t="n">
         <v>-288428</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="12" t="n">
         <v>-290041</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="N5" s="12" t="n">
         <v>-288103</v>
       </c>
-      <c r="N5" s="14" t="n">
-        <v>-291052</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -896,8 +896,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="13" t="n">
-        <v>-8199</v>
+      <c r="S5" s="11" t="n">
+        <v>11204</v>
       </c>
     </row>
     <row r="6">
@@ -906,13 +906,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>-502</v>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>6237</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-2108</v>
+        <v>-2132</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -928,28 +928,28 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>1606</v>
+        <v>8369</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="12" t="n">
+        <v>44016</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>35647</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="12" t="n">
         <v>34041</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>38235</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="12" t="n">
         <v>42255</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>37867</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>7</v>
+        <v>11702</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-1881</v>
+        <v>2551</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-1881</v>
+        <v>2551</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="13" t="n">
-        <v>39124</v>
+      <c r="S7" s="11" t="n">
+        <v>-36828</v>
       </c>
     </row>
     <row r="8">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>213</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1091,50 +1091,50 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>196373</v>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>246761</v>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G9" s="13" t="n">
-        <v>-50388</v>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>-1109893</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>-1233187</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>123294</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="14" t="n">
+      <c r="J9" s="12" t="n">
+        <v>305921</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>182627</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="L9" s="12" t="n">
         <v>233015</v>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="M9" s="12" t="n">
         <v>290398</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="N9" s="12" t="n">
         <v>298330</v>
       </c>
-      <c r="N9" s="14" t="n">
-        <v>434768</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>498</v>
+        <v>4517</v>
       </c>
     </row>
     <row r="10">
@@ -1166,15 +1166,15 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>698</v>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="n">
-        <v>200</v>
+        <v>3902</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>-615</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -1182,36 +1182,36 @@
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>498</v>
+        <v>4517</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="12" t="n">
+        <v>10634</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>6117</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="12" t="n">
         <v>5619</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="12" t="n">
         <v>4249</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="12" t="n">
         <v>3576</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>3391</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="13" t="n">
-        <v>12275</v>
+      <c r="S10" s="11" t="n">
+        <v>-6371</v>
       </c>
     </row>
     <row r="11">
@@ -1229,67 +1229,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="n">
-        <v>33571</v>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>21525</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>-162682</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>-162664</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>-18</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-256374</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-256356</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-268402</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-282892</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-288206</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>12046</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="14" t="n">
-        <v>-256356</v>
-      </c>
-      <c r="K11" s="14" t="n">
-        <v>-268402</v>
-      </c>
-      <c r="L11" s="14" t="n">
-        <v>-282892</v>
-      </c>
-      <c r="M11" s="14" t="n">
-        <v>-288206</v>
-      </c>
-      <c r="N11" s="14" t="n">
-        <v>-313041</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S11" s="11" t="n">
-        <v>22098</v>
+        <v>5601</v>
       </c>
     </row>
     <row r="12">
@@ -1298,67 +1298,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>45834</v>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>7989</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>-433669</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>-305877</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>-127792</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>-60180</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>67612</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>29767</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>-11755</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>-13701</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>37845</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="n">
-        <v>67612</v>
-      </c>
-      <c r="K12" s="14" t="n">
-        <v>29767</v>
-      </c>
-      <c r="L12" s="14" t="n">
-        <v>-11755</v>
-      </c>
-      <c r="M12" s="14" t="n">
-        <v>-13701</v>
-      </c>
-      <c r="N12" s="14" t="n">
-        <v>-125118</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="13" t="n">
-        <v>-15554</v>
+      <c r="S12" s="11" t="n">
+        <v>2582</v>
       </c>
     </row>
     <row r="13">
@@ -1369,11 +1369,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>276476</v>
+        <v>-1702342</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>276475</v>
+        <v>-1702343</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-467</v>
+        <v>-1080</v>
       </c>
     </row>
     <row r="14">
@@ -1463,7 +1463,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="12" t="inlineStr">
+      <c r="Q14" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="13" t="n">
-        <v>-2118</v>
+      <c r="S14" s="14" t="n">
+        <v>-12362</v>
       </c>
     </row>
     <row r="15">
@@ -1483,67 +1483,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="n">
-        <v>664875</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="n">
-        <v>696019</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>-1870981</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>-1971667</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>100686</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>-727055</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>-827741</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>-796597</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>-712178</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>-610634</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>-31144</v>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J15" s="14" t="n">
-        <v>-827741</v>
-      </c>
-      <c r="K15" s="14" t="n">
-        <v>-796597</v>
-      </c>
-      <c r="L15" s="14" t="n">
-        <v>-712178</v>
-      </c>
-      <c r="M15" s="14" t="n">
-        <v>-610634</v>
-      </c>
-      <c r="N15" s="14" t="n">
-        <v>-787481</v>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q15" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="11" t="n">
-        <v>12046</v>
+      <c r="S15" s="14" t="n">
+        <v>-18</v>
       </c>
     </row>
     <row r="16">
@@ -1552,67 +1552,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>12075</v>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="n">
-        <v>-200</v>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>-6371</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>-6371</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>63189</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>69560</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>57285</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>54835</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>50325</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="13" t="n">
-        <v>12275</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J16" s="14" t="n">
-        <v>69560</v>
-      </c>
-      <c r="K16" s="14" t="n">
-        <v>57285</v>
-      </c>
-      <c r="L16" s="14" t="n">
-        <v>54835</v>
-      </c>
-      <c r="M16" s="14" t="n">
-        <v>50325</v>
-      </c>
-      <c r="N16" s="14" t="n">
-        <v>53470</v>
-      </c>
-      <c r="P16" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q16" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R16" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="13" t="n">
-        <v>7977</v>
+      <c r="S16" s="14" t="n">
+        <v>3796</v>
       </c>
     </row>
     <row r="17">
@@ -1621,50 +1621,50 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>94585</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="n">
-        <v>86608</v>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>-326774</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>-330570</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
-        <v>7977</v>
+      <c r="G17" s="14" t="n">
+        <v>3796</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="14" t="n">
+      <c r="J17" s="12" t="n">
+        <v>642226</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>638430</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="L17" s="12" t="n">
         <v>630453</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="M17" s="12" t="n">
         <v>612710</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="N17" s="12" t="n">
         <v>580162</v>
       </c>
-      <c r="N17" s="14" t="n">
-        <v>678520</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="11" t="n">
-        <v>3923</v>
+        <v>2156</v>
       </c>
     </row>
     <row r="18">
@@ -1690,67 +1690,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="n">
-        <v>224718</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>213825</v>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>-707567</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>-609456</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>-98111</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>21640</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>119751</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>108858</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>44633</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>-19854</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="13" t="n">
-        <v>10893</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="14" t="n">
-        <v>119751</v>
-      </c>
-      <c r="K18" s="14" t="n">
-        <v>108858</v>
-      </c>
-      <c r="L18" s="14" t="n">
-        <v>44633</v>
-      </c>
-      <c r="M18" s="14" t="n">
-        <v>-19854</v>
-      </c>
-      <c r="N18" s="14" t="n">
-        <v>55491</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="11" t="n">
-        <v>3444</v>
+        <v>3571</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>996253</v>
+        <v>-2911693</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>996252</v>
+        <v>-2911693</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="11" t="n">
-        <v>-5130</v>
+      <c r="S19" s="14" t="n">
+        <v>3905</v>
       </c>
     </row>
     <row r="20">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>1606</v>
+        <v>8369</v>
       </c>
     </row>
     <row r="21">
@@ -1881,61 +1881,61 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>9600</v>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
+        <v>19442</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="13" t="n">
-        <v>17799</v>
-      </c>
-      <c r="F21" s="12" t="inlineStr">
+      <c r="E21" s="14" t="n">
+        <v>8238</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>11204</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3242722</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3231518</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3239717</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3228282</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3217004</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="13" t="n">
-        <v>-8199</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="14" t="n">
-        <v>3231518</v>
-      </c>
-      <c r="K21" s="14" t="n">
-        <v>3239717</v>
-      </c>
-      <c r="L21" s="14" t="n">
-        <v>3228282</v>
-      </c>
-      <c r="M21" s="14" t="n">
-        <v>3217004</v>
-      </c>
-      <c r="N21" s="14" t="n">
-        <v>3241565</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>37845</v>
+      <c r="S21" s="14" t="n">
+        <v>-127792</v>
       </c>
     </row>
     <row r="22">
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>6188</v>
+        <v>2849</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>-15910</v>
+        <v>-2752</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
@@ -1966,36 +1966,36 @@
         </is>
       </c>
       <c r="G22" s="11" t="n">
-        <v>22098</v>
+        <v>5601</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="14" t="n">
+      <c r="J22" s="12" t="n">
+        <v>-4205892</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4211493</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4233591</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4253368</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4252604</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-4249116</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="13" t="n">
-        <v>10893</v>
+      <c r="S22" s="11" t="n">
+        <v>-98111</v>
       </c>
     </row>
     <row r="23">
@@ -2019,15 +2019,15 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>9676</v>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
+        <v>17991</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="13" t="n">
-        <v>5753</v>
+      <c r="E23" s="14" t="n">
+        <v>15835</v>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
@@ -2035,34 +2035,34 @@
         </is>
       </c>
       <c r="G23" s="11" t="n">
-        <v>3923</v>
+        <v>2156</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="14" t="n">
+      <c r="J23" s="12" t="n">
+        <v>506874</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>504718</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="L23" s="12" t="n">
         <v>500795</v>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="M23" s="12" t="n">
         <v>539565</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="N23" s="12" t="n">
         <v>536077</v>
       </c>
-      <c r="N23" s="14" t="n">
-        <v>500013</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="12" t="inlineStr">
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="13" t="n">
-        <v>-17822</v>
+      <c r="S23" s="14" t="n">
+        <v>-18961</v>
       </c>
     </row>
     <row r="24">
@@ -2088,52 +2088,52 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>9223</v>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
+        <v>17379</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="13" t="n">
-        <v>27045</v>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
+      <c r="E24" s="14" t="n">
+        <v>36340</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="13" t="n">
-        <v>-17822</v>
+      <c r="G24" s="14" t="n">
+        <v>-18961</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="14" t="n">
+      <c r="J24" s="12" t="n">
+        <v>456296</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>475257</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="12" t="n">
         <v>493079</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="12" t="n">
         <v>485521</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="12" t="n">
         <v>499523</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>507538</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q24" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="11" t="n">
-        <v>12103</v>
+      <c r="S24" s="14" t="n">
+        <v>-17855</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>34687</v>
+        <v>57661</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>34687</v>
+        <v>57661</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="11" t="n">
-        <v>-33527</v>
+      <c r="S25" s="14" t="n">
+        <v>34003</v>
       </c>
     </row>
     <row r="26">
@@ -2249,21 +2249,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="n">
-        <v>19378</v>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="n">
-        <v>19371</v>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>-6942</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>-18644</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,27 +2271,27 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>7</v>
+        <v>11702</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>1368959</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1357257</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>1357250</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>1369345</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="12" t="n">
         <v>1423115</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>1432784</v>
       </c>
     </row>
     <row r="28">
@@ -2300,49 +2300,49 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="n">
-        <v>-830</v>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="n">
-        <v>14724</v>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="n">
-        <v>-15554</v>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>600</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>-1982</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="n">
+        <v>2582</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-411167</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-413749</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-398195</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-399462</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="12" t="n">
         <v>-396840</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-388889</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,15 +2365,15 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>16334</v>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
+        <v>8631</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="13" t="n">
-        <v>12890</v>
+      <c r="E29" s="14" t="n">
+        <v>5060</v>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
@@ -2381,31 +2381,31 @@
         </is>
       </c>
       <c r="G29" s="11" t="n">
-        <v>3444</v>
+        <v>3571</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-262773</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-266344</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-269788</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-263108</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="12" t="n">
         <v>-255037</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-244034</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 21-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 22-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,51 +2424,51 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>26867</v>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
+        <v>28776</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="13" t="n">
-        <v>14764</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G30" s="11" t="n">
-        <v>12103</v>
+      <c r="E30" s="14" t="n">
+        <v>46631</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>-17855</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-695019</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-677164</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-689267</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-706775</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="12" t="n">
         <v>-771238</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-799861</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23330.2</v>
+        <v>23454.05</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23466.8</v>
+        <v>23489</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>61749</v>
+        <v>31065</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>61749</v>
+        <v>31065</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23314.8</v>
+        <v>23285.75</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23414.3</v>
+        <v>23329</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23634.46666666666</v>
+        <v>23653.33333333334</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23406.46666666666</v>
+        <v>23348.45833333334</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2597,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v>53154</v>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>-24743</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,43 +2611,43 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>14030</v>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G33" s="13" t="n">
-        <v>39124</v>
+        <v>12085</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>-36828</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="14" t="n">
+      <c r="J33" s="12" t="n">
+        <v>-397348</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-360520</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="12" t="n">
         <v>-399644</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="12" t="n">
         <v>-392641</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="12" t="n">
         <v>-395375</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-447481</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23550.63333333333</v>
+        <v>23571.16666666667</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23398.63333333333</v>
+        <v>23367.91666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>-66</v>
+        <v>-153</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>401</v>
+        <v>927</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,35 +2686,35 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-467</v>
+        <v>-1080</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="14" t="n">
+      <c r="J34" s="12" t="n">
+        <v>19239</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>20319</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="12" t="n">
         <v>20786</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="12" t="n">
         <v>21431</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="12" t="n">
         <v>21007</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>21158</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23482.46666666666</v>
+        <v>23450.08333333334</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23390.8</v>
+        <v>23387.375</v>
       </c>
     </row>
     <row r="35">
@@ -2731,13 +2731,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="13" t="n">
-        <v>7148</v>
+      <c r="C35" s="14" t="n">
+        <v>8036</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,43 +2745,43 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>12278</v>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G35" s="11" t="n">
-        <v>-5130</v>
+        <v>4131</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>3905</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="14" t="n">
+      <c r="J35" s="12" t="n">
+        <v>208180</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>204275</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="12" t="n">
         <v>209405</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="12" t="n">
         <v>194874</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="12" t="n">
         <v>199455</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>197217</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23398.63333333333</v>
+        <v>23367.91666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,13 +2792,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="13" t="n">
-        <v>8273</v>
+      <c r="C36" s="14" t="n">
+        <v>44604</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,43 +2806,43 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>41800</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="n">
-        <v>-33527</v>
+        <v>10601</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>34003</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="14" t="n">
+      <c r="J36" s="12" t="n">
+        <v>169929</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>135926</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="12" t="n">
         <v>169453</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="12" t="n">
         <v>176336</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="12" t="n">
         <v>174913</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>229106</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23330.46666666666</v>
+        <v>23246.83333333334</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>68509</v>
+        <v>27744</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>68509</v>
+        <v>27744</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23246.63333333333</v>
+        <v>23164.66666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23178.46666666666</v>
+        <v>23043.58333333334</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.25</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.39</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>12.29</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>13.17</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>13.43</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9768793036226828</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9805221830332062</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9778148328815047</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9744981133829045</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9721766836399037</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9679688193651542</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,414    PCR(OI) 1.46    Max Pain 23,400</t>
+          <t>Spot 23,329    PCR(OI) 0.88    Max Pain 23,350</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23881.14879032258</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23879.4189516129</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23876.09516129032</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23879.57419354839</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23882.07862903226</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23883.62056451613</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23329</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23414.3</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23346.4</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23270.6</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23217.6</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23118.6</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23500</v>
-      </c>
-      <c r="Q45" s="14" t="n">
-        <v>178853</v>
+        <v>23350</v>
+      </c>
+      <c r="Q45" s="12" t="n">
+        <v>342913</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>36912</v>
-      </c>
-      <c r="S45" s="14" t="n">
-        <v>7146984</v>
+        <v>303410</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>19149392</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.960516959670768</v>
+        <v>0.9570447338803717</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9581623376424576</v>
@@ -3173,20 +3173,20 @@
         <v>0.9933791141865997</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23600</v>
-      </c>
-      <c r="Q46" s="14" t="n">
-        <v>164756</v>
+        <v>23400</v>
+      </c>
+      <c r="Q46" s="12" t="n">
+        <v>318073</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>43079</v>
-      </c>
-      <c r="S46" s="14" t="n">
-        <v>3860663</v>
-      </c>
-      <c r="T46" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>185715</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>26471078</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24376.7689516129</v>
+        <v>24376.0810483871</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24365.80846774194</v>
@@ -3212,20 +3212,20 @@
         <v>24336.7810483871</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>23700</v>
-      </c>
-      <c r="Q47" s="14" t="n">
-        <v>145155</v>
-      </c>
-      <c r="R47" s="13" t="n">
-        <v>-933</v>
-      </c>
-      <c r="S47" s="14" t="n">
-        <v>2459258</v>
-      </c>
-      <c r="T47" s="31" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>23500</v>
+      </c>
+      <c r="Q47" s="12" t="n">
+        <v>196697</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>17844</v>
+      </c>
+      <c r="S47" s="12" t="n">
+        <v>19082903</v>
+      </c>
+      <c r="T47" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23414.3</v>
+        <v>23329</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23346.4</v>
@@ -3250,7 +3250,7 @@
       <c r="N48" s="18" t="n">
         <v>24175.65</v>
       </c>
-      <c r="P48" s="32" t="inlineStr">
+      <c r="P48" s="30" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="30" t="inlineStr">
-        <is>
-          <t>21-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="30" t="inlineStr">
+      <c r="J49" s="31" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="31" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="30" t="inlineStr">
+      <c r="L49" s="31" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="30" t="inlineStr">
+      <c r="M49" s="31" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="N49" s="30" t="inlineStr">
+      <c r="N49" s="31" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
@@ -3318,17 +3318,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
-        <v>23400</v>
-      </c>
-      <c r="Q50" s="14" t="n">
-        <v>247382</v>
+      <c r="P50" s="32" t="n">
+        <v>23350</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>208701</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>173731</v>
-      </c>
-      <c r="S50" s="14" t="n">
-        <v>8115411</v>
+        <v>53445</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>24191120</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3337,38 +3337,38 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="33" t="n">
+      <c r="P51" s="32" t="n">
         <v>23300</v>
       </c>
-      <c r="Q51" s="14" t="n">
-        <v>243496</v>
+      <c r="Q51" s="12" t="n">
+        <v>337341</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>48318</v>
-      </c>
-      <c r="S51" s="14" t="n">
-        <v>5246181</v>
-      </c>
-      <c r="T51" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>93845</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>27406236</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="33" t="n">
+      <c r="P52" s="32" t="n">
         <v>22500</v>
       </c>
-      <c r="Q52" s="14" t="n">
-        <v>191934</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>53126</v>
-      </c>
-      <c r="S52" s="14" t="n">
-        <v>1363091</v>
-      </c>
-      <c r="T52" s="31" t="inlineStr">
+      <c r="Q52" s="12" t="n">
+        <v>176416</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>-15518</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>1021060</v>
+      </c>
+      <c r="T52" s="33" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 21-Sep-2026    1 DAY AGO = 18-Sep-2026    2 DAYS AGO = 17-Sep-2026    3 DAYS AGO = 16-Sep-2026    4 DAYS AGO = 15-Sep-2026    (generated 21-Sep-2026 20:32 IST)</t>
+          <t>TODAY = 22-Sep-2026    1 DAY AGO = 21-Sep-2026    2 DAYS AGO = 18-Sep-2026    3 DAYS AGO = 17-Sep-2026    4 DAYS AGO = 16-Sep-2026    (generated 22-Sep-2026 20:57 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-23
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -190,6 +190,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -198,9 +201,6 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>3992</v>
+        <v>-5466</v>
       </c>
     </row>
     <row r="3">
@@ -701,48 +701,48 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>3787</v>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
+        <v>-6607</v>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E3" s="11" t="n">
-        <v>-205</v>
+      <c r="E3" s="13" t="n">
+        <v>-1141</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>3992</v>
+        <v>-5466</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="14" t="n">
+        <v>240245</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>245711</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="14" t="n">
         <v>241719</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="14" t="n">
         <v>241420</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>238948</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>233302</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>123294</v>
+        <v>-117111</v>
       </c>
     </row>
     <row r="4">
@@ -770,65 +770,65 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+        <v>-979</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="14" t="n">
+      <c r="E4" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>-979</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>12202</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>13181</v>
+      </c>
+      <c r="L4" s="14" t="n">
+        <v>13180</v>
+      </c>
+      <c r="M4" s="14" t="n">
+        <v>12967</v>
+      </c>
+      <c r="N4" s="14" t="n">
+        <v>12858</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>13181</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>13180</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>12967</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>12858</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>12546</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>100686</v>
+      <c r="S4" s="11" t="n">
+        <v>36095</v>
       </c>
     </row>
     <row r="5">
@@ -837,56 +837,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="n">
-        <v>-7474</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>4888</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G5" s="14" t="n">
-        <v>-12362</v>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>354</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>-3941</v>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>4295</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="14" t="n">
+        <v>-298613</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-302908</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="14" t="n">
         <v>-290546</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="14" t="n">
         <v>-288428</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="14" t="n">
         <v>-290041</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-288103</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
+      <c r="Q5" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -896,8 +896,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>11204</v>
+      <c r="S5" s="13" t="n">
+        <v>4202</v>
       </c>
     </row>
     <row r="6">
@@ -906,50 +906,50 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>6237</v>
+      <c r="C6" s="13" t="n">
+        <v>2396</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-2132</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+        <v>246</v>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>8369</v>
+      <c r="G6" s="13" t="n">
+        <v>2150</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
+        <v>46166</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>44016</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>35647</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="14" t="n">
         <v>34041</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="14" t="n">
         <v>38235</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>42255</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -957,7 +957,7 @@
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R6" s="10" t="inlineStr">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>11702</v>
+        <v>-45914</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>2551</v>
+        <v>-4836</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>2551</v>
+        <v>-4836</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-36828</v>
+        <v>37415</v>
       </c>
     </row>
     <row r="8">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>1</v>
+        <v>-979</v>
       </c>
     </row>
     <row r="9">
@@ -1091,67 +1091,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>-1109893</v>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>320821</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>-1233187</v>
+        <v>437932</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>-117111</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>188810</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>305921</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>182627</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <v>233015</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <v>290398</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="12" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>123294</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>305921</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>182627</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>233015</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>290398</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>298330</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>4517</v>
+      <c r="S9" s="13" t="n">
+        <v>288</v>
       </c>
     </row>
     <row r="10">
@@ -1160,50 +1160,50 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
-        <v>3902</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="C10" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n">
-        <v>-615</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="E10" s="13" t="n">
+        <v>-253</v>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>4517</v>
+      <c r="G10" s="13" t="n">
+        <v>288</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
+        <v>10922</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>10634</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>6117</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="14" t="n">
         <v>5619</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="14" t="n">
         <v>4249</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>3576</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>-6371</v>
+        <v>18297</v>
       </c>
     </row>
     <row r="11">
@@ -1229,56 +1229,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="n">
-        <v>-162682</v>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>143614</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>-162664</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G11" s="14" t="n">
-        <v>-18</v>
+        <v>76037</v>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>67577</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="14" t="n">
+        <v>-188797</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-256374</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="14" t="n">
         <v>-256356</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="14" t="n">
         <v>-268402</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="14" t="n">
         <v>-282892</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-288206</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="Q11" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>5601</v>
+      <c r="S11" s="13" t="n">
+        <v>1638</v>
       </c>
     </row>
     <row r="12">
@@ -1298,56 +1298,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>-433669</v>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="n">
+        <v>176138</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>-305877</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G12" s="14" t="n">
-        <v>-127792</v>
+        <v>126893</v>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="n">
+        <v>49245</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="14" t="n">
+        <v>-10935</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>-60180</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <v>67612</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="14" t="n">
         <v>29767</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="14" t="n">
         <v>-11755</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>-13701</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>2582</v>
+      <c r="S12" s="13" t="n">
+        <v>334</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-1702342</v>
+        <v>640608</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-1702343</v>
+        <v>640609</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
+      <c r="Q13" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>-1080</v>
+      <c r="S13" s="13" t="n">
+        <v>-259</v>
       </c>
     </row>
     <row r="14">
@@ -1463,9 +1463,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q14" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>-12362</v>
+      <c r="S14" s="13" t="n">
+        <v>4295</v>
       </c>
     </row>
     <row r="15">
@@ -1485,56 +1485,56 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>-1870981</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>-1971667</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
+        <v>646880</v>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>610785</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="14" t="n">
-        <v>100686</v>
+      <c r="G15" s="11" t="n">
+        <v>36095</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-690960</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-727055</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-827741</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>-796597</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>-712178</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-610634</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q15" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>-18</v>
+      <c r="S15" s="13" t="n">
+        <v>67577</v>
       </c>
     </row>
     <row r="16">
@@ -1554,65 +1554,65 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>-6371</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+        <v>18297</v>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="13" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>18297</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>81486</v>
+      </c>
+      <c r="K16" s="14" t="n">
+        <v>63189</v>
+      </c>
+      <c r="L16" s="14" t="n">
+        <v>69560</v>
+      </c>
+      <c r="M16" s="14" t="n">
+        <v>57285</v>
+      </c>
+      <c r="N16" s="14" t="n">
+        <v>54835</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q16" s="12" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>-6371</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>63189</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>69560</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>57285</v>
-      </c>
-      <c r="M16" s="12" t="n">
-        <v>54835</v>
-      </c>
-      <c r="N16" s="12" t="n">
-        <v>50325</v>
-      </c>
-      <c r="P16" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R16" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>3796</v>
+      <c r="S16" s="13" t="n">
+        <v>-89862</v>
       </c>
     </row>
     <row r="17">
@@ -1623,65 +1623,65 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>-326774</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>-330570</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+        <v>65844</v>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>155706</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>-89862</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>552364</v>
+      </c>
+      <c r="K17" s="14" t="n">
+        <v>642226</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <v>638430</v>
+      </c>
+      <c r="M17" s="14" t="n">
+        <v>630453</v>
+      </c>
+      <c r="N17" s="14" t="n">
+        <v>612710</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>3796</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>642226</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>638430</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>630453</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>612710</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>580162</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>2156</v>
+      <c r="S17" s="13" t="n">
+        <v>2397</v>
       </c>
     </row>
     <row r="18">
@@ -1692,54 +1692,54 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>-707567</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>-609456</v>
+        <v>229522</v>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>194053</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G18" s="11" t="n">
-        <v>-98111</v>
+        <v>35469</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="12" t="n">
+      <c r="J18" s="14" t="n">
+        <v>57109</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>21640</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="14" t="n">
         <v>119751</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="14" t="n">
         <v>108858</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="14" t="n">
         <v>44633</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>-19854</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="9" t="inlineStr">
+      <c r="Q18" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="11" t="n">
-        <v>3571</v>
+      <c r="S18" s="13" t="n">
+        <v>3963</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-2911693</v>
+        <v>960543</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-2911693</v>
+        <v>960544</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q19" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>3905</v>
+      <c r="S19" s="13" t="n">
+        <v>-4740</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
+      <c r="Q20" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>8369</v>
+      <c r="S20" s="13" t="n">
+        <v>2150</v>
       </c>
     </row>
     <row r="21">
@@ -1875,58 +1875,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C21" s="11" t="n">
-        <v>19442</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="C21" s="13" t="n">
+        <v>17903</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
-        <v>8238</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="E21" s="11" t="n">
+        <v>13701</v>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>11204</v>
+      <c r="G21" s="13" t="n">
+        <v>4202</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="14" t="n">
+        <v>3246924</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3242722</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <v>3231518</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="14" t="n">
         <v>3239717</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="14" t="n">
         <v>3228282</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3217004</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-127792</v>
+      <c r="S21" s="13" t="n">
+        <v>49245</v>
       </c>
     </row>
     <row r="22">
@@ -1946,48 +1946,48 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>2849</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
+        <v>-726</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E22" s="11" t="n">
-        <v>-2752</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="E22" s="13" t="n">
+        <v>-2364</v>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>5601</v>
+      <c r="G22" s="13" t="n">
+        <v>1638</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J22" s="14" t="n">
+        <v>-4204254</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-4205892</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="14" t="n">
         <v>-4211493</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="14" t="n">
         <v>-4233591</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="14" t="n">
         <v>-4253368</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4252604</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="Q22" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="11" t="n">
-        <v>-98111</v>
+        <v>35469</v>
       </c>
     </row>
     <row r="23">
@@ -2013,56 +2013,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n">
-        <v>17991</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="C23" s="13" t="n">
+        <v>20318</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n">
-        <v>15835</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="E23" s="11" t="n">
+        <v>17921</v>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>2156</v>
+      <c r="G23" s="13" t="n">
+        <v>2397</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="J23" s="14" t="n">
+        <v>509271</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>506874</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <v>504718</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="14" t="n">
         <v>500795</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="14" t="n">
         <v>539565</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>536077</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-18961</v>
+      <c r="S23" s="11" t="n">
+        <v>-8237</v>
       </c>
     </row>
     <row r="24">
@@ -2082,58 +2082,58 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C24" s="11" t="n">
-        <v>17379</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="C24" s="13" t="n">
+        <v>25174</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>36340</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+      <c r="E24" s="11" t="n">
+        <v>33411</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-18961</v>
+      <c r="G24" s="11" t="n">
+        <v>-8237</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J24" s="14" t="n">
+        <v>448059</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>456296</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="14" t="n">
         <v>475257</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="14" t="n">
         <v>493079</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="14" t="n">
         <v>485521</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>499523</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q24" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>-17855</v>
+      <c r="S24" s="13" t="n">
+        <v>41617</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>57661</v>
+        <v>62669</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>57661</v>
+        <v>62669</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q25" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>34003</v>
+      <c r="S25" s="13" t="n">
+        <v>-32416</v>
       </c>
     </row>
     <row r="26">
@@ -2249,49 +2249,49 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
-        <v>-6942</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="C27" s="11" t="n">
+        <v>-58473</v>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>-18644</v>
+      <c r="E27" s="13" t="n">
+        <v>-12559</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>11702</v>
+        <v>-45914</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>1323045</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>1368959</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>1357257</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="14" t="n">
         <v>1357250</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>1369345</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1423115</v>
       </c>
     </row>
     <row r="28">
@@ -2300,49 +2300,49 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="11" t="n">
-        <v>600</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="C28" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>-1982</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="13" t="n">
+        <v>-326</v>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>2582</v>
+      <c r="G28" s="13" t="n">
+        <v>334</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-410833</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-411167</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-413749</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="14" t="n">
         <v>-398195</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>-399462</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-396840</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2361,51 +2361,51 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>8631</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="n">
-        <v>5060</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
+        <v>-1275</v>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>-5238</v>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G29" s="11" t="n">
-        <v>3571</v>
+      <c r="G29" s="13" t="n">
+        <v>3963</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-258810</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-262773</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-266344</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="14" t="n">
         <v>-269788</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>-263108</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-255037</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 22-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 23-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,57 +2418,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
-        <v>28776</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E30" s="14" t="n">
-        <v>46631</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G30" s="14" t="n">
-        <v>-17855</v>
+      <c r="C30" s="13" t="n">
+        <v>35367</v>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>-6250</v>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>41617</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-653402</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-695019</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-677164</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="14" t="n">
         <v>-689267</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="14" t="n">
         <v>-706775</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-771238</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23454.05</v>
+        <v>23352.15</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23489</v>
+        <v>23466.9</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>31065</v>
+        <v>-24373</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>31065</v>
+        <v>-24373</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23285.75</v>
+        <v>23349.55</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23329</v>
+        <v>23446.8</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23653.33333333334</v>
+        <v>23609.96666666667</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23348.45833333334</v>
+        <v>23433.94166666667</v>
       </c>
     </row>
     <row r="33">
@@ -2599,55 +2599,55 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>-24743</v>
+        <v>34042</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>12085</v>
+        <v>-3373</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-36828</v>
+        <v>37415</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-359933</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-397348</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-360520</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="14" t="n">
         <v>-399644</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="14" t="n">
         <v>-392641</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-395375</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23571.16666666667</v>
+        <v>23538.43333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23367.91666666667</v>
+        <v>23421.08333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2666,55 +2666,55 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>-153</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
+        <v>412</v>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="11" t="n">
-        <v>927</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="E34" s="13" t="n">
+        <v>671</v>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="11" t="n">
-        <v>-1080</v>
+      <c r="G34" s="13" t="n">
+        <v>-259</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>18980</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>19239</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>20319</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="14" t="n">
         <v>20786</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="14" t="n">
         <v>21431</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>21007</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23450.08333333334</v>
+        <v>23492.61666666666</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23387.375</v>
+        <v>23408.225</v>
       </c>
     </row>
     <row r="35">
@@ -2731,57 +2731,57 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C35" s="14" t="n">
-        <v>8036</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="n">
+        <v>-390</v>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="11" t="n">
-        <v>4131</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="n">
-        <v>3905</v>
+      <c r="E35" s="13" t="n">
+        <v>4350</v>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="n">
+        <v>-4740</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>203440</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>208180</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>204275</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="14" t="n">
         <v>209405</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="14" t="n">
         <v>194874</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>199455</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23367.91666666667</v>
+        <v>23421.08333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,57 +2792,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>44604</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="C36" s="11" t="n">
+        <v>10982</v>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
-        <v>10601</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>34003</v>
+      <c r="E36" s="13" t="n">
+        <v>43398</v>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="n">
+        <v>-32416</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>137513</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>169929</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>135926</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="14" t="n">
         <v>169453</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="14" t="n">
         <v>176336</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>174913</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23246.83333333334</v>
+        <v>23375.26666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>27744</v>
+        <v>45046</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>27744</v>
+        <v>45046</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23164.66666666667</v>
+        <v>23303.73333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23043.58333333334</v>
+        <v>23257.91666666666</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.25</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.39</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>12.29</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>13.17</v>
       </c>
     </row>
     <row r="41">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 22-Sep-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 29-Sep-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9815024431531654</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9768793036226828</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9805221830332062</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9778148328815047</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9744981133829045</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9721766836399037</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,329    PCR(OI) 0.88    Max Pain 23,350</t>
+          <t>Spot 23,447    PCR(OI) 1.02    Max Pain 23,500</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23888.68225806452</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23881.14879032258</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23879.4189516129</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23876.09516129032</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23879.57419354839</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23882.07862903226</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23446.8</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23329</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23414.3</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23346.4</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23270.6</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23217.6</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23350</v>
-      </c>
-      <c r="Q45" s="12" t="n">
-        <v>342913</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>303410</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>19149392</v>
+        <v>23500</v>
+      </c>
+      <c r="Q45" s="14" t="n">
+        <v>158186</v>
+      </c>
+      <c r="R45" s="13" t="n">
+        <v>20040</v>
+      </c>
+      <c r="S45" s="14" t="n">
+        <v>2695454</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9570447338803717</v>
+        <v>0.9618398546344451</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9581623376424576</v>
@@ -3173,20 +3173,20 @@
         <v>0.9933791141865997</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23400</v>
-      </c>
-      <c r="Q46" s="12" t="n">
-        <v>318073</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>185715</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>26471078</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>24000</v>
+      </c>
+      <c r="Q46" s="14" t="n">
+        <v>235377</v>
+      </c>
+      <c r="R46" s="13" t="n">
+        <v>17887</v>
+      </c>
+      <c r="S46" s="14" t="n">
+        <v>743158</v>
+      </c>
+      <c r="T46" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24376.0810483871</v>
+        <v>24377.0310483871</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24365.80846774194</v>
@@ -3212,20 +3212,20 @@
         <v>24336.7810483871</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>23500</v>
-      </c>
-      <c r="Q47" s="12" t="n">
-        <v>196697</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>17844</v>
-      </c>
-      <c r="S47" s="12" t="n">
-        <v>19082903</v>
-      </c>
-      <c r="T47" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>25000</v>
+      </c>
+      <c r="Q47" s="14" t="n">
+        <v>181976</v>
+      </c>
+      <c r="R47" s="13" t="n">
+        <v>5912</v>
+      </c>
+      <c r="S47" s="14" t="n">
+        <v>211199</v>
+      </c>
+      <c r="T47" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23329</v>
+        <v>23446.8</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23346.4</v>
@@ -3250,7 +3250,7 @@
       <c r="N48" s="18" t="n">
         <v>24175.65</v>
       </c>
-      <c r="P48" s="30" t="inlineStr">
+      <c r="P48" s="31" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="31" t="inlineStr">
-        <is>
-          <t>22-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="31" t="inlineStr">
+      <c r="J49" s="32" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="32" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="31" t="inlineStr">
+      <c r="L49" s="32" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="31" t="inlineStr">
+      <c r="M49" s="32" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="N49" s="31" t="inlineStr">
+      <c r="N49" s="32" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
@@ -3318,17 +3318,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
-        <v>23350</v>
-      </c>
-      <c r="Q50" s="12" t="n">
-        <v>208701</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>53445</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>24191120</v>
+      <c r="P50" s="33" t="n">
+        <v>23400</v>
+      </c>
+      <c r="Q50" s="14" t="n">
+        <v>178381</v>
+      </c>
+      <c r="R50" s="13" t="n">
+        <v>84357</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>3567548</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3337,38 +3337,38 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="32" t="n">
+      <c r="P51" s="33" t="n">
         <v>23300</v>
       </c>
-      <c r="Q51" s="12" t="n">
-        <v>337341</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>93845</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>27406236</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="Q51" s="14" t="n">
+        <v>141700</v>
+      </c>
+      <c r="R51" s="13" t="n">
+        <v>35187</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>1757172</v>
+      </c>
+      <c r="T51" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>22500</v>
-      </c>
-      <c r="Q52" s="12" t="n">
-        <v>176416</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>-15518</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>1021060</v>
-      </c>
-      <c r="T52" s="33" t="inlineStr">
+      <c r="P52" s="33" t="n">
+        <v>23000</v>
+      </c>
+      <c r="Q52" s="14" t="n">
+        <v>195011.7692307692</v>
+      </c>
+      <c r="R52" s="13" t="n">
+        <v>48608.76923076923</v>
+      </c>
+      <c r="S52" s="14" t="n">
+        <v>890889</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 22-Sep-2026    1 DAY AGO = 21-Sep-2026    2 DAYS AGO = 18-Sep-2026    3 DAYS AGO = 17-Sep-2026    4 DAYS AGO = 16-Sep-2026    (generated 22-Sep-2026 20:57 IST)</t>
+          <t>TODAY = 23-Sep-2026    1 DAY AGO = 22-Sep-2026    2 DAYS AGO = 21-Sep-2026    3 DAYS AGO = 18-Sep-2026    4 DAYS AGO = 17-Sep-2026    (generated 23-Sep-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-24
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -187,7 +187,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,11 +196,11 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-5466</v>
+        <v>5866</v>
       </c>
     </row>
     <row r="3">
@@ -701,27 +701,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-6607</v>
+        <v>16361</v>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E3" s="13" t="n">
-        <v>-1141</v>
+        <v>10495</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-5466</v>
+        <v>5866</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="14" t="n">
+        <v>246111</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>240245</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="14" t="n">
         <v>245711</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="14" t="n">
         <v>241719</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="14" t="n">
         <v>241420</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>238948</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>-117111</v>
+        <v>201934</v>
       </c>
     </row>
     <row r="4">
@@ -770,27 +770,27 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>-979</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
+        <v>8</v>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="E4" s="13" t="n">
+        <v>4764</v>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>-979</v>
+      <c r="G4" s="13" t="n">
+        <v>-4756</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,20 +798,20 @@
         </is>
       </c>
       <c r="J4" s="14" t="n">
+        <v>7446</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>12202</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="14" t="n">
         <v>13181</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="14" t="n">
         <v>13180</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="14" t="n">
         <v>12967</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>12858</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -819,7 +819,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>36095</v>
+        <v>-276540</v>
       </c>
     </row>
     <row r="5">
@@ -837,67 +837,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
-        <v>354</v>
+      <c r="C5" s="11" t="n">
+        <v>3132</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E5" s="13" t="n">
-        <v>-3941</v>
+        <v>14341</v>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>-11209</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>-309822</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>-298613</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>-302908</v>
+      </c>
+      <c r="M5" s="14" t="n">
+        <v>-290546</v>
+      </c>
+      <c r="N5" s="14" t="n">
+        <v>-288428</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n">
-        <v>4295</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="n">
-        <v>-298613</v>
-      </c>
-      <c r="K5" s="14" t="n">
-        <v>-302908</v>
-      </c>
-      <c r="L5" s="14" t="n">
-        <v>-290546</v>
-      </c>
-      <c r="M5" s="14" t="n">
-        <v>-288428</v>
-      </c>
-      <c r="N5" s="14" t="n">
-        <v>-290041</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="13" t="n">
-        <v>4202</v>
+      <c r="S5" s="11" t="n">
+        <v>31425</v>
       </c>
     </row>
     <row r="6">
@@ -906,29 +906,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
-        <v>2396</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="C6" s="11" t="n">
+        <v>14329</v>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
-        <v>246</v>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="E6" s="13" t="n">
+        <v>4230</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="13" t="n">
-        <v>2150</v>
+      <c r="G6" s="11" t="n">
+        <v>10099</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,20 +936,20 @@
         </is>
       </c>
       <c r="J6" s="14" t="n">
+        <v>56265</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>46166</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="14" t="n">
         <v>44016</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="14" t="n">
         <v>35647</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="14" t="n">
         <v>34041</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>38235</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -957,7 +957,7 @@
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R6" s="10" t="inlineStr">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>-45914</v>
+        <v>81592</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-4836</v>
+        <v>33830</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-4836</v>
+        <v>33830</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>37415</v>
+        <v>-67540</v>
       </c>
     </row>
     <row r="8">
@@ -1071,7 +1071,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
+      <c r="Q8" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>-979</v>
+      <c r="S8" s="13" t="n">
+        <v>-4756</v>
       </c>
     </row>
     <row r="9">
@@ -1091,67 +1091,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
-        <v>320821</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="C9" s="11" t="n">
+        <v>1071907</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="11" t="n">
-        <v>437932</v>
+      <c r="E9" s="13" t="n">
+        <v>869973</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>201934</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>390744</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>188810</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>305921</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <v>182627</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <v>233015</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="12" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>-117111</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>188810</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>305921</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>182627</v>
-      </c>
-      <c r="M9" s="14" t="n">
-        <v>233015</v>
-      </c>
-      <c r="N9" s="14" t="n">
-        <v>290398</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S9" s="13" t="n">
-        <v>288</v>
+        <v>-783</v>
       </c>
     </row>
     <row r="10">
@@ -1162,65 +1162,65 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>35</v>
+        <v>-510</v>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E10" s="13" t="n">
-        <v>-253</v>
+        <v>273</v>
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>-783</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="n">
+        <v>10139</v>
+      </c>
+      <c r="K10" s="14" t="n">
+        <v>10922</v>
+      </c>
+      <c r="L10" s="14" t="n">
+        <v>10634</v>
+      </c>
+      <c r="M10" s="14" t="n">
+        <v>6117</v>
+      </c>
+      <c r="N10" s="14" t="n">
+        <v>5619</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q10" s="12" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="13" t="n">
-        <v>288</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J10" s="14" t="n">
-        <v>10922</v>
-      </c>
-      <c r="K10" s="14" t="n">
-        <v>10634</v>
-      </c>
-      <c r="L10" s="14" t="n">
-        <v>6117</v>
-      </c>
-      <c r="M10" s="14" t="n">
-        <v>5619</v>
-      </c>
-      <c r="N10" s="14" t="n">
-        <v>4249</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q10" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>18297</v>
+      <c r="S10" s="13" t="n">
+        <v>1404</v>
       </c>
     </row>
     <row r="11">
@@ -1229,29 +1229,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
-        <v>143614</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="C11" s="11" t="n">
+        <v>179332</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E11" s="11" t="n">
-        <v>76037</v>
+      <c r="E11" s="13" t="n">
+        <v>251528</v>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G11" s="13" t="n">
-        <v>67577</v>
+        <v>-72196</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,20 +1259,20 @@
         </is>
       </c>
       <c r="J11" s="14" t="n">
+        <v>-260993</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-188797</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="14" t="n">
         <v>-256374</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="M11" s="14" t="n">
         <v>-256356</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="14" t="n">
         <v>-268402</v>
       </c>
-      <c r="N11" s="14" t="n">
-        <v>-282892</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1280,7 +1280,7 @@
       </c>
       <c r="Q11" s="12" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="S11" s="13" t="n">
-        <v>1638</v>
+        <v>-4563</v>
       </c>
     </row>
     <row r="12">
@@ -1298,29 +1298,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n">
-        <v>176138</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="C12" s="11" t="n">
+        <v>278692</v>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E12" s="11" t="n">
-        <v>126893</v>
+      <c r="E12" s="13" t="n">
+        <v>407648</v>
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G12" s="13" t="n">
-        <v>49245</v>
+        <v>-128956</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,20 +1328,20 @@
         </is>
       </c>
       <c r="J12" s="14" t="n">
+        <v>-139891</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>-10935</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="14" t="n">
         <v>-60180</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="M12" s="14" t="n">
         <v>67612</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="14" t="n">
         <v>29767</v>
       </c>
-      <c r="N12" s="14" t="n">
-        <v>-11755</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="Q12" s="12" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R12" s="10" t="inlineStr">
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="S12" s="13" t="n">
-        <v>334</v>
+        <v>-877</v>
       </c>
     </row>
     <row r="13">
@@ -1369,11 +1369,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>640608</v>
+        <v>1529421</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>640609</v>
+        <v>1529422</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="Q13" s="12" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="13" t="n">
-        <v>-259</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Q14" s="12" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="13" t="n">
-        <v>4295</v>
+        <v>-11209</v>
       </c>
     </row>
     <row r="15">
@@ -1485,27 +1485,27 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>646880</v>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
+        <v>-105845</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="13" t="n">
-        <v>610785</v>
+      <c r="E15" s="11" t="n">
+        <v>170695</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>36095</v>
+        <v>-276540</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="14" t="n">
+        <v>-967500</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-690960</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="14" t="n">
         <v>-727055</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="14" t="n">
         <v>-827741</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="14" t="n">
         <v>-796597</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-712178</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="Q15" s="12" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="13" t="n">
-        <v>67577</v>
+        <v>-72196</v>
       </c>
     </row>
     <row r="16">
@@ -1552,29 +1552,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>18297</v>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="C16" s="13" t="n">
+        <v>1404</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>18297</v>
+      <c r="G16" s="13" t="n">
+        <v>1404</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="14" t="n">
+        <v>82890</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>81486</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="14" t="n">
         <v>63189</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="14" t="n">
         <v>69560</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="14" t="n">
         <v>57285</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>54835</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="Q16" s="12" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="13" t="n">
-        <v>-89862</v>
+        <v>133789</v>
       </c>
     </row>
     <row r="17">
@@ -1621,67 +1621,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
-        <v>65844</v>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="C17" s="13" t="n">
+        <v>176700</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="13" t="n">
-        <v>155706</v>
+      <c r="E17" s="11" t="n">
+        <v>42911</v>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>133789</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>686153</v>
+      </c>
+      <c r="K17" s="14" t="n">
+        <v>552364</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <v>642226</v>
+      </c>
+      <c r="M17" s="14" t="n">
+        <v>638430</v>
+      </c>
+      <c r="N17" s="14" t="n">
+        <v>630453</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="12" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
-        <v>-89862</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="14" t="n">
-        <v>552364</v>
-      </c>
-      <c r="K17" s="14" t="n">
-        <v>642226</v>
-      </c>
-      <c r="L17" s="14" t="n">
-        <v>638430</v>
-      </c>
-      <c r="M17" s="14" t="n">
-        <v>630453</v>
-      </c>
-      <c r="N17" s="14" t="n">
-        <v>612710</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S17" s="13" t="n">
-        <v>2397</v>
+        <v>-27191</v>
       </c>
     </row>
     <row r="18">
@@ -1690,29 +1690,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n">
-        <v>229522</v>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="C18" s="13" t="n">
+        <v>163967</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="13" t="n">
-        <v>194053</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="E18" s="11" t="n">
+        <v>22619</v>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>35469</v>
+      <c r="G18" s="13" t="n">
+        <v>141348</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,20 +1720,20 @@
         </is>
       </c>
       <c r="J18" s="14" t="n">
+        <v>198457</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>57109</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="14" t="n">
         <v>21640</v>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="M18" s="14" t="n">
         <v>119751</v>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="N18" s="14" t="n">
         <v>108858</v>
       </c>
-      <c r="N18" s="14" t="n">
-        <v>44633</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="Q18" s="12" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R18" s="10" t="inlineStr">
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="S18" s="13" t="n">
-        <v>3963</v>
+        <v>-36877</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>960543</v>
+        <v>236226</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>960544</v>
+        <v>236225</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Q19" s="12" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="13" t="n">
-        <v>-4740</v>
+        <v>34491</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="12" t="inlineStr">
+      <c r="Q20" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="13" t="n">
-        <v>2150</v>
+      <c r="S20" s="11" t="n">
+        <v>10099</v>
       </c>
     </row>
     <row r="21">
@@ -1875,29 +1875,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n">
-        <v>17903</v>
+      <c r="C21" s="11" t="n">
+        <v>15837</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>13701</v>
-      </c>
-      <c r="F21" s="12" t="inlineStr">
+        <v>-15588</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="13" t="n">
-        <v>4202</v>
+      <c r="G21" s="11" t="n">
+        <v>31425</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,20 +1905,20 @@
         </is>
       </c>
       <c r="J21" s="14" t="n">
+        <v>3278349</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3246924</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="14" t="n">
         <v>3242722</v>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="M21" s="14" t="n">
         <v>3231518</v>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="N21" s="14" t="n">
         <v>3239717</v>
       </c>
-      <c r="N21" s="14" t="n">
-        <v>3228282</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="Q21" s="12" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="S21" s="13" t="n">
-        <v>49245</v>
+        <v>-128956</v>
       </c>
     </row>
     <row r="22">
@@ -1944,67 +1944,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
-        <v>-726</v>
+      <c r="C22" s="13" t="n">
+        <v>-1676</v>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E22" s="13" t="n">
-        <v>-2364</v>
+        <v>2887</v>
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>-4563</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>-4208817</v>
+      </c>
+      <c r="K22" s="14" t="n">
+        <v>-4204254</v>
+      </c>
+      <c r="L22" s="14" t="n">
+        <v>-4205892</v>
+      </c>
+      <c r="M22" s="14" t="n">
+        <v>-4211493</v>
+      </c>
+      <c r="N22" s="14" t="n">
+        <v>-4233591</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q22" s="12" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="13" t="n">
-        <v>1638</v>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J22" s="14" t="n">
-        <v>-4204254</v>
-      </c>
-      <c r="K22" s="14" t="n">
-        <v>-4205892</v>
-      </c>
-      <c r="L22" s="14" t="n">
-        <v>-4211493</v>
-      </c>
-      <c r="M22" s="14" t="n">
-        <v>-4233591</v>
-      </c>
-      <c r="N22" s="14" t="n">
-        <v>-4253368</v>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>35469</v>
+      <c r="S22" s="13" t="n">
+        <v>141348</v>
       </c>
     </row>
     <row r="23">
@@ -2015,65 +2015,65 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C23" s="13" t="n">
-        <v>20318</v>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+        <v>-26305</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="11" t="n">
-        <v>17921</v>
+      <c r="E23" s="13" t="n">
+        <v>886</v>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="n">
+        <v>-27191</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="n">
+        <v>482080</v>
+      </c>
+      <c r="K23" s="14" t="n">
+        <v>509271</v>
+      </c>
+      <c r="L23" s="14" t="n">
+        <v>506874</v>
+      </c>
+      <c r="M23" s="14" t="n">
+        <v>504718</v>
+      </c>
+      <c r="N23" s="14" t="n">
+        <v>500795</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="13" t="n">
-        <v>2397</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="14" t="n">
-        <v>509271</v>
-      </c>
-      <c r="K23" s="14" t="n">
-        <v>506874</v>
-      </c>
-      <c r="L23" s="14" t="n">
-        <v>504718</v>
-      </c>
-      <c r="M23" s="14" t="n">
-        <v>500795</v>
-      </c>
-      <c r="N23" s="14" t="n">
-        <v>539565</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>-8237</v>
+        <v>329</v>
       </c>
     </row>
     <row r="24">
@@ -2084,65 +2084,65 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C24" s="13" t="n">
-        <v>25174</v>
+        <v>-8789</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E24" s="11" t="n">
-        <v>33411</v>
+        <v>-9118</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>329</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="n">
+        <v>448388</v>
+      </c>
+      <c r="K24" s="14" t="n">
+        <v>448059</v>
+      </c>
+      <c r="L24" s="14" t="n">
+        <v>456296</v>
+      </c>
+      <c r="M24" s="14" t="n">
+        <v>475257</v>
+      </c>
+      <c r="N24" s="14" t="n">
+        <v>493079</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q24" s="12" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>-8237</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="14" t="n">
-        <v>448059</v>
-      </c>
-      <c r="K24" s="14" t="n">
-        <v>456296</v>
-      </c>
-      <c r="L24" s="14" t="n">
-        <v>475257</v>
-      </c>
-      <c r="M24" s="14" t="n">
-        <v>493079</v>
-      </c>
-      <c r="N24" s="14" t="n">
-        <v>485521</v>
-      </c>
-      <c r="P24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q24" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S24" s="13" t="n">
-        <v>41617</v>
+        <v>-43838</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>62669</v>
+        <v>-20933</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>62669</v>
+        <v>-20933</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="12" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="13" t="n">
-        <v>-32416</v>
+        <v>33044</v>
       </c>
     </row>
     <row r="26">
@@ -2251,27 +2251,27 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>-58473</v>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
+        <v>38257</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E27" s="13" t="n">
-        <v>-12559</v>
+      <c r="E27" s="11" t="n">
+        <v>-43335</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>-45914</v>
+        <v>81592</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="14" t="n">
+        <v>1404637</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>1323045</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="14" t="n">
         <v>1368959</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="14" t="n">
         <v>1357257</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="14" t="n">
         <v>1357250</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>1369345</v>
       </c>
     </row>
     <row r="28">
@@ -2302,27 +2302,27 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C28" s="13" t="n">
-        <v>8</v>
+        <v>-433</v>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E28" s="13" t="n">
-        <v>-326</v>
+        <v>444</v>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G28" s="13" t="n">
-        <v>334</v>
+        <v>-877</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="14" t="n">
+        <v>-411710</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-410833</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="14" t="n">
         <v>-411167</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="14" t="n">
         <v>-413749</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="14" t="n">
         <v>-398195</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-399462</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
-        <v>-1275</v>
+      <c r="C29" s="13" t="n">
+        <v>-13206</v>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E29" s="13" t="n">
-        <v>-5238</v>
+        <v>23671</v>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G29" s="13" t="n">
-        <v>3963</v>
+        <v>-36877</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="14" t="n">
+        <v>-295687</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-258810</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="14" t="n">
         <v>-262773</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="14" t="n">
         <v>-266344</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="14" t="n">
         <v>-269788</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-263108</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 23-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 24-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,29 +2418,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="13" t="n">
-        <v>35367</v>
+      <c r="C30" s="11" t="n">
+        <v>30263</v>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E30" s="13" t="n">
-        <v>-6250</v>
+        <v>74101</v>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G30" s="13" t="n">
-        <v>41617</v>
+        <v>-43838</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="14" t="n">
+        <v>-697240</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-653402</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="14" t="n">
         <v>-695019</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="14" t="n">
         <v>-677164</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="14" t="n">
         <v>-689267</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-706775</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23352.15</v>
+        <v>23221.8</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23466.9</v>
+        <v>23281.95</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-24373</v>
+        <v>54881</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-24373</v>
+        <v>54881</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23349.55</v>
+        <v>23046.15</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23446.8</v>
+        <v>23063.1</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23609.96666666667</v>
+        <v>23450.45000000001</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23433.94166666667</v>
+        <v>23096.75000000001</v>
       </c>
     </row>
     <row r="33">
@@ -2599,27 +2599,27 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>34042</v>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
+        <v>-76910</v>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E33" s="11" t="n">
-        <v>-3373</v>
+      <c r="E33" s="13" t="n">
+        <v>-9370</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>37415</v>
+        <v>-67540</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="14" t="n">
+        <v>-427473</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-359933</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="14" t="n">
         <v>-397348</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="14" t="n">
         <v>-360520</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="14" t="n">
         <v>-399644</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-392641</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23538.43333333333</v>
+        <v>23366.2</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23421.08333333333</v>
+        <v>23130.40000000001</v>
       </c>
     </row>
     <row r="34">
@@ -2664,29 +2664,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>412</v>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="C34" s="13" t="n">
+        <v>1713</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="13" t="n">
-        <v>671</v>
+      <c r="E34" s="11" t="n">
+        <v>1708</v>
       </c>
       <c r="F34" s="12" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-259</v>
+        <v>5</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="14" t="n">
+        <v>18985</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>18980</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="14" t="n">
         <v>19239</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="14" t="n">
         <v>20319</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="14" t="n">
         <v>20786</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>21431</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23492.61666666666</v>
+        <v>23214.65000000001</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23408.225</v>
+        <v>23164.05</v>
       </c>
     </row>
     <row r="35">
@@ -2733,27 +2733,27 @@
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C35" s="13" t="n">
-        <v>-390</v>
+        <v>17836</v>
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E35" s="13" t="n">
-        <v>4350</v>
+        <v>-16655</v>
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-4740</v>
+        <v>34491</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="14" t="n">
+        <v>237931</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>203440</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="14" t="n">
         <v>208180</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="14" t="n">
         <v>204275</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="14" t="n">
         <v>209405</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>194874</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23421.08333333333</v>
+        <v>23130.40000000001</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,29 +2792,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>10982</v>
-      </c>
-      <c r="D36" s="12" t="inlineStr">
+      <c r="C36" s="13" t="n">
+        <v>66916</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="13" t="n">
-        <v>43398</v>
+      <c r="E36" s="11" t="n">
+        <v>33872</v>
       </c>
       <c r="F36" s="12" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-32416</v>
+        <v>33044</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="14" t="n">
+        <v>170557</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>137513</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="14" t="n">
         <v>169929</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="14" t="n">
         <v>135926</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="14" t="n">
         <v>169453</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>176336</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23375.26666666666</v>
+        <v>22978.85000000001</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>45046</v>
+        <v>9555</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>45046</v>
+        <v>9555</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23303.73333333333</v>
+        <v>22894.60000000001</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23257.91666666666</v>
+        <v>22743.05000000001</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>12.69</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>10.35</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.25</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.39</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>12.29</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9653913300442524</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9815024431531654</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9768793036226828</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9805221830332062</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9778148328815047</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9744981133829045</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,447    PCR(OI) 1.02    Max Pain 23,500</t>
+          <t>Spot 23,063    PCR(OI) 0.72    Max Pain 23,300</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23889.89758064516</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23888.68225806452</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23881.14879032258</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23879.4189516129</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23876.09516129032</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23879.57419354839</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23063.1</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23446.8</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23329</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23414.3</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23346.4</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23270.6</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3137,17 +3137,17 @@
         <v>23500</v>
       </c>
       <c r="Q45" s="14" t="n">
-        <v>158186</v>
-      </c>
-      <c r="R45" s="13" t="n">
-        <v>20040</v>
+        <v>208801</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>50615</v>
       </c>
       <c r="S45" s="14" t="n">
-        <v>2695454</v>
+        <v>1321364</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9618398546344451</v>
+        <v>0.9462197383200984</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9581623376424576</v>
@@ -3176,17 +3176,17 @@
         <v>24000</v>
       </c>
       <c r="Q46" s="14" t="n">
-        <v>235377</v>
-      </c>
-      <c r="R46" s="13" t="n">
-        <v>17887</v>
+        <v>298613</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>63236</v>
       </c>
       <c r="S46" s="14" t="n">
-        <v>743158</v>
-      </c>
-      <c r="T46" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>1144027</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24377.0310483871</v>
+        <v>24373.93669354838</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24365.80846774194</v>
@@ -3212,16 +3212,16 @@
         <v>24336.7810483871</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>25000</v>
+        <v>24500</v>
       </c>
       <c r="Q47" s="14" t="n">
-        <v>181976</v>
-      </c>
-      <c r="R47" s="13" t="n">
-        <v>5912</v>
+        <v>195348</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>58611</v>
       </c>
       <c r="S47" s="14" t="n">
-        <v>211199</v>
+        <v>649177</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23446.8</v>
+        <v>23063.1</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23346.4</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="32" t="inlineStr">
-        <is>
-          <t>23-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="32" t="inlineStr">
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="32" t="inlineStr">
+      <c r="L49" s="29" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="32" t="inlineStr">
+      <c r="M49" s="29" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="N49" s="32" t="inlineStr">
+      <c r="N49" s="29" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
@@ -3318,55 +3318,55 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
-        <v>23400</v>
+      <c r="P50" s="32" t="n">
+        <v>23000</v>
       </c>
       <c r="Q50" s="14" t="n">
-        <v>178381</v>
+        <v>180885.3846153846</v>
       </c>
       <c r="R50" s="13" t="n">
-        <v>84357</v>
+        <v>-14126.38461538462</v>
       </c>
       <c r="S50" s="14" t="n">
-        <v>3567548</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
+        <v>2432163</v>
+      </c>
+      <c r="T50" s="33" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="33" t="n">
-        <v>23300</v>
+      <c r="P51" s="32" t="n">
+        <v>22000</v>
       </c>
       <c r="Q51" s="14" t="n">
-        <v>141700</v>
-      </c>
-      <c r="R51" s="13" t="n">
-        <v>35187</v>
+        <v>186656</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>73837</v>
       </c>
       <c r="S51" s="14" t="n">
-        <v>1757172</v>
-      </c>
-      <c r="T51" s="32" t="inlineStr">
+        <v>859869</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="33" t="n">
-        <v>23000</v>
+      <c r="P52" s="32" t="n">
+        <v>21000</v>
       </c>
       <c r="Q52" s="14" t="n">
-        <v>195011.7692307692</v>
-      </c>
-      <c r="R52" s="13" t="n">
-        <v>48608.76923076923</v>
+        <v>170050</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>30670</v>
       </c>
       <c r="S52" s="14" t="n">
-        <v>890889</v>
+        <v>283218</v>
       </c>
       <c r="T52" s="30" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 23-Sep-2026    1 DAY AGO = 22-Sep-2026    2 DAYS AGO = 21-Sep-2026    3 DAYS AGO = 18-Sep-2026    4 DAYS AGO = 17-Sep-2026    (generated 23-Sep-2026 20:32 IST)</t>
+          <t>TODAY = 24-Sep-2026    1 DAY AGO = 23-Sep-2026    2 DAYS AGO = 22-Sep-2026    3 DAYS AGO = 21-Sep-2026    4 DAYS AGO = 18-Sep-2026    (generated 24-Sep-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-25
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,13 +187,13 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>5866</v>
+        <v>-1712</v>
       </c>
     </row>
     <row r="3">
@@ -701,48 +701,48 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>16361</v>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
+        <v>-280</v>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E3" s="13" t="n">
-        <v>10495</v>
+      <c r="E3" s="11" t="n">
+        <v>1432</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>5866</v>
+        <v>-1712</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>244399</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>246111</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>240245</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>245711</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="12" t="n">
         <v>241719</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>241420</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>201934</v>
+        <v>-217249</v>
       </c>
     </row>
     <row r="4">
@@ -768,50 +768,50 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C4" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="C4" s="14" t="n">
+        <v>214</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="13" t="n">
-        <v>4764</v>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
+      <c r="E4" s="11" t="n">
+        <v>1089</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="13" t="n">
-        <v>-4756</v>
+      <c r="G4" s="11" t="n">
+        <v>-875</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="12" t="n">
+        <v>6571</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>7446</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="12" t="n">
         <v>12202</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="12" t="n">
         <v>13181</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="12" t="n">
         <v>13180</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>12967</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -819,7 +819,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-276540</v>
+        <v>25090</v>
       </c>
     </row>
     <row r="5">
@@ -837,56 +837,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="11" t="n">
-        <v>3132</v>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="C5" s="14" t="n">
+        <v>2562</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
-        <v>14341</v>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="E5" s="11" t="n">
+        <v>4741</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n">
-        <v>-11209</v>
+      <c r="G5" s="11" t="n">
+        <v>-2179</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="14" t="n">
+      <c r="J5" s="12" t="n">
+        <v>-312001</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-309822</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="12" t="n">
         <v>-298613</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="12" t="n">
         <v>-302908</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="N5" s="12" t="n">
         <v>-290546</v>
       </c>
-      <c r="N5" s="14" t="n">
-        <v>-288428</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
+      <c r="Q5" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -896,8 +896,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>31425</v>
+      <c r="S5" s="14" t="n">
+        <v>16335</v>
       </c>
     </row>
     <row r="6">
@@ -906,50 +906,50 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>14329</v>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="n">
-        <v>4230</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="C6" s="14" t="n">
+        <v>4142</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>-624</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>10099</v>
+      <c r="G6" s="14" t="n">
+        <v>4766</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="12" t="n">
+        <v>61031</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>56265</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="12" t="n">
         <v>46166</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>44016</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="12" t="n">
         <v>35647</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>34041</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -957,7 +957,7 @@
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R6" s="10" t="inlineStr">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>81592</v>
+        <v>-76852</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>33830</v>
+        <v>6638</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>33830</v>
+        <v>6638</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-67540</v>
+        <v>60557</v>
       </c>
     </row>
     <row r="8">
@@ -1071,7 +1071,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="12" t="inlineStr">
+      <c r="Q8" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="13" t="n">
-        <v>-4756</v>
+      <c r="S8" s="11" t="n">
+        <v>-875</v>
       </c>
     </row>
     <row r="9">
@@ -1093,65 +1093,65 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>1071907</v>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
+        <v>-180855</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="13" t="n">
-        <v>869973</v>
+      <c r="E9" s="11" t="n">
+        <v>36394</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>-217249</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>173495</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>390744</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>188810</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>305921</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>182627</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>201934</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>390744</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>188810</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>305921</v>
-      </c>
-      <c r="M9" s="14" t="n">
-        <v>182627</v>
-      </c>
-      <c r="N9" s="14" t="n">
-        <v>233015</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="13" t="n">
-        <v>-783</v>
+      <c r="S9" s="14" t="n">
+        <v>259</v>
       </c>
     </row>
     <row r="10">
@@ -1160,67 +1160,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="n">
-        <v>-510</v>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>350</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="13" t="n">
-        <v>273</v>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="n">
+        <v>91</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>259</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>10398</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>10139</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>10922</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>10634</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>6117</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="13" t="n">
-        <v>-783</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J10" s="14" t="n">
-        <v>10139</v>
-      </c>
-      <c r="K10" s="14" t="n">
-        <v>10922</v>
-      </c>
-      <c r="L10" s="14" t="n">
-        <v>10634</v>
-      </c>
-      <c r="M10" s="14" t="n">
-        <v>6117</v>
-      </c>
-      <c r="N10" s="14" t="n">
-        <v>5619</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q10" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="13" t="n">
-        <v>1404</v>
+      <c r="S10" s="14" t="n">
+        <v>-4223</v>
       </c>
     </row>
     <row r="11">
@@ -1231,65 +1231,65 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>179332</v>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>251528</v>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
+        <v>-27687</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>-47711</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>20024</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-240969</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-260993</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-188797</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-256374</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-256356</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="13" t="n">
-        <v>-72196</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="14" t="n">
-        <v>-260993</v>
-      </c>
-      <c r="K11" s="14" t="n">
-        <v>-188797</v>
-      </c>
-      <c r="L11" s="14" t="n">
-        <v>-256374</v>
-      </c>
-      <c r="M11" s="14" t="n">
-        <v>-256356</v>
-      </c>
-      <c r="N11" s="14" t="n">
-        <v>-268402</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="13" t="n">
-        <v>-4563</v>
+      <c r="S11" s="11" t="n">
+        <v>-21936</v>
       </c>
     </row>
     <row r="12">
@@ -1298,67 +1298,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>278692</v>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>407648</v>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
+      <c r="C12" s="14" t="n">
+        <v>118321</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>-78647</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>196968</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>57077</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>-139891</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>-10935</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>-60180</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>67612</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="13" t="n">
-        <v>-128956</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="n">
-        <v>-139891</v>
-      </c>
-      <c r="K12" s="14" t="n">
-        <v>-10935</v>
-      </c>
-      <c r="L12" s="14" t="n">
-        <v>-60180</v>
-      </c>
-      <c r="M12" s="14" t="n">
-        <v>67612</v>
-      </c>
-      <c r="N12" s="14" t="n">
-        <v>29767</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="13" t="n">
-        <v>-877</v>
+      <c r="S12" s="11" t="n">
+        <v>-2375</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1529421</v>
+        <v>-89871</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1529422</v>
+        <v>-89873</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,9 +1394,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q13" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="13" t="n">
-        <v>5</v>
+      <c r="S13" s="14" t="n">
+        <v>-2085</v>
       </c>
     </row>
     <row r="14">
@@ -1463,7 +1463,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="12" t="inlineStr">
+      <c r="Q14" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="13" t="n">
-        <v>-11209</v>
+      <c r="S14" s="11" t="n">
+        <v>-2179</v>
       </c>
     </row>
     <row r="15">
@@ -1485,56 +1485,56 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>-105845</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
+        <v>506024</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="11" t="n">
-        <v>170695</v>
+      <c r="E15" s="14" t="n">
+        <v>480934</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-276540</v>
+        <v>25090</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="12" t="n">
+        <v>-942410</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-967500</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="12" t="n">
         <v>-690960</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="12" t="n">
         <v>-727055</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="12" t="n">
         <v>-827741</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-796597</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="13" t="n">
-        <v>-72196</v>
+      <c r="S15" s="14" t="n">
+        <v>20024</v>
       </c>
     </row>
     <row r="16">
@@ -1552,58 +1552,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>1404</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>-4223</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="n">
-        <v>1404</v>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>-4223</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="14" t="n">
+      <c r="J16" s="12" t="n">
+        <v>78667</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>82890</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="12" t="n">
         <v>81486</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="12" t="n">
         <v>63189</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="12" t="n">
         <v>69560</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>57285</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="13" t="n">
-        <v>133789</v>
+      <c r="S16" s="14" t="n">
+        <v>-2370</v>
       </c>
     </row>
     <row r="17">
@@ -1621,67 +1621,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="13" t="n">
-        <v>176700</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="C17" s="11" t="n">
+        <v>92342</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n">
-        <v>42911</v>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="E17" s="14" t="n">
+        <v>94712</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>-2370</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>683783</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>686153</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>552364</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>642226</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>638430</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
-        <v>133789</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="14" t="n">
-        <v>686153</v>
-      </c>
-      <c r="K17" s="14" t="n">
-        <v>552364</v>
-      </c>
-      <c r="L17" s="14" t="n">
-        <v>642226</v>
-      </c>
-      <c r="M17" s="14" t="n">
-        <v>638430</v>
-      </c>
-      <c r="N17" s="14" t="n">
-        <v>630453</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="13" t="n">
-        <v>-27191</v>
+      <c r="S17" s="14" t="n">
+        <v>12931</v>
       </c>
     </row>
     <row r="18">
@@ -1690,56 +1690,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="13" t="n">
-        <v>163967</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="C18" s="11" t="n">
+        <v>187399</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
-        <v>22619</v>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G18" s="13" t="n">
-        <v>141348</v>
+      <c r="E18" s="14" t="n">
+        <v>205895</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>-18496</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="14" t="n">
+      <c r="J18" s="12" t="n">
+        <v>179961</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>198457</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="12" t="n">
         <v>57109</v>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="M18" s="12" t="n">
         <v>21640</v>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="N18" s="12" t="n">
         <v>119751</v>
       </c>
-      <c r="N18" s="14" t="n">
-        <v>108858</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="12" t="inlineStr">
+      <c r="Q18" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="13" t="n">
-        <v>-36877</v>
+      <c r="S18" s="11" t="n">
+        <v>-7207</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>236226</v>
+        <v>781542</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>236225</v>
+        <v>781541</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="13" t="n">
-        <v>34491</v>
+      <c r="S19" s="14" t="n">
+        <v>-4103</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>10099</v>
+      <c r="S20" s="14" t="n">
+        <v>4766</v>
       </c>
     </row>
     <row r="21">
@@ -1875,58 +1875,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C21" s="11" t="n">
-        <v>15837</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="C21" s="14" t="n">
+        <v>12538</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>-15588</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="E21" s="14" t="n">
+        <v>-3797</v>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>31425</v>
+      <c r="G21" s="14" t="n">
+        <v>16335</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="14" t="n">
+      <c r="J21" s="12" t="n">
+        <v>3294684</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3278349</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="12" t="n">
         <v>3246924</v>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="M21" s="12" t="n">
         <v>3242722</v>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="N21" s="12" t="n">
         <v>3231518</v>
       </c>
-      <c r="N21" s="14" t="n">
-        <v>3239717</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="13" t="n">
-        <v>-128956</v>
+      <c r="S21" s="14" t="n">
+        <v>196968</v>
       </c>
     </row>
     <row r="22">
@@ -1944,58 +1944,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="13" t="n">
-        <v>-1676</v>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>8951</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="13" t="n">
-        <v>2887</v>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="n">
+        <v>30887</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="13" t="n">
-        <v>-4563</v>
+      <c r="G22" s="11" t="n">
+        <v>-21936</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="14" t="n">
+      <c r="J22" s="12" t="n">
+        <v>-4230753</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4208817</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4204254</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4205892</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4211493</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-4233591</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="13" t="n">
-        <v>141348</v>
+      <c r="S22" s="14" t="n">
+        <v>-18496</v>
       </c>
     </row>
     <row r="23">
@@ -2013,67 +2013,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="13" t="n">
-        <v>-26305</v>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>28212</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="13" t="n">
-        <v>886</v>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="E23" s="11" t="n">
+        <v>15281</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>12931</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>495011</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>482080</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>509271</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>506874</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>504718</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="13" t="n">
-        <v>-27191</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="14" t="n">
-        <v>482080</v>
-      </c>
-      <c r="K23" s="14" t="n">
-        <v>509271</v>
-      </c>
-      <c r="L23" s="14" t="n">
-        <v>506874</v>
-      </c>
-      <c r="M23" s="14" t="n">
-        <v>504718</v>
-      </c>
-      <c r="N23" s="14" t="n">
-        <v>500795</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>329</v>
+        <v>-7330</v>
       </c>
     </row>
     <row r="24">
@@ -2082,67 +2082,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="n">
-        <v>-8789</v>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>3188</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E24" s="11" t="n">
-        <v>-9118</v>
+        <v>10518</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>-7330</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="n">
+        <v>441058</v>
+      </c>
+      <c r="K24" s="12" t="n">
+        <v>448388</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>448059</v>
+      </c>
+      <c r="M24" s="12" t="n">
+        <v>456296</v>
+      </c>
+      <c r="N24" s="12" t="n">
+        <v>475257</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q24" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>329</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="14" t="n">
-        <v>448388</v>
-      </c>
-      <c r="K24" s="14" t="n">
-        <v>448059</v>
-      </c>
-      <c r="L24" s="14" t="n">
-        <v>456296</v>
-      </c>
-      <c r="M24" s="14" t="n">
-        <v>475257</v>
-      </c>
-      <c r="N24" s="14" t="n">
-        <v>493079</v>
-      </c>
-      <c r="P24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q24" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="13" t="n">
-        <v>-43838</v>
+      <c r="S24" s="14" t="n">
+        <v>86434</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-20933</v>
+        <v>52889</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-20933</v>
+        <v>52889</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="13" t="n">
-        <v>33044</v>
+      <c r="S25" s="14" t="n">
+        <v>-54369</v>
       </c>
     </row>
     <row r="26">
@@ -2251,47 +2251,47 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>38257</v>
+        <v>-69960</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E27" s="11" t="n">
-        <v>-43335</v>
+        <v>6892</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>81592</v>
+        <v>-76852</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>1327785</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1404637</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>1323045</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>1368959</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="12" t="n">
         <v>1357257</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>1357250</v>
       </c>
     </row>
     <row r="28">
@@ -2300,49 +2300,49 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C28" s="13" t="n">
-        <v>-433</v>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="C28" s="11" t="n">
+        <v>-215</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="13" t="n">
-        <v>444</v>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="n">
+        <v>2160</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="13" t="n">
-        <v>-877</v>
+      <c r="G28" s="11" t="n">
+        <v>-2375</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-414085</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-411710</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-410833</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-411167</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="12" t="n">
         <v>-413749</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-398195</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,53 +2359,53 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C29" s="13" t="n">
-        <v>-13206</v>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="n">
-        <v>23671</v>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>-19100</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>-11893</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="13" t="n">
-        <v>-36877</v>
+      <c r="G29" s="11" t="n">
+        <v>-7207</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-302894</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-295687</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-258810</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-262773</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="12" t="n">
         <v>-266344</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-269788</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 24-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 25-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,57 +2418,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
-        <v>30263</v>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="n">
-        <v>74101</v>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="n">
-        <v>-43838</v>
+      <c r="C30" s="14" t="n">
+        <v>33817</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>-52617</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>86434</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-610806</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-697240</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-653402</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-695019</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="12" t="n">
         <v>-677164</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-689267</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23221.8</v>
+        <v>23035</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23281.95</v>
+        <v>23162.7</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>54881</v>
+        <v>-55458</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>54881</v>
+        <v>-55458</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23046.15</v>
+        <v>23020.95</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23063.1</v>
+        <v>23140.5</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23450.45000000001</v>
+        <v>23336.9</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23096.75000000001</v>
+        <v>23124.275</v>
       </c>
     </row>
     <row r="33">
@@ -2599,55 +2599,55 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>-76910</v>
-      </c>
-      <c r="D33" s="12" t="inlineStr">
+        <v>46335</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E33" s="13" t="n">
-        <v>-9370</v>
+      <c r="E33" s="11" t="n">
+        <v>-14222</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-67540</v>
+        <v>60557</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="14" t="n">
+      <c r="J33" s="12" t="n">
+        <v>-366916</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-427473</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="12" t="n">
         <v>-359933</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="12" t="n">
         <v>-397348</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="12" t="n">
         <v>-360520</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-399644</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23366.2</v>
+        <v>23249.8</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23130.40000000001</v>
+        <v>23108.05</v>
       </c>
     </row>
     <row r="34">
@@ -2664,57 +2664,57 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C34" s="13" t="n">
-        <v>1713</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="n">
+        <v>-1794</v>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="11" t="n">
-        <v>1708</v>
-      </c>
-      <c r="F34" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G34" s="13" t="n">
-        <v>5</v>
+      <c r="E34" s="14" t="n">
+        <v>291</v>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>-2085</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="14" t="n">
+      <c r="J34" s="12" t="n">
+        <v>16900</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>18985</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="12" t="n">
         <v>18980</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="12" t="n">
         <v>19239</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="12" t="n">
         <v>20319</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>20786</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23214.65000000001</v>
+        <v>23195.15</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23164.05</v>
+        <v>23091.825</v>
       </c>
     </row>
     <row r="35">
@@ -2731,57 +2731,57 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C35" s="13" t="n">
-        <v>17836</v>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E35" s="13" t="n">
-        <v>-16655</v>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G35" s="13" t="n">
-        <v>34491</v>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="n">
+        <v>-3744</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="n">
+        <v>359</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>-4103</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="14" t="n">
+      <c r="J35" s="12" t="n">
+        <v>233828</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>237931</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="12" t="n">
         <v>203440</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="12" t="n">
         <v>208180</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="12" t="n">
         <v>204275</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>209405</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23130.40000000001</v>
+        <v>23108.05</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,57 +2792,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C36" s="13" t="n">
-        <v>66916</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="n">
+        <v>-7951</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
-        <v>33872</v>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="13" t="n">
-        <v>33044</v>
+      <c r="E36" s="14" t="n">
+        <v>46418</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>-54369</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="14" t="n">
+      <c r="J36" s="12" t="n">
+        <v>116188</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>170557</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="12" t="n">
         <v>137513</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="12" t="n">
         <v>169929</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="12" t="n">
         <v>135926</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>169453</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22978.85000000001</v>
+        <v>23053.4</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>9555</v>
+        <v>32846</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>9555</v>
+        <v>32846</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22894.60000000001</v>
+        <v>22966.3</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22743.05000000001</v>
+        <v>22911.65</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>12.69</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>10.35</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.25</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.39</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9686854587751691</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9653913300442524</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9815024431531654</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9768793036226828</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9805221830332062</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9778148328815047</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,063    PCR(OI) 0.72    Max Pain 23,300</t>
+          <t>Spot 23,140    PCR(OI) 0.93    Max Pain 23,250</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23888.55927419355</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23889.89758064516</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23888.68225806452</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23881.14879032258</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23879.4189516129</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23876.09516129032</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23140.5</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23063.1</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23446.8</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23329</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23414.3</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23346.4</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3136,18 +3136,18 @@
       <c r="P45" s="28" t="n">
         <v>23500</v>
       </c>
-      <c r="Q45" s="14" t="n">
-        <v>208801</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>50615</v>
-      </c>
-      <c r="S45" s="14" t="n">
-        <v>1321364</v>
+      <c r="Q45" s="12" t="n">
+        <v>217592</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>8791</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>2113409</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9462197383200984</v>
+        <v>0.9493709489654826</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9581623376424576</v>
@@ -3175,18 +3175,18 @@
       <c r="P46" s="28" t="n">
         <v>24000</v>
       </c>
-      <c r="Q46" s="14" t="n">
-        <v>298613</v>
+      <c r="Q46" s="12" t="n">
+        <v>240151</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>63236</v>
-      </c>
-      <c r="S46" s="14" t="n">
-        <v>1144027</v>
+        <v>-58462</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>1319868</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24373.93669354838</v>
+        <v>24374.56088709677</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24365.80846774194</v>
@@ -3214,16 +3214,16 @@
       <c r="P47" s="28" t="n">
         <v>24500</v>
       </c>
-      <c r="Q47" s="14" t="n">
-        <v>195348</v>
+      <c r="Q47" s="12" t="n">
+        <v>156478</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>58611</v>
-      </c>
-      <c r="S47" s="14" t="n">
-        <v>649177</v>
-      </c>
-      <c r="T47" s="30" t="inlineStr">
+        <v>-38870</v>
+      </c>
+      <c r="S47" s="12" t="n">
+        <v>504459</v>
+      </c>
+      <c r="T47" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23063.1</v>
+        <v>23140.5</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23346.4</v>
@@ -3250,7 +3250,7 @@
       <c r="N48" s="18" t="n">
         <v>24175.65</v>
       </c>
-      <c r="P48" s="31" t="inlineStr">
+      <c r="P48" s="30" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="29" t="inlineStr">
-        <is>
-          <t>24-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="29" t="inlineStr">
+      <c r="J49" s="31" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="31" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="29" t="inlineStr">
+      <c r="L49" s="31" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="29" t="inlineStr">
+      <c r="M49" s="31" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
       </c>
-      <c r="N49" s="29" t="inlineStr">
+      <c r="N49" s="31" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
@@ -3319,16 +3319,16 @@
     </row>
     <row r="50">
       <c r="P50" s="32" t="n">
-        <v>23000</v>
-      </c>
-      <c r="Q50" s="14" t="n">
-        <v>180885.3846153846</v>
-      </c>
-      <c r="R50" s="13" t="n">
-        <v>-14126.38461538462</v>
-      </c>
-      <c r="S50" s="14" t="n">
-        <v>2432163</v>
+        <v>23100</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>168406</v>
+      </c>
+      <c r="R50" s="14" t="n">
+        <v>51698</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>7190858</v>
       </c>
       <c r="T50" s="33" t="inlineStr">
         <is>
@@ -3338,37 +3338,37 @@
     </row>
     <row r="51">
       <c r="P51" s="32" t="n">
-        <v>22000</v>
-      </c>
-      <c r="Q51" s="14" t="n">
-        <v>186656</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>73837</v>
-      </c>
-      <c r="S51" s="14" t="n">
-        <v>859869</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>23000</v>
+      </c>
+      <c r="Q51" s="12" t="n">
+        <v>222071.7692307692</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>41186.38461538462</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>6262310</v>
+      </c>
+      <c r="T51" s="33" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="P52" s="32" t="n">
-        <v>21000</v>
-      </c>
-      <c r="Q52" s="14" t="n">
-        <v>170050</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>30670</v>
-      </c>
-      <c r="S52" s="14" t="n">
-        <v>283218</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
+        <v>22000</v>
+      </c>
+      <c r="Q52" s="12" t="n">
+        <v>201855</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>15199</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>893153</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 24-Sep-2026    1 DAY AGO = 23-Sep-2026    2 DAYS AGO = 22-Sep-2026    3 DAYS AGO = 21-Sep-2026    4 DAYS AGO = 18-Sep-2026    (generated 24-Sep-2026 20:32 IST)</t>
+          <t>TODAY = 25-Sep-2026    1 DAY AGO = 24-Sep-2026    2 DAYS AGO = 23-Sep-2026    3 DAYS AGO = 22-Sep-2026    4 DAYS AGO = 21-Sep-2026    (generated 25-Sep-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-28
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -187,13 +187,13 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-1712</v>
+        <v>13119</v>
       </c>
     </row>
     <row r="3">
@@ -701,27 +701,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-280</v>
+        <v>10680</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>1432</v>
+        <v>-2439</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-1712</v>
+        <v>13119</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>257518</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>244399</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>246111</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>240245</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>245711</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>241719</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>-217249</v>
+        <v>262150</v>
       </c>
     </row>
     <row r="4">
@@ -770,27 +770,27 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>214</v>
+        <v>-843</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>1089</v>
+        <v>-1260</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>-875</v>
+        <v>417</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,26 +798,26 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>6988</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>6571</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>7446</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>12202</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>13181</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>13180</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="9" t="inlineStr">
+      <c r="Q4" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -827,8 +827,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>25090</v>
+      <c r="S4" s="14" t="n">
+        <v>29522</v>
       </c>
     </row>
     <row r="5">
@@ -837,29 +837,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
-        <v>2562</v>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="C5" s="11" t="n">
+        <v>5262</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="11" t="n">
-        <v>4741</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="E5" s="14" t="n">
+        <v>12930</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="11" t="n">
-        <v>-2179</v>
+      <c r="G5" s="14" t="n">
+        <v>-7668</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -867,20 +867,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-319669</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-312001</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-309822</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-298613</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-302908</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-290546</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -888,7 +888,7 @@
       </c>
       <c r="Q5" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="S5" s="14" t="n">
-        <v>16335</v>
+        <v>-13736</v>
       </c>
     </row>
     <row r="6">
@@ -908,27 +908,27 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>4142</v>
+        <v>-4583</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>-624</v>
+        <v>1285</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G6" s="14" t="n">
-        <v>4766</v>
+        <v>-5868</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,26 +936,26 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>55163</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>61031</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>56265</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>46166</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>44016</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>35647</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="9" t="inlineStr">
+      <c r="Q6" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -965,8 +965,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="11" t="n">
-        <v>-76852</v>
+      <c r="S6" s="14" t="n">
+        <v>-51167</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>6638</v>
+        <v>10516</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>6638</v>
+        <v>10516</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,7 +1002,7 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
+      <c r="Q7" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>60557</v>
+      <c r="S7" s="14" t="n">
+        <v>16867</v>
       </c>
     </row>
     <row r="8">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>-875</v>
+        <v>417</v>
       </c>
     </row>
     <row r="9">
@@ -1093,27 +1093,27 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>-180855</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
+        <v>1273453</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="11" t="n">
-        <v>36394</v>
+      <c r="E9" s="14" t="n">
+        <v>1011303</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>-217249</v>
+        <v>262150</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,26 +1121,26 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>435645</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>173495</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>390744</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>188810</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>305921</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>182627</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>259</v>
+      <c r="S9" s="11" t="n">
+        <v>448</v>
       </c>
     </row>
     <row r="10">
@@ -1160,29 +1160,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>350</v>
+      <c r="C10" s="11" t="n">
+        <v>250</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>91</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+        <v>-198</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>259</v>
+      <c r="G10" s="11" t="n">
+        <v>448</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,26 +1190,26 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>10846</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>10398</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>10139</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>10922</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>10634</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>6117</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
+      <c r="Q10" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>-4223</v>
+      <c r="S10" s="11" t="n">
+        <v>-26200</v>
       </c>
     </row>
     <row r="11">
@@ -1231,27 +1231,27 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>-27687</v>
+        <v>286497</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>-47711</v>
+        <v>292003</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>20024</v>
+        <v>-5506</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,26 +1259,26 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-246475</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-240969</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-260993</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-188797</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-256374</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-256356</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>-21936</v>
+      <c r="S11" s="14" t="n">
+        <v>-59</v>
       </c>
     </row>
     <row r="12">
@@ -1298,67 +1298,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n">
-        <v>118321</v>
+      <c r="C12" s="11" t="n">
+        <v>263259</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>-78647</v>
+        <v>520351</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>-257092</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>-200015</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>57077</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>-139891</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>-10935</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>-60180</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>196968</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>57077</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>-139891</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>-10935</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>-60180</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>67612</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S12" s="11" t="n">
-        <v>-2375</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-89871</v>
+        <v>1823459</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-89873</v>
+        <v>1823459</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
+      <c r="Q13" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="14" t="n">
-        <v>-2085</v>
+      <c r="S13" s="11" t="n">
+        <v>-1627</v>
       </c>
     </row>
     <row r="14">
@@ -1463,7 +1463,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="9" t="inlineStr">
+      <c r="Q14" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="11" t="n">
-        <v>-2179</v>
+      <c r="S14" s="14" t="n">
+        <v>-7668</v>
       </c>
     </row>
     <row r="15">
@@ -1485,27 +1485,27 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>506024</v>
+        <v>-43112</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E15" s="14" t="n">
-        <v>480934</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+        <v>-72634</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>25090</v>
+      <c r="G15" s="14" t="n">
+        <v>29522</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-912888</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-942410</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-967500</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-690960</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-727055</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-827741</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>20024</v>
+        <v>-5506</v>
       </c>
     </row>
     <row r="16">
@@ -1552,29 +1552,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
-        <v>-4223</v>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="C16" s="11" t="n">
+        <v>-25600</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="E16" s="11" t="n">
+        <v>600</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>-4223</v>
+      <c r="G16" s="11" t="n">
+        <v>-26200</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,26 +1582,26 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>52467</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>78667</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>82890</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>81486</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>63189</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>69560</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
+      <c r="Q16" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>-2370</v>
+      <c r="S16" s="11" t="n">
+        <v>-9989</v>
       </c>
     </row>
     <row r="17">
@@ -1621,29 +1621,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
-        <v>92342</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="C17" s="14" t="n">
+        <v>37980</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="14" t="n">
-        <v>94712</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="E17" s="11" t="n">
+        <v>47969</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>-2370</v>
+      <c r="G17" s="11" t="n">
+        <v>-9989</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,26 +1651,26 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>673794</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>683783</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>686153</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>552364</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>642226</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>638430</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1680,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>12931</v>
+      <c r="S17" s="11" t="n">
+        <v>16641</v>
       </c>
     </row>
     <row r="18">
@@ -1692,27 +1692,27 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>187399</v>
+        <v>-24098</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>205895</v>
+        <v>-30764</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-18496</v>
+        <v>6666</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,20 +1720,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>186627</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>179961</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>198457</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>57109</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>21640</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>119751</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="Q18" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R18" s="10" t="inlineStr">
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="S18" s="11" t="n">
-        <v>-7207</v>
+        <v>9595</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>781542</v>
+        <v>-54830</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>781541</v>
+        <v>-54829</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>-4103</v>
+        <v>11609</v>
       </c>
     </row>
     <row r="20">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="14" t="n">
-        <v>4766</v>
+        <v>-5868</v>
       </c>
     </row>
     <row r="21">
@@ -1877,27 +1877,27 @@
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C21" s="14" t="n">
-        <v>12538</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+        <v>-32150</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
-        <v>-3797</v>
+      <c r="E21" s="11" t="n">
+        <v>-18414</v>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G21" s="14" t="n">
-        <v>16335</v>
+        <v>-13736</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,20 +1905,20 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3280948</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3294684</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3278349</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3246924</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>3242722</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3231518</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="Q21" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>196968</v>
+        <v>-257092</v>
       </c>
     </row>
     <row r="22">
@@ -1944,29 +1944,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n">
-        <v>8951</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="C22" s="11" t="n">
+        <v>9990</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="11" t="n">
-        <v>30887</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="E22" s="14" t="n">
+        <v>10049</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>-21936</v>
+      <c r="G22" s="14" t="n">
+        <v>-59</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4230812</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4230753</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4208817</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4204254</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4205892</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4211493</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>-18496</v>
+        <v>6666</v>
       </c>
     </row>
     <row r="23">
@@ -2013,29 +2013,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n">
-        <v>28212</v>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="C23" s="11" t="n">
+        <v>39430</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="11" t="n">
-        <v>15281</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
+      <c r="E23" s="14" t="n">
+        <v>22789</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>12931</v>
+      <c r="G23" s="11" t="n">
+        <v>16641</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,26 +2043,26 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>511652</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>495011</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>482080</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>509271</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>506874</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>504718</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>-7330</v>
+      <c r="S23" s="14" t="n">
+        <v>-2846</v>
       </c>
     </row>
     <row r="24">
@@ -2084,27 +2084,27 @@
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C24" s="14" t="n">
-        <v>3188</v>
+        <v>-18641</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E24" s="11" t="n">
-        <v>10518</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
+        <v>-15795</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>-7330</v>
+      <c r="G24" s="14" t="n">
+        <v>-2846</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,26 +2112,26 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>438212</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>441058</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>448388</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>448059</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>456296</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>475257</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
+      <c r="Q24" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>86434</v>
+      <c r="S24" s="11" t="n">
+        <v>38957</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>52889</v>
+        <v>-1371</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>52889</v>
+        <v>-1371</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,7 +2178,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
+      <c r="Q25" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>-54369</v>
+      <c r="S25" s="11" t="n">
+        <v>-26849</v>
       </c>
     </row>
     <row r="26">
@@ -2249,29 +2249,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C27" s="11" t="n">
-        <v>-69960</v>
+      <c r="C27" s="14" t="n">
+        <v>-122314</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E27" s="11" t="n">
-        <v>6892</v>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
+        <v>-71147</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G27" s="11" t="n">
-        <v>-76852</v>
+      <c r="G27" s="14" t="n">
+        <v>-51167</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1276618</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1327785</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1404637</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1323045</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1368959</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1357257</v>
       </c>
     </row>
     <row r="28">
@@ -2302,27 +2302,27 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>-215</v>
+        <v>279</v>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E28" s="11" t="n">
-        <v>2160</v>
+        <v>-2336</v>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G28" s="11" t="n">
-        <v>-2375</v>
+        <v>2615</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-411470</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-414085</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-411710</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-410833</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-411167</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-413749</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
-        <v>-19100</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="n">
+        <v>-17191</v>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>-11893</v>
+      <c r="E29" s="11" t="n">
+        <v>-26786</v>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G29" s="11" t="n">
-        <v>-7207</v>
+        <v>9595</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-293299</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-302894</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-295687</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-258810</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-262773</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-266344</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 25-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 28-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,27 +2420,27 @@
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C30" s="14" t="n">
-        <v>33817</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
+        <v>-31525</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>-52617</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
+      <c r="E30" s="11" t="n">
+        <v>-70482</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>86434</v>
+      <c r="G30" s="11" t="n">
+        <v>38957</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-571849</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-610806</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-697240</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-653402</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-695019</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-677164</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23035</v>
+        <v>23064.9</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23162.7</v>
+        <v>23080.25</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-55458</v>
+        <v>-170751</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-55458</v>
+        <v>-170751</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23020.95</v>
+        <v>22762.2</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23140.5</v>
+        <v>22780.25</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23336.9</v>
+        <v>23304.31666666667</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23124.275</v>
+        <v>22827.24166666667</v>
       </c>
     </row>
     <row r="33">
@@ -2599,27 +2599,27 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>46335</v>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
+        <v>-42546</v>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E33" s="11" t="n">
-        <v>-14222</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="E33" s="14" t="n">
+        <v>-59413</v>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G33" s="11" t="n">
-        <v>60557</v>
+      <c r="G33" s="14" t="n">
+        <v>16867</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-350049</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-366916</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-427473</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-359933</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-397348</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-360520</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23249.8</v>
+        <v>23192.28333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23108.05</v>
+        <v>22874.23333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2666,27 +2666,27 @@
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>-1794</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
+        <v>291</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>291</v>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
+      <c r="E34" s="11" t="n">
+        <v>1918</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>-2085</v>
+      <c r="G34" s="11" t="n">
+        <v>-1627</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>15273</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>16900</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>18985</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>18980</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>19239</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>20319</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23195.15</v>
+        <v>22986.26666666667</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23091.825</v>
+        <v>22921.225</v>
       </c>
     </row>
     <row r="35">
@@ -2731,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>-3744</v>
+      <c r="C35" s="11" t="n">
+        <v>-19064</v>
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E35" s="14" t="n">
-        <v>359</v>
+        <v>-30673</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>-4103</v>
+        <v>11609</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>245437</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>233828</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>237931</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>203440</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>208180</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>204275</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23108.05</v>
+        <v>22874.23333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,29 +2792,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>-7951</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="11" t="n">
+        <v>-20294</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>46418</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
+      <c r="E36" s="11" t="n">
+        <v>6555</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>-54369</v>
+      <c r="G36" s="11" t="n">
+        <v>-26849</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>89339</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>116188</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>170557</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>137513</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>169929</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>135926</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23053.4</v>
+        <v>22668.21666666667</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>32846</v>
+        <v>-81613</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>32846</v>
+        <v>-81613</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22966.3</v>
+        <v>22556.18333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22911.65</v>
+        <v>22350.16666666667</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>12.16</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>12.69</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>10.35</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.25</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9536176861203818</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9686854587751691</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9653913300442524</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9815024431531654</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9768793036226828</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9805221830332062</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,140    PCR(OI) 0.93    Max Pain 23,250</t>
+          <t>Spot 22,780    PCR(OI) 0.62    Max Pain 22,950</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23888.24193548387</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23888.55927419355</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23889.89758064516</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23888.68225806452</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23881.14879032258</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23879.4189516129</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22780.25</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23140.5</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23063.1</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23446.8</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23329</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23414.3</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23500</v>
+        <v>23000</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>217592</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>8791</v>
+        <v>325815</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>275374</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>2113409</v>
+        <v>6386340</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3158,33 +3158,33 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
+        <v>0.9345051638525492</v>
+      </c>
+      <c r="K46" s="25" t="n">
         <v>0.9493709489654826</v>
       </c>
-      <c r="K46" s="25" t="n">
+      <c r="L46" s="25" t="n">
         <v>0.9581623376424576</v>
       </c>
-      <c r="L46" s="25" t="n">
+      <c r="M46" s="25" t="n">
         <v>0.9605609315602034</v>
       </c>
-      <c r="M46" s="25" t="n">
+      <c r="N46" s="25" t="n">
         <v>0.9813887944889631</v>
       </c>
-      <c r="N46" s="25" t="n">
-        <v>0.9933791141865997</v>
-      </c>
       <c r="P46" s="28" t="n">
-        <v>24000</v>
+        <v>23500</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>240151</v>
+        <v>257957</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>-58462</v>
+        <v>40365</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>1319868</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
+        <v>1848120</v>
+      </c>
+      <c r="T46" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3197,33 +3197,33 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
+        <v>24376.80483870968</v>
+      </c>
+      <c r="K47" s="18" t="n">
         <v>24374.56088709677</v>
       </c>
-      <c r="K47" s="18" t="n">
+      <c r="L47" s="18" t="n">
         <v>24365.80846774194</v>
       </c>
-      <c r="L47" s="18" t="n">
+      <c r="M47" s="18" t="n">
         <v>24358.78790322581</v>
       </c>
-      <c r="M47" s="18" t="n">
+      <c r="N47" s="18" t="n">
         <v>24350.89959677419</v>
       </c>
-      <c r="N47" s="18" t="n">
-        <v>24336.7810483871</v>
-      </c>
       <c r="P47" s="28" t="n">
-        <v>24500</v>
+        <v>24000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>156478</v>
+        <v>274956</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>-38870</v>
+        <v>34805</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>504459</v>
-      </c>
-      <c r="T47" s="29" t="inlineStr">
+        <v>2022133</v>
+      </c>
+      <c r="T47" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3236,21 +3236,21 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
+        <v>22780.25</v>
+      </c>
+      <c r="K48" s="18" t="n">
         <v>23140.5</v>
       </c>
-      <c r="K48" s="18" t="n">
+      <c r="L48" s="18" t="n">
         <v>23346.4</v>
       </c>
-      <c r="L48" s="18" t="n">
+      <c r="M48" s="18" t="n">
         <v>23398.1</v>
       </c>
-      <c r="M48" s="18" t="n">
+      <c r="N48" s="18" t="n">
         <v>23897.7</v>
       </c>
-      <c r="N48" s="18" t="n">
-        <v>24175.65</v>
-      </c>
-      <c r="P48" s="30" t="inlineStr">
+      <c r="P48" s="31" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3266,29 +3266,29 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="31" t="inlineStr">
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
         <is>
           <t>25-Sep-2026</t>
         </is>
       </c>
-      <c r="K49" s="31" t="inlineStr">
+      <c r="L49" s="29" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="31" t="inlineStr">
+      <c r="M49" s="29" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="31" t="inlineStr">
+      <c r="N49" s="29" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
-        </is>
-      </c>
-      <c r="N49" s="31" t="inlineStr">
-        <is>
-          <t>28-Aug-2026</t>
         </is>
       </c>
       <c r="P49" s="27" t="inlineStr">
@@ -3319,16 +3319,16 @@
     </row>
     <row r="50">
       <c r="P50" s="32" t="n">
-        <v>23100</v>
+        <v>22800</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>168406</v>
-      </c>
-      <c r="R50" s="14" t="n">
-        <v>51698</v>
+        <v>191935</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>53808</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>7190858</v>
+        <v>11147805</v>
       </c>
       <c r="T50" s="33" t="inlineStr">
         <is>
@@ -3338,20 +3338,20 @@
     </row>
     <row r="51">
       <c r="P51" s="32" t="n">
-        <v>23000</v>
+        <v>22500</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>222071.7692307692</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>41186.38461538462</v>
+        <v>171043</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>10163</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>6262310</v>
-      </c>
-      <c r="T51" s="33" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>3293052</v>
+      </c>
+      <c r="T51" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3360,15 +3360,15 @@
         <v>22000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>201855</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>15199</v>
+        <v>214561</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>12706</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>893153</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
+        <v>1387354</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 25-Sep-2026    1 DAY AGO = 24-Sep-2026    2 DAYS AGO = 23-Sep-2026    3 DAYS AGO = 22-Sep-2026    4 DAYS AGO = 21-Sep-2026    (generated 25-Sep-2026 20:32 IST)</t>
+          <t>TODAY = 28-Sep-2026    1 DAY AGO = 25-Sep-2026    2 DAYS AGO = 24-Sep-2026    3 DAYS AGO = 23-Sep-2026    4 DAYS AGO = 22-Sep-2026    (generated 28-Sep-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-29
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,6 +187,9 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -198,9 +201,6 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>13119</v>
+        <v>-33705</v>
       </c>
     </row>
     <row r="3">
@@ -701,48 +701,48 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>10680</v>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
+        <v>-36802</v>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E3" s="11" t="n">
-        <v>-2439</v>
+      <c r="E3" s="13" t="n">
+        <v>-3097</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>13119</v>
+        <v>-33705</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="14" t="n">
+        <v>223813</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>257518</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="14" t="n">
         <v>244399</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="14" t="n">
         <v>246111</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>240245</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>245711</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>262150</v>
+        <v>-118989</v>
       </c>
     </row>
     <row r="4">
@@ -768,56 +768,56 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>-843</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>10720</v>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n">
-        <v>-1260</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="E4" s="13" t="n">
+        <v>-17800</v>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>417</v>
+      <c r="G4" s="13" t="n">
+        <v>28520</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="14" t="n">
+        <v>35508</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>6988</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="14" t="n">
         <v>6571</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="14" t="n">
         <v>7446</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="14" t="n">
         <v>12202</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>13181</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="13" t="inlineStr">
+      <c r="Q4" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -827,8 +827,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>29522</v>
+      <c r="S4" s="11" t="n">
+        <v>166920</v>
       </c>
     </row>
     <row r="5">
@@ -839,65 +839,65 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>5262</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>12930</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
+        <v>-23688</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>-76050</v>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>52362</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>-267307</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>-319669</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>-312001</v>
+      </c>
+      <c r="M5" s="14" t="n">
+        <v>-309822</v>
+      </c>
+      <c r="N5" s="14" t="n">
+        <v>-298613</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-7668</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-319669</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-312001</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-309822</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-298613</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-302908</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="14" t="n">
-        <v>-13736</v>
+      <c r="S5" s="11" t="n">
+        <v>-5527</v>
       </c>
     </row>
     <row r="6">
@@ -906,56 +906,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
-        <v>-4583</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>1285</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="C6" s="11" t="n">
+        <v>-55055</v>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>-7878</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>-5868</v>
+      <c r="G6" s="11" t="n">
+        <v>-47177</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
+        <v>7986</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>55163</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>61031</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="14" t="n">
         <v>56265</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="14" t="n">
         <v>46166</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>44016</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="13" t="inlineStr">
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -965,8 +965,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="14" t="n">
-        <v>-51167</v>
+      <c r="S6" s="11" t="n">
+        <v>-772432</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>10516</v>
+        <v>-104825</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>10516</v>
+        <v>-104825</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,7 +1002,7 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="13" t="inlineStr">
+      <c r="Q7" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="14" t="n">
-        <v>16867</v>
+      <c r="S7" s="11" t="n">
+        <v>89125</v>
       </c>
     </row>
     <row r="8">
@@ -1071,7 +1071,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
+      <c r="Q8" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>417</v>
+      <c r="S8" s="13" t="n">
+        <v>28520</v>
       </c>
     </row>
     <row r="9">
@@ -1093,48 +1093,48 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>1273453</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>1011303</v>
+        <v>-2801541</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>-2682552</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>262150</v>
+        <v>-118989</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="14" t="n">
+        <v>316656</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>435645</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="14" t="n">
         <v>173495</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="14" t="n">
         <v>390744</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="14" t="n">
         <v>188810</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>305921</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>448</v>
+        <v>-6274</v>
       </c>
     </row>
     <row r="10">
@@ -1162,54 +1162,54 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>250</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
+        <v>-7786</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n">
-        <v>-198</v>
+      <c r="E10" s="13" t="n">
+        <v>-1512</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>448</v>
+        <v>-6274</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
+        <v>4572</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>10846</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>10398</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="14" t="n">
         <v>10139</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="14" t="n">
         <v>10922</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>10634</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
+      <c r="Q10" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>-26200</v>
+      <c r="S10" s="13" t="n">
+        <v>-3073</v>
       </c>
     </row>
     <row r="11">
@@ -1231,54 +1231,54 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>286497</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>292003</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+        <v>-802184</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>-627196</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-5506</v>
+      <c r="G11" s="11" t="n">
+        <v>-174988</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="14" t="n">
+        <v>-421463</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-246475</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="14" t="n">
         <v>-240969</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="14" t="n">
         <v>-260993</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="14" t="n">
         <v>-188797</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-256374</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="13" t="inlineStr">
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>-59</v>
+      <c r="S11" s="11" t="n">
+        <v>-69743</v>
       </c>
     </row>
     <row r="12">
@@ -1300,54 +1300,54 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>263259</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>520351</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G12" s="14" t="n">
-        <v>-257092</v>
+        <v>-728508</v>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>-1028758</v>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="n">
+        <v>300250</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="14" t="n">
+        <v>100235</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>-200015</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <v>57077</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="14" t="n">
         <v>-139891</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="14" t="n">
         <v>-10935</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>-60180</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>2615</v>
+      <c r="S12" s="13" t="n">
+        <v>286037</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1823459</v>
+        <v>-4340019</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1823459</v>
+        <v>-4340018</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="Q13" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-1627</v>
+        <v>8990</v>
       </c>
     </row>
     <row r="14">
@@ -1463,9 +1463,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q14" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>-7668</v>
+      <c r="S14" s="13" t="n">
+        <v>52362</v>
       </c>
     </row>
     <row r="15">
@@ -1483,56 +1483,56 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
-        <v>-43112</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="C15" s="13" t="n">
+        <v>-1292133</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E15" s="14" t="n">
-        <v>-72634</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="E15" s="11" t="n">
+        <v>-1459053</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="14" t="n">
-        <v>29522</v>
+      <c r="G15" s="11" t="n">
+        <v>166920</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-745968</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-912888</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-942410</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>-967500</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>-690960</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-727055</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
+      <c r="Q15" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>-5506</v>
+      <c r="S15" s="11" t="n">
+        <v>-174988</v>
       </c>
     </row>
     <row r="16">
@@ -1552,56 +1552,56 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>-25600</v>
+      <c r="C16" s="13" t="n">
+        <v>-3373</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>600</v>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
+        <v>-300</v>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>-26200</v>
+      <c r="G16" s="13" t="n">
+        <v>-3073</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="14" t="n">
+        <v>49394</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>52467</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <v>78667</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="14" t="n">
         <v>82890</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="14" t="n">
         <v>81486</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>63189</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="9" t="inlineStr">
+      <c r="Q16" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>-9989</v>
+      <c r="S16" s="13" t="n">
+        <v>-22537</v>
       </c>
     </row>
     <row r="17">
@@ -1621,50 +1621,50 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="n">
-        <v>37980</v>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>-508939</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>47969</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+        <v>-486402</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>-9989</v>
+      <c r="G17" s="13" t="n">
+        <v>-22537</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="12" t="n">
+      <c r="J17" s="14" t="n">
+        <v>651257</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <v>673794</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="14" t="n">
         <v>683783</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="14" t="n">
         <v>686153</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="14" t="n">
         <v>552364</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>642226</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="Q17" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="11" t="n">
-        <v>16641</v>
+        <v>-15244</v>
       </c>
     </row>
     <row r="18">
@@ -1690,67 +1690,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n">
-        <v>-24098</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="C18" s="13" t="n">
+        <v>-665778</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E18" s="14" t="n">
-        <v>-30764</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="E18" s="11" t="n">
+        <v>-524469</v>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>-141309</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="n">
+        <v>45318</v>
+      </c>
+      <c r="K18" s="14" t="n">
+        <v>186627</v>
+      </c>
+      <c r="L18" s="14" t="n">
+        <v>179961</v>
+      </c>
+      <c r="M18" s="14" t="n">
+        <v>198457</v>
+      </c>
+      <c r="N18" s="14" t="n">
+        <v>57109</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>6666</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>186627</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>179961</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>198457</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>57109</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>21640</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="11" t="n">
-        <v>9595</v>
+      <c r="S18" s="13" t="n">
+        <v>213463</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-54830</v>
+        <v>-2470223</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-54829</v>
+        <v>-2470224</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q19" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>11609</v>
+      <c r="S19" s="13" t="n">
+        <v>-122266</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
+      <c r="Q20" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>-5868</v>
+      <c r="S20" s="11" t="n">
+        <v>-47177</v>
       </c>
     </row>
     <row r="21">
@@ -1875,58 +1875,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n">
-        <v>-32150</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="C21" s="11" t="n">
+        <v>-89996</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>-18414</v>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
+      <c r="E21" s="13" t="n">
+        <v>-84469</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="14" t="n">
-        <v>-13736</v>
+      <c r="G21" s="11" t="n">
+        <v>-5527</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="14" t="n">
+        <v>3275421</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3280948</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <v>3294684</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="14" t="n">
         <v>3278349</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="14" t="n">
         <v>3246924</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3242722</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-257092</v>
+      <c r="S21" s="13" t="n">
+        <v>300250</v>
       </c>
     </row>
     <row r="22">
@@ -1946,56 +1946,56 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>9990</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="n">
-        <v>10049</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+        <v>-150803</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>-81060</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>-59</v>
+      <c r="G22" s="11" t="n">
+        <v>-69743</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J22" s="14" t="n">
+        <v>-4300555</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-4230812</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="14" t="n">
         <v>-4230753</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="14" t="n">
         <v>-4208817</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="14" t="n">
         <v>-4204254</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4205892</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q22" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>6666</v>
+      <c r="S22" s="13" t="n">
+        <v>-141309</v>
       </c>
     </row>
     <row r="23">
@@ -2015,65 +2015,65 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>39430</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="n">
-        <v>22789</v>
+        <v>-188105</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>-172861</v>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>-15244</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="n">
+        <v>496408</v>
+      </c>
+      <c r="K23" s="14" t="n">
+        <v>511652</v>
+      </c>
+      <c r="L23" s="14" t="n">
+        <v>495011</v>
+      </c>
+      <c r="M23" s="14" t="n">
+        <v>482080</v>
+      </c>
+      <c r="N23" s="14" t="n">
+        <v>509271</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="12" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>16641</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>511652</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>495011</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>482080</v>
-      </c>
-      <c r="M23" s="12" t="n">
-        <v>509271</v>
-      </c>
-      <c r="N23" s="12" t="n">
-        <v>506874</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-2846</v>
+      <c r="S23" s="13" t="n">
+        <v>90514</v>
       </c>
     </row>
     <row r="24">
@@ -2082,56 +2082,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C24" s="14" t="n">
-        <v>-18641</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="C24" s="11" t="n">
+        <v>-116636</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>-15795</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G24" s="14" t="n">
-        <v>-2846</v>
+      <c r="E24" s="13" t="n">
+        <v>-207150</v>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>90514</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J24" s="14" t="n">
+        <v>528726</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>438212</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="14" t="n">
         <v>441058</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="14" t="n">
         <v>448388</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="14" t="n">
         <v>448059</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>456296</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="9" t="inlineStr">
+      <c r="Q24" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="11" t="n">
-        <v>38957</v>
+      <c r="S24" s="13" t="n">
+        <v>272932</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-1371</v>
+        <v>-545540</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-1371</v>
+        <v>-545540</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="11" t="n">
-        <v>-26849</v>
+        <v>24151</v>
       </c>
     </row>
     <row r="26">
@@ -2249,49 +2249,49 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
-        <v>-122314</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="C27" s="11" t="n">
+        <v>-1549707</v>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>-71147</v>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="E27" s="13" t="n">
+        <v>-777275</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n">
-        <v>-51167</v>
+      <c r="G27" s="11" t="n">
+        <v>-772432</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>504186</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>1276618</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>1327785</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="14" t="n">
         <v>1404637</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>1323045</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1368959</v>
       </c>
     </row>
     <row r="28">
@@ -2302,47 +2302,47 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>279</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+        <v>-4355</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>-2336</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="13" t="n">
+        <v>-290392</v>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>2615</v>
+      <c r="G28" s="13" t="n">
+        <v>286037</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-125433</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-411470</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-414085</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="14" t="n">
         <v>-411710</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>-410833</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-411167</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,53 +2359,53 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>-17191</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>-138295</v>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
-        <v>-26786</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="E29" s="13" t="n">
+        <v>-351758</v>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G29" s="11" t="n">
-        <v>9595</v>
+      <c r="G29" s="13" t="n">
+        <v>213463</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-79836</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-293299</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-302894</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="14" t="n">
         <v>-295687</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>-258810</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-262773</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 28-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 29-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,57 +2418,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
-        <v>-31525</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="C30" s="11" t="n">
+        <v>-657150</v>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n">
-        <v>-70482</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="E30" s="13" t="n">
+        <v>-930082</v>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G30" s="11" t="n">
-        <v>38957</v>
+      <c r="G30" s="13" t="n">
+        <v>272932</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-298917</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-571849</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-610806</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="14" t="n">
         <v>-697240</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="14" t="n">
         <v>-653402</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-695019</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23064.9</v>
+        <v>22732.45</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23080.25</v>
+        <v>22753.25</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-170751</v>
+        <v>-2349507</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-170751</v>
+        <v>-2349507</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22762.2</v>
+        <v>22569.65</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22780.25</v>
+        <v>22716.2</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23304.31666666667</v>
+        <v>22973.35</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22827.24166666667</v>
+        <v>22697.95</v>
       </c>
     </row>
     <row r="33">
@@ -2597,57 +2597,57 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>-42546</v>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="C33" s="13" t="n">
+        <v>-369137</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E33" s="14" t="n">
-        <v>-59413</v>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
+      <c r="E33" s="11" t="n">
+        <v>-458262</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>16867</v>
+      <c r="G33" s="11" t="n">
+        <v>89125</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-260924</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-350049</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-366916</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="14" t="n">
         <v>-427473</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="14" t="n">
         <v>-359933</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-397348</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23192.28333333333</v>
+        <v>22863.3</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22874.23333333333</v>
+        <v>22679.7</v>
       </c>
     </row>
     <row r="34">
@@ -2664,57 +2664,57 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="n">
-        <v>291</v>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="n">
+        <v>-11101</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>1918</v>
+        <v>-20091</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-1627</v>
+        <v>8990</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>24263</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>15273</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>16900</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="14" t="n">
         <v>18985</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="14" t="n">
         <v>18980</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>19239</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22986.26666666667</v>
+        <v>22789.75</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22921.225</v>
+        <v>22661.45</v>
       </c>
     </row>
     <row r="35">
@@ -2731,57 +2731,57 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>-19064</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="13" t="n">
+        <v>-277672</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>-30673</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="n">
-        <v>11609</v>
+      <c r="E35" s="11" t="n">
+        <v>-155406</v>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="n">
+        <v>-122266</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>123171</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>245437</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>233828</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="14" t="n">
         <v>237931</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="14" t="n">
         <v>203440</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>208180</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22874.23333333333</v>
+        <v>22679.7</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,57 +2792,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>-20294</v>
+      <c r="C36" s="13" t="n">
+        <v>-573919</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>6555</v>
+        <v>-598070</v>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G36" s="11" t="n">
-        <v>-26849</v>
+        <v>24151</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>113490</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>89339</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>116188</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="14" t="n">
         <v>170557</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="14" t="n">
         <v>137513</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>169929</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22668.21666666667</v>
+        <v>22606.15</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-81613</v>
+        <v>-1231829</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-81613</v>
+        <v>-1231829</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22556.18333333333</v>
+        <v>22496.1</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22350.16666666667</v>
+        <v>22422.55</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>13.64</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>12.16</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>12.69</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>10.35</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9508129344180111</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9536176861203818</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9686854587751691</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9653913300442524</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9815024431531654</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9768793036226828</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,780    PCR(OI) 0.62    Max Pain 22,950</t>
+          <t>Spot 22,716    PCR(OI) 0.88    Max Pain 22,750</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23891.34516129032</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23888.24193548387</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23888.55927419355</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23889.89758064516</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23888.68225806452</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23881.14879032258</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22716.2</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22780.25</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23140.5</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23063.1</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23446.8</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23329</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23000</v>
-      </c>
-      <c r="Q45" s="12" t="n">
-        <v>325815</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>275374</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>6386340</v>
+        <v>22700</v>
+      </c>
+      <c r="Q45" s="14" t="n">
+        <v>205026</v>
+      </c>
+      <c r="R45" s="13" t="n">
+        <v>185967</v>
+      </c>
+      <c r="S45" s="14" t="n">
+        <v>26340483</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9345051638525492</v>
+        <v>0.9318974125354335</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9493709489654826</v>
@@ -3173,20 +3173,20 @@
         <v>0.9813887944889631</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23500</v>
-      </c>
-      <c r="Q46" s="12" t="n">
-        <v>257957</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>40365</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>1848120</v>
+        <v>22750</v>
+      </c>
+      <c r="Q46" s="14" t="n">
+        <v>171522</v>
+      </c>
+      <c r="R46" s="13" t="n">
+        <v>139483</v>
+      </c>
+      <c r="S46" s="14" t="n">
+        <v>16480733</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24376.80483870968</v>
+        <v>24376.28830645161</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24374.56088709677</v>
@@ -3212,18 +3212,18 @@
         <v>24350.89959677419</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>24000</v>
-      </c>
-      <c r="Q47" s="12" t="n">
-        <v>274956</v>
+        <v>23500</v>
+      </c>
+      <c r="Q47" s="14" t="n">
+        <v>186031</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>34805</v>
-      </c>
-      <c r="S47" s="12" t="n">
-        <v>2022133</v>
-      </c>
-      <c r="T47" s="30" t="inlineStr">
+        <v>-70233</v>
+      </c>
+      <c r="S47" s="14" t="n">
+        <v>1988526</v>
+      </c>
+      <c r="T47" s="31" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22780.25</v>
+        <v>22716.2</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23140.5</v>
@@ -3250,7 +3250,7 @@
       <c r="N48" s="18" t="n">
         <v>23897.7</v>
       </c>
-      <c r="P48" s="31" t="inlineStr">
+      <c r="P48" s="32" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="29" t="inlineStr">
-        <is>
-          <t>28-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="29" t="inlineStr">
+      <c r="J49" s="30" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="30" t="inlineStr">
         <is>
           <t>25-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="29" t="inlineStr">
+      <c r="L49" s="30" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="29" t="inlineStr">
+      <c r="M49" s="30" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="N49" s="29" t="inlineStr">
+      <c r="N49" s="30" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
@@ -3318,66 +3318,66 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
-        <v>22800</v>
-      </c>
-      <c r="Q50" s="12" t="n">
-        <v>191935</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>53808</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>11147805</v>
-      </c>
-      <c r="T50" s="33" t="inlineStr">
+      <c r="P50" s="33" t="n">
+        <v>22700</v>
+      </c>
+      <c r="Q50" s="14" t="n">
+        <v>308746</v>
+      </c>
+      <c r="R50" s="13" t="n">
+        <v>173979</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>19810182</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="32" t="n">
-        <v>22500</v>
-      </c>
-      <c r="Q51" s="12" t="n">
-        <v>171043</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>10163</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>3293052</v>
-      </c>
-      <c r="T51" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="P51" s="33" t="n">
+        <v>22650</v>
+      </c>
+      <c r="Q51" s="14" t="n">
+        <v>199264</v>
+      </c>
+      <c r="R51" s="13" t="n">
+        <v>128742</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>21312030</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>22000</v>
-      </c>
-      <c r="Q52" s="12" t="n">
-        <v>214561</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>12706</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>1387354</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="P52" s="33" t="n">
+        <v>22600</v>
+      </c>
+      <c r="Q52" s="14" t="n">
+        <v>222523</v>
+      </c>
+      <c r="R52" s="13" t="n">
+        <v>100312</v>
+      </c>
+      <c r="S52" s="14" t="n">
+        <v>25179081</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 28-Sep-2026    1 DAY AGO = 25-Sep-2026    2 DAYS AGO = 24-Sep-2026    3 DAYS AGO = 23-Sep-2026    4 DAYS AGO = 22-Sep-2026    (generated 28-Sep-2026 20:31 IST)</t>
+          <t>TODAY = 29-Sep-2026    1 DAY AGO = 28-Sep-2026    2 DAYS AGO = 25-Sep-2026    3 DAYS AGO = 24-Sep-2026    4 DAYS AGO = 23-Sep-2026    (generated 29-Sep-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-30
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -190,13 +190,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-33705</v>
+        <v>18613</v>
       </c>
     </row>
     <row r="3">
@@ -701,48 +701,48 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-36802</v>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
+        <v>16837</v>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E3" s="13" t="n">
-        <v>-3097</v>
+      <c r="E3" s="11" t="n">
+        <v>-1776</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-33705</v>
+        <v>18613</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>242426</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>223813</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>257518</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>244399</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="12" t="n">
         <v>246111</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>240245</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>-118989</v>
+        <v>117121</v>
       </c>
     </row>
     <row r="4">
@@ -768,50 +768,50 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>10720</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="n">
-        <v>-17800</v>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G4" s="13" t="n">
-        <v>28520</v>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>-433</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>3025</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>-3458</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="12" t="n">
+        <v>32050</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>35508</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="12" t="n">
         <v>6988</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="12" t="n">
         <v>6571</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="12" t="n">
         <v>7446</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>12202</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -819,7 +819,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>166920</v>
+        <v>-96725</v>
       </c>
     </row>
     <row r="5">
@@ -839,65 +839,65 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>-23688</v>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="n">
-        <v>-76050</v>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+        <v>1515</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>17078</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>-15563</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-282870</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-267307</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-319669</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-312001</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-309822</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n">
-        <v>52362</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="n">
-        <v>-267307</v>
-      </c>
-      <c r="K5" s="14" t="n">
-        <v>-319669</v>
-      </c>
-      <c r="L5" s="14" t="n">
-        <v>-312001</v>
-      </c>
-      <c r="M5" s="14" t="n">
-        <v>-309822</v>
-      </c>
-      <c r="N5" s="14" t="n">
-        <v>-298613</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>-5527</v>
+        <v>23941</v>
       </c>
     </row>
     <row r="6">
@@ -908,48 +908,48 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>-55055</v>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="n">
-        <v>-7878</v>
+        <v>3713</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>3305</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>-47177</v>
+        <v>408</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="12" t="n">
+        <v>8394</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>7986</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="12" t="n">
         <v>55163</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>61031</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="12" t="n">
         <v>56265</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>46166</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -957,7 +957,7 @@
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R6" s="10" t="inlineStr">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>-772432</v>
+        <v>94345</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-104825</v>
+        <v>21632</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-104825</v>
+        <v>21632</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>89125</v>
+        <v>-29976</v>
       </c>
     </row>
     <row r="8">
@@ -1071,9 +1071,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="13" t="n">
-        <v>28520</v>
+      <c r="S8" s="14" t="n">
+        <v>-3458</v>
       </c>
     </row>
     <row r="9">
@@ -1093,48 +1093,48 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>-2801541</v>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>-2682552</v>
+        <v>959422</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>842301</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>-118989</v>
+        <v>117121</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="14" t="n">
+      <c r="J9" s="12" t="n">
+        <v>433777</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>316656</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="L9" s="12" t="n">
         <v>435645</v>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="M9" s="12" t="n">
         <v>173495</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="N9" s="12" t="n">
         <v>390744</v>
       </c>
-      <c r="N9" s="14" t="n">
-        <v>188810</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>-6274</v>
+        <v>979</v>
       </c>
     </row>
     <row r="10">
@@ -1162,65 +1162,65 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>-7786</v>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="n">
-        <v>-1512</v>
+        <v>3535</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>2556</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>979</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>5551</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>4572</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>10846</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>10398</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>10139</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>-6274</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J10" s="14" t="n">
-        <v>4572</v>
-      </c>
-      <c r="K10" s="14" t="n">
-        <v>10846</v>
-      </c>
-      <c r="L10" s="14" t="n">
-        <v>10398</v>
-      </c>
-      <c r="M10" s="14" t="n">
-        <v>10139</v>
-      </c>
-      <c r="N10" s="14" t="n">
-        <v>10922</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q10" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="13" t="n">
-        <v>-3073</v>
+      <c r="S10" s="11" t="n">
+        <v>-2736</v>
       </c>
     </row>
     <row r="11">
@@ -1231,54 +1231,54 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>-802184</v>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>-627196</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+        <v>125075</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>169195</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>-174988</v>
+      <c r="G11" s="14" t="n">
+        <v>-44120</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="14" t="n">
+      <c r="J11" s="12" t="n">
+        <v>-465583</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-421463</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="12" t="n">
         <v>-246475</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="M11" s="12" t="n">
         <v>-240969</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="12" t="n">
         <v>-260993</v>
       </c>
-      <c r="N11" s="14" t="n">
-        <v>-188797</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>-69743</v>
+      <c r="S11" s="14" t="n">
+        <v>-9000</v>
       </c>
     </row>
     <row r="12">
@@ -1300,56 +1300,56 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>-728508</v>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>-1028758</v>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G12" s="13" t="n">
-        <v>300250</v>
+        <v>221106</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>295087</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>-73981</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="14" t="n">
+      <c r="J12" s="12" t="n">
+        <v>26254</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>100235</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="12" t="n">
         <v>-200015</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="M12" s="12" t="n">
         <v>57077</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="12" t="n">
         <v>-139891</v>
       </c>
-      <c r="N12" s="14" t="n">
-        <v>-10935</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q12" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R12" s="10" t="inlineStr">
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="13" t="n">
-        <v>286037</v>
+      <c r="S12" s="14" t="n">
+        <v>-50187</v>
       </c>
     </row>
     <row r="13">
@@ -1369,11 +1369,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-4340019</v>
+        <v>1309138</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-4340018</v>
+        <v>1309139</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="Q13" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>8990</v>
+        <v>-1044</v>
       </c>
     </row>
     <row r="14">
@@ -1463,9 +1463,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q14" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="13" t="n">
-        <v>52362</v>
+      <c r="S14" s="14" t="n">
+        <v>-15563</v>
       </c>
     </row>
     <row r="15">
@@ -1483,56 +1483,56 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="n">
-        <v>-1292133</v>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>380962</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>-1459053</v>
+        <v>477687</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>166920</v>
+        <v>-96725</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="12" t="n">
+        <v>-842693</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-745968</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="12" t="n">
         <v>-912888</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="12" t="n">
         <v>-942410</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="12" t="n">
         <v>-967500</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-690960</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="11" t="n">
-        <v>-174988</v>
+      <c r="S15" s="14" t="n">
+        <v>-44120</v>
       </c>
     </row>
     <row r="16">
@@ -1552,58 +1552,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
-        <v>-3373</v>
+      <c r="C16" s="11" t="n">
+        <v>-2736</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>-300</v>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G16" s="13" t="n">
-        <v>-3073</v>
+      <c r="G16" s="11" t="n">
+        <v>-2736</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="14" t="n">
+      <c r="J16" s="12" t="n">
+        <v>46658</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>49394</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="12" t="n">
         <v>52467</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="12" t="n">
         <v>78667</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="12" t="n">
         <v>82890</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>81486</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="13" t="n">
-        <v>-22537</v>
+      <c r="S16" s="14" t="n">
+        <v>16868</v>
       </c>
     </row>
     <row r="17">
@@ -1621,67 +1621,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>-508939</v>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>101225</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>-486402</v>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
+        <v>84357</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>16868</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>668125</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>651257</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>673794</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>683783</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>686153</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
-        <v>-22537</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="14" t="n">
-        <v>651257</v>
-      </c>
-      <c r="K17" s="14" t="n">
-        <v>673794</v>
-      </c>
-      <c r="L17" s="14" t="n">
-        <v>683783</v>
-      </c>
-      <c r="M17" s="14" t="n">
-        <v>686153</v>
-      </c>
-      <c r="N17" s="14" t="n">
-        <v>552364</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>-15244</v>
+      <c r="S17" s="14" t="n">
+        <v>-6859</v>
       </c>
     </row>
     <row r="18">
@@ -1690,67 +1690,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="n">
-        <v>-665778</v>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>189051</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>-524469</v>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
+        <v>106459</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>82592</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>127910</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>45318</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>186627</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>179961</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>198457</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="13" t="n">
-        <v>-141309</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="14" t="n">
-        <v>45318</v>
-      </c>
-      <c r="K18" s="14" t="n">
-        <v>186627</v>
-      </c>
-      <c r="L18" s="14" t="n">
-        <v>179961</v>
-      </c>
-      <c r="M18" s="14" t="n">
-        <v>198457</v>
-      </c>
-      <c r="N18" s="14" t="n">
-        <v>57109</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="13" t="n">
-        <v>213463</v>
+      <c r="S18" s="14" t="n">
+        <v>-7787</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-2470223</v>
+        <v>668502</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-2470224</v>
+        <v>668503</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="13" t="n">
-        <v>-122266</v>
+      <c r="S19" s="14" t="n">
+        <v>4077</v>
       </c>
     </row>
     <row r="20">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Q20" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>-47177</v>
+        <v>408</v>
       </c>
     </row>
     <row r="21">
@@ -1877,65 +1877,65 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-89996</v>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="n">
-        <v>-84469</v>
+        <v>30803</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>6862</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>23941</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3299362</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3275421</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3280948</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3294684</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3278349</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>-5527</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="14" t="n">
-        <v>3275421</v>
-      </c>
-      <c r="K21" s="14" t="n">
-        <v>3280948</v>
-      </c>
-      <c r="L21" s="14" t="n">
-        <v>3294684</v>
-      </c>
-      <c r="M21" s="14" t="n">
-        <v>3278349</v>
-      </c>
-      <c r="N21" s="14" t="n">
-        <v>3246924</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="13" t="n">
-        <v>300250</v>
+      <c r="S21" s="14" t="n">
+        <v>-73981</v>
       </c>
     </row>
     <row r="22">
@@ -1946,56 +1946,56 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>-150803</v>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="n">
-        <v>-81060</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+        <v>4755</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>13755</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>-69743</v>
+      <c r="G22" s="14" t="n">
+        <v>-9000</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="14" t="n">
+      <c r="J22" s="12" t="n">
+        <v>-4309555</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4300555</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4230812</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4230753</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4208817</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-4204254</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="13" t="n">
-        <v>-141309</v>
+      <c r="S22" s="14" t="n">
+        <v>82592</v>
       </c>
     </row>
     <row r="23">
@@ -2015,56 +2015,56 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>-188105</v>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="n">
-        <v>-172861</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+        <v>10452</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>17311</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>-15244</v>
+      <c r="G23" s="14" t="n">
+        <v>-6859</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="14" t="n">
+      <c r="J23" s="12" t="n">
+        <v>489549</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>496408</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="L23" s="12" t="n">
         <v>511652</v>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="M23" s="12" t="n">
         <v>495011</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="N23" s="12" t="n">
         <v>482080</v>
       </c>
-      <c r="N23" s="14" t="n">
-        <v>509271</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q23" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="13" t="n">
-        <v>90514</v>
+      <c r="S23" s="14" t="n">
+        <v>-8082</v>
       </c>
     </row>
     <row r="24">
@@ -2084,56 +2084,56 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>-116636</v>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="n">
-        <v>-207150</v>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="n">
-        <v>90514</v>
+        <v>8832</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>16914</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>-8082</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="14" t="n">
+      <c r="J24" s="12" t="n">
+        <v>520644</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>528726</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="12" t="n">
         <v>438212</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="12" t="n">
         <v>441058</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="12" t="n">
         <v>448388</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>448059</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q24" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="13" t="n">
-        <v>272932</v>
+      <c r="S24" s="14" t="n">
+        <v>-36371</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-545540</v>
+        <v>54842</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-545540</v>
+        <v>54842</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,7 +2178,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
+      <c r="Q25" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="11" t="n">
-        <v>24151</v>
+      <c r="S25" s="14" t="n">
+        <v>26943</v>
       </c>
     </row>
     <row r="26">
@@ -2251,47 +2251,47 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>-1549707</v>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="n">
-        <v>-777275</v>
+        <v>232783</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="n">
+        <v>138438</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>-772432</v>
+        <v>94345</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>598531</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>504186</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>1276618</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>1327785</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="12" t="n">
         <v>1404637</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>1323045</v>
       </c>
     </row>
     <row r="28">
@@ -2302,47 +2302,47 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>-4355</v>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="n">
-        <v>-290392</v>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="n">
-        <v>286037</v>
+        <v>2032</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>52219</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>-50187</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-175620</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-125433</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-411470</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-414085</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="12" t="n">
         <v>-411710</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-410833</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2361,51 +2361,51 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>-138295</v>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="n">
-        <v>-351758</v>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G29" s="13" t="n">
-        <v>213463</v>
+        <v>24812</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>32599</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>-7787</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-87623</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-79836</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-293299</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-302894</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="12" t="n">
         <v>-295687</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-258810</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 29-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 30-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,55 +2420,55 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>-657150</v>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="n">
-        <v>-930082</v>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="n">
-        <v>272932</v>
+        <v>94085</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>130456</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>-36371</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-335288</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-298917</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-571849</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-610806</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="12" t="n">
         <v>-697240</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-653402</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22732.45</v>
+        <v>22665</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>22753.25</v>
+        <v>22809.35</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-2349507</v>
+        <v>353712</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-2349507</v>
+        <v>353712</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22569.65</v>
+        <v>22595.2</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22716.2</v>
+        <v>22620.45</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>22973.35</v>
+        <v>22968.95</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22697.95</v>
+        <v>22647.725</v>
       </c>
     </row>
     <row r="33">
@@ -2597,57 +2597,57 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v>-369137</v>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>44433</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>-458262</v>
+        <v>74409</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>89125</v>
+        <v>-29976</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="14" t="n">
+      <c r="J33" s="12" t="n">
+        <v>-290900</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-260924</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="12" t="n">
         <v>-350049</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="12" t="n">
         <v>-366916</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="12" t="n">
         <v>-427473</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-359933</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>22863.3</v>
+        <v>22889.15</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22679.7</v>
+        <v>22675</v>
       </c>
     </row>
     <row r="34">
@@ -2664,57 +2664,57 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C34" s="13" t="n">
-        <v>-11101</v>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="n">
+        <v>8403</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>-20091</v>
+        <v>9447</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>8990</v>
+        <v>-1044</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="14" t="n">
+      <c r="J34" s="12" t="n">
+        <v>23219</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>24263</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="12" t="n">
         <v>15273</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="12" t="n">
         <v>16900</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="12" t="n">
         <v>18985</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>18980</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22789.75</v>
+        <v>22754.8</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22661.45</v>
+        <v>22702.275</v>
       </c>
     </row>
     <row r="35">
@@ -2731,57 +2731,57 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C35" s="13" t="n">
-        <v>-277672</v>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="n">
+        <v>34491</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>-155406</v>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G35" s="13" t="n">
-        <v>-122266</v>
+        <v>30414</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>4077</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="14" t="n">
+      <c r="J35" s="12" t="n">
+        <v>127248</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>123171</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="12" t="n">
         <v>245437</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="12" t="n">
         <v>233828</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="12" t="n">
         <v>237931</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>203440</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22679.7</v>
+        <v>22675</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,57 +2792,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C36" s="13" t="n">
-        <v>-573919</v>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="n">
+        <v>95956</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>-598070</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
+        <v>69013</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G36" s="11" t="n">
-        <v>24151</v>
+      <c r="G36" s="14" t="n">
+        <v>26943</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="14" t="n">
+      <c r="J36" s="12" t="n">
+        <v>140433</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>113490</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="12" t="n">
         <v>89339</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="12" t="n">
         <v>116188</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="12" t="n">
         <v>170557</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>137513</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22606.15</v>
+        <v>22540.65</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-1231829</v>
+        <v>183283</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-1231829</v>
+        <v>183283</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22496.1</v>
+        <v>22460.85</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22422.55</v>
+        <v>22326.5</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>13.41</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>13.64</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>12.16</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>12.69</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>10.35</v>
       </c>
     </row>
     <row r="41">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 29-Sep-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 06-Oct-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.946824047390084</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9508129344180111</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9536176861203818</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9686854587751691</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9653913300442524</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9815024431531654</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,716    PCR(OI) 0.88    Max Pain 22,750</t>
+          <t>Spot 22,620    PCR(OI) 0.65    Max Pain 22,700</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23890.86975806452</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23891.34516129032</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23888.24193548387</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23888.55927419355</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23889.89758064516</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23888.68225806452</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22620.45</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22716.2</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22780.25</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23140.5</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23063.1</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23446.8</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>22700</v>
-      </c>
-      <c r="Q45" s="14" t="n">
-        <v>205026</v>
-      </c>
-      <c r="R45" s="13" t="n">
-        <v>185967</v>
-      </c>
-      <c r="S45" s="14" t="n">
-        <v>26340483</v>
+        <v>23000</v>
+      </c>
+      <c r="Q45" s="12" t="n">
+        <v>180405</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>77303</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>2395137</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9318974125354335</v>
+        <v>0.9279988116049818</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9493709489654826</v>
@@ -3173,20 +3173,20 @@
         <v>0.9813887944889631</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>22750</v>
-      </c>
-      <c r="Q46" s="14" t="n">
-        <v>171522</v>
-      </c>
-      <c r="R46" s="13" t="n">
-        <v>139483</v>
-      </c>
-      <c r="S46" s="14" t="n">
-        <v>16480733</v>
+        <v>23500</v>
+      </c>
+      <c r="Q46" s="12" t="n">
+        <v>150623</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>46939</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>741731</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24376.28830645161</v>
+        <v>24375.51612903226</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24374.56088709677</v>
@@ -3212,18 +3212,18 @@
         <v>24350.89959677419</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>23500</v>
-      </c>
-      <c r="Q47" s="14" t="n">
-        <v>186031</v>
+        <v>24000</v>
+      </c>
+      <c r="Q47" s="12" t="n">
+        <v>141164</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>-70233</v>
-      </c>
-      <c r="S47" s="14" t="n">
-        <v>1988526</v>
-      </c>
-      <c r="T47" s="31" t="inlineStr">
+        <v>56571</v>
+      </c>
+      <c r="S47" s="12" t="n">
+        <v>601953</v>
+      </c>
+      <c r="T47" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22716.2</v>
+        <v>22620.45</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23140.5</v>
@@ -3250,7 +3250,7 @@
       <c r="N48" s="18" t="n">
         <v>23897.7</v>
       </c>
-      <c r="P48" s="32" t="inlineStr">
+      <c r="P48" s="31" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="30" t="inlineStr">
-        <is>
-          <t>29-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="30" t="inlineStr">
+      <c r="J49" s="32" t="inlineStr">
+        <is>
+          <t>30-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="32" t="inlineStr">
         <is>
           <t>25-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="30" t="inlineStr">
+      <c r="L49" s="32" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="30" t="inlineStr">
+      <c r="M49" s="32" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="N49" s="30" t="inlineStr">
+      <c r="N49" s="32" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
@@ -3319,16 +3319,16 @@
     </row>
     <row r="50">
       <c r="P50" s="33" t="n">
-        <v>22700</v>
-      </c>
-      <c r="Q50" s="14" t="n">
-        <v>308746</v>
-      </c>
-      <c r="R50" s="13" t="n">
-        <v>173979</v>
-      </c>
-      <c r="S50" s="14" t="n">
-        <v>19810182</v>
+        <v>22500</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>101975</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>39507</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>2063409</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3338,46 +3338,46 @@
     </row>
     <row r="51">
       <c r="P51" s="33" t="n">
-        <v>22650</v>
-      </c>
-      <c r="Q51" s="14" t="n">
-        <v>199264</v>
-      </c>
-      <c r="R51" s="13" t="n">
-        <v>128742</v>
-      </c>
-      <c r="S51" s="14" t="n">
-        <v>21312030</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>22000</v>
+      </c>
+      <c r="Q51" s="12" t="n">
+        <v>121373</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>32680</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>891746</v>
+      </c>
+      <c r="T51" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="P52" s="33" t="n">
-        <v>22600</v>
-      </c>
-      <c r="Q52" s="14" t="n">
-        <v>222523</v>
-      </c>
-      <c r="R52" s="13" t="n">
-        <v>100312</v>
-      </c>
-      <c r="S52" s="14" t="n">
-        <v>25179081</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>20500</v>
+      </c>
+      <c r="Q52" s="12" t="n">
+        <v>92756</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>14912</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>152009</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 29-Sep-2026    1 DAY AGO = 28-Sep-2026    2 DAYS AGO = 25-Sep-2026    3 DAYS AGO = 24-Sep-2026    4 DAYS AGO = 23-Sep-2026    (generated 29-Sep-2026 20:32 IST)</t>
+          <t>TODAY = 30-Sep-2026    1 DAY AGO = 29-Sep-2026    2 DAYS AGO = 28-Sep-2026    3 DAYS AGO = 25-Sep-2026    4 DAYS AGO = 24-Sep-2026    (generated 30-Sep-2026 20:33 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-01
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -187,7 +187,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,11 +196,11 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>18613</v>
+        <v>7386</v>
       </c>
     </row>
     <row r="3">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>16837</v>
+        <v>5526</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-1776</v>
+        <v>-1860</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>18613</v>
+        <v>7386</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,28 +729,28 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>249812</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>242426</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>223813</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>257518</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>244399</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>246111</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>117121</v>
+      <c r="S3" s="14" t="n">
+        <v>-138293</v>
       </c>
     </row>
     <row r="4">
@@ -774,61 +774,61 @@
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>-433</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="n">
-        <v>3025</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+        <v>-1523</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>-2730</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>1207</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>33257</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>32050</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>35508</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>6988</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>6571</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>-3458</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>32050</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>35508</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>6988</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>6571</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>7446</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-96725</v>
+        <v>-455</v>
       </c>
     </row>
     <row r="5">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>1515</v>
+        <v>211</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>17078</v>
+        <v>27515</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-15563</v>
+        <v>-27304</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -867,28 +867,28 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-310174</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-282870</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-267307</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-319669</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-312001</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-309822</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -896,8 +896,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>23941</v>
+      <c r="S5" s="14" t="n">
+        <v>-31754</v>
       </c>
     </row>
     <row r="6">
@@ -912,15 +912,15 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>3713</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>3305</v>
+        <v>15823</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>-2888</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>408</v>
+        <v>18711</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,20 +936,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>27105</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>8394</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>7986</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>55163</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>61031</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>56265</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>94345</v>
+        <v>84237</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>21632</v>
+        <v>20037</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>21632</v>
+        <v>20037</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-29976</v>
+        <v>-13164</v>
       </c>
     </row>
     <row r="8">
@@ -1071,9 +1071,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>-3458</v>
+      <c r="S8" s="11" t="n">
+        <v>1207</v>
       </c>
     </row>
     <row r="9">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>959422</v>
+        <v>409331</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
@@ -1105,15 +1105,15 @@
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>842301</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>117121</v>
+        <v>547624</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>-138293</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,28 +1121,28 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>295484</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>433777</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>316656</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>435645</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>173495</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>390744</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>979</v>
+      <c r="S9" s="14" t="n">
+        <v>-575</v>
       </c>
     </row>
     <row r="10">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>3535</v>
+        <v>50</v>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
@@ -1174,15 +1174,15 @@
         </is>
       </c>
       <c r="E10" s="14" t="n">
-        <v>2556</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>979</v>
+        <v>625</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>-575</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,20 +1190,20 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>4976</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>5551</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>4572</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>10846</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>10398</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>10139</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>-2736</v>
+        <v>-7132</v>
       </c>
     </row>
     <row r="11">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>125075</v>
+        <v>203970</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
@@ -1243,53 +1243,53 @@
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>169195</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+        <v>169852</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>34118</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-431465</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-465583</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-421463</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-246475</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-240969</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-44120</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-465583</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-421463</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-246475</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-240969</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-260993</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S11" s="14" t="n">
-        <v>-9000</v>
+        <v>-697</v>
       </c>
     </row>
     <row r="12">
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>221106</v>
+        <v>284865</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
@@ -1312,53 +1312,53 @@
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>295087</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+        <v>180114</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>104751</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>131005</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>26254</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>100235</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>-200015</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>57077</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-73981</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>26254</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>100235</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>-200015</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>57077</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>-139891</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-50187</v>
+        <v>-19277</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1309138</v>
+        <v>898216</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1309139</v>
+        <v>898215</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-1044</v>
+        <v>-2463</v>
       </c>
     </row>
     <row r="14">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-15563</v>
+        <v>-27304</v>
       </c>
     </row>
     <row r="15">
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>380962</v>
+        <v>382104</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>477687</v>
+        <v>382559</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-96725</v>
+        <v>-455</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,28 +1513,28 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-843148</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-842693</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-745968</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-912888</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-942410</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-967500</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>-44120</v>
+      <c r="S15" s="11" t="n">
+        <v>34118</v>
       </c>
     </row>
     <row r="16">
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>-2736</v>
+        <v>-6556</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>0</v>
+        <v>576</v>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="G16" s="11" t="n">
-        <v>-2736</v>
+        <v>-7132</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,28 +1582,28 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>39526</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>46658</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>49394</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>52467</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>78667</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>82890</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>16868</v>
+      <c r="S16" s="11" t="n">
+        <v>-1547</v>
       </c>
     </row>
     <row r="17">
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="C17" s="14" t="n">
-        <v>101225</v>
+        <v>82725</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1635,53 +1635,53 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>84357</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+        <v>84272</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>-1547</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>666578</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>668125</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>651257</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>673794</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>683783</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>16868</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>668125</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>651257</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>673794</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>683783</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>686153</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>-6859</v>
+      <c r="S17" s="11" t="n">
+        <v>45532</v>
       </c>
     </row>
     <row r="18">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>189051</v>
+        <v>169091</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>106459</v>
+        <v>159957</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="G18" s="14" t="n">
-        <v>82592</v>
+        <v>9134</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,20 +1720,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>137044</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>127910</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>45318</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>186627</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>179961</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>198457</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-7787</v>
+        <v>-6869</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>668502</v>
+        <v>627364</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>668503</v>
+        <v>627364</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>4077</v>
+        <v>10023</v>
       </c>
     </row>
     <row r="20">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>408</v>
+        <v>18711</v>
       </c>
     </row>
     <row r="21">
@@ -1875,13 +1875,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="n">
-        <v>30803</v>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>-31295</v>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
@@ -1889,53 +1889,53 @@
         </is>
       </c>
       <c r="E21" s="14" t="n">
-        <v>6862</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
+        <v>459</v>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>-31754</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3267608</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3299362</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3275421</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3280948</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3294684</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>23941</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>3299362</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>3275421</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>3280948</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>3294684</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>3278349</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-73981</v>
+      <c r="S21" s="11" t="n">
+        <v>104751</v>
       </c>
     </row>
     <row r="22">
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>4755</v>
+        <v>18890</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>13755</v>
+        <v>19587</v>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-9000</v>
+        <v>-697</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4310252</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4309555</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4300555</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4230812</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4230753</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4208817</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>82592</v>
+        <v>9134</v>
       </c>
     </row>
     <row r="23">
@@ -2019,61 +2019,61 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>10452</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="n">
-        <v>17311</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
+        <v>33479</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>-12053</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>45532</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>535081</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>489549</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>496408</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>511652</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>495011</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>-6859</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>489549</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>496408</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>511652</v>
-      </c>
-      <c r="M23" s="12" t="n">
-        <v>495011</v>
-      </c>
-      <c r="N23" s="12" t="n">
-        <v>482080</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S23" s="14" t="n">
-        <v>-8082</v>
+        <v>-13081</v>
       </c>
     </row>
     <row r="24">
@@ -2082,13 +2082,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="n">
-        <v>8832</v>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>-8729</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
@@ -2096,7 +2096,7 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>16914</v>
+        <v>4352</v>
       </c>
       <c r="F24" s="13" t="inlineStr">
         <is>
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-8082</v>
+        <v>-13081</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,20 +2112,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>507563</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>520644</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>528726</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>438212</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>441058</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>448388</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-36371</v>
+        <v>-58091</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>54842</v>
+        <v>12345</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>54842</v>
+        <v>12345</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>26943</v>
+        <v>5604</v>
       </c>
     </row>
     <row r="26">
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>232783</v>
+        <v>198052</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>138438</v>
+        <v>113815</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>94345</v>
+        <v>84237</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>682768</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>598531</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>504186</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1276618</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1327785</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1404637</v>
       </c>
     </row>
     <row r="28">
@@ -2306,7 +2306,7 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>2032</v>
+        <v>7299</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>52219</v>
+        <v>26576</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-50187</v>
+        <v>-19277</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-194897</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-175620</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-125433</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-411470</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-414085</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-411710</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>24812</v>
+        <v>20260</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>32599</v>
+        <v>27129</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-7787</v>
+        <v>-6869</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-94492</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-87623</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-79836</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-293299</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-302894</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-295687</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 30-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 01-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>94085</v>
+        <v>75085</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>130456</v>
+        <v>133176</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-36371</v>
+        <v>-58091</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-393379</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-335288</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-298917</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-571849</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-610806</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-697240</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22665</v>
+        <v>22543.7</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>22809.35</v>
+        <v>22610.6</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>353712</v>
+        <v>300696</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>353712</v>
+        <v>300696</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22595.2</v>
+        <v>22217.3</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22620.45</v>
+        <v>22421.95</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>22968.95</v>
+        <v>23009.23333333333</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22647.725</v>
+        <v>22419.28333333333</v>
       </c>
     </row>
     <row r="33">
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="C33" s="14" t="n">
-        <v>44433</v>
+        <v>28340</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>74409</v>
+        <v>41504</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-29976</v>
+        <v>-13164</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-304064</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-290900</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-260924</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-350049</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-366916</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-427473</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>22889.15</v>
+        <v>22809.91666666666</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22675</v>
+        <v>22416.61666666666</v>
       </c>
     </row>
     <row r="34">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>8403</v>
+        <v>54</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>9447</v>
+        <v>2517</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-1044</v>
+        <v>-2463</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>20756</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>23219</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>24263</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>15273</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>16900</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>18985</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22754.8</v>
+        <v>22615.93333333333</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22702.275</v>
+        <v>22413.95</v>
       </c>
     </row>
     <row r="35">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>34491</v>
+        <v>29344</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>30414</v>
+        <v>19321</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>4077</v>
+        <v>10023</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>137271</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>127248</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>123171</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>245437</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>233828</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>237931</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22675</v>
+        <v>22416.61666666666</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>95956</v>
+        <v>79078</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>69013</v>
+        <v>73474</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
@@ -2814,7 +2814,7 @@
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>26943</v>
+        <v>5604</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>146037</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>140433</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>113490</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>89339</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>116188</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>170557</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22540.65</v>
+        <v>22222.63333333333</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>183283</v>
+        <v>136816</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>183283</v>
+        <v>136816</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22460.85</v>
+        <v>22023.31666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22326.5</v>
+        <v>21829.33333333333</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>14.46</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>13.49</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>13.41</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>13.64</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>12.16</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>12.69</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9386076799537314</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.946824047390084</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9508129344180111</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9536176861203818</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9686854587751691</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9653913300442524</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,620    PCR(OI) 0.65    Max Pain 22,700</t>
+          <t>Spot 22,422    PCR(OI) 0.69    Max Pain 22,550</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23888.52177419355</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23890.86975806452</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23891.34516129032</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23888.24193548387</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23888.55927419355</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23889.89758064516</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22421.95</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22620.45</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22716.2</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22780.25</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>23140.5</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23063.1</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3137,17 +3137,17 @@
         <v>23000</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>180405</v>
+        <v>211765</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>77303</v>
+        <v>31360</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>2395137</v>
+        <v>1799484</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9279988116049818</v>
+        <v>0.9199158076678682</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9493709489654826</v>
@@ -3176,17 +3176,17 @@
         <v>23500</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>150623</v>
+        <v>192261</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>46939</v>
+        <v>41638</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>741731</v>
-      </c>
-      <c r="T46" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>1367162</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24375.51612903226</v>
+        <v>24373.91532258064</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24374.56088709677</v>
@@ -3215,13 +3215,13 @@
         <v>24000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>141164</v>
+        <v>170754</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>56571</v>
+        <v>29590</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>601953</v>
+        <v>772072</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22620.45</v>
+        <v>22421.95</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23140.5</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="32" t="inlineStr">
-        <is>
-          <t>30-Sep-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="32" t="inlineStr">
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>01-Oct-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
         <is>
           <t>25-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="32" t="inlineStr">
+      <c r="L49" s="29" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="32" t="inlineStr">
+      <c r="M49" s="29" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
       </c>
-      <c r="N49" s="32" t="inlineStr">
+      <c r="N49" s="29" t="inlineStr">
         <is>
           <t>04-Sep-2026</t>
         </is>
@@ -3318,66 +3318,66 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
-        <v>22500</v>
+      <c r="P50" s="32" t="n">
+        <v>22300</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>101975</v>
+        <v>125716</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>39507</v>
+        <v>68992</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>2063409</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
+        <v>2858337</v>
+      </c>
+      <c r="T50" s="33" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="33" t="n">
+      <c r="P51" s="32" t="n">
         <v>22000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>121373</v>
+        <v>154746</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>32680</v>
+        <v>33373</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>891746</v>
-      </c>
-      <c r="T51" s="32" t="inlineStr">
+        <v>2126540</v>
+      </c>
+      <c r="T51" s="33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="P52" s="32" t="n">
+        <v>21500</v>
+      </c>
+      <c r="Q52" s="12" t="n">
+        <v>147958</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>63996</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>1165561</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="P52" s="33" t="n">
-        <v>20500</v>
-      </c>
-      <c r="Q52" s="12" t="n">
-        <v>92756</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>14912</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>152009</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 30-Sep-2026    1 DAY AGO = 29-Sep-2026    2 DAYS AGO = 28-Sep-2026    3 DAYS AGO = 25-Sep-2026    4 DAYS AGO = 24-Sep-2026    (generated 30-Sep-2026 20:33 IST)</t>
+          <t>TODAY = 01-Oct-2026    1 DAY AGO = 30-Sep-2026    2 DAYS AGO = 29-Sep-2026    3 DAYS AGO = 28-Sep-2026    4 DAYS AGO = 25-Sep-2026    (generated 01-Oct-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-05
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>7386</v>
+        <v>-7779</v>
       </c>
     </row>
     <row r="3">
@@ -701,27 +701,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>5526</v>
+        <v>-4879</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-1860</v>
+        <v>2900</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>7386</v>
+        <v>-7779</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,26 +729,26 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>242033</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>249812</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>242426</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>223813</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>257518</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>244399</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
+      <c r="Q3" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="14" t="n">
-        <v>-138293</v>
+      <c r="S3" s="11" t="n">
+        <v>-176222</v>
       </c>
     </row>
     <row r="4">
@@ -768,67 +768,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
-        <v>-1523</v>
+      <c r="C4" s="11" t="n">
+        <v>-419</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>-2730</v>
+        <v>10</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>-429</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>32828</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>33257</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>32050</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>35508</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>6988</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>1207</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>33257</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>32050</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>35508</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>6988</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>6571</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-455</v>
+        <v>208051</v>
       </c>
     </row>
     <row r="5">
@@ -839,65 +839,65 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>211</v>
+        <v>-488</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>27515</v>
+        <v>-8271</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>7783</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-302391</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-310174</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-282870</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-267307</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-319669</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-27304</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-310174</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-282870</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-267307</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-319669</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-312001</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="14" t="n">
-        <v>-31754</v>
+      <c r="S5" s="11" t="n">
+        <v>-10134</v>
       </c>
     </row>
     <row r="6">
@@ -906,29 +906,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>15823</v>
+      <c r="C6" s="14" t="n">
+        <v>3408</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-2888</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+        <v>2983</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>18711</v>
+      <c r="G6" s="14" t="n">
+        <v>425</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,26 +936,26 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>27530</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>27105</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>8394</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>7986</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>55163</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>61031</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="9" t="inlineStr">
+      <c r="Q6" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -965,8 +965,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="11" t="n">
-        <v>84237</v>
+      <c r="S6" s="14" t="n">
+        <v>36124</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>20037</v>
+        <v>-2378</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>20037</v>
+        <v>-2378</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-13164</v>
+        <v>27504</v>
       </c>
     </row>
     <row r="8">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>1207</v>
+        <v>-429</v>
       </c>
     </row>
     <row r="9">
@@ -1091,29 +1091,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C9" s="11" t="n">
-        <v>409331</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="n">
+        <v>287664</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="14" t="n">
-        <v>547624</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="E9" s="11" t="n">
+        <v>463886</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>-138293</v>
+      <c r="G9" s="11" t="n">
+        <v>-176222</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,20 +1121,20 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>119262</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>295484</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>433777</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>316656</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>435645</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>173495</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="14" t="n">
-        <v>-575</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="10">
@@ -1160,29 +1160,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
-        <v>50</v>
+      <c r="C10" s="14" t="n">
+        <v>18810</v>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E10" s="14" t="n">
-        <v>625</v>
+        <v>-100</v>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-575</v>
+        <v>18910</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,20 +1190,20 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>23886</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>4976</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>5551</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>4572</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>10846</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>10398</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>-7132</v>
+        <v>13789</v>
       </c>
     </row>
     <row r="11">
@@ -1231,27 +1231,27 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>203970</v>
+        <v>-53957</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>169852</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+        <v>-119691</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>34118</v>
+      <c r="G11" s="14" t="n">
+        <v>65734</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,26 +1259,26 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-365731</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-431465</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-465583</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-421463</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-246475</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-240969</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="13" t="inlineStr">
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>-697</v>
+      <c r="S11" s="11" t="n">
+        <v>-2683</v>
       </c>
     </row>
     <row r="12">
@@ -1298,29 +1298,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>284865</v>
+      <c r="C12" s="14" t="n">
+        <v>60076</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>180114</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
+        <v>-31503</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>104751</v>
+      <c r="G12" s="14" t="n">
+        <v>91579</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,26 +1328,26 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>222584</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>131005</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>26254</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>100235</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>-200015</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>57077</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="13" t="inlineStr">
+      <c r="Q12" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>-19277</v>
+      <c r="S12" s="11" t="n">
+        <v>-33670</v>
       </c>
     </row>
     <row r="13">
@@ -1369,11 +1369,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>898216</v>
+        <v>312593</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>898215</v>
+        <v>312592</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>-2463</v>
+      <c r="S13" s="14" t="n">
+        <v>-1373</v>
       </c>
     </row>
     <row r="14">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-27304</v>
+        <v>7783</v>
       </c>
     </row>
     <row r="15">
@@ -1483,29 +1483,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
-        <v>382104</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="C15" s="11" t="n">
+        <v>917279</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="11" t="n">
-        <v>382559</v>
+      <c r="E15" s="14" t="n">
+        <v>709228</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-455</v>
+        <v>208051</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,26 +1513,26 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-635097</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-843148</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-842693</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-745968</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-912888</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-942410</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="11" t="n">
-        <v>34118</v>
+      <c r="S15" s="14" t="n">
+        <v>65734</v>
       </c>
     </row>
     <row r="16">
@@ -1554,65 +1554,65 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>-6556</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+        <v>13789</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
-        <v>576</v>
+      <c r="E16" s="14" t="n">
+        <v>0</v>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>13789</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>53315</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>39526</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>46658</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>49394</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>52467</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>-7132</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>39526</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>46658</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>49394</v>
-      </c>
-      <c r="M16" s="12" t="n">
-        <v>52467</v>
-      </c>
-      <c r="N16" s="12" t="n">
-        <v>78667</v>
-      </c>
-      <c r="P16" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q16" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R16" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>-1547</v>
+      <c r="S16" s="14" t="n">
+        <v>-78263</v>
       </c>
     </row>
     <row r="17">
@@ -1621,29 +1621,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n">
-        <v>82725</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="C17" s="11" t="n">
+        <v>60465</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n">
-        <v>84272</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="E17" s="14" t="n">
+        <v>138728</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>-1547</v>
+      <c r="G17" s="14" t="n">
+        <v>-78263</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,26 +1651,26 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>588315</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>666578</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>668125</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>651257</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>673794</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>683783</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="9" t="inlineStr">
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1680,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>45532</v>
+      <c r="S17" s="14" t="n">
+        <v>31907</v>
       </c>
     </row>
     <row r="18">
@@ -1690,29 +1690,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
-        <v>169091</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="C18" s="11" t="n">
+        <v>159406</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
-        <v>159957</v>
+      <c r="E18" s="14" t="n">
+        <v>302983</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G18" s="14" t="n">
-        <v>9134</v>
+        <v>-143577</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,26 +1720,26 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>-6533</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>137044</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>127910</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>45318</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>186627</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>179961</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="13" t="inlineStr">
+      <c r="Q18" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>-6869</v>
+      <c r="S18" s="11" t="n">
+        <v>-13619</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>627364</v>
+        <v>1150939</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>627364</v>
+        <v>1150939</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1786,7 +1786,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
+      <c r="Q19" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>10023</v>
+      <c r="S19" s="11" t="n">
+        <v>2828</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>18711</v>
+      <c r="S20" s="14" t="n">
+        <v>425</v>
       </c>
     </row>
     <row r="21">
@@ -1875,29 +1875,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n">
-        <v>-31295</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="C21" s="11" t="n">
+        <v>-5264</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
-        <v>459</v>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
+      <c r="E21" s="11" t="n">
+        <v>4870</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="14" t="n">
-        <v>-31754</v>
+      <c r="G21" s="11" t="n">
+        <v>-10134</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,26 +1905,26 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3257474</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3267608</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3299362</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3275421</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>3280948</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3294684</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="9" t="inlineStr">
+      <c r="Q21" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>104751</v>
+      <c r="S21" s="14" t="n">
+        <v>91579</v>
       </c>
     </row>
     <row r="22">
@@ -1946,27 +1946,27 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>18890</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
+        <v>-1313</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
-        <v>19587</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="E22" s="11" t="n">
+        <v>1370</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>-697</v>
+      <c r="G22" s="11" t="n">
+        <v>-2683</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4312935</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4310252</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4309555</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4300555</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4230812</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4230753</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>9134</v>
+        <v>-143577</v>
       </c>
     </row>
     <row r="23">
@@ -2013,29 +2013,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n">
-        <v>33479</v>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="C23" s="14" t="n">
+        <v>26776</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E23" s="11" t="n">
-        <v>-12053</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="E23" s="14" t="n">
+        <v>-5131</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>45532</v>
+      <c r="G23" s="14" t="n">
+        <v>31907</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,26 +2043,26 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>566988</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>535081</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>489549</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>496408</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>511652</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>495011</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-13081</v>
+      <c r="S23" s="11" t="n">
+        <v>-19090</v>
       </c>
     </row>
     <row r="24">
@@ -2082,29 +2082,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C24" s="14" t="n">
-        <v>-8729</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="C24" s="11" t="n">
+        <v>-4579</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>4352</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+      <c r="E24" s="11" t="n">
+        <v>14511</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-13081</v>
+      <c r="G24" s="11" t="n">
+        <v>-19090</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,20 +2112,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>488473</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>507563</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>520644</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>528726</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>438212</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>441058</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="Q24" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-58091</v>
+        <v>11165</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>12345</v>
+        <v>15620</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>12345</v>
+        <v>15620</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>5604</v>
+        <v>-28959</v>
       </c>
     </row>
     <row r="26">
@@ -2249,29 +2249,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C27" s="11" t="n">
-        <v>198052</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="C27" s="14" t="n">
+        <v>126688</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
-        <v>113815</v>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="E27" s="11" t="n">
+        <v>90564</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G27" s="11" t="n">
-        <v>84237</v>
+      <c r="G27" s="14" t="n">
+        <v>36124</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>718892</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>682768</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>598531</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>504186</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1276618</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1327785</v>
       </c>
     </row>
     <row r="28">
@@ -2302,27 +2302,27 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>7299</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+        <v>-1521</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="14" t="n">
-        <v>26576</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="E28" s="11" t="n">
+        <v>32149</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>-19277</v>
+      <c r="G28" s="11" t="n">
+        <v>-33670</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-228567</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-194897</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-175620</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-125433</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-411470</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-414085</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
-        <v>20260</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="n">
+        <v>17029</v>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>27129</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
+      <c r="E29" s="11" t="n">
+        <v>30648</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>-6869</v>
+      <c r="G29" s="11" t="n">
+        <v>-13619</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-108111</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-94492</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-87623</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-79836</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-293299</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-302894</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 01-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 05-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,29 +2418,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
-        <v>75085</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="C30" s="14" t="n">
+        <v>50640</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>133176</v>
+      <c r="E30" s="11" t="n">
+        <v>39475</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-58091</v>
+        <v>11165</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-382214</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-393379</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-335288</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-298917</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-571849</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-610806</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22543.7</v>
+        <v>22532.4</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>22610.6</v>
+        <v>22621.8</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>300696</v>
+        <v>192836</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>300696</v>
+        <v>192836</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22217.3</v>
+        <v>22397.1</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22421.95</v>
+        <v>22555.75</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23009.23333333333</v>
+        <v>22877.36666666666</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22419.28333333333</v>
+        <v>22540.31666666667</v>
       </c>
     </row>
     <row r="33">
@@ -2597,29 +2597,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
-        <v>28340</v>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="C33" s="11" t="n">
+        <v>81734</v>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="11" t="n">
-        <v>41504</v>
+      <c r="E33" s="14" t="n">
+        <v>54230</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-13164</v>
+        <v>27504</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-276560</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-304064</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-290900</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-260924</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-350049</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-366916</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>22809.91666666666</v>
+        <v>22749.58333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22416.61666666666</v>
+        <v>22524.88333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2666,27 +2666,27 @@
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>54</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
+        <v>-18</v>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="11" t="n">
-        <v>2517</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="E34" s="14" t="n">
+        <v>1355</v>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="11" t="n">
-        <v>-2463</v>
+      <c r="G34" s="14" t="n">
+        <v>-1373</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>19383</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>20756</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>23219</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>24263</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>15273</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>16900</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22615.93333333333</v>
+        <v>22652.66666666666</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22413.95</v>
+        <v>22509.45</v>
       </c>
     </row>
     <row r="35">
@@ -2731,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>29344</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="C35" s="11" t="n">
+        <v>17310</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="11" t="n">
-        <v>19321</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
+      <c r="E35" s="14" t="n">
+        <v>14482</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>10023</v>
+      <c r="G35" s="11" t="n">
+        <v>2828</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>140099</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>137271</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>127248</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>123171</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>245437</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>233828</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22416.61666666666</v>
+        <v>22524.88333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,29 +2792,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>79078</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="C36" s="11" t="n">
+        <v>26661</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
-        <v>73474</v>
+      <c r="E36" s="14" t="n">
+        <v>55620</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>5604</v>
+        <v>-28959</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>117078</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>146037</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>140433</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>113490</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>89339</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>116188</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22222.63333333333</v>
+        <v>22427.96666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>136816</v>
+        <v>125687</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>136816</v>
+        <v>125687</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22023.31666666667</v>
+        <v>22300.18333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>21829.33333333333</v>
+        <v>22203.26666666666</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>14.78</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>14.46</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>13.49</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>13.41</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>13.64</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>12.16</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9443402010193789</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9386076799537314</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.946824047390084</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9508129344180111</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9536176861203818</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9686854587751691</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,422    PCR(OI) 0.69    Max Pain 22,550</t>
+          <t>Spot 22,556    PCR(OI) 0.89    Max Pain 22,550</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23885.19516129032</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23888.52177419355</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23890.86975806452</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23891.34516129032</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23888.24193548387</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23888.55927419355</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22555.75</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22421.95</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22620.45</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22716.2</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22780.25</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>23140.5</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23000</v>
+        <v>22800</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>211765</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>31360</v>
+        <v>221193</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>83607</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>1799484</v>
+        <v>5342437</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,35 +3158,35 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
+        <v>0.9255281866927508</v>
+      </c>
+      <c r="K46" s="25" t="n">
         <v>0.9199158076678682</v>
       </c>
-      <c r="K46" s="25" t="n">
+      <c r="L46" s="25" t="n">
         <v>0.9493709489654826</v>
       </c>
-      <c r="L46" s="25" t="n">
+      <c r="M46" s="25" t="n">
         <v>0.9581623376424576</v>
       </c>
-      <c r="M46" s="25" t="n">
+      <c r="N46" s="25" t="n">
         <v>0.9605609315602034</v>
       </c>
-      <c r="N46" s="25" t="n">
-        <v>0.9813887944889631</v>
-      </c>
       <c r="P46" s="28" t="n">
-        <v>23500</v>
+        <v>23000</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>192261</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>41638</v>
+        <v>225585</v>
+      </c>
+      <c r="R46" s="14" t="n">
+        <v>13820</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>1367162</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>2736232</v>
+      </c>
+      <c r="T46" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3197,31 +3197,31 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
+        <v>24370.67862903226</v>
+      </c>
+      <c r="K47" s="18" t="n">
         <v>24373.91532258064</v>
       </c>
-      <c r="K47" s="18" t="n">
+      <c r="L47" s="18" t="n">
         <v>24374.56088709677</v>
       </c>
-      <c r="L47" s="18" t="n">
+      <c r="M47" s="18" t="n">
         <v>24365.80846774194</v>
       </c>
-      <c r="M47" s="18" t="n">
+      <c r="N47" s="18" t="n">
         <v>24358.78790322581</v>
       </c>
-      <c r="N47" s="18" t="n">
-        <v>24350.89959677419</v>
-      </c>
       <c r="P47" s="28" t="n">
-        <v>24000</v>
+        <v>23500</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>170754</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>29590</v>
+        <v>205470</v>
+      </c>
+      <c r="R47" s="14" t="n">
+        <v>13209</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>772072</v>
+        <v>1412013</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
@@ -3236,19 +3236,19 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
+        <v>22555.75</v>
+      </c>
+      <c r="K48" s="18" t="n">
         <v>22421.95</v>
       </c>
-      <c r="K48" s="18" t="n">
+      <c r="L48" s="18" t="n">
         <v>23140.5</v>
       </c>
-      <c r="L48" s="18" t="n">
+      <c r="M48" s="18" t="n">
         <v>23346.4</v>
       </c>
-      <c r="M48" s="18" t="n">
+      <c r="N48" s="18" t="n">
         <v>23398.1</v>
-      </c>
-      <c r="N48" s="18" t="n">
-        <v>23897.7</v>
       </c>
       <c r="P48" s="31" t="inlineStr">
         <is>
@@ -3268,27 +3268,27 @@
       </c>
       <c r="J49" s="29" t="inlineStr">
         <is>
+          <t>05-Oct-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
+        <is>
           <t>01-Oct-2026</t>
         </is>
       </c>
-      <c r="K49" s="29" t="inlineStr">
+      <c r="L49" s="29" t="inlineStr">
         <is>
           <t>25-Sep-2026</t>
         </is>
       </c>
-      <c r="L49" s="29" t="inlineStr">
+      <c r="M49" s="29" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="29" t="inlineStr">
+      <c r="N49" s="29" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
-        </is>
-      </c>
-      <c r="N49" s="29" t="inlineStr">
-        <is>
-          <t>04-Sep-2026</t>
         </is>
       </c>
       <c r="P49" s="27" t="inlineStr">
@@ -3319,16 +3319,16 @@
     </row>
     <row r="50">
       <c r="P50" s="32" t="n">
-        <v>22300</v>
+        <v>22500</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>125716</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>68992</v>
+        <v>188172</v>
+      </c>
+      <c r="R50" s="14" t="n">
+        <v>112545</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>2858337</v>
+        <v>13269393</v>
       </c>
       <c r="T50" s="33" t="inlineStr">
         <is>
@@ -3341,17 +3341,17 @@
         <v>22000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>154746</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>33373</v>
+        <v>196668</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>41922</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>2126540</v>
-      </c>
-      <c r="T51" s="33" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>3581139</v>
+      </c>
+      <c r="T51" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3360,24 +3360,24 @@
         <v>21500</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>147958</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>63996</v>
+        <v>226555</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>78597</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>1165561</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>1745808</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 01-Oct-2026    1 DAY AGO = 30-Sep-2026    2 DAYS AGO = 29-Sep-2026    3 DAYS AGO = 28-Sep-2026    4 DAYS AGO = 25-Sep-2026    (generated 01-Oct-2026 20:32 IST)</t>
+          <t>TODAY = 05-Oct-2026    1 DAY AGO = 01-Oct-2026    2 DAYS AGO = 30-Sep-2026    3 DAYS AGO = 29-Sep-2026    4 DAYS AGO = 28-Sep-2026    (generated 05-Oct-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-06
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -187,6 +187,9 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -198,9 +201,6 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-7779</v>
+        <v>-4933</v>
       </c>
     </row>
     <row r="3">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-4879</v>
+        <v>-4339</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>2900</v>
+        <v>594</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-7779</v>
+        <v>-4933</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,28 +729,28 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>237100</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>242033</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>249812</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>242426</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>223813</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>257518</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>-176222</v>
+      <c r="S3" s="14" t="n">
+        <v>87245</v>
       </c>
     </row>
     <row r="4">
@@ -768,67 +768,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>-419</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>273</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>-800</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>1073</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>33901</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>32828</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>33257</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>32050</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>35508</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>-429</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>32828</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>33257</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>32050</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>35508</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>6988</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>208051</v>
+      <c r="S4" s="14" t="n">
+        <v>-22660</v>
       </c>
     </row>
     <row r="5">
@@ -837,13 +837,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>-488</v>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>1168</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>-8271</v>
+        <v>-7498</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>7783</v>
+        <v>8666</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -867,20 +867,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-293725</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-302391</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-310174</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-282870</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-267307</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-319669</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>-10134</v>
+        <v>-17248</v>
       </c>
     </row>
     <row r="6">
@@ -906,13 +906,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>3408</v>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>-1907</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -920,15 +920,15 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>2983</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>425</v>
+        <v>2899</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>-4806</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,28 +936,28 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>22724</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>27530</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>27105</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>8394</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>7986</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>55163</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R6" s="10" t="inlineStr">
@@ -965,8 +965,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="14" t="n">
-        <v>36124</v>
+      <c r="S6" s="11" t="n">
+        <v>-32547</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-2378</v>
+        <v>-4805</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-2378</v>
+        <v>-4805</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>27504</v>
+        <v>28082</v>
       </c>
     </row>
     <row r="8">
@@ -1071,9 +1071,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>-429</v>
+      <c r="S8" s="14" t="n">
+        <v>1073</v>
       </c>
     </row>
     <row r="9">
@@ -1091,29 +1091,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>287664</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>463886</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>-176222</v>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>-1784356</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>-1871601</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>87245</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,20 +1121,20 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>206507</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>119262</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>295484</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>433777</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>316656</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>435645</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="14" t="n">
-        <v>18910</v>
+        <v>3885</v>
       </c>
     </row>
     <row r="10">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>18810</v>
+        <v>2834</v>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="E10" s="14" t="n">
-        <v>-100</v>
+        <v>-1051</v>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="G10" s="14" t="n">
-        <v>18910</v>
+        <v>3885</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,20 +1190,20 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>27771</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>23886</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>4976</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>5551</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>4572</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>10846</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>13789</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>-53957</v>
+        <v>-223082</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>-119691</v>
+        <v>-241329</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>65734</v>
+        <v>18247</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,20 +1259,20 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-347484</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-365731</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-431465</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-465583</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-421463</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-246475</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="S11" s="11" t="n">
-        <v>-2683</v>
+        <v>-1287</v>
       </c>
     </row>
     <row r="12">
@@ -1298,13 +1298,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>60076</v>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>-550365</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
@@ -1312,15 +1312,15 @@
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>-31503</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G12" s="14" t="n">
-        <v>91579</v>
+        <v>-440988</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>-109377</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,20 +1328,20 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>113207</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>222584</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>131005</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>26254</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>100235</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>-200015</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="S12" s="11" t="n">
-        <v>-33670</v>
+        <v>-26743</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>312593</v>
+        <v>-2554969</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>312592</v>
+        <v>-2554969</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="14" t="n">
-        <v>-1373</v>
+        <v>-4721</v>
       </c>
     </row>
     <row r="14">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>7783</v>
+        <v>8666</v>
       </c>
     </row>
     <row r="15">
@@ -1483,67 +1483,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="n">
-        <v>917279</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>709228</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>-1364022</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>-1341362</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>-22660</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>-657757</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>-635097</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>-843148</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>-842693</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>-745968</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>208051</v>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>-635097</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>-843148</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>-842693</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>-745968</v>
-      </c>
-      <c r="N15" s="12" t="n">
-        <v>-912888</v>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>65734</v>
+        <v>18247</v>
       </c>
     </row>
     <row r="16">
@@ -1552,21 +1552,21 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>13789</v>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="n">
-        <v>0</v>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>-150</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>-376</v>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="G16" s="11" t="n">
-        <v>13789</v>
+        <v>226</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>53541</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>53315</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>39526</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>46658</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>49394</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>52467</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>-78263</v>
+        <v>-20549</v>
       </c>
     </row>
     <row r="17">
@@ -1621,21 +1621,21 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="n">
-        <v>60465</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>138728</v>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>-248566</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>-228017</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-78263</v>
+        <v>-20549</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,20 +1651,20 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>567766</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>588315</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>666578</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>668125</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>651257</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>673794</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="14" t="n">
-        <v>31907</v>
+        <v>43509</v>
       </c>
     </row>
     <row r="18">
@@ -1690,29 +1690,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="n">
-        <v>159406</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>302983</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="n">
-        <v>-143577</v>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>-404592</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>-447575</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>42983</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,28 +1720,28 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>36450</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>-6533</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>137044</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>127910</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>45318</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>186627</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R18" s="10" t="inlineStr">
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="11" t="n">
-        <v>-13619</v>
+      <c r="S18" s="14" t="n">
+        <v>722</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>1150939</v>
+        <v>-2017330</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>1150939</v>
+        <v>-2017330</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="11" t="n">
-        <v>2828</v>
+      <c r="S19" s="14" t="n">
+        <v>-8839</v>
       </c>
     </row>
     <row r="20">
@@ -1855,9 +1855,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>425</v>
+      <c r="S20" s="11" t="n">
+        <v>-4806</v>
       </c>
     </row>
     <row r="21">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-5264</v>
+        <v>-5752</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>4870</v>
+        <v>11496</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>-10134</v>
+        <v>-17248</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,28 +1905,28 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3240226</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3257474</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3267608</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3299362</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>3275421</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3280948</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>91579</v>
+      <c r="S21" s="11" t="n">
+        <v>-109377</v>
       </c>
     </row>
     <row r="22">
@@ -1944,13 +1944,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="n">
-        <v>-1313</v>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>5264</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>1370</v>
+        <v>6551</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="G22" s="11" t="n">
-        <v>-2683</v>
+        <v>-1287</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,28 +1974,28 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4314222</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4312935</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4310252</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4309555</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4300555</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4230812</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>-143577</v>
+      <c r="S22" s="11" t="n">
+        <v>42983</v>
       </c>
     </row>
     <row r="23">
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>26776</v>
+        <v>21621</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>-5131</v>
+        <v>-21888</v>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="G23" s="14" t="n">
-        <v>31907</v>
+        <v>43509</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,20 +2043,20 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>610497</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>566988</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>535081</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>489549</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>496408</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>511652</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>-19090</v>
+        <v>-24974</v>
       </c>
     </row>
     <row r="24">
@@ -2088,7 +2088,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>-4579</v>
+        <v>-14287</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
@@ -2096,7 +2096,7 @@
         </is>
       </c>
       <c r="E24" s="11" t="n">
-        <v>14511</v>
+        <v>10687</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>-19090</v>
+        <v>-24974</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,20 +2112,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>463499</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>488473</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>507563</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>520644</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>528726</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>438212</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>11165</v>
+        <v>58568</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>15620</v>
+        <v>6846</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>15620</v>
+        <v>6846</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>-28959</v>
+        <v>-14522</v>
       </c>
     </row>
     <row r="26">
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="C27" s="14" t="n">
-        <v>126688</v>
+        <v>23278</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
@@ -2263,15 +2263,15 @@
         </is>
       </c>
       <c r="E27" s="11" t="n">
-        <v>90564</v>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G27" s="14" t="n">
-        <v>36124</v>
+        <v>55825</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="n">
+        <v>-32547</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>686345</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>718892</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>682768</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>598531</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>504186</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1276618</v>
       </c>
     </row>
     <row r="28">
@@ -2300,13 +2300,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="n">
-        <v>-1521</v>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>700</v>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="E28" s="11" t="n">
-        <v>32149</v>
+        <v>27443</v>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="G28" s="11" t="n">
-        <v>-33670</v>
+        <v>-26743</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-255310</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-228567</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-194897</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-175620</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-125433</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-411470</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C29" s="14" t="n">
-        <v>17029</v>
+        <v>22848</v>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
@@ -2373,15 +2373,15 @@
         </is>
       </c>
       <c r="E29" s="11" t="n">
-        <v>30648</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G29" s="11" t="n">
-        <v>-13619</v>
+        <v>22126</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>722</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-107389</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-108111</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-94492</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-87623</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-79836</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-293299</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 05-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 06-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="C30" s="14" t="n">
-        <v>50640</v>
+        <v>69562</v>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="E30" s="11" t="n">
-        <v>39475</v>
+        <v>10994</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>11165</v>
+        <v>58568</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-323646</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-382214</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-393379</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-335288</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-298917</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-571849</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22532.4</v>
+        <v>22603.25</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>22621.8</v>
+        <v>22776.1</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>192836</v>
+        <v>116388</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>192836</v>
+        <v>116388</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22397.1</v>
+        <v>22561.6</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22555.75</v>
+        <v>22776.1</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>22877.36666666666</v>
+        <v>23062.09999999999</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22540.31666666667</v>
+        <v>22740.34999999999</v>
       </c>
     </row>
     <row r="33">
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>81734</v>
+        <v>59750</v>
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="E33" s="14" t="n">
-        <v>54230</v>
+        <v>31668</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>27504</v>
+        <v>28082</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-248478</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-276560</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-304064</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-290900</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-260924</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-350049</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>22749.58333333333</v>
+        <v>22919.09999999999</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22524.88333333333</v>
+        <v>22704.59999999999</v>
       </c>
     </row>
     <row r="34">
@@ -2664,13 +2664,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="n">
-        <v>-18</v>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>62</v>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="14" t="n">
-        <v>1355</v>
+        <v>4783</v>
       </c>
       <c r="F34" s="13" t="inlineStr">
         <is>
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-1373</v>
+        <v>-4721</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>14662</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>19383</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>20756</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>23219</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>24263</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>15273</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22652.66666666666</v>
+        <v>22847.59999999999</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22509.45</v>
+        <v>22668.85</v>
       </c>
     </row>
     <row r="35">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="C35" s="11" t="n">
-        <v>17310</v>
+        <v>13093</v>
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
@@ -2745,15 +2745,15 @@
         </is>
       </c>
       <c r="E35" s="14" t="n">
-        <v>14482</v>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G35" s="11" t="n">
-        <v>2828</v>
+        <v>21932</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>-8839</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>131260</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>140099</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>137271</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>127248</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>123171</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>245437</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22524.88333333333</v>
+        <v>22704.59999999999</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="C36" s="11" t="n">
-        <v>26661</v>
+        <v>21068</v>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="E36" s="14" t="n">
-        <v>55620</v>
+        <v>35590</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
@@ -2814,7 +2814,7 @@
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-28959</v>
+        <v>-14522</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>102556</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>117078</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>146037</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>140433</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>113490</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>89339</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22427.96666666666</v>
+        <v>22633.09999999999</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>125687</v>
+        <v>93973</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>125687</v>
+        <v>93973</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22300.18333333333</v>
+        <v>22490.09999999999</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22203.26666666666</v>
+        <v>22418.59999999999</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>13.61</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>14.78</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>14.46</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>13.49</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>13.41</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>13.64</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9536774908049497</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9443402010193789</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9386076799537314</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.946824047390084</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9508129344180111</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9536176861203818</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,556    PCR(OI) 0.89    Max Pain 22,550</t>
+          <t>Spot 22,776    PCR(OI) 1.45    Max Pain 22,750</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23882.39233870968</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23885.19516129032</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23888.52177419355</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23890.86975806452</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23891.34516129032</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23888.24193548387</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22776.1</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22555.75</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22421.95</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22620.45</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22716.2</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22780.25</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3137,17 +3137,17 @@
         <v>22800</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>221193</v>
+        <v>338466</v>
       </c>
       <c r="R45" s="14" t="n">
-        <v>83607</v>
+        <v>117273</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>5342437</v>
+        <v>22937164</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9255281866927508</v>
+        <v>0.9345016493863957</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9199158076678682</v>
@@ -3173,20 +3173,20 @@
         <v>0.9605609315602034</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23000</v>
+        <v>22900</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>225585</v>
-      </c>
-      <c r="R46" s="14" t="n">
-        <v>13820</v>
+        <v>171063</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>-1238</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>2736232</v>
+        <v>8780604</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24370.67862903226</v>
+        <v>24372.45564516129</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24373.91532258064</v>
@@ -3212,18 +3212,18 @@
         <v>24358.78790322581</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>23500</v>
+        <v>23000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>205470</v>
-      </c>
-      <c r="R47" s="14" t="n">
-        <v>13209</v>
+        <v>200099</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>-25486</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>1412013</v>
-      </c>
-      <c r="T47" s="30" t="inlineStr">
+        <v>3661418</v>
+      </c>
+      <c r="T47" s="31" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22555.75</v>
+        <v>22776.1</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>22421.95</v>
@@ -3250,7 +3250,7 @@
       <c r="N48" s="18" t="n">
         <v>23398.1</v>
       </c>
-      <c r="P48" s="31" t="inlineStr">
+      <c r="P48" s="32" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="29" t="inlineStr">
-        <is>
-          <t>05-Oct-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="29" t="inlineStr">
+      <c r="J49" s="30" t="inlineStr">
+        <is>
+          <t>06-Oct-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="30" t="inlineStr">
         <is>
           <t>01-Oct-2026</t>
         </is>
       </c>
-      <c r="L49" s="29" t="inlineStr">
+      <c r="L49" s="30" t="inlineStr">
         <is>
           <t>25-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="29" t="inlineStr">
+      <c r="M49" s="30" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="N49" s="29" t="inlineStr">
+      <c r="N49" s="30" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
@@ -3318,66 +3318,66 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
-        <v>22500</v>
+      <c r="P50" s="33" t="n">
+        <v>22750</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>188172</v>
+        <v>284265</v>
       </c>
       <c r="R50" s="14" t="n">
-        <v>112545</v>
+        <v>273343</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>13269393</v>
-      </c>
-      <c r="T50" s="33" t="inlineStr">
+        <v>10173699</v>
+      </c>
+      <c r="T50" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="P51" s="33" t="n">
+        <v>22700</v>
+      </c>
+      <c r="Q51" s="12" t="n">
+        <v>406319</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>372567</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>25605423</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="P51" s="32" t="n">
-        <v>22000</v>
-      </c>
-      <c r="Q51" s="12" t="n">
-        <v>196668</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>41922</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>3581139</v>
-      </c>
-      <c r="T51" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>21500</v>
+      <c r="P52" s="33" t="n">
+        <v>22600</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>226555</v>
+        <v>221466</v>
       </c>
       <c r="R52" s="14" t="n">
-        <v>78597</v>
+        <v>143438</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>1745808</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>23617674</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 05-Oct-2026    1 DAY AGO = 01-Oct-2026    2 DAYS AGO = 30-Sep-2026    3 DAYS AGO = 29-Sep-2026    4 DAYS AGO = 28-Sep-2026    (generated 05-Oct-2026 20:31 IST)</t>
+          <t>TODAY = 06-Oct-2026    1 DAY AGO = 05-Oct-2026    2 DAYS AGO = 01-Oct-2026    3 DAYS AGO = 30-Sep-2026    4 DAYS AGO = 29-Sep-2026    (generated 06-Oct-2026 20:35 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-07
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -193,14 +193,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-4933</v>
+        <v>8300</v>
       </c>
     </row>
     <row r="3">
@@ -701,27 +701,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-4339</v>
+        <v>5721</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>594</v>
+        <v>-2579</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-4933</v>
+        <v>8300</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,26 +729,26 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>245400</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>237100</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>242033</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>249812</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>242426</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>223813</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
+      <c r="Q3" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="14" t="n">
-        <v>87245</v>
+      <c r="S3" s="11" t="n">
+        <v>36119</v>
       </c>
     </row>
     <row r="4">
@@ -768,29 +768,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
-        <v>273</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="C4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E4" s="14" t="n">
-        <v>-800</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="E4" s="11" t="n">
+        <v>-17</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>1073</v>
+      <c r="G4" s="11" t="n">
+        <v>18</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,26 +798,26 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>33919</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>33901</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>32828</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>33257</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>32050</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>35508</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="13" t="inlineStr">
+      <c r="Q4" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -827,8 +827,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>-22660</v>
+      <c r="S4" s="11" t="n">
+        <v>-57123</v>
       </c>
     </row>
     <row r="5">
@@ -837,67 +837,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
-        <v>1168</v>
+      <c r="C5" s="11" t="n">
+        <v>3141</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>-7498</v>
+        <v>7701</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>-4560</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-298285</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-293725</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-302391</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-310174</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-282870</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>8666</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-293725</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-302391</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-310174</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-282870</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-267307</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>-17248</v>
+        <v>35758</v>
       </c>
     </row>
     <row r="6">
@@ -908,27 +908,27 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>-1907</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
+        <v>1035</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
-        <v>2899</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="E6" s="14" t="n">
+        <v>4793</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>-4806</v>
+      <c r="G6" s="14" t="n">
+        <v>-3758</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,20 +936,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>18966</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>22724</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>27530</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>27105</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>8394</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>7986</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -957,7 +957,7 @@
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R6" s="10" t="inlineStr">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>-32547</v>
+        <v>158075</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-4805</v>
+        <v>9898</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-4805</v>
+        <v>9898</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>28082</v>
+        <v>-53841</v>
       </c>
     </row>
     <row r="8">
@@ -1071,7 +1071,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
+      <c r="Q8" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>1073</v>
+      <c r="S8" s="11" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -1093,27 +1093,27 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>-1784356</v>
+        <v>761996</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>-1871601</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+        <v>725877</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>87245</v>
+      <c r="G9" s="11" t="n">
+        <v>36119</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,26 +1121,26 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>242626</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>206507</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>119262</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>295484</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>433777</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>316656</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>3885</v>
+      <c r="S9" s="11" t="n">
+        <v>33672</v>
       </c>
     </row>
     <row r="10">
@@ -1160,29 +1160,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>2834</v>
+      <c r="C10" s="11" t="n">
+        <v>33722</v>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E10" s="14" t="n">
-        <v>-1051</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+        <v>50</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>3885</v>
+      <c r="G10" s="11" t="n">
+        <v>33672</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,26 +1190,26 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>61443</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>27771</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>23886</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>4976</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>5551</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>4572</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>226</v>
+      <c r="S10" s="14" t="n">
+        <v>1150</v>
       </c>
     </row>
     <row r="11">
@@ -1231,65 +1231,65 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>-223082</v>
+        <v>113286</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>-241329</v>
+        <v>165881</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>-52595</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-400079</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-347484</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-365731</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-431465</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-465583</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>18247</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-347484</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-365731</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-431465</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-465583</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-421463</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S11" s="11" t="n">
-        <v>-1287</v>
+        <v>11280</v>
       </c>
     </row>
     <row r="12">
@@ -1300,27 +1300,27 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>-550365</v>
+        <v>252495</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>-440988</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
+        <v>269691</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>-109377</v>
+      <c r="G12" s="14" t="n">
+        <v>-17196</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,26 +1328,26 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>96011</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>113207</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>222584</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>131005</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>26254</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>100235</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>-26743</v>
+      <c r="S12" s="14" t="n">
+        <v>-42248</v>
       </c>
     </row>
     <row r="13">
@@ -1369,11 +1369,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-2554969</v>
+        <v>1161499</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-2554969</v>
+        <v>1161499</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
+      <c r="Q13" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="14" t="n">
-        <v>-4721</v>
+      <c r="S13" s="11" t="n">
+        <v>-1791</v>
       </c>
     </row>
     <row r="14">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>8666</v>
+        <v>-4560</v>
       </c>
     </row>
     <row r="15">
@@ -1485,27 +1485,27 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>-1364022</v>
+        <v>322550</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>-1341362</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
+        <v>379673</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G15" s="14" t="n">
-        <v>-22660</v>
+      <c r="G15" s="11" t="n">
+        <v>-57123</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-714880</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-657757</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-635097</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-843148</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-842693</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-745968</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>18247</v>
+        <v>-52595</v>
       </c>
     </row>
     <row r="16">
@@ -1554,27 +1554,27 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>-150</v>
+        <v>1150</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>-376</v>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>226</v>
+      <c r="G16" s="14" t="n">
+        <v>1150</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>54691</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>53541</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>53315</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>39526</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>46658</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>49394</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>-20549</v>
+        <v>6899</v>
       </c>
     </row>
     <row r="17">
@@ -1623,65 +1623,65 @@
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C17" s="14" t="n">
-        <v>-248566</v>
+        <v>63743</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>-228017</v>
+        <v>56844</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>6899</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>574665</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>567766</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>588315</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>666578</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>668125</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>-20549</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>567766</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>588315</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>666578</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>668125</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>651257</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S17" s="14" t="n">
-        <v>43509</v>
+        <v>-29795</v>
       </c>
     </row>
     <row r="18">
@@ -1692,27 +1692,27 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>-404592</v>
+        <v>155323</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>-447575</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+        <v>106249</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>42983</v>
+      <c r="G18" s="14" t="n">
+        <v>49074</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,20 +1720,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>85524</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>36450</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>-6533</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>137044</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>127910</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>45318</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="Q18" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R18" s="10" t="inlineStr">
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>722</v>
+        <v>-27176</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-2017330</v>
+        <v>542766</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-2017330</v>
+        <v>542766</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>-8839</v>
+        <v>2768</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>-4806</v>
+      <c r="S20" s="14" t="n">
+        <v>-3758</v>
       </c>
     </row>
     <row r="21">
@@ -1877,65 +1877,65 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-5752</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
+        <v>41224</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>11496</v>
+      <c r="E21" s="14" t="n">
+        <v>5466</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>35758</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3275984</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3240226</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3257474</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3267608</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3299362</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>-17248</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>3240226</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>3257474</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>3267608</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>3299362</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>3275421</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>-109377</v>
+      <c r="S21" s="14" t="n">
+        <v>-17196</v>
       </c>
     </row>
     <row r="22">
@@ -1944,29 +1944,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n">
-        <v>5264</v>
+      <c r="C22" s="11" t="n">
+        <v>8779</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>6551</v>
+        <v>-2501</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G22" s="11" t="n">
-        <v>-1287</v>
+        <v>11280</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,26 +1974,26 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4302942</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4314222</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4312935</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4310252</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4309555</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4300555</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="9" t="inlineStr">
+      <c r="Q22" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>42983</v>
+      <c r="S22" s="14" t="n">
+        <v>49074</v>
       </c>
     </row>
     <row r="23">
@@ -2013,29 +2013,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n">
-        <v>21621</v>
+      <c r="C23" s="11" t="n">
+        <v>23645</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>-21888</v>
+        <v>53440</v>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G23" s="14" t="n">
-        <v>43509</v>
+        <v>-29795</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,26 +2043,26 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>580702</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>610497</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>566988</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>535081</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>489549</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>496408</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>-24974</v>
+      <c r="S23" s="14" t="n">
+        <v>-17243</v>
       </c>
     </row>
     <row r="24">
@@ -2084,27 +2084,27 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>-14287</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+        <v>5186</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>10687</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="E24" s="14" t="n">
+        <v>22429</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>-24974</v>
+      <c r="G24" s="14" t="n">
+        <v>-17243</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,20 +2112,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>446256</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>463499</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>488473</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>507563</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>520644</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>528726</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="Q24" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>58568</v>
+        <v>-88651</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>6846</v>
+        <v>78834</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>6846</v>
+        <v>78834</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>-14522</v>
+        <v>52864</v>
       </c>
     </row>
     <row r="26">
@@ -2249,29 +2249,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
-        <v>23278</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="C27" s="11" t="n">
+        <v>217694</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>55825</v>
+      <c r="E27" s="14" t="n">
+        <v>59619</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>-32547</v>
+        <v>158075</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>844420</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>686345</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>718892</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>682768</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>598531</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>504186</v>
       </c>
     </row>
     <row r="28">
@@ -2300,29 +2300,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="14" t="n">
-        <v>700</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="C28" s="11" t="n">
+        <v>1537</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>27443</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>43785</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>-26743</v>
+      <c r="G28" s="14" t="n">
+        <v>-42248</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-297558</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-255310</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-228567</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-194897</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-175620</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-125433</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>22848</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>10395</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
-        <v>22126</v>
+      <c r="E29" s="14" t="n">
+        <v>37571</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>722</v>
+        <v>-27176</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-134565</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-107389</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-108111</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-94492</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-87623</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-79836</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 06-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 07-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,29 +2418,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
-        <v>69562</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="C30" s="11" t="n">
+        <v>17480</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n">
-        <v>10994</v>
+      <c r="E30" s="14" t="n">
+        <v>106131</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>58568</v>
+        <v>-88651</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-412297</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-323646</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-382214</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-393379</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-335288</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-298917</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22603.25</v>
+        <v>22690.45</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>22776.1</v>
+        <v>22717.65</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>116388</v>
+        <v>247106</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>116388</v>
+        <v>247106</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22561.6</v>
+        <v>22546.3</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22776.1</v>
+        <v>22603.05</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23062.09999999999</v>
+        <v>22869.71666666667</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22740.34999999999</v>
+        <v>22612.69166666667</v>
       </c>
     </row>
     <row r="33">
@@ -2597,29 +2597,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>59750</v>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="C33" s="14" t="n">
+        <v>22811</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="14" t="n">
-        <v>31668</v>
+      <c r="E33" s="11" t="n">
+        <v>76652</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>28082</v>
+        <v>-53841</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-302319</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-248478</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-276560</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-304064</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-290900</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-260924</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>22919.09999999999</v>
+        <v>22793.68333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22704.59999999999</v>
+        <v>22622.33333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2664,29 +2664,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>62</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="C34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>4783</v>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
+      <c r="E34" s="11" t="n">
+        <v>1791</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>-4721</v>
+      <c r="G34" s="11" t="n">
+        <v>-1791</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>12871</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>14662</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>19383</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>20756</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>23219</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>24263</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22847.59999999999</v>
+        <v>22698.36666666666</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22668.85</v>
+        <v>22631.975</v>
       </c>
     </row>
     <row r="35">
@@ -2731,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>13093</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="n">
+        <v>19084</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>21932</v>
+      <c r="E35" s="11" t="n">
+        <v>16316</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>-8839</v>
+        <v>2768</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>134028</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>131260</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>140099</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>137271</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>127248</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>123171</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22704.59999999999</v>
+        <v>22622.33333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,29 +2792,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>21068</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="14" t="n">
+        <v>62832</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>35590</v>
+      <c r="E36" s="11" t="n">
+        <v>9968</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-14522</v>
+        <v>52864</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>155420</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>102556</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>117078</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>146037</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>140433</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>113490</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22633.09999999999</v>
+        <v>22527.01666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>93973</v>
+        <v>104727</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>93973</v>
+        <v>104727</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22490.09999999999</v>
+        <v>22450.98333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22418.59999999999</v>
+        <v>22355.66666666666</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>13.89</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>13.61</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>14.78</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>14.46</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>13.49</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>13.41</v>
       </c>
     </row>
     <row r="41">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 06-Oct-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 13-Oct-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9468773774630451</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9536774908049497</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9443402010193789</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9386076799537314</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.946824047390084</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9508129344180111</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,776    PCR(OI) 1.45    Max Pain 22,750</t>
+          <t>Spot 22,603    PCR(OI) 0.81    Max Pain 22,650</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23871.14798387097</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23882.39233870968</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23885.19516129032</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23888.52177419355</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23890.86975806452</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23891.34516129032</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22603.05</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22776.1</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22555.75</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22421.95</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22620.45</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22716.2</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>22800</v>
+        <v>22700</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>338466</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>117273</v>
+        <v>132447</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>60582</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>22937164</v>
+        <v>3511063</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9345016493863957</v>
+        <v>0.9274545270170964</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9199158076678682</v>
@@ -3173,16 +3173,16 @@
         <v>0.9605609315602034</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>22900</v>
+        <v>22800</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>171063</v>
+        <v>145498</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>-1238</v>
+        <v>81624</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>8780604</v>
+        <v>2518903</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24372.45564516129</v>
+        <v>24371.06008064516</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24373.91532258064</v>
@@ -3215,17 +3215,17 @@
         <v>23000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>200099</v>
+        <v>148173</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>-25486</v>
+        <v>63333</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>3661418</v>
-      </c>
-      <c r="T47" s="31" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>1878895</v>
+      </c>
+      <c r="T47" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22776.1</v>
+        <v>22603.05</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>22421.95</v>
@@ -3250,7 +3250,7 @@
       <c r="N48" s="18" t="n">
         <v>23398.1</v>
       </c>
-      <c r="P48" s="32" t="inlineStr">
+      <c r="P48" s="31" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
-          <t>06-Oct-2026</t>
+          <t>07-Oct-2026</t>
         </is>
       </c>
       <c r="K49" s="30" t="inlineStr">
@@ -3318,66 +3318,66 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
-        <v>22750</v>
+      <c r="P50" s="32" t="n">
+        <v>22600</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>284265</v>
-      </c>
-      <c r="R50" s="14" t="n">
-        <v>273343</v>
+        <v>96163</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>34732</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>10173699</v>
-      </c>
-      <c r="T50" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>4392616</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="33" t="n">
-        <v>22700</v>
+      <c r="P51" s="32" t="n">
+        <v>22000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>406319</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>372567</v>
+        <v>109171</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>30762</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>25605423</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>1297662</v>
+      </c>
+      <c r="T51" s="33" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="33" t="n">
-        <v>22600</v>
+      <c r="P52" s="32" t="n">
+        <v>21500</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>221466</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>143438</v>
+        <v>109328</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>3051</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>23617674</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>688694</v>
+      </c>
+      <c r="T52" s="33" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 06-Oct-2026    1 DAY AGO = 05-Oct-2026    2 DAYS AGO = 01-Oct-2026    3 DAYS AGO = 30-Sep-2026    4 DAYS AGO = 29-Sep-2026    (generated 06-Oct-2026 20:35 IST)</t>
+          <t>TODAY = 07-Oct-2026    1 DAY AGO = 06-Oct-2026    2 DAYS AGO = 05-Oct-2026    3 DAYS AGO = 01-Oct-2026    4 DAYS AGO = 30-Sep-2026    (generated 07-Oct-2026 20:40 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-08
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,10 +187,10 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -199,7 +199,7 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>8300</v>
+        <v>1993</v>
       </c>
     </row>
     <row r="3">
@@ -705,15 +705,15 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>5721</v>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="n">
-        <v>-2579</v>
+        <v>4595</v>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>2602</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,28 +721,28 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>8300</v>
+        <v>1993</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="14" t="n">
+        <v>247393</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>245400</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="14" t="n">
         <v>237100</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="14" t="n">
         <v>242033</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>249812</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>242426</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>36119</v>
+        <v>167405</v>
       </c>
     </row>
     <row r="4">
@@ -768,13 +768,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>1</v>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>-182</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>-17</v>
+        <v>-2513</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -790,28 +790,28 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>18</v>
+        <v>2331</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="14" t="n">
+        <v>36250</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>33919</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="14" t="n">
         <v>33901</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="14" t="n">
         <v>32828</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="14" t="n">
         <v>33257</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>32050</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-57123</v>
+        <v>-111739</v>
       </c>
     </row>
     <row r="5">
@@ -837,58 +837,58 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>3141</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>-1843</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n">
-        <v>7701</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="E5" s="13" t="n">
+        <v>6981</v>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-4560</v>
+      <c r="G5" s="13" t="n">
+        <v>-8824</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="14" t="n">
+        <v>-307109</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-298285</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="14" t="n">
         <v>-293725</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="14" t="n">
         <v>-302391</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="14" t="n">
         <v>-310174</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-282870</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q5" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -896,8 +896,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>35758</v>
+      <c r="S5" s="13" t="n">
+        <v>-22854</v>
       </c>
     </row>
     <row r="6">
@@ -906,50 +906,50 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>1035</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>4793</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>-3758</v>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>-478</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>-4978</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>4500</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
+        <v>23466</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>18966</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>22724</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="14" t="n">
         <v>27530</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="14" t="n">
         <v>27105</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>8394</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>158075</v>
+        <v>170525</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>9898</v>
+        <v>2092</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>9898</v>
+        <v>2092</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-53841</v>
+        <v>-36508</v>
       </c>
     </row>
     <row r="8">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>18</v>
+        <v>2331</v>
       </c>
     </row>
     <row r="9">
@@ -1097,15 +1097,15 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>761996</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
+        <v>1184767</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="14" t="n">
-        <v>725877</v>
+      <c r="E9" s="13" t="n">
+        <v>1017362</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -1113,28 +1113,28 @@
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>36119</v>
+        <v>167405</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="14" t="n">
+        <v>410031</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>242626</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="14" t="n">
         <v>206507</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="14" t="n">
         <v>119262</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="14" t="n">
         <v>295484</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>433777</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>33672</v>
+        <v>23456</v>
       </c>
     </row>
     <row r="10">
@@ -1166,15 +1166,15 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>33722</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
+        <v>23761</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="14" t="n">
-        <v>50</v>
+      <c r="E10" s="13" t="n">
+        <v>305</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -1182,34 +1182,34 @@
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>33672</v>
+        <v>23456</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
+        <v>84899</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>61443</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>27771</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="14" t="n">
         <v>23886</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="14" t="n">
         <v>4976</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>5551</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
+      <c r="Q10" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>1150</v>
+      <c r="S10" s="13" t="n">
+        <v>1693</v>
       </c>
     </row>
     <row r="11">
@@ -1235,52 +1235,52 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>113286</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
+        <v>230429</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E11" s="14" t="n">
-        <v>165881</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="E11" s="13" t="n">
+        <v>234628</v>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-52595</v>
+      <c r="G11" s="13" t="n">
+        <v>-4199</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="14" t="n">
+        <v>-404278</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-400079</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="14" t="n">
         <v>-347484</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="14" t="n">
         <v>-365731</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="14" t="n">
         <v>-431465</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-465583</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q11" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>11280</v>
+      <c r="S11" s="13" t="n">
+        <v>-19775</v>
       </c>
     </row>
     <row r="12">
@@ -1304,50 +1304,50 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>252495</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
+        <v>265265</v>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E12" s="14" t="n">
-        <v>269691</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="E12" s="13" t="n">
+        <v>451928</v>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-17196</v>
+      <c r="G12" s="13" t="n">
+        <v>-186663</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="14" t="n">
+        <v>-90652</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>96011</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <v>113207</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="14" t="n">
         <v>222584</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="14" t="n">
         <v>131005</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>26254</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="13" t="inlineStr">
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>-42248</v>
+      <c r="S12" s="13" t="n">
+        <v>-27621</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1161499</v>
+        <v>1704222</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1161499</v>
+        <v>1704223</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-1791</v>
+        <v>-2105</v>
       </c>
     </row>
     <row r="14">
@@ -1463,7 +1463,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
+      <c r="Q14" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>-4560</v>
+      <c r="S14" s="13" t="n">
+        <v>-8824</v>
       </c>
     </row>
     <row r="15">
@@ -1483,13 +1483,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
-        <v>322550</v>
+      <c r="C15" s="13" t="n">
+        <v>214358</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>379673</v>
+        <v>326097</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1505,34 +1505,34 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-57123</v>
+        <v>-111739</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-826619</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-714880</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-657757</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>-635097</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>-843148</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-842693</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
+      <c r="Q15" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>-52595</v>
+      <c r="S15" s="13" t="n">
+        <v>-4199</v>
       </c>
     </row>
     <row r="16">
@@ -1552,13 +1552,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
-        <v>1150</v>
+      <c r="C16" s="13" t="n">
+        <v>2093</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1566,42 +1566,42 @@
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
+        <v>400</v>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>1150</v>
+      <c r="G16" s="13" t="n">
+        <v>1693</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="14" t="n">
+        <v>56384</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>54691</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <v>53541</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="14" t="n">
         <v>53315</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="14" t="n">
         <v>39526</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>46658</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
+      <c r="Q16" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>6899</v>
+      <c r="S16" s="13" t="n">
+        <v>91418</v>
       </c>
     </row>
     <row r="17">
@@ -1621,13 +1621,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n">
-        <v>63743</v>
+      <c r="C17" s="13" t="n">
+        <v>132428</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1635,44 +1635,44 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>56844</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+        <v>41010</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>6899</v>
+      <c r="G17" s="13" t="n">
+        <v>91418</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="12" t="n">
+      <c r="J17" s="14" t="n">
+        <v>666083</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <v>574665</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="14" t="n">
         <v>567766</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="14" t="n">
         <v>588315</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="14" t="n">
         <v>666578</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>668125</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1680,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>-29795</v>
+      <c r="S17" s="11" t="n">
+        <v>29144</v>
       </c>
     </row>
     <row r="18">
@@ -1690,13 +1690,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
-        <v>155323</v>
+      <c r="C18" s="13" t="n">
+        <v>214825</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1704,42 +1704,42 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>106249</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
+        <v>196197</v>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>49074</v>
+      <c r="G18" s="13" t="n">
+        <v>18628</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="12" t="n">
+      <c r="J18" s="14" t="n">
+        <v>104152</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>85524</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="14" t="n">
         <v>36450</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="14" t="n">
         <v>-6533</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="14" t="n">
         <v>137044</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>127910</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="13" t="inlineStr">
+      <c r="Q18" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>-27176</v>
+      <c r="S18" s="13" t="n">
+        <v>-25913</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>542766</v>
+        <v>563704</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>542766</v>
+        <v>563704</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1786,7 +1786,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
+      <c r="Q19" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>2768</v>
+      <c r="S19" s="13" t="n">
+        <v>16793</v>
       </c>
     </row>
     <row r="20">
@@ -1855,9 +1855,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>-3758</v>
+      <c r="S20" s="11" t="n">
+        <v>4500</v>
       </c>
     </row>
     <row r="21">
@@ -1875,56 +1875,56 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="n">
-        <v>41224</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="n">
-        <v>5466</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G21" s="11" t="n">
-        <v>35758</v>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="n">
+        <v>-22876</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>-22</v>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>-22854</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="14" t="n">
+        <v>3253130</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3275984</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <v>3240226</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="14" t="n">
         <v>3257474</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="14" t="n">
         <v>3267608</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3299362</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
+      <c r="Q21" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-17196</v>
+      <c r="S21" s="13" t="n">
+        <v>-186663</v>
       </c>
     </row>
     <row r="22">
@@ -1950,61 +1950,61 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>8779</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>-2501</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+        <v>7073</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>26848</v>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>-19775</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>-4322717</v>
+      </c>
+      <c r="K22" s="14" t="n">
+        <v>-4302942</v>
+      </c>
+      <c r="L22" s="14" t="n">
+        <v>-4314222</v>
+      </c>
+      <c r="M22" s="14" t="n">
+        <v>-4312935</v>
+      </c>
+      <c r="N22" s="14" t="n">
+        <v>-4310252</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q22" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>11280</v>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J22" s="12" t="n">
-        <v>-4302942</v>
-      </c>
-      <c r="K22" s="12" t="n">
-        <v>-4314222</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>-4312935</v>
-      </c>
-      <c r="M22" s="12" t="n">
-        <v>-4310252</v>
-      </c>
-      <c r="N22" s="12" t="n">
-        <v>-4309555</v>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q22" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>49074</v>
+      <c r="S22" s="13" t="n">
+        <v>18628</v>
       </c>
     </row>
     <row r="23">
@@ -2019,52 +2019,52 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>23645</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+        <v>39303</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n">
-        <v>53440</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="n">
-        <v>-29795</v>
+      <c r="E23" s="13" t="n">
+        <v>10159</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>29144</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="J23" s="14" t="n">
+        <v>609846</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>580702</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <v>610497</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="14" t="n">
         <v>566988</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="14" t="n">
         <v>535081</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>489549</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-17243</v>
+      <c r="S23" s="11" t="n">
+        <v>13485</v>
       </c>
     </row>
     <row r="24">
@@ -2088,61 +2088,61 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>5186</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+        <v>21776</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>22429</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+      <c r="E24" s="13" t="n">
+        <v>8291</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>13485</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="n">
+        <v>459741</v>
+      </c>
+      <c r="K24" s="14" t="n">
+        <v>446256</v>
+      </c>
+      <c r="L24" s="14" t="n">
+        <v>463499</v>
+      </c>
+      <c r="M24" s="14" t="n">
+        <v>488473</v>
+      </c>
+      <c r="N24" s="14" t="n">
+        <v>507563</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q24" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-17243</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="12" t="n">
-        <v>446256</v>
-      </c>
-      <c r="K24" s="12" t="n">
-        <v>463499</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>488473</v>
-      </c>
-      <c r="M24" s="12" t="n">
-        <v>507563</v>
-      </c>
-      <c r="N24" s="12" t="n">
-        <v>520644</v>
-      </c>
-      <c r="P24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>-88651</v>
+      <c r="S24" s="13" t="n">
+        <v>-116991</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>78834</v>
+        <v>45276</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>78834</v>
+        <v>45276</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,7 +2178,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
+      <c r="Q25" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>52864</v>
+      <c r="S25" s="13" t="n">
+        <v>21820</v>
       </c>
     </row>
     <row r="26">
@@ -2255,15 +2255,15 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>217694</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+        <v>225816</v>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
-        <v>59619</v>
+      <c r="E27" s="13" t="n">
+        <v>55291</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,27 +2271,27 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>158075</v>
+        <v>170525</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>1014945</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>844420</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>686345</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="14" t="n">
         <v>718892</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>682768</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>598531</v>
       </c>
     </row>
     <row r="28">
@@ -2306,43 +2306,43 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>1537</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+        <v>732</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="14" t="n">
-        <v>43785</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="E28" s="13" t="n">
+        <v>28353</v>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>-42248</v>
+      <c r="G28" s="13" t="n">
+        <v>-27621</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-325179</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-297558</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-255310</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="14" t="n">
         <v>-228567</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>-194897</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-175620</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,47 +2365,47 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>10395</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+        <v>6832</v>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>37571</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
+      <c r="E29" s="13" t="n">
+        <v>32745</v>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>-27176</v>
+      <c r="G29" s="13" t="n">
+        <v>-25913</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-160478</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-134565</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-107389</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="14" t="n">
         <v>-108111</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>-94492</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-87623</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 07-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 08-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,51 +2424,51 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>17480</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
+        <v>21446</v>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>106131</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
+      <c r="E30" s="13" t="n">
+        <v>138437</v>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>-88651</v>
+      <c r="G30" s="13" t="n">
+        <v>-116991</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-529288</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-412297</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-323646</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="14" t="n">
         <v>-382214</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="14" t="n">
         <v>-393379</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-335288</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22690.45</v>
+        <v>22599.05</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>22717.65</v>
+        <v>22599.05</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>247106</v>
+        <v>254826</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>247106</v>
+        <v>254826</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22546.3</v>
+        <v>22179.9</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22603.05</v>
+        <v>22231.8</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>22869.71666666667</v>
+        <v>22913.08333333333</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22612.69166666667</v>
+        <v>22284.35833333334</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2597,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="14" t="n">
-        <v>22811</v>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>-6163</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>76652</v>
+        <v>30345</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2619,35 +2619,35 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-53841</v>
+        <v>-36508</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-338827</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-302319</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-248478</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="14" t="n">
         <v>-276560</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="14" t="n">
         <v>-304064</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-290900</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>22793.68333333333</v>
+        <v>22756.06666666667</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22622.33333333333</v>
+        <v>22336.91666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2664,12 +2664,12 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="14" t="n">
+      <c r="C34" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>1791</v>
+        <v>2105</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,35 +2686,35 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-1791</v>
+        <v>-2105</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>10766</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>12871</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>14662</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="14" t="n">
         <v>19383</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="14" t="n">
         <v>20756</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>23219</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22698.36666666666</v>
+        <v>22493.93333333333</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22631.975</v>
+        <v>22389.475</v>
       </c>
     </row>
     <row r="35">
@@ -2731,13 +2731,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>19084</v>
+      <c r="C35" s="13" t="n">
+        <v>28576</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,43 +2745,43 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>16316</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
+        <v>11783</v>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>2768</v>
+      <c r="G35" s="13" t="n">
+        <v>16793</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>150821</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>134028</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>131260</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="14" t="n">
         <v>140099</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="14" t="n">
         <v>137271</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>127248</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22622.33333333333</v>
+        <v>22336.91666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,13 +2792,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>62832</v>
+      <c r="C36" s="13" t="n">
+        <v>52549</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,43 +2806,43 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>9968</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
+        <v>30729</v>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>52864</v>
+      <c r="G36" s="13" t="n">
+        <v>21820</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>177240</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>155420</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>102556</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="14" t="n">
         <v>117078</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="14" t="n">
         <v>146037</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>140433</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22527.01666666666</v>
+        <v>22074.78333333334</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>104727</v>
+        <v>74962</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>104727</v>
+        <v>74962</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22450.98333333333</v>
+        <v>21917.76666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22355.66666666666</v>
+        <v>21655.63333333334</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>15.28</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>13.89</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>13.61</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>14.78</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>14.46</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>13.49</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.931810958742466</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9468773774630451</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9536774908049497</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9443402010193789</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9386076799537314</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.946824047390084</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,603    PCR(OI) 0.81    Max Pain 22,650</t>
+          <t>Spot 22,232    PCR(OI) 0.62    Max Pain 22,400</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23858.70201612903</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23871.14798387097</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23882.39233870968</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23885.19516129032</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23888.52177419355</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23890.86975806452</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22231.8</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22603.05</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22776.1</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22555.75</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22421.95</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22620.45</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>22700</v>
-      </c>
-      <c r="Q45" s="12" t="n">
-        <v>132447</v>
+        <v>23000</v>
+      </c>
+      <c r="Q45" s="14" t="n">
+        <v>219523</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>60582</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>3511063</v>
+        <v>71350</v>
+      </c>
+      <c r="S45" s="14" t="n">
+        <v>1326199</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9274545270170964</v>
+        <v>0.9123333744368372</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9199158076678682</v>
@@ -3173,18 +3173,18 @@
         <v>0.9605609315602034</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>22800</v>
-      </c>
-      <c r="Q46" s="12" t="n">
-        <v>145498</v>
+        <v>23500</v>
+      </c>
+      <c r="Q46" s="14" t="n">
+        <v>197443</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>81624</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>2518903</v>
-      </c>
-      <c r="T46" s="30" t="inlineStr">
+        <v>95851</v>
+      </c>
+      <c r="S46" s="14" t="n">
+        <v>1350677</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24371.06008064516</v>
+        <v>24368.06612903226</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24373.91532258064</v>
@@ -3212,20 +3212,20 @@
         <v>24358.78790322581</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>23000</v>
-      </c>
-      <c r="Q47" s="12" t="n">
-        <v>148173</v>
+        <v>24000</v>
+      </c>
+      <c r="Q47" s="14" t="n">
+        <v>213581</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>63333</v>
-      </c>
-      <c r="S47" s="12" t="n">
-        <v>1878895</v>
+        <v>82743</v>
+      </c>
+      <c r="S47" s="14" t="n">
+        <v>549841</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22603.05</v>
+        <v>22231.8</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>22421.95</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="30" t="inlineStr">
-        <is>
-          <t>07-Oct-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="30" t="inlineStr">
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>08-Oct-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
         <is>
           <t>01-Oct-2026</t>
         </is>
       </c>
-      <c r="L49" s="30" t="inlineStr">
+      <c r="L49" s="29" t="inlineStr">
         <is>
           <t>25-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="30" t="inlineStr">
+      <c r="M49" s="29" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="N49" s="30" t="inlineStr">
+      <c r="N49" s="29" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
@@ -3319,18 +3319,18 @@
     </row>
     <row r="50">
       <c r="P50" s="32" t="n">
-        <v>22600</v>
-      </c>
-      <c r="Q50" s="12" t="n">
-        <v>96163</v>
+        <v>22000</v>
+      </c>
+      <c r="Q50" s="14" t="n">
+        <v>161230</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>34732</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>4392616</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
+        <v>52059</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>2177699</v>
+      </c>
+      <c r="T50" s="33" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3338,46 +3338,46 @@
     </row>
     <row r="51">
       <c r="P51" s="32" t="n">
-        <v>22000</v>
-      </c>
-      <c r="Q51" s="12" t="n">
-        <v>109171</v>
+        <v>21500</v>
+      </c>
+      <c r="Q51" s="14" t="n">
+        <v>149240</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>30762</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>1297662</v>
-      </c>
-      <c r="T51" s="33" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>39912</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>1004025</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="P52" s="32" t="n">
-        <v>21500</v>
-      </c>
-      <c r="Q52" s="12" t="n">
-        <v>109328</v>
+        <v>21000</v>
+      </c>
+      <c r="Q52" s="14" t="n">
+        <v>180823</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>3051</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>688694</v>
-      </c>
-      <c r="T52" s="33" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>97906</v>
+      </c>
+      <c r="S52" s="14" t="n">
+        <v>773129</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 07-Oct-2026    1 DAY AGO = 06-Oct-2026    2 DAYS AGO = 05-Oct-2026    3 DAYS AGO = 01-Oct-2026    4 DAYS AGO = 30-Sep-2026    (generated 07-Oct-2026 20:40 IST)</t>
+          <t>TODAY = 08-Oct-2026    1 DAY AGO = 07-Oct-2026    2 DAYS AGO = 06-Oct-2026    3 DAYS AGO = 05-Oct-2026    4 DAYS AGO = 01-Oct-2026    (generated 08-Oct-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-09
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,10 +187,10 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>1993</v>
+        <v>-17870</v>
       </c>
     </row>
     <row r="3">
@@ -701,48 +701,48 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>4595</v>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
+        <v>-16037</v>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E3" s="13" t="n">
-        <v>2602</v>
+      <c r="E3" s="11" t="n">
+        <v>1833</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>1993</v>
+        <v>-17870</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>229523</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>247393</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>245400</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>237100</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="12" t="n">
         <v>242033</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>249812</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>167405</v>
+        <v>-351296</v>
       </c>
     </row>
     <row r="4">
@@ -768,67 +768,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>-182</v>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>304</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>-2513</v>
+        <v>4624</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>-4320</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>31930</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>36250</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>33919</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>33901</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>32828</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>2331</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="14" t="n">
-        <v>36250</v>
-      </c>
-      <c r="K4" s="14" t="n">
-        <v>33919</v>
-      </c>
-      <c r="L4" s="14" t="n">
-        <v>33901</v>
-      </c>
-      <c r="M4" s="14" t="n">
-        <v>32828</v>
-      </c>
-      <c r="N4" s="14" t="n">
-        <v>33257</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-111739</v>
+        <v>195618</v>
       </c>
     </row>
     <row r="5">
@@ -837,67 +837,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>-1843</v>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="n">
-        <v>6981</v>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>3360</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>-9761</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>13121</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-293988</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-307109</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-298285</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-293725</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-302391</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n">
-        <v>-8824</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="n">
-        <v>-307109</v>
-      </c>
-      <c r="K5" s="14" t="n">
-        <v>-298285</v>
-      </c>
-      <c r="L5" s="14" t="n">
-        <v>-293725</v>
-      </c>
-      <c r="M5" s="14" t="n">
-        <v>-302391</v>
-      </c>
-      <c r="N5" s="14" t="n">
-        <v>-310174</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="13" t="n">
-        <v>-22854</v>
+      <c r="S5" s="11" t="n">
+        <v>-35559</v>
       </c>
     </row>
     <row r="6">
@@ -906,50 +906,50 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>-478</v>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>10844</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-4978</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+        <v>1775</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>4500</v>
+      <c r="G6" s="14" t="n">
+        <v>9069</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="12" t="n">
+        <v>32535</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>23466</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="12" t="n">
         <v>18966</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>22724</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="12" t="n">
         <v>27530</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>27105</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -957,7 +957,7 @@
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R6" s="10" t="inlineStr">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>170525</v>
+        <v>-116384</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>2092</v>
+        <v>-1529</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>2092</v>
+        <v>-1529</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-36508</v>
+        <v>79705</v>
       </c>
     </row>
     <row r="8">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>2331</v>
+        <v>-4320</v>
       </c>
     </row>
     <row r="9">
@@ -1093,65 +1093,65 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>1184767</v>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>1017362</v>
+        <v>-797789</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>-446493</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>-351296</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>58735</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>410031</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>242626</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>206507</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>119262</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>167405</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>410031</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>242626</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>206507</v>
-      </c>
-      <c r="M9" s="14" t="n">
-        <v>119262</v>
-      </c>
-      <c r="N9" s="14" t="n">
-        <v>295484</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>23456</v>
+      <c r="S9" s="14" t="n">
+        <v>2096</v>
       </c>
     </row>
     <row r="10">
@@ -1160,56 +1160,56 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
-        <v>23761</v>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="C10" s="14" t="n">
+        <v>3123</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="13" t="n">
-        <v>305</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="E10" s="11" t="n">
+        <v>1027</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>23456</v>
+      <c r="G10" s="14" t="n">
+        <v>2096</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="12" t="n">
+        <v>86995</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>84899</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="12" t="n">
         <v>61443</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="12" t="n">
         <v>27771</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="12" t="n">
         <v>23886</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>4976</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="12" t="inlineStr">
+      <c r="Q10" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="13" t="n">
-        <v>1693</v>
+      <c r="S10" s="11" t="n">
+        <v>5088</v>
       </c>
     </row>
     <row r="11">
@@ -1231,65 +1231,65 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>230429</v>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>234628</v>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
+        <v>-137125</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>-194585</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>57460</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-346818</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-404278</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-400079</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-347484</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-365731</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="13" t="n">
-        <v>-4199</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="14" t="n">
-        <v>-404278</v>
-      </c>
-      <c r="K11" s="14" t="n">
-        <v>-400079</v>
-      </c>
-      <c r="L11" s="14" t="n">
-        <v>-347484</v>
-      </c>
-      <c r="M11" s="14" t="n">
-        <v>-365731</v>
-      </c>
-      <c r="N11" s="14" t="n">
-        <v>-431465</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="13" t="n">
-        <v>-19775</v>
+      <c r="S11" s="11" t="n">
+        <v>-33922</v>
       </c>
     </row>
     <row r="12">
@@ -1300,65 +1300,65 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>265265</v>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>451928</v>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
+        <v>-47786</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>-339525</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>291739</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>201087</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>-90652</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>96011</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>113207</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>222584</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="13" t="n">
-        <v>-186663</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="n">
-        <v>-90652</v>
-      </c>
-      <c r="K12" s="14" t="n">
-        <v>96011</v>
-      </c>
-      <c r="L12" s="14" t="n">
-        <v>113207</v>
-      </c>
-      <c r="M12" s="14" t="n">
-        <v>222584</v>
-      </c>
-      <c r="N12" s="14" t="n">
-        <v>131005</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="13" t="n">
-        <v>-27621</v>
+      <c r="S12" s="11" t="n">
+        <v>-12378</v>
       </c>
     </row>
     <row r="13">
@@ -1369,11 +1369,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1704222</v>
+        <v>-979577</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1704223</v>
+        <v>-979576</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>-2105</v>
+      <c r="S13" s="14" t="n">
+        <v>-1293</v>
       </c>
     </row>
     <row r="14">
@@ -1463,9 +1463,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q14" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="13" t="n">
-        <v>-8824</v>
+      <c r="S14" s="14" t="n">
+        <v>13121</v>
       </c>
     </row>
     <row r="15">
@@ -1483,58 +1483,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n">
-        <v>214358</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="C15" s="11" t="n">
+        <v>965687</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="11" t="n">
-        <v>326097</v>
+      <c r="E15" s="14" t="n">
+        <v>770069</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-111739</v>
+        <v>195618</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="12" t="n">
+        <v>-631001</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-826619</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="12" t="n">
         <v>-714880</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="12" t="n">
         <v>-657757</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="12" t="n">
         <v>-635097</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-843148</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="13" t="n">
-        <v>-4199</v>
+      <c r="S15" s="14" t="n">
+        <v>57460</v>
       </c>
     </row>
     <row r="16">
@@ -1552,58 +1552,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
-        <v>2093</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="C16" s="11" t="n">
+        <v>5640</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
-        <v>400</v>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="E16" s="14" t="n">
+        <v>552</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="13" t="n">
-        <v>1693</v>
+      <c r="G16" s="11" t="n">
+        <v>5088</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="14" t="n">
+      <c r="J16" s="12" t="n">
+        <v>61472</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>56384</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="12" t="n">
         <v>54691</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="12" t="n">
         <v>53541</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="12" t="n">
         <v>53315</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>39526</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="13" t="n">
-        <v>91418</v>
+      <c r="S16" s="14" t="n">
+        <v>-125591</v>
       </c>
     </row>
     <row r="17">
@@ -1621,67 +1621,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="13" t="n">
-        <v>132428</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="C17" s="11" t="n">
+        <v>122321</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n">
-        <v>41010</v>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="E17" s="14" t="n">
+        <v>247912</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>-125591</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>540492</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>666083</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>574665</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>567766</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>588315</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
-        <v>91418</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="14" t="n">
-        <v>666083</v>
-      </c>
-      <c r="K17" s="14" t="n">
-        <v>574665</v>
-      </c>
-      <c r="L17" s="14" t="n">
-        <v>567766</v>
-      </c>
-      <c r="M17" s="14" t="n">
-        <v>588315</v>
-      </c>
-      <c r="N17" s="14" t="n">
-        <v>666578</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>29144</v>
+      <c r="S17" s="14" t="n">
+        <v>65622</v>
       </c>
     </row>
     <row r="18">
@@ -1690,67 +1690,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="13" t="n">
-        <v>214825</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="C18" s="11" t="n">
+        <v>211168</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
-        <v>196197</v>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
+      <c r="E18" s="14" t="n">
+        <v>286283</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>-75115</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>29037</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>104152</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>85524</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>36450</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>-6533</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="13" t="n">
-        <v>18628</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="14" t="n">
-        <v>104152</v>
-      </c>
-      <c r="K18" s="14" t="n">
-        <v>85524</v>
-      </c>
-      <c r="L18" s="14" t="n">
-        <v>36450</v>
-      </c>
-      <c r="M18" s="14" t="n">
-        <v>-6533</v>
-      </c>
-      <c r="N18" s="14" t="n">
-        <v>137044</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="13" t="n">
-        <v>-25913</v>
+      <c r="S18" s="14" t="n">
+        <v>10277</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>563704</v>
+        <v>1304816</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>563704</v>
+        <v>1304816</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="13" t="n">
-        <v>16793</v>
+      <c r="S19" s="14" t="n">
+        <v>-21168</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>4500</v>
+      <c r="S20" s="14" t="n">
+        <v>9069</v>
       </c>
     </row>
     <row r="21">
@@ -1875,58 +1875,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n">
-        <v>-22876</v>
+      <c r="C21" s="11" t="n">
+        <v>-27093</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>-22</v>
-      </c>
-      <c r="F21" s="12" t="inlineStr">
+        <v>8466</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="13" t="n">
-        <v>-22854</v>
+      <c r="G21" s="11" t="n">
+        <v>-35559</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="14" t="n">
+      <c r="J21" s="12" t="n">
+        <v>3217571</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3253130</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="12" t="n">
         <v>3275984</v>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="M21" s="12" t="n">
         <v>3240226</v>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="N21" s="12" t="n">
         <v>3257474</v>
       </c>
-      <c r="N21" s="14" t="n">
-        <v>3267608</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="13" t="n">
-        <v>-186663</v>
+      <c r="S21" s="14" t="n">
+        <v>291739</v>
       </c>
     </row>
     <row r="22">
@@ -1944,58 +1944,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
-        <v>7073</v>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="C22" s="14" t="n">
+        <v>5330</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="13" t="n">
-        <v>26848</v>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="n">
+        <v>39252</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="13" t="n">
-        <v>-19775</v>
+      <c r="G22" s="11" t="n">
+        <v>-33922</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="14" t="n">
+      <c r="J22" s="12" t="n">
+        <v>-4356639</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4322717</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4302942</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4314222</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4312935</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-4310252</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="13" t="n">
-        <v>18628</v>
+      <c r="S22" s="14" t="n">
+        <v>-75115</v>
       </c>
     </row>
     <row r="23">
@@ -2013,56 +2013,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n">
-        <v>39303</v>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="n">
-        <v>10159</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="C23" s="14" t="n">
+        <v>37869</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>-27753</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>29144</v>
+      <c r="G23" s="14" t="n">
+        <v>65622</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="14" t="n">
+      <c r="J23" s="12" t="n">
+        <v>675468</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>609846</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="L23" s="12" t="n">
         <v>580702</v>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="M23" s="12" t="n">
         <v>610497</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="N23" s="12" t="n">
         <v>566988</v>
       </c>
-      <c r="N23" s="14" t="n">
-        <v>535081</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>13485</v>
+      <c r="S23" s="14" t="n">
+        <v>3859</v>
       </c>
     </row>
     <row r="24">
@@ -2082,58 +2082,58 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C24" s="11" t="n">
-        <v>21776</v>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="C24" s="14" t="n">
+        <v>7635</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="13" t="n">
-        <v>8291</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="E24" s="11" t="n">
+        <v>3776</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>13485</v>
+      <c r="G24" s="14" t="n">
+        <v>3859</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="14" t="n">
+      <c r="J24" s="12" t="n">
+        <v>463600</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>459741</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="12" t="n">
         <v>446256</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="12" t="n">
         <v>463499</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="12" t="n">
         <v>488473</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>507563</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q24" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="13" t="n">
-        <v>-116991</v>
+      <c r="S24" s="14" t="n">
+        <v>118485</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>45276</v>
+        <v>23741</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>45276</v>
+        <v>23741</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="13" t="n">
-        <v>21820</v>
+      <c r="S25" s="14" t="n">
+        <v>-57244</v>
       </c>
     </row>
     <row r="26">
@@ -2251,47 +2251,47 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>225816</v>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
+        <v>-55609</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="13" t="n">
-        <v>55291</v>
+      <c r="E27" s="11" t="n">
+        <v>60775</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>170525</v>
+        <v>-116384</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>898561</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1014945</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>844420</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>686345</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="12" t="n">
         <v>718892</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>682768</v>
       </c>
     </row>
     <row r="28">
@@ -2300,49 +2300,49 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="11" t="n">
-        <v>732</v>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="C28" s="14" t="n">
+        <v>1251</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="13" t="n">
-        <v>28353</v>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="n">
+        <v>13629</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="13" t="n">
-        <v>-27621</v>
+      <c r="G28" s="11" t="n">
+        <v>-12378</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-337557</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-325179</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-297558</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-255310</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="12" t="n">
         <v>-228567</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-194897</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,53 +2359,53 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
-        <v>6832</v>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="C29" s="14" t="n">
+        <v>27855</v>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="13" t="n">
-        <v>32745</v>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G29" s="13" t="n">
-        <v>-25913</v>
+      <c r="E29" s="11" t="n">
+        <v>17578</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>10277</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-150201</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-160478</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-134565</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-107389</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="12" t="n">
         <v>-108111</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-94492</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 08-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 09-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,57 +2418,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
-        <v>21446</v>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="n">
-        <v>138437</v>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="n">
-        <v>-116991</v>
+      <c r="C30" s="14" t="n">
+        <v>88256</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>-30229</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>118485</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-410803</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-529288</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-412297</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-323646</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="12" t="n">
         <v>-382214</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-393379</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22599.05</v>
+        <v>22314.95</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>22599.05</v>
+        <v>22580.75</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>254826</v>
+        <v>61753</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>254826</v>
+        <v>61753</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22179.9</v>
+        <v>22294.75</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22231.8</v>
+        <v>22520.45</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>22913.08333333333</v>
+        <v>22921.88333333333</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22284.35833333334</v>
+        <v>22492.88333333333</v>
       </c>
     </row>
     <row r="33">
@@ -2599,55 +2599,55 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>-6163</v>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
+        <v>93085</v>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="11" t="n">
-        <v>30345</v>
+      <c r="E33" s="14" t="n">
+        <v>13380</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-36508</v>
+        <v>79705</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="14" t="n">
+      <c r="J33" s="12" t="n">
+        <v>-259122</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-338827</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="12" t="n">
         <v>-302319</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="12" t="n">
         <v>-248478</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="12" t="n">
         <v>-276560</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-304064</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>22756.06666666667</v>
+        <v>22751.31666666667</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22336.91666666667</v>
+        <v>22465.31666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2664,57 +2664,57 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="C34" s="11" t="n">
+        <v>146</v>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="11" t="n">
-        <v>2105</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="E34" s="14" t="n">
+        <v>1439</v>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="11" t="n">
-        <v>-2105</v>
+      <c r="G34" s="14" t="n">
+        <v>-1293</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="14" t="n">
+      <c r="J34" s="12" t="n">
+        <v>9473</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>10766</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="12" t="n">
         <v>12871</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="12" t="n">
         <v>14662</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="12" t="n">
         <v>19383</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>20756</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22493.93333333333</v>
+        <v>22635.88333333333</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22389.475</v>
+        <v>22437.75</v>
       </c>
     </row>
     <row r="35">
@@ -2731,57 +2731,57 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="13" t="n">
-        <v>28576</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="C35" s="11" t="n">
+        <v>10457</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="11" t="n">
-        <v>11783</v>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G35" s="13" t="n">
-        <v>16793</v>
+      <c r="E35" s="14" t="n">
+        <v>31625</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>-21168</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="14" t="n">
+      <c r="J35" s="12" t="n">
+        <v>129653</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>150821</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="12" t="n">
         <v>134028</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="12" t="n">
         <v>131260</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="12" t="n">
         <v>140099</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>137271</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22336.91666666667</v>
+        <v>22465.31666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,57 +2792,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="13" t="n">
-        <v>52549</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="C36" s="11" t="n">
+        <v>16331</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
-        <v>30729</v>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="13" t="n">
-        <v>21820</v>
+      <c r="E36" s="14" t="n">
+        <v>73575</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>-57244</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="14" t="n">
+      <c r="J36" s="12" t="n">
+        <v>119996</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>177240</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="12" t="n">
         <v>155420</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="12" t="n">
         <v>102556</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="12" t="n">
         <v>117078</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>146037</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22074.78333333334</v>
+        <v>22349.88333333333</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>74962</v>
+        <v>120019</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>74962</v>
+        <v>120019</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>21917.76666666667</v>
+        <v>22179.31666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>21655.63333333334</v>
+        <v>22063.88333333333</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>14.38</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>15.28</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>13.89</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>13.61</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>14.78</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>14.46</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9443977202311479</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.931810958742466</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9468773774630451</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9536774908049497</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9443402010193789</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9386076799537314</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,232    PCR(OI) 0.62    Max Pain 22,400</t>
+          <t>Spot 22,520    PCR(OI) 1.28    Max Pain 22,500</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23846.36209677419</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23858.70201612903</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23871.14798387097</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23882.39233870968</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23885.19516129032</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23888.52177419355</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22520.45</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22231.8</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22603.05</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22776.1</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22555.75</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22421.95</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23000</v>
-      </c>
-      <c r="Q45" s="14" t="n">
-        <v>219523</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>71350</v>
-      </c>
-      <c r="S45" s="14" t="n">
-        <v>1326199</v>
+        <v>22900</v>
+      </c>
+      <c r="Q45" s="12" t="n">
+        <v>147165</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>35249</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>2002225</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9123333744368372</v>
+        <v>0.9240905192059701</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9199158076678682</v>
@@ -3173,18 +3173,18 @@
         <v>0.9605609315602034</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23500</v>
-      </c>
-      <c r="Q46" s="14" t="n">
-        <v>197443</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>95851</v>
-      </c>
-      <c r="S46" s="14" t="n">
-        <v>1350677</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
+        <v>23000</v>
+      </c>
+      <c r="Q46" s="12" t="n">
+        <v>218522</v>
+      </c>
+      <c r="R46" s="14" t="n">
+        <v>2620</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>2330762</v>
+      </c>
+      <c r="T46" s="30" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24368.06612903226</v>
+        <v>24370.3939516129</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24373.91532258064</v>
@@ -3212,18 +3212,18 @@
         <v>24358.78790322581</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>24000</v>
-      </c>
-      <c r="Q47" s="14" t="n">
-        <v>213581</v>
+        <v>23500</v>
+      </c>
+      <c r="Q47" s="12" t="n">
+        <v>146941</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>82743</v>
-      </c>
-      <c r="S47" s="14" t="n">
-        <v>549841</v>
-      </c>
-      <c r="T47" s="30" t="inlineStr">
+        <v>-50463</v>
+      </c>
+      <c r="S47" s="12" t="n">
+        <v>865343</v>
+      </c>
+      <c r="T47" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22231.8</v>
+        <v>22520.45</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>22421.95</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="29" t="inlineStr">
-        <is>
-          <t>08-Oct-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="29" t="inlineStr">
+      <c r="J49" s="30" t="inlineStr">
+        <is>
+          <t>09-Oct-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="30" t="inlineStr">
         <is>
           <t>01-Oct-2026</t>
         </is>
       </c>
-      <c r="L49" s="29" t="inlineStr">
+      <c r="L49" s="30" t="inlineStr">
         <is>
           <t>25-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="29" t="inlineStr">
+      <c r="M49" s="30" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
         </is>
       </c>
-      <c r="N49" s="29" t="inlineStr">
+      <c r="N49" s="30" t="inlineStr">
         <is>
           <t>11-Sep-2026</t>
         </is>
@@ -3319,16 +3319,16 @@
     </row>
     <row r="50">
       <c r="P50" s="32" t="n">
-        <v>22000</v>
-      </c>
-      <c r="Q50" s="14" t="n">
-        <v>161230</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>52059</v>
-      </c>
-      <c r="S50" s="14" t="n">
-        <v>2177699</v>
+        <v>22500</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>198319</v>
+      </c>
+      <c r="R50" s="14" t="n">
+        <v>153132</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>6894888</v>
       </c>
       <c r="T50" s="33" t="inlineStr">
         <is>
@@ -3340,18 +3340,18 @@
       <c r="P51" s="32" t="n">
         <v>21500</v>
       </c>
-      <c r="Q51" s="14" t="n">
-        <v>149240</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>39912</v>
-      </c>
-      <c r="S51" s="14" t="n">
-        <v>1004025</v>
+      <c r="Q51" s="12" t="n">
+        <v>198195</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>49767</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>1290579</v>
       </c>
       <c r="T51" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3359,25 +3359,25 @@
       <c r="P52" s="32" t="n">
         <v>21000</v>
       </c>
-      <c r="Q52" s="14" t="n">
-        <v>180823</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>97906</v>
-      </c>
-      <c r="S52" s="14" t="n">
-        <v>773129</v>
+      <c r="Q52" s="12" t="n">
+        <v>193137</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>11662</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>1084148</v>
       </c>
       <c r="T52" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 08-Oct-2026    1 DAY AGO = 07-Oct-2026    2 DAYS AGO = 06-Oct-2026    3 DAYS AGO = 05-Oct-2026    4 DAYS AGO = 01-Oct-2026    (generated 08-Oct-2026 20:32 IST)</t>
+          <t>TODAY = 09-Oct-2026    1 DAY AGO = 08-Oct-2026    2 DAYS AGO = 07-Oct-2026    3 DAYS AGO = 06-Oct-2026    4 DAYS AGO = 05-Oct-2026    (generated 09-Oct-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-12
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -187,7 +187,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -199,7 +199,7 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-17870</v>
+        <v>13406</v>
       </c>
     </row>
     <row r="3">
@@ -701,27 +701,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-16037</v>
+        <v>9441</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>1833</v>
+        <v>-3965</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-17870</v>
+        <v>13406</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>242929</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>229523</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>247393</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>245400</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>237100</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>242033</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>-351296</v>
+        <v>329296</v>
       </c>
     </row>
     <row r="4">
@@ -768,67 +768,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
-        <v>304</v>
+      <c r="C4" s="11" t="n">
+        <v>414</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>4624</v>
+        <v>-1817</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>2231</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>34161</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>31930</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>36250</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>33919</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>33901</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>-4320</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>31930</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>36250</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>33919</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>33901</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>32828</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>195618</v>
+        <v>-102156</v>
       </c>
     </row>
     <row r="5">
@@ -839,65 +839,65 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>3360</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+        <v>-2675</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n">
-        <v>-9761</v>
+      <c r="E5" s="11" t="n">
+        <v>-803</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>-1872</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-295860</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-293988</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-307109</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-298285</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-293725</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>13121</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-293988</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-307109</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-298285</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-293725</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-302391</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>-35559</v>
+        <v>15133</v>
       </c>
     </row>
     <row r="6">
@@ -908,65 +908,65 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>10844</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
+        <v>-9621</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
-        <v>1775</v>
+      <c r="E6" s="14" t="n">
+        <v>4144</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>-13765</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>18770</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>32535</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>23466</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>18966</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>22724</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>9069</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>32535</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>23466</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>18966</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>22724</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>27530</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>-116384</v>
+        <v>120776</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-1529</v>
+        <v>-2441</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-1529</v>
+        <v>-2441</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>79705</v>
+        <v>-23424</v>
       </c>
     </row>
     <row r="8">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>-4320</v>
+        <v>2231</v>
       </c>
     </row>
     <row r="9">
@@ -1093,27 +1093,27 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>-797789</v>
+        <v>1529245</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>-446493</v>
+        <v>1199949</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>-351296</v>
+        <v>329296</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,26 +1121,26 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>388031</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>58735</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>410031</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>242626</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>206507</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>119262</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>2096</v>
+      <c r="S9" s="11" t="n">
+        <v>648</v>
       </c>
     </row>
     <row r="10">
@@ -1160,29 +1160,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>3123</v>
+      <c r="C10" s="11" t="n">
+        <v>304</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>1027</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+        <v>-344</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>2096</v>
+      <c r="G10" s="11" t="n">
+        <v>648</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,26 +1190,26 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>87643</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>86995</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>84899</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>61443</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>27771</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>23886</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>5088</v>
+      <c r="S10" s="14" t="n">
+        <v>5812</v>
       </c>
     </row>
     <row r="11">
@@ -1231,27 +1231,27 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>-137125</v>
+        <v>246084</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>-194585</v>
+        <v>261052</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>57460</v>
+        <v>-14968</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,26 +1259,26 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-361786</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-346818</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-404278</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-400079</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-347484</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-365731</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>-33922</v>
+      <c r="S11" s="14" t="n">
+        <v>-11545</v>
       </c>
     </row>
     <row r="12">
@@ -1300,27 +1300,27 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>-47786</v>
+        <v>201034</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>-339525</v>
+        <v>516009</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G12" s="14" t="n">
-        <v>291739</v>
+        <v>-314975</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,26 +1328,26 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>-113888</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>201087</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>-90652</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>96011</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>113207</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>222584</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>-12378</v>
+      <c r="S12" s="14" t="n">
+        <v>-6011</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-979577</v>
+        <v>1976667</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-979576</v>
+        <v>1976666</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
+      <c r="Q13" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="14" t="n">
-        <v>-1293</v>
+      <c r="S13" s="11" t="n">
+        <v>-764</v>
       </c>
     </row>
     <row r="14">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>13121</v>
+        <v>-1872</v>
       </c>
     </row>
     <row r="15">
@@ -1485,27 +1485,27 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>965687</v>
+        <v>-297569</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E15" s="14" t="n">
-        <v>770069</v>
+        <v>-195413</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>195618</v>
+        <v>-102156</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-733157</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-631001</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-826619</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-714880</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-657757</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-635097</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>57460</v>
+        <v>-14968</v>
       </c>
     </row>
     <row r="16">
@@ -1552,29 +1552,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>5640</v>
+      <c r="C16" s="14" t="n">
+        <v>5725</v>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E16" s="14" t="n">
-        <v>552</v>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
+        <v>-87</v>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>5088</v>
+      <c r="G16" s="14" t="n">
+        <v>5812</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>67284</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>61472</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>56384</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>54691</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>53541</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>53315</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>-125591</v>
+        <v>45931</v>
       </c>
     </row>
     <row r="17">
@@ -1623,27 +1623,27 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>122321</v>
+        <v>-86673</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E17" s="14" t="n">
-        <v>247912</v>
+        <v>-132604</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-125591</v>
+        <v>45931</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,26 +1651,26 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>586423</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>540492</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>666083</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>574665</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>567766</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>588315</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1680,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>65622</v>
+      <c r="S17" s="11" t="n">
+        <v>10110</v>
       </c>
     </row>
     <row r="18">
@@ -1692,65 +1692,65 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>211168</v>
+        <v>-168760</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>286283</v>
+        <v>-219173</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>50413</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>79450</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>29037</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>104152</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>85524</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>36450</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>-75115</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>29037</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>104152</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>85524</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>36450</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>-6533</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>10277</v>
+        <v>-18949</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>1304816</v>
+        <v>-547277</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>1304816</v>
+        <v>-547277</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>-21168</v>
+        <v>7571</v>
       </c>
     </row>
     <row r="20">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="14" t="n">
-        <v>9069</v>
+        <v>-13765</v>
       </c>
     </row>
     <row r="21">
@@ -1877,65 +1877,65 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-27093</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
+        <v>19747</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>8466</v>
+      <c r="E21" s="14" t="n">
+        <v>4614</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>15133</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3232704</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3217571</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3253130</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3275984</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3240226</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>-35559</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>3217571</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>3253130</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>3275984</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>3240226</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>3257474</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>291739</v>
+        <v>-314975</v>
       </c>
     </row>
     <row r="22">
@@ -1944,29 +1944,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n">
-        <v>5330</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="C22" s="11" t="n">
+        <v>3855</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="11" t="n">
-        <v>39252</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="E22" s="14" t="n">
+        <v>15400</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>-33922</v>
+      <c r="G22" s="14" t="n">
+        <v>-11545</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4368184</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4356639</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4322717</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4302942</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4314222</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4312935</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>-75115</v>
+        <v>50413</v>
       </c>
     </row>
     <row r="23">
@@ -2013,29 +2013,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n">
-        <v>37869</v>
+      <c r="C23" s="11" t="n">
+        <v>16482</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>-27753</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
+        <v>6372</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>65622</v>
+      <c r="G23" s="11" t="n">
+        <v>10110</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,20 +2043,20 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>685578</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>675468</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>609846</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>580702</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>610497</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>566988</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="Q23" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="S23" s="14" t="n">
-        <v>3859</v>
+        <v>-13698</v>
       </c>
     </row>
     <row r="24">
@@ -2084,27 +2084,27 @@
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C24" s="14" t="n">
-        <v>7635</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+        <v>-2043</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>3776</v>
+      <c r="E24" s="14" t="n">
+        <v>11655</v>
       </c>
       <c r="F24" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G24" s="14" t="n">
-        <v>3859</v>
+        <v>-13698</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,20 +2112,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>449902</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>463600</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>459741</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>446256</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>463499</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>488473</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="Q24" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>118485</v>
+        <v>-95816</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>23741</v>
+        <v>38041</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>23741</v>
+        <v>38041</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>-57244</v>
+        <v>16617</v>
       </c>
     </row>
     <row r="26">
@@ -2251,27 +2251,27 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>-55609</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+        <v>160879</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>60775</v>
+      <c r="E27" s="14" t="n">
+        <v>40103</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>-116384</v>
+        <v>120776</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1019337</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>898561</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1014945</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>844420</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>686345</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>718892</v>
       </c>
     </row>
     <row r="28">
@@ -2300,29 +2300,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="14" t="n">
-        <v>1251</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="C28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>13629</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>6011</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>-12378</v>
+      <c r="G28" s="14" t="n">
+        <v>-6011</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-343568</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-337557</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-325179</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-297558</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-255310</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-228567</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>27855</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>12804</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
-        <v>17578</v>
+      <c r="E29" s="14" t="n">
+        <v>31753</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>10277</v>
+        <v>-18949</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-169150</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-150201</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-160478</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-134565</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-107389</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-108111</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 09-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 12-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,29 +2418,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
-        <v>88256</v>
+      <c r="C30" s="11" t="n">
+        <v>3589</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>-30229</v>
+        <v>99405</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>118485</v>
+        <v>-95816</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-506619</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-410803</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-529288</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-412297</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-323646</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-382214</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22314.95</v>
+        <v>22593.2</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>22580.75</v>
+        <v>22651.1</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>61753</v>
+        <v>177272</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>61753</v>
+        <v>177272</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22294.75</v>
+        <v>22304.45</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22520.45</v>
+        <v>22363.35</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>22921.88333333333</v>
+        <v>22921.46666666666</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22492.88333333333</v>
+        <v>22401.49166666666</v>
       </c>
     </row>
     <row r="33">
@@ -2597,29 +2597,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>93085</v>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="C33" s="14" t="n">
+        <v>4550</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="14" t="n">
-        <v>13380</v>
+      <c r="E33" s="11" t="n">
+        <v>27974</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>79705</v>
+        <v>-23424</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-282546</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-259122</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-338827</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-302319</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-248478</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-276560</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>22751.31666666667</v>
+        <v>22786.28333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22465.31666666667</v>
+        <v>22439.63333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2664,29 +2664,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>146</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="C34" s="14" t="n">
+        <v>1268</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>1439</v>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
+      <c r="E34" s="11" t="n">
+        <v>2032</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>-1293</v>
+      <c r="G34" s="11" t="n">
+        <v>-764</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>8709</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>9473</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>10766</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>12871</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>14662</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>19383</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22635.88333333333</v>
+        <v>22574.81666666666</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22437.75</v>
+        <v>22477.775</v>
       </c>
     </row>
     <row r="35">
@@ -2731,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>10457</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="n">
+        <v>21893</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>31625</v>
+      <c r="E35" s="11" t="n">
+        <v>14322</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>-21168</v>
+        <v>7571</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>137224</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>129653</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>150821</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>134028</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>131260</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>140099</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22465.31666666667</v>
+        <v>22439.63333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,29 +2792,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>16331</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="14" t="n">
+        <v>25543</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>73575</v>
+      <c r="E36" s="11" t="n">
+        <v>8926</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-57244</v>
+        <v>16617</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>136613</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>119996</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>177240</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>155420</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>102556</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>117078</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22349.88333333333</v>
+        <v>22228.16666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>120019</v>
+        <v>53254</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>120019</v>
+        <v>53254</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22179.31666666667</v>
+        <v>22092.98333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22063.88333333333</v>
+        <v>21881.51666666667</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>14.38</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>15.28</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>13.89</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>13.61</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>14.78</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9382791147640293</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9443977202311479</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.931810958742466</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9468773774630451</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9536774908049497</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9443402010193789</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,520    PCR(OI) 1.28    Max Pain 22,500</t>
+          <t>Spot 22,363    PCR(OI) 0.59    Max Pain 22,400</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23834.43225806452</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23846.36209677419</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23858.70201612903</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23871.14798387097</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23882.39233870968</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23885.19516129032</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22363.35</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22520.45</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22231.8</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22603.05</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22776.1</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22555.75</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>22900</v>
+        <v>22500</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>147165</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>35249</v>
+        <v>254972</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>108443</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>2002225</v>
+        <v>7774457</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3158,35 +3158,35 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
+        <v>0.9176949934665591</v>
+      </c>
+      <c r="K46" s="25" t="n">
         <v>0.9240905192059701</v>
       </c>
-      <c r="K46" s="25" t="n">
+      <c r="L46" s="25" t="n">
         <v>0.9199158076678682</v>
       </c>
-      <c r="L46" s="25" t="n">
+      <c r="M46" s="25" t="n">
         <v>0.9493709489654826</v>
       </c>
-      <c r="M46" s="25" t="n">
+      <c r="N46" s="25" t="n">
         <v>0.9581623376424576</v>
       </c>
-      <c r="N46" s="25" t="n">
-        <v>0.9605609315602034</v>
-      </c>
       <c r="P46" s="28" t="n">
-        <v>23000</v>
+        <v>22600</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>218522</v>
-      </c>
-      <c r="R46" s="14" t="n">
-        <v>2620</v>
+        <v>272030</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>158441</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>2330762</v>
-      </c>
-      <c r="T46" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>7082621</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3197,35 +3197,35 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
+        <v>24369.04435483871</v>
+      </c>
+      <c r="K47" s="18" t="n">
         <v>24370.3939516129</v>
       </c>
-      <c r="K47" s="18" t="n">
+      <c r="L47" s="18" t="n">
         <v>24373.91532258064</v>
       </c>
-      <c r="L47" s="18" t="n">
+      <c r="M47" s="18" t="n">
         <v>24374.56088709677</v>
       </c>
-      <c r="M47" s="18" t="n">
+      <c r="N47" s="18" t="n">
         <v>24365.80846774194</v>
       </c>
-      <c r="N47" s="18" t="n">
-        <v>24358.78790322581</v>
-      </c>
       <c r="P47" s="28" t="n">
-        <v>23500</v>
+        <v>23000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>146941</v>
+        <v>258562</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>-50463</v>
+        <v>40040</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>865343</v>
-      </c>
-      <c r="T47" s="29" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>2985848</v>
+      </c>
+      <c r="T47" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3236,19 +3236,19 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
+        <v>22363.35</v>
+      </c>
+      <c r="K48" s="18" t="n">
         <v>22520.45</v>
       </c>
-      <c r="K48" s="18" t="n">
+      <c r="L48" s="18" t="n">
         <v>22421.95</v>
       </c>
-      <c r="L48" s="18" t="n">
+      <c r="M48" s="18" t="n">
         <v>23140.5</v>
       </c>
-      <c r="M48" s="18" t="n">
+      <c r="N48" s="18" t="n">
         <v>23346.4</v>
-      </c>
-      <c r="N48" s="18" t="n">
-        <v>23398.1</v>
       </c>
       <c r="P48" s="31" t="inlineStr">
         <is>
@@ -3268,27 +3268,27 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
+          <t>12-Oct-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="30" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="K49" s="30" t="inlineStr">
+      <c r="L49" s="30" t="inlineStr">
         <is>
           <t>01-Oct-2026</t>
         </is>
       </c>
-      <c r="L49" s="30" t="inlineStr">
+      <c r="M49" s="30" t="inlineStr">
         <is>
           <t>25-Sep-2026</t>
         </is>
       </c>
-      <c r="M49" s="30" t="inlineStr">
+      <c r="N49" s="30" t="inlineStr">
         <is>
           <t>18-Sep-2026</t>
-        </is>
-      </c>
-      <c r="N49" s="30" t="inlineStr">
-        <is>
-          <t>11-Sep-2026</t>
         </is>
       </c>
       <c r="P49" s="27" t="inlineStr">
@@ -3319,18 +3319,18 @@
     </row>
     <row r="50">
       <c r="P50" s="32" t="n">
-        <v>22500</v>
+        <v>22200</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>198319</v>
-      </c>
-      <c r="R50" s="14" t="n">
-        <v>153132</v>
+        <v>156058</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>23349</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>6894888</v>
-      </c>
-      <c r="T50" s="33" t="inlineStr">
+        <v>5950750</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3338,37 +3338,37 @@
     </row>
     <row r="51">
       <c r="P51" s="32" t="n">
-        <v>21500</v>
+        <v>22000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>198195</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>49767</v>
+        <v>198067</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>6605</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>1290579</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>4028297</v>
+      </c>
+      <c r="T51" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="P52" s="32" t="n">
-        <v>21000</v>
+        <v>21500</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>193137</v>
+        <v>154449</v>
       </c>
       <c r="R52" s="14" t="n">
-        <v>11662</v>
+        <v>-43746</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>1084148</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
+        <v>1487297</v>
+      </c>
+      <c r="T52" s="33" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 09-Oct-2026    1 DAY AGO = 08-Oct-2026    2 DAYS AGO = 07-Oct-2026    3 DAYS AGO = 06-Oct-2026    4 DAYS AGO = 05-Oct-2026    (generated 09-Oct-2026 20:31 IST)</t>
+          <t>TODAY = 12-Oct-2026    1 DAY AGO = 09-Oct-2026    2 DAYS AGO = 08-Oct-2026    3 DAYS AGO = 07-Oct-2026    4 DAYS AGO = 06-Oct-2026    (generated 12-Oct-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-13
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -193,14 +193,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>13406</v>
+        <v>-13072</v>
       </c>
     </row>
     <row r="3">
@@ -701,27 +701,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>9441</v>
+        <v>-11981</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-3965</v>
+        <v>1091</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>13406</v>
+        <v>-13072</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>229857</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>242929</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>229523</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>247393</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>245400</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>237100</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>329296</v>
+        <v>-276579</v>
       </c>
     </row>
     <row r="4">
@@ -768,29 +768,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C4" s="11" t="n">
-        <v>414</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="C4" s="14" t="n">
+        <v>321</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n">
-        <v>-1817</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="E4" s="14" t="n">
+        <v>-49</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>2231</v>
+      <c r="G4" s="14" t="n">
+        <v>370</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,20 +798,20 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>34531</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>34161</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>31930</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>36250</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>33919</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>33901</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -819,7 +819,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-102156</v>
+        <v>146322</v>
       </c>
     </row>
     <row r="5">
@@ -839,65 +839,65 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>-2675</v>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
+        <v>3148</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E5" s="11" t="n">
-        <v>-803</v>
+      <c r="E5" s="14" t="n">
+        <v>-3217</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>6365</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-289495</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-295860</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-293988</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-307109</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-298285</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-1872</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-295860</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-293988</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-307109</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-298285</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-293725</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>15133</v>
+        <v>-20095</v>
       </c>
     </row>
     <row r="6">
@@ -908,65 +908,65 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>-9621</v>
+        <v>3285</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>4144</v>
+        <v>-3052</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>6337</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>25107</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>18770</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>32535</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>23466</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>18966</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>-13765</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>18770</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>32535</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>23466</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>18966</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>22724</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>120776</v>
+        <v>-155741</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-2441</v>
+        <v>-5227</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-2441</v>
+        <v>-5227</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-23424</v>
+        <v>80542</v>
       </c>
     </row>
     <row r="8">
@@ -1071,7 +1071,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
+      <c r="Q8" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>2231</v>
+      <c r="S8" s="14" t="n">
+        <v>370</v>
       </c>
     </row>
     <row r="9">
@@ -1093,65 +1093,65 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>1529245</v>
+        <v>-2656825</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>1199949</v>
+        <v>-2380246</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>-276579</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>111452</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>388031</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>58735</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>410031</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>242626</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>329296</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>388031</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>58735</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>410031</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>242626</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>206507</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>648</v>
+      <c r="S9" s="14" t="n">
+        <v>7205</v>
       </c>
     </row>
     <row r="10">
@@ -1160,29 +1160,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
-        <v>304</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="C10" s="14" t="n">
+        <v>5546</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n">
-        <v>-344</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="E10" s="14" t="n">
+        <v>-1659</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>648</v>
+      <c r="G10" s="14" t="n">
+        <v>7205</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,26 +1190,26 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>94848</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>87643</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>86995</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>84899</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>61443</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>27771</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
+      <c r="Q10" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>5812</v>
+      <c r="S10" s="11" t="n">
+        <v>7081</v>
       </c>
     </row>
     <row r="11">
@@ -1231,65 +1231,65 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>246084</v>
+        <v>-339611</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>261052</v>
+        <v>-412402</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>72791</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-288995</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-361786</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-346818</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-404278</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-400079</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-14968</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-361786</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-346818</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-404278</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-400079</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-347484</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>-11545</v>
+      <c r="S11" s="11" t="n">
+        <v>-66855</v>
       </c>
     </row>
     <row r="12">
@@ -1300,65 +1300,65 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>201034</v>
+        <v>-646874</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>516009</v>
+        <v>-843457</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>196583</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>82695</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>-113888</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>201087</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>-90652</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>96011</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-314975</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>-113888</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>201087</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>-90652</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>96011</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>113207</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>-6011</v>
+      <c r="S12" s="11" t="n">
+        <v>-10444</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1976667</v>
+        <v>-3637764</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1976666</v>
+        <v>-3637764</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>-764</v>
+      <c r="S13" s="14" t="n">
+        <v>-1113</v>
       </c>
     </row>
     <row r="14">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-1872</v>
+        <v>6365</v>
       </c>
     </row>
     <row r="15">
@@ -1483,29 +1483,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
-        <v>-297569</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="C15" s="14" t="n">
+        <v>-821652</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E15" s="14" t="n">
-        <v>-195413</v>
+      <c r="E15" s="11" t="n">
+        <v>-967974</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-102156</v>
+        <v>146322</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-586835</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-733157</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-631001</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-826619</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-714880</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-657757</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>-14968</v>
+        <v>72791</v>
       </c>
     </row>
     <row r="16">
@@ -1552,29 +1552,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
-        <v>5725</v>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="C16" s="11" t="n">
+        <v>5716</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E16" s="14" t="n">
-        <v>-87</v>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="E16" s="11" t="n">
+        <v>-1365</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>5812</v>
+      <c r="G16" s="11" t="n">
+        <v>7081</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>74365</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>67284</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>61472</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>56384</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>54691</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>53541</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>45931</v>
+        <v>-21085</v>
       </c>
     </row>
     <row r="17">
@@ -1621,67 +1621,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
-        <v>-86673</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="C17" s="14" t="n">
+        <v>-129774</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E17" s="14" t="n">
-        <v>-132604</v>
+      <c r="E17" s="11" t="n">
+        <v>-108689</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>-21085</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>565338</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>586423</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>540492</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>666083</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>574665</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>45931</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>586423</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>540492</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>666083</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>574665</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>567766</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>10110</v>
+      <c r="S17" s="14" t="n">
+        <v>88442</v>
       </c>
     </row>
     <row r="18">
@@ -1690,67 +1690,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n">
-        <v>-168760</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="C18" s="14" t="n">
+        <v>-275963</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E18" s="14" t="n">
-        <v>-219173</v>
+      <c r="E18" s="11" t="n">
+        <v>-143645</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>-132318</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>-52868</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>79450</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>29037</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>104152</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>85524</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>50413</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>79450</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>29037</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>104152</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>85524</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>36450</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-18949</v>
+        <v>16666</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-547277</v>
+        <v>-1221673</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-547277</v>
+        <v>-1221673</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>7571</v>
+        <v>-12931</v>
       </c>
     </row>
     <row r="20">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="14" t="n">
-        <v>-13765</v>
+        <v>6337</v>
       </c>
     </row>
     <row r="21">
@@ -1877,65 +1877,65 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>19747</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+        <v>-4944</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
-        <v>4614</v>
+      <c r="E21" s="11" t="n">
+        <v>15151</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>-20095</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3212609</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3232704</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3217571</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3253130</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3275984</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>15133</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>3232704</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>3217571</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>3253130</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>3275984</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>3240226</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>-314975</v>
+        <v>196583</v>
       </c>
     </row>
     <row r="22">
@@ -1944,29 +1944,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
-        <v>3855</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="n">
+        <v>4762</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
-        <v>15400</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="E22" s="11" t="n">
+        <v>71617</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>-11545</v>
+      <c r="G22" s="11" t="n">
+        <v>-66855</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4435039</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4368184</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4356639</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4322717</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4302942</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4314222</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>50413</v>
+        <v>-132318</v>
       </c>
     </row>
     <row r="23">
@@ -2013,29 +2013,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n">
-        <v>16482</v>
+      <c r="C23" s="14" t="n">
+        <v>49077</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>6372</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+        <v>-39365</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>10110</v>
+      <c r="G23" s="14" t="n">
+        <v>88442</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,26 +2043,26 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>774020</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>685578</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>675468</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>609846</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>580702</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>610497</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-13698</v>
+      <c r="S23" s="11" t="n">
+        <v>-1492</v>
       </c>
     </row>
     <row r="24">
@@ -2084,27 +2084,27 @@
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C24" s="14" t="n">
-        <v>-2043</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+        <v>10680</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>11655</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+      <c r="E24" s="11" t="n">
+        <v>12172</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-13698</v>
+      <c r="G24" s="11" t="n">
+        <v>-1492</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,20 +2112,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>448410</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>449902</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>463600</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>459741</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>446256</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>463499</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="Q24" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-95816</v>
+        <v>149519</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>38041</v>
+        <v>59575</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>38041</v>
+        <v>59575</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>16617</v>
+        <v>-66498</v>
       </c>
     </row>
     <row r="26">
@@ -2251,27 +2251,27 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>160879</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+        <v>-118251</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
-        <v>40103</v>
+      <c r="E27" s="11" t="n">
+        <v>37490</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>120776</v>
+        <v>-155741</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>863596</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1019337</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>898561</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1014945</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>844420</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>686345</v>
       </c>
     </row>
     <row r="28">
@@ -2300,29 +2300,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="C28" s="14" t="n">
+        <v>135</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="14" t="n">
-        <v>6011</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="E28" s="11" t="n">
+        <v>10579</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>-6011</v>
+      <c r="G28" s="11" t="n">
+        <v>-10444</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-354012</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-343568</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-337557</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-325179</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-297558</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-255310</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
-        <v>12804</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="n">
+        <v>36131</v>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>31753</v>
+      <c r="E29" s="11" t="n">
+        <v>19465</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-18949</v>
+        <v>16666</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-152484</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-169150</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-150201</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-160478</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-134565</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-107389</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 12-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 13-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,29 +2418,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
-        <v>3589</v>
+      <c r="C30" s="14" t="n">
+        <v>113834</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>99405</v>
+        <v>-35685</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-95816</v>
+        <v>149519</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-357100</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-506619</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-410803</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-529288</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-412297</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-323646</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22593.2</v>
+        <v>22364.15</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>22651.1</v>
+        <v>22721.95</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>177272</v>
+        <v>31849</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>177272</v>
+        <v>31849</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22304.45</v>
+        <v>22288.45</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22363.35</v>
+        <v>22721.95</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>22921.46666666666</v>
+        <v>23299.95</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22401.49166666666</v>
+        <v>22649.7</v>
       </c>
     </row>
     <row r="33">
@@ -2597,29 +2597,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
-        <v>4550</v>
+      <c r="C33" s="11" t="n">
+        <v>78703</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>27974</v>
+        <v>-1839</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-23424</v>
+        <v>80542</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-202004</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-282546</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-259122</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-338827</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-302319</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-248478</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>22786.28333333333</v>
+        <v>23010.95</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22439.63333333333</v>
+        <v>22577.45</v>
       </c>
     </row>
     <row r="34">
@@ -2664,29 +2664,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="14" t="n">
-        <v>1268</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="C34" s="11" t="n">
+        <v>588</v>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="11" t="n">
-        <v>2032</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="E34" s="14" t="n">
+        <v>1701</v>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="11" t="n">
-        <v>-764</v>
+      <c r="G34" s="14" t="n">
+        <v>-1113</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>7596</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>8709</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>9473</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>10766</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>12871</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>14662</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22574.81666666666</v>
+        <v>22866.45</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22477.775</v>
+        <v>22505.2</v>
       </c>
     </row>
     <row r="35">
@@ -2731,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>21893</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="C35" s="11" t="n">
+        <v>16883</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="11" t="n">
-        <v>14322</v>
+      <c r="E35" s="14" t="n">
+        <v>29814</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>7571</v>
+        <v>-12931</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>124293</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>137224</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>129653</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>150821</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>134028</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>131260</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22439.63333333333</v>
+        <v>22577.45</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,29 +2792,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>25543</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="C36" s="11" t="n">
+        <v>10766</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
-        <v>8926</v>
+      <c r="E36" s="14" t="n">
+        <v>77264</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>16617</v>
+        <v>-66498</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>70115</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>136613</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>119996</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>177240</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>155420</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>102556</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22228.16666666666</v>
+        <v>22432.95</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>53254</v>
+        <v>106940</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>53254</v>
+        <v>106940</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22092.98333333333</v>
+        <v>22143.95</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>21881.51666666667</v>
+        <v>21999.45</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>14.12</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>15.25</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>14.38</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>15.28</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>13.89</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>13.61</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9538116838234366</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9382791147640293</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9443977202311479</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.931810958742466</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9468773774630451</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9536774908049497</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,363    PCR(OI) 0.59    Max Pain 22,400</t>
+          <t>Spot 22,722    PCR(OI) 1.40    Max Pain 22,700</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23822.26008064516</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23834.43225806452</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23846.36209677419</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23858.70201612903</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23871.14798387097</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23882.39233870968</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22721.95</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22363.35</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22520.45</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22231.8</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22603.05</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22776.1</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>22500</v>
+        <v>22750</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>254972</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>108443</v>
+        <v>311637</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>184649</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>7774457</v>
+        <v>23606930</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9176949934665591</v>
+        <v>0.9322997454667669</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9240905192059701</v>
@@ -3173,20 +3173,20 @@
         <v>0.9581623376424576</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>22600</v>
+        <v>22800</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>272030</v>
+        <v>189523</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>158441</v>
+        <v>-27679</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>7082621</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>13773080</v>
+      </c>
+      <c r="T46" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24369.04435483871</v>
+        <v>24371.93629032258</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24370.3939516129</v>
@@ -3215,17 +3215,17 @@
         <v>23000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>258562</v>
+        <v>219628</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>40040</v>
+        <v>-38934</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>2985848</v>
-      </c>
-      <c r="T47" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>3490217</v>
+      </c>
+      <c r="T47" s="31" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22363.35</v>
+        <v>22721.95</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>22520.45</v>
@@ -3250,7 +3250,7 @@
       <c r="N48" s="18" t="n">
         <v>23346.4</v>
       </c>
-      <c r="P48" s="31" t="inlineStr">
+      <c r="P48" s="32" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
-          <t>12-Oct-2026</t>
+          <t>13-Oct-2026</t>
         </is>
       </c>
       <c r="K49" s="30" t="inlineStr">
@@ -3318,66 +3318,66 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
-        <v>22200</v>
+      <c r="P50" s="33" t="n">
+        <v>22700</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>156058</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>23349</v>
+        <v>371827</v>
+      </c>
+      <c r="R50" s="14" t="n">
+        <v>350293</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>5950750</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
+        <v>11023046</v>
+      </c>
+      <c r="T50" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="P51" s="33" t="n">
+        <v>22550</v>
+      </c>
+      <c r="Q51" s="12" t="n">
+        <v>269159</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>247074</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>22795276</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="P51" s="32" t="n">
-        <v>22000</v>
-      </c>
-      <c r="Q51" s="12" t="n">
-        <v>198067</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>6605</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>4028297</v>
-      </c>
-      <c r="T51" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>21500</v>
+      <c r="P52" s="33" t="n">
+        <v>22500</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>154449</v>
+        <v>233808</v>
       </c>
       <c r="R52" s="14" t="n">
-        <v>-43746</v>
+        <v>175410</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>1487297</v>
-      </c>
-      <c r="T52" s="33" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>30318873</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 12-Oct-2026    1 DAY AGO = 09-Oct-2026    2 DAYS AGO = 08-Oct-2026    3 DAYS AGO = 07-Oct-2026    4 DAYS AGO = 06-Oct-2026    (generated 12-Oct-2026 20:31 IST)</t>
+          <t>TODAY = 13-Oct-2026    1 DAY AGO = 12-Oct-2026    2 DAYS AGO = 09-Oct-2026    3 DAYS AGO = 08-Oct-2026    4 DAYS AGO = 07-Oct-2026    (generated 13-Oct-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-14
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-13072</v>
+        <v>15501</v>
       </c>
     </row>
     <row r="3">
@@ -701,27 +701,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-11981</v>
+        <v>7731</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>1091</v>
+        <v>-7770</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-13072</v>
+        <v>15501</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>245358</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>229857</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>242929</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>229523</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>247393</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>245400</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>-276579</v>
+        <v>75969</v>
       </c>
     </row>
     <row r="4">
@@ -768,29 +768,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
-        <v>321</v>
+      <c r="C4" s="11" t="n">
+        <v>152</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>-49</v>
+        <v>4661</v>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G4" s="14" t="n">
-        <v>370</v>
+        <v>-4509</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,20 +798,20 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>30022</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>34531</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>34161</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>31930</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>36250</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>33919</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -819,7 +819,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>146322</v>
+        <v>-119666</v>
       </c>
     </row>
     <row r="5">
@@ -839,65 +839,65 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>3148</v>
+        <v>-1134</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>-3217</v>
+        <v>6068</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>-7202</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-296697</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-289495</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-295860</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-293988</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-307109</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>6365</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-289495</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-295860</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-293988</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-307109</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-298285</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>-20095</v>
+        <v>9466</v>
       </c>
     </row>
     <row r="6">
@@ -908,65 +908,65 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>3285</v>
+        <v>-2982</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>-3052</v>
+        <v>808</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>-3790</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>21317</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>25107</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>18770</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>32535</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>23466</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>6337</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>25107</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>18770</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>32535</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>23466</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>18966</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>-155741</v>
+        <v>124017</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-5227</v>
+        <v>3767</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-5227</v>
+        <v>3767</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>80542</v>
+        <v>-16394</v>
       </c>
     </row>
     <row r="8">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="14" t="n">
-        <v>370</v>
+        <v>-4509</v>
       </c>
     </row>
     <row r="9">
@@ -1093,27 +1093,27 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>-2656825</v>
+        <v>902620</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>-2380246</v>
+        <v>826651</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>-276579</v>
+        <v>75969</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,26 +1121,26 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>187421</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>111452</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>388031</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>58735</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>410031</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>242626</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>7205</v>
+      <c r="S9" s="11" t="n">
+        <v>3535</v>
       </c>
     </row>
     <row r="10">
@@ -1160,29 +1160,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>5546</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="C10" s="11" t="n">
+        <v>3490</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E10" s="14" t="n">
-        <v>-1659</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="E10" s="11" t="n">
+        <v>-45</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>7205</v>
+      <c r="G10" s="11" t="n">
+        <v>3535</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,26 +1190,26 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>98383</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>94848</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>87643</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>86995</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>84899</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>61443</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>7081</v>
+      <c r="S10" s="14" t="n">
+        <v>1585</v>
       </c>
     </row>
     <row r="11">
@@ -1231,65 +1231,65 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>-339611</v>
+        <v>169250</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>-412402</v>
+        <v>213161</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>-43911</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-332906</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-288995</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-361786</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-346818</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-404278</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>72791</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-288995</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-361786</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-346818</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-404278</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-400079</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S11" s="11" t="n">
-        <v>-66855</v>
+        <v>37958</v>
       </c>
     </row>
     <row r="12">
@@ -1300,27 +1300,27 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>-646874</v>
+        <v>184722</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>-843457</v>
+        <v>220316</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G12" s="14" t="n">
-        <v>196583</v>
+        <v>-35594</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,26 +1328,26 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>47101</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>82695</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>-113888</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>201087</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>-90652</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>96011</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>-10444</v>
+      <c r="S12" s="14" t="n">
+        <v>-13984</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-3637764</v>
+        <v>1260082</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-3637764</v>
+        <v>1260083</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
+      <c r="Q13" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="14" t="n">
-        <v>-1113</v>
+      <c r="S13" s="11" t="n">
+        <v>-3276</v>
       </c>
     </row>
     <row r="14">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>6365</v>
+        <v>-7202</v>
       </c>
     </row>
     <row r="15">
@@ -1485,27 +1485,27 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>-821652</v>
+        <v>189598</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>-967974</v>
+        <v>309264</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>146322</v>
+        <v>-119666</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-706501</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-586835</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-733157</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-631001</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-826619</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-714880</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>72791</v>
+        <v>-43911</v>
       </c>
     </row>
     <row r="16">
@@ -1552,29 +1552,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>5716</v>
+      <c r="C16" s="14" t="n">
+        <v>1585</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>-1365</v>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>7081</v>
+      <c r="G16" s="14" t="n">
+        <v>1585</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,26 +1582,26 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>75950</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>74365</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>67284</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>61472</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>56384</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>54691</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
+      <c r="Q16" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>-21085</v>
+      <c r="S16" s="11" t="n">
+        <v>-20573</v>
       </c>
     </row>
     <row r="17">
@@ -1623,27 +1623,27 @@
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C17" s="14" t="n">
-        <v>-129774</v>
+        <v>67183</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>-108689</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+        <v>87756</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>-21085</v>
+      <c r="G17" s="11" t="n">
+        <v>-20573</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,20 +1651,20 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>544765</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>565338</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>586423</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>540492</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>666083</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>574665</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="Q17" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="14" t="n">
-        <v>88442</v>
+        <v>-30034</v>
       </c>
     </row>
     <row r="18">
@@ -1692,65 +1692,65 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>-275963</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
+        <v>47218</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
-        <v>-143645</v>
+      <c r="E18" s="14" t="n">
+        <v>-91436</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>138654</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>85786</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>-52868</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>79450</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>29037</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>104152</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>-132318</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>-52868</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>79450</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>29037</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>104152</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>85524</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>16666</v>
+        <v>-13503</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-1221673</v>
+        <v>305584</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-1221673</v>
+        <v>305584</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>-12931</v>
+        <v>8773</v>
       </c>
     </row>
     <row r="20">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="14" t="n">
-        <v>6337</v>
+        <v>-3790</v>
       </c>
     </row>
     <row r="21">
@@ -1877,65 +1877,65 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-4944</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
+        <v>25226</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>15151</v>
+      <c r="E21" s="14" t="n">
+        <v>15760</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>9466</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3222075</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3212609</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3232704</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3217571</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3253130</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>-20095</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>3212609</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>3232704</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>3217571</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>3253130</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>3275984</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>196583</v>
+        <v>-35594</v>
       </c>
     </row>
     <row r="22">
@@ -1944,29 +1944,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n">
-        <v>4762</v>
+      <c r="C22" s="11" t="n">
+        <v>13400</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>71617</v>
+        <v>-24558</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G22" s="11" t="n">
-        <v>-66855</v>
+        <v>37958</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4397081</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4435039</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4368184</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4356639</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4322717</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4302942</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>-132318</v>
+        <v>138654</v>
       </c>
     </row>
     <row r="23">
@@ -2015,27 +2015,27 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>49077</v>
+        <v>-13876</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>-39365</v>
+        <v>16158</v>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G23" s="14" t="n">
-        <v>88442</v>
+        <v>-30034</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,26 +2043,26 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>743986</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>774020</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>685578</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>675468</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>609846</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>580702</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>-1492</v>
+      <c r="S23" s="14" t="n">
+        <v>-17390</v>
       </c>
     </row>
     <row r="24">
@@ -2082,29 +2082,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C24" s="14" t="n">
-        <v>10680</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="C24" s="11" t="n">
+        <v>1495</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>12172</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="E24" s="14" t="n">
+        <v>18885</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>-1492</v>
+      <c r="G24" s="14" t="n">
+        <v>-17390</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,20 +2112,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>431020</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>448410</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>449902</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>463600</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>459741</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>446256</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="Q24" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>149519</v>
+        <v>-96530</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>59575</v>
+        <v>26245</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>59575</v>
+        <v>26245</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>-66498</v>
+        <v>10897</v>
       </c>
     </row>
     <row r="26">
@@ -2251,27 +2251,27 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>-118251</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+        <v>158243</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>37490</v>
+      <c r="E27" s="14" t="n">
+        <v>34226</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>-155741</v>
+        <v>124017</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>987613</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>863596</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1019337</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>898561</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1014945</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>844420</v>
       </c>
     </row>
     <row r="28">
@@ -2300,29 +2300,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="14" t="n">
-        <v>135</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="C28" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>10579</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>14059</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>-10444</v>
+      <c r="G28" s="14" t="n">
+        <v>-13984</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-367996</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-354012</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-343568</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-337557</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-325179</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-297558</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>36131</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>12450</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
-        <v>19465</v>
+      <c r="E29" s="14" t="n">
+        <v>25953</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>16666</v>
+        <v>-13503</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-165987</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-152484</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-169150</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-150201</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-160478</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-134565</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 13-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 14-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,27 +2420,27 @@
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C30" s="14" t="n">
-        <v>113834</v>
+        <v>-4253</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>-35685</v>
+        <v>92277</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>149519</v>
+        <v>-96530</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-453630</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-357100</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-506619</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-410803</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-529288</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-412297</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22364.15</v>
+        <v>22715.75</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>22721.95</v>
+        <v>22757.95</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>31849</v>
+        <v>166515</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>31849</v>
+        <v>166515</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22288.45</v>
+        <v>22558.95</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22721.95</v>
+        <v>22622.7</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23299.95</v>
+        <v>22933.11666666667</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22649.7</v>
+        <v>22634.61666666667</v>
       </c>
     </row>
     <row r="33">
@@ -2597,29 +2597,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>78703</v>
+      <c r="C33" s="14" t="n">
+        <v>19881</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>-1839</v>
+        <v>36275</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>80542</v>
+        <v>-16394</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-218398</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-202004</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-282546</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-259122</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-338827</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-302319</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23010.95</v>
+        <v>22845.53333333334</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22577.45</v>
+        <v>22646.53333333334</v>
       </c>
     </row>
     <row r="34">
@@ -2664,29 +2664,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>588</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="C34" s="14" t="n">
+        <v>603</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>1701</v>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
+      <c r="E34" s="11" t="n">
+        <v>3879</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>-1113</v>
+      <c r="G34" s="11" t="n">
+        <v>-3276</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>4320</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>7596</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>8709</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>9473</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>10766</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>12871</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22866.45</v>
+        <v>22734.11666666667</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22505.2</v>
+        <v>22658.45</v>
       </c>
     </row>
     <row r="35">
@@ -2731,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>16883</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="n">
+        <v>16925</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>29814</v>
+      <c r="E35" s="11" t="n">
+        <v>8152</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>-12931</v>
+        <v>8773</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>133066</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>124293</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>137224</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>129653</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>150821</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>134028</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22577.45</v>
+        <v>22646.53333333334</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,29 +2792,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>10766</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="14" t="n">
+        <v>30045</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>77264</v>
+      <c r="E36" s="11" t="n">
+        <v>19148</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-66498</v>
+        <v>10897</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>81012</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>70115</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>136613</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>119996</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>177240</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>155420</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22432.95</v>
+        <v>22535.11666666667</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>106940</v>
+        <v>67454</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>106940</v>
+        <v>67454</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22143.95</v>
+        <v>22447.53333333334</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>21999.45</v>
+        <v>22336.11666666667</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>14.63</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>14.12</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>15.25</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>14.38</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>15.28</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>13.89</v>
       </c>
     </row>
     <row r="41">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 13-Oct-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 19-Oct-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9501517111819584</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9538116838234366</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9382791147640293</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9443977202311479</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.931810958742466</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9468773774630451</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,722    PCR(OI) 1.40    Max Pain 22,700</t>
+          <t>Spot 22,623    PCR(OI) 0.86    Max Pain 22,600</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23809.56612903226</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23822.26008064516</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23834.43225806452</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23846.36209677419</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23858.70201612903</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23871.14798387097</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22622.7</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22721.95</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22363.35</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22520.45</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22231.8</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22603.05</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>22750</v>
+        <v>22700</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>311637</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>184649</v>
+        <v>139221</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>78873</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>23606930</v>
+        <v>4618025</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9322997454667669</v>
+        <v>0.9282579238326566</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9240905192059701</v>
@@ -3173,16 +3173,16 @@
         <v>0.9581623376424576</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>22800</v>
+        <v>23000</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>189523</v>
+        <v>173840</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>-27679</v>
+        <v>76798</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>13773080</v>
+        <v>2744359</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24371.93629032258</v>
+        <v>24371.13588709677</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24370.3939516129</v>
@@ -3212,16 +3212,16 @@
         <v>24365.80846774194</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>23000</v>
+        <v>23500</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>219628</v>
+        <v>150883</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>-38934</v>
+        <v>66994</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>3490217</v>
+        <v>1053008</v>
       </c>
       <c r="T47" s="31" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22721.95</v>
+        <v>22622.7</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>22520.45</v>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
-          <t>13-Oct-2026</t>
+          <t>14-Oct-2026</t>
         </is>
       </c>
       <c r="K49" s="30" t="inlineStr">
@@ -3319,65 +3319,65 @@
     </row>
     <row r="50">
       <c r="P50" s="33" t="n">
-        <v>22700</v>
+        <v>22500</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>371827</v>
+        <v>105653</v>
       </c>
       <c r="R50" s="14" t="n">
-        <v>350293</v>
+        <v>-9436</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>11023046</v>
-      </c>
-      <c r="T50" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>3076694</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="P51" s="33" t="n">
-        <v>22550</v>
+        <v>22000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>269159</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>247074</v>
+        <v>115380</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>32337</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>22795276</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>1277644</v>
+      </c>
+      <c r="T51" s="31" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="P52" s="33" t="n">
-        <v>22500</v>
+        <v>21000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>233808</v>
+        <v>102260</v>
       </c>
       <c r="R52" s="14" t="n">
-        <v>175410</v>
+        <v>-7494</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>30318873</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>413250</v>
+      </c>
+      <c r="T52" s="31" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 13-Oct-2026    1 DAY AGO = 12-Oct-2026    2 DAYS AGO = 09-Oct-2026    3 DAYS AGO = 08-Oct-2026    4 DAYS AGO = 07-Oct-2026    (generated 13-Oct-2026 20:32 IST)</t>
+          <t>TODAY = 14-Oct-2026    1 DAY AGO = 13-Oct-2026    2 DAYS AGO = 12-Oct-2026    3 DAYS AGO = 09-Oct-2026    4 DAYS AGO = 08-Oct-2026    (generated 14-Oct-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-15
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>15501</v>
+        <v>-26046</v>
       </c>
     </row>
     <row r="3">
@@ -701,27 +701,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>7731</v>
+        <v>-22453</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-7770</v>
+        <v>3593</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>15501</v>
+        <v>-26046</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>219312</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>245358</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>229857</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>242929</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>229523</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>247393</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>75969</v>
+        <v>-129508</v>
       </c>
     </row>
     <row r="4">
@@ -768,29 +768,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C4" s="11" t="n">
-        <v>152</v>
+      <c r="C4" s="14" t="n">
+        <v>1768</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>4661</v>
+        <v>-4651</v>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G4" s="14" t="n">
-        <v>-4509</v>
+        <v>6419</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,20 +798,20 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>36441</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>30022</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>34531</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>34161</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>31930</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>36250</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -819,7 +819,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-119666</v>
+        <v>234460</v>
       </c>
     </row>
     <row r="5">
@@ -839,65 +839,65 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>-1134</v>
+        <v>4267</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>6068</v>
+        <v>-12603</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>16870</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-279827</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-296697</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-289495</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-295860</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-293988</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-7202</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-296697</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-289495</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-295860</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-293988</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-307109</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>9466</v>
+        <v>-43005</v>
       </c>
     </row>
     <row r="6">
@@ -906,67 +906,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
-        <v>-2982</v>
+      <c r="C6" s="11" t="n">
+        <v>-3670</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>808</v>
+        <v>-6427</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>2757</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>24074</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>21317</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>25107</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>18770</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>32535</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>-3790</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>21317</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>25107</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>18770</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>32535</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>23466</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>124017</v>
+        <v>-43924</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>3767</v>
+        <v>-20088</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>3767</v>
+        <v>-20088</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-16394</v>
+        <v>43081</v>
       </c>
     </row>
     <row r="8">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="14" t="n">
-        <v>-4509</v>
+        <v>6419</v>
       </c>
     </row>
     <row r="9">
@@ -1093,27 +1093,27 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>902620</v>
+        <v>-248261</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>826651</v>
+        <v>-118753</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>75969</v>
+        <v>-129508</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,20 +1121,20 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>57913</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>187421</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>111452</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>388031</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>58735</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>410031</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>3535</v>
+        <v>-79278</v>
       </c>
     </row>
     <row r="10">
@@ -1162,65 +1162,65 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>3490</v>
+        <v>-79118</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>-45</v>
+        <v>160</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>-79278</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>19105</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>98383</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>94848</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>87643</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>86995</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>3535</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>98383</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>94848</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>87643</v>
-      </c>
-      <c r="M10" s="12" t="n">
-        <v>86995</v>
-      </c>
-      <c r="N10" s="12" t="n">
-        <v>84899</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q10" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>1585</v>
+      <c r="S10" s="11" t="n">
+        <v>5711</v>
       </c>
     </row>
     <row r="11">
@@ -1229,29 +1229,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
-        <v>169250</v>
+      <c r="C11" s="14" t="n">
+        <v>8264</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>213161</v>
+        <v>-116761</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-43911</v>
+        <v>125025</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,26 +1259,26 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-207881</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-332906</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-288995</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-361786</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-346818</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-404278</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>37958</v>
+      <c r="S11" s="14" t="n">
+        <v>20527</v>
       </c>
     </row>
     <row r="12">
@@ -1300,65 +1300,65 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>184722</v>
+        <v>-4402</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>220316</v>
+        <v>-88164</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>83762</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>130863</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>47101</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>82695</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>-113888</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>201087</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-35594</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>47101</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>82695</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>-113888</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>201087</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>-90652</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>-13984</v>
+      <c r="S12" s="11" t="n">
+        <v>-36108</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1260082</v>
+        <v>-323517</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1260083</v>
+        <v>-323518</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>-3276</v>
+      <c r="S13" s="14" t="n">
+        <v>-573</v>
       </c>
     </row>
     <row r="14">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-7202</v>
+        <v>16870</v>
       </c>
     </row>
     <row r="15">
@@ -1483,29 +1483,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
-        <v>189598</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="C15" s="11" t="n">
+        <v>1076630</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="11" t="n">
-        <v>309264</v>
+      <c r="E15" s="14" t="n">
+        <v>842170</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-119666</v>
+        <v>234460</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-472041</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-706501</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-586835</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-733157</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-631001</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-826619</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>-43911</v>
+        <v>125025</v>
       </c>
     </row>
     <row r="16">
@@ -1552,29 +1552,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
-        <v>1585</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="C16" s="11" t="n">
+        <v>5711</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>1585</v>
+      <c r="G16" s="11" t="n">
+        <v>5711</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,26 +1582,26 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>81661</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>75950</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>74365</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>67284</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>61472</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>56384</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="9" t="inlineStr">
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>-20573</v>
+      <c r="S16" s="14" t="n">
+        <v>-97738</v>
       </c>
     </row>
     <row r="17">
@@ -1621,29 +1621,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n">
-        <v>67183</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="C17" s="11" t="n">
+        <v>160469</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n">
-        <v>87756</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="E17" s="14" t="n">
+        <v>258207</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>-20573</v>
+      <c r="G17" s="14" t="n">
+        <v>-97738</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,20 +1651,20 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>447027</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>544765</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>565338</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>586423</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>540492</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>666083</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="Q17" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="14" t="n">
-        <v>-30034</v>
+        <v>42575</v>
       </c>
     </row>
     <row r="18">
@@ -1690,67 +1690,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
-        <v>47218</v>
+      <c r="C18" s="11" t="n">
+        <v>364435</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>-91436</v>
+        <v>506868</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>-142433</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>-56647</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>85786</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>-52868</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>79450</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>29037</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>138654</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>85786</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>-52868</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>79450</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>29037</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>104152</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-13503</v>
+        <v>16397</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>305584</v>
+        <v>1607245</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>305584</v>
+        <v>1607245</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>8773</v>
+        <v>-13695</v>
       </c>
     </row>
     <row r="20">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="14" t="n">
-        <v>-3790</v>
+        <v>2757</v>
       </c>
     </row>
     <row r="21">
@@ -1877,65 +1877,65 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>25226</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+        <v>-12222</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
-        <v>15760</v>
+      <c r="E21" s="11" t="n">
+        <v>30783</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>-43005</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3179070</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3222075</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3212609</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3232704</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3217571</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>9466</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>3222075</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>3212609</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>3232704</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>3217571</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>3253130</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>-35594</v>
+        <v>83762</v>
       </c>
     </row>
     <row r="22">
@@ -1944,29 +1944,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
-        <v>13400</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="C22" s="14" t="n">
+        <v>14795</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E22" s="11" t="n">
-        <v>-24558</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="E22" s="14" t="n">
+        <v>-5732</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>37958</v>
+      <c r="G22" s="14" t="n">
+        <v>20527</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4376554</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4397081</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4435039</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4368184</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4356639</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4322717</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>138654</v>
+        <v>-142433</v>
       </c>
     </row>
     <row r="23">
@@ -2015,65 +2015,65 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>-13876</v>
+        <v>12856</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>16158</v>
+        <v>-29719</v>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>42575</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>786561</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>743986</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>774020</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>685578</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>675468</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>-30034</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>743986</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>774020</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>685578</v>
-      </c>
-      <c r="M23" s="12" t="n">
-        <v>675468</v>
-      </c>
-      <c r="N23" s="12" t="n">
-        <v>609846</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-17390</v>
+      <c r="S23" s="11" t="n">
+        <v>-20097</v>
       </c>
     </row>
     <row r="24">
@@ -2082,29 +2082,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C24" s="11" t="n">
-        <v>1495</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="C24" s="14" t="n">
+        <v>9022</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>18885</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+      <c r="E24" s="11" t="n">
+        <v>29119</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-17390</v>
+      <c r="G24" s="11" t="n">
+        <v>-20097</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,20 +2112,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>410923</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>431020</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>448410</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>449902</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>463600</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>459741</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="Q24" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-96530</v>
+        <v>63635</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>26245</v>
+        <v>24451</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>26245</v>
+        <v>24451</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>10897</v>
+        <v>-28813</v>
       </c>
     </row>
     <row r="26">
@@ -2251,27 +2251,27 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>158243</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+        <v>-39331</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
-        <v>34226</v>
+      <c r="E27" s="11" t="n">
+        <v>4593</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>124017</v>
+        <v>-43924</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>943689</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>987613</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>863596</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1019337</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>898561</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1014945</v>
       </c>
     </row>
     <row r="28">
@@ -2302,27 +2302,27 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>75</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+        <v>-7195</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="14" t="n">
-        <v>14059</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="E28" s="11" t="n">
+        <v>28913</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>-13984</v>
+      <c r="G28" s="11" t="n">
+        <v>-36108</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-404104</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-367996</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-354012</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-343568</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-337557</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-325179</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
-        <v>12450</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="n">
+        <v>34243</v>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>25953</v>
+      <c r="E29" s="11" t="n">
+        <v>17846</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-13503</v>
+        <v>16397</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-149590</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-165987</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-152484</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-169150</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-150201</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-160478</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 14-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 15-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,27 +2420,27 @@
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C30" s="14" t="n">
-        <v>-4253</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
+        <v>66328</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>92277</v>
+      <c r="E30" s="11" t="n">
+        <v>2693</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-96530</v>
+        <v>63635</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-389995</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-453630</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-357100</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-506619</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-410803</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-529288</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22715.75</v>
+        <v>22671.3</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>22757.95</v>
+        <v>23056.4</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>166515</v>
+        <v>54045</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>166515</v>
+        <v>54045</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22558.95</v>
+        <v>22637.4</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22622.7</v>
+        <v>22997.35</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>22933.11666666667</v>
+        <v>23575.7</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22634.61666666667</v>
+        <v>22947.2</v>
       </c>
     </row>
     <row r="33">
@@ -2597,29 +2597,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
-        <v>19881</v>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="C33" s="11" t="n">
+        <v>54952</v>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="11" t="n">
-        <v>36275</v>
+      <c r="E33" s="14" t="n">
+        <v>11871</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-16394</v>
+        <v>43081</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-175317</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-218398</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-202004</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-282546</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-259122</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-338827</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>22845.53333333334</v>
+        <v>23316.05</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22646.53333333334</v>
+        <v>22897.05</v>
       </c>
     </row>
     <row r="34">
@@ -2664,29 +2664,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="14" t="n">
-        <v>603</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="C34" s="11" t="n">
+        <v>90</v>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="11" t="n">
-        <v>3879</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="E34" s="14" t="n">
+        <v>663</v>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="11" t="n">
-        <v>-3276</v>
+      <c r="G34" s="14" t="n">
+        <v>-573</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>3747</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>4320</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>7596</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>8709</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>9473</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>10766</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>22734.11666666667</v>
+        <v>23156.7</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22658.45</v>
+        <v>22846.9</v>
       </c>
     </row>
     <row r="35">
@@ -2731,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>16925</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="C35" s="11" t="n">
+        <v>16767</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="11" t="n">
-        <v>8152</v>
+      <c r="E35" s="14" t="n">
+        <v>30462</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>8773</v>
+        <v>-13695</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>119371</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>133066</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>124293</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>137224</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>129653</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>150821</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22646.53333333334</v>
+        <v>22897.05</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,29 +2792,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>30045</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="C36" s="11" t="n">
+        <v>10521</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
-        <v>19148</v>
+      <c r="E36" s="14" t="n">
+        <v>39334</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>10897</v>
+        <v>-28813</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>52199</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>81012</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>70115</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>136613</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>119996</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>177240</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22535.11666666667</v>
+        <v>22737.7</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>67454</v>
+        <v>82330</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>67454</v>
+        <v>82330</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22447.53333333334</v>
+        <v>22478.05</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22336.11666666667</v>
+        <v>22318.7</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>14.03</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>14.63</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>14.12</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>15.25</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>14.38</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>15.28</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9663308743049036</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9501517111819584</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9538116838234366</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9382791147640293</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9443977202311479</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.931810958742466</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,623    PCR(OI) 0.86    Max Pain 22,600</t>
+          <t>Spot 22,997    PCR(OI) 1.66    Max Pain 22,900</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23798.62903225806</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23809.56612903226</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23822.26008064516</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23834.43225806452</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23846.36209677419</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23858.70201612903</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22997.35</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22622.7</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22721.95</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22363.35</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22520.45</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22231.8</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>22700</v>
+        <v>23000</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>139221</v>
+        <v>126323</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>78873</v>
+        <v>-47517</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>4618025</v>
+        <v>4888084</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9282579238326566</v>
+        <v>0.9435136467083808</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9240905192059701</v>
@@ -3173,16 +3173,16 @@
         <v>0.9581623376424576</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23000</v>
+        <v>23500</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>173840</v>
+        <v>144645</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>76798</v>
+        <v>-6238</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>2744359</v>
+        <v>1838543</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24371.13588709677</v>
+        <v>24374.15725806452</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24370.3939516129</v>
@@ -3212,16 +3212,16 @@
         <v>24365.80846774194</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>23500</v>
+        <v>24000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>150883</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>66994</v>
+        <v>153607</v>
+      </c>
+      <c r="R47" s="14" t="n">
+        <v>14618</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>1053008</v>
+        <v>981119</v>
       </c>
       <c r="T47" s="31" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22622.7</v>
+        <v>22997.35</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>22520.45</v>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
-          <t>14-Oct-2026</t>
+          <t>15-Oct-2026</t>
         </is>
       </c>
       <c r="K49" s="30" t="inlineStr">
@@ -3319,54 +3319,54 @@
     </row>
     <row r="50">
       <c r="P50" s="33" t="n">
-        <v>22500</v>
+        <v>22700</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>105653</v>
+        <v>170492</v>
       </c>
       <c r="R50" s="14" t="n">
-        <v>-9436</v>
+        <v>106948</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>3076694</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>2167043</v>
+      </c>
+      <c r="T50" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="P51" s="33" t="n">
-        <v>22000</v>
+        <v>22500</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>115380</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>32337</v>
+        <v>199031</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>93378</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>1277644</v>
-      </c>
-      <c r="T51" s="31" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>1636842</v>
+      </c>
+      <c r="T51" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="P52" s="33" t="n">
-        <v>21000</v>
+        <v>22000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>102260</v>
+        <v>188301</v>
       </c>
       <c r="R52" s="14" t="n">
-        <v>-7494</v>
+        <v>72921</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>413250</v>
+        <v>1180605</v>
       </c>
       <c r="T52" s="31" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 14-Oct-2026    1 DAY AGO = 13-Oct-2026    2 DAYS AGO = 12-Oct-2026    3 DAYS AGO = 09-Oct-2026    4 DAYS AGO = 08-Oct-2026    (generated 14-Oct-2026 20:31 IST)</t>
+          <t>TODAY = 15-Oct-2026    1 DAY AGO = 14-Oct-2026    2 DAYS AGO = 13-Oct-2026    3 DAYS AGO = 12-Oct-2026    4 DAYS AGO = 09-Oct-2026    (generated 15-Oct-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-16
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-26046</v>
+        <v>602</v>
       </c>
     </row>
     <row r="3">
@@ -701,65 +701,65 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-22453</v>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
+        <v>2253</v>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E3" s="11" t="n">
-        <v>3593</v>
+      <c r="E3" s="13" t="n">
+        <v>1651</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>602</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="n">
+        <v>219914</v>
+      </c>
+      <c r="K3" s="14" t="n">
+        <v>219312</v>
+      </c>
+      <c r="L3" s="14" t="n">
+        <v>245358</v>
+      </c>
+      <c r="M3" s="14" t="n">
+        <v>229857</v>
+      </c>
+      <c r="N3" s="14" t="n">
+        <v>242929</v>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q3" s="12" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G3" s="11" t="n">
-        <v>-26046</v>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n">
-        <v>219312</v>
-      </c>
-      <c r="K3" s="12" t="n">
-        <v>245358</v>
-      </c>
-      <c r="L3" s="12" t="n">
-        <v>229857</v>
-      </c>
-      <c r="M3" s="12" t="n">
-        <v>242929</v>
-      </c>
-      <c r="N3" s="12" t="n">
-        <v>229523</v>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>-129508</v>
+      <c r="S3" s="13" t="n">
+        <v>-1388</v>
       </c>
     </row>
     <row r="4">
@@ -768,50 +768,50 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
-        <v>1768</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="n">
-        <v>-4651</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="C4" s="11" t="n">
+        <v>752</v>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>6419</v>
+      <c r="G4" s="11" t="n">
+        <v>752</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="14" t="n">
+        <v>37193</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>36441</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="14" t="n">
         <v>30022</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="14" t="n">
         <v>34531</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="14" t="n">
         <v>34161</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>31930</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -819,7 +819,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>234460</v>
+        <v>-19445</v>
       </c>
     </row>
     <row r="5">
@@ -837,56 +837,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
-        <v>4267</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="C5" s="11" t="n">
+        <v>1417</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n">
-        <v>-12603</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="E5" s="11" t="n">
+        <v>-5411</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>16870</v>
+      <c r="G5" s="11" t="n">
+        <v>6828</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="14" t="n">
+        <v>-272999</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-279827</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="14" t="n">
         <v>-296697</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="14" t="n">
         <v>-289495</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="14" t="n">
         <v>-295860</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-293988</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
+      <c r="Q5" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -896,8 +896,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>-43005</v>
+      <c r="S5" s="13" t="n">
+        <v>-20284</v>
       </c>
     </row>
     <row r="6">
@@ -906,67 +906,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>-3670</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>-6427</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="C6" s="13" t="n">
+        <v>-5127</v>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>3055</v>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>-8182</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="n">
+        <v>15892</v>
+      </c>
+      <c r="K6" s="14" t="n">
+        <v>24074</v>
+      </c>
+      <c r="L6" s="14" t="n">
+        <v>21317</v>
+      </c>
+      <c r="M6" s="14" t="n">
+        <v>25107</v>
+      </c>
+      <c r="N6" s="14" t="n">
+        <v>18770</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>2757</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>24074</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>21317</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>25107</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>18770</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>32535</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>-43924</v>
+        <v>87900</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-20088</v>
+        <v>-705</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-20088</v>
+        <v>-705</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,7 +1002,7 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
+      <c r="Q7" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>43081</v>
+      <c r="S7" s="13" t="n">
+        <v>34058</v>
       </c>
     </row>
     <row r="8">
@@ -1071,7 +1071,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
+      <c r="Q8" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>6419</v>
+      <c r="S8" s="11" t="n">
+        <v>752</v>
       </c>
     </row>
     <row r="9">
@@ -1093,54 +1093,54 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>-248261</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>-118753</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
+        <v>900722</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>902110</v>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>-129508</v>
+      <c r="G9" s="13" t="n">
+        <v>-1388</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="14" t="n">
+        <v>56525</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>57913</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="14" t="n">
         <v>187421</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="14" t="n">
         <v>111452</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="14" t="n">
         <v>388031</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>58735</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="9" t="inlineStr">
+      <c r="Q9" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>-79278</v>
+      <c r="S9" s="13" t="n">
+        <v>-10430</v>
       </c>
     </row>
     <row r="10">
@@ -1160,56 +1160,56 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
-        <v>-79118</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="C10" s="13" t="n">
+        <v>-10430</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n">
-        <v>160</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="E10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>-79278</v>
+      <c r="G10" s="13" t="n">
+        <v>-10430</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
+        <v>8675</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>19105</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>98383</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="14" t="n">
         <v>94848</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="14" t="n">
         <v>87643</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>86995</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
+      <c r="Q10" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>5711</v>
+      <c r="S10" s="13" t="n">
+        <v>8220</v>
       </c>
     </row>
     <row r="11">
@@ -1229,67 +1229,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
-        <v>8264</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>-116761</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="C11" s="11" t="n">
+        <v>23506</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>89300</v>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>-65794</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="n">
+        <v>-273675</v>
+      </c>
+      <c r="K11" s="14" t="n">
+        <v>-207881</v>
+      </c>
+      <c r="L11" s="14" t="n">
+        <v>-332906</v>
+      </c>
+      <c r="M11" s="14" t="n">
+        <v>-288995</v>
+      </c>
+      <c r="N11" s="14" t="n">
+        <v>-361786</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>125025</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-207881</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-332906</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-288995</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-361786</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-346818</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>20527</v>
+      <c r="S11" s="11" t="n">
+        <v>48957</v>
       </c>
     </row>
     <row r="12">
@@ -1300,54 +1300,54 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>-4402</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>-88164</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+        <v>171587</v>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>93975</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>83762</v>
+      <c r="G12" s="11" t="n">
+        <v>77612</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="14" t="n">
+        <v>208475</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>130863</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <v>47101</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="14" t="n">
         <v>82695</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="14" t="n">
         <v>-113888</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>201087</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>-36108</v>
+      <c r="S12" s="13" t="n">
+        <v>-18924</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-323517</v>
+        <v>1085385</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-323518</v>
+        <v>1085385</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
+      <c r="Q13" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="14" t="n">
-        <v>-573</v>
+      <c r="S13" s="11" t="n">
+        <v>-564</v>
       </c>
     </row>
     <row r="14">
@@ -1463,7 +1463,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
+      <c r="Q14" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>16870</v>
+      <c r="S14" s="11" t="n">
+        <v>6828</v>
       </c>
     </row>
     <row r="15">
@@ -1483,58 +1483,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
-        <v>1076630</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="C15" s="13" t="n">
+        <v>625270</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="14" t="n">
-        <v>842170</v>
+      <c r="E15" s="11" t="n">
+        <v>644715</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>234460</v>
+        <v>-19445</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-491486</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-472041</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-706501</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>-586835</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>-733157</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-631001</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q15" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>125025</v>
+      <c r="S15" s="13" t="n">
+        <v>-65794</v>
       </c>
     </row>
     <row r="16">
@@ -1552,58 +1552,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>5711</v>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="C16" s="13" t="n">
+        <v>8220</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>5711</v>
+      <c r="G16" s="13" t="n">
+        <v>8220</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="14" t="n">
+        <v>89881</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>81661</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <v>75950</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="14" t="n">
         <v>74365</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="14" t="n">
         <v>67284</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>61472</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q16" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>-97738</v>
+      <c r="S16" s="13" t="n">
+        <v>74210</v>
       </c>
     </row>
     <row r="17">
@@ -1621,67 +1621,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
-        <v>160469</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>258207</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="C17" s="13" t="n">
+        <v>61927</v>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>-12283</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>74210</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>521237</v>
+      </c>
+      <c r="K17" s="14" t="n">
+        <v>447027</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <v>544765</v>
+      </c>
+      <c r="M17" s="14" t="n">
+        <v>565338</v>
+      </c>
+      <c r="N17" s="14" t="n">
+        <v>586423</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>-97738</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>447027</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>544765</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>565338</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>586423</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>540492</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>42575</v>
+      <c r="S17" s="13" t="n">
+        <v>-9897</v>
       </c>
     </row>
     <row r="18">
@@ -1692,56 +1692,56 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>364435</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+        <v>-14153</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="14" t="n">
-        <v>506868</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="E18" s="11" t="n">
+        <v>48831</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>-142433</v>
+      <c r="G18" s="11" t="n">
+        <v>-62984</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="12" t="n">
+      <c r="J18" s="14" t="n">
+        <v>-119631</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>-56647</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="14" t="n">
         <v>85786</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="14" t="n">
         <v>-52868</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="14" t="n">
         <v>79450</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>29037</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q18" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R18" s="10" t="inlineStr">
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>16397</v>
+      <c r="S18" s="13" t="n">
+        <v>-8070</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>1607245</v>
+        <v>681264</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>1607245</v>
+        <v>681263</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q19" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>-13695</v>
+      <c r="S19" s="13" t="n">
+        <v>4839</v>
       </c>
     </row>
     <row r="20">
@@ -1855,9 +1855,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q20" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>2757</v>
+      <c r="S20" s="13" t="n">
+        <v>-8182</v>
       </c>
     </row>
     <row r="21">
@@ -1877,54 +1877,54 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-12222</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
+        <v>22923</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>30783</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="E21" s="13" t="n">
+        <v>43207</v>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>-43005</v>
+      <c r="G21" s="13" t="n">
+        <v>-20284</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="14" t="n">
+        <v>3158786</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3179070</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <v>3222075</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="14" t="n">
         <v>3212609</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="14" t="n">
         <v>3232704</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3217571</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
+      <c r="Q21" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>83762</v>
+      <c r="S21" s="11" t="n">
+        <v>77612</v>
       </c>
     </row>
     <row r="22">
@@ -1944,56 +1944,56 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n">
-        <v>14795</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="C22" s="11" t="n">
+        <v>26287</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
-        <v>-5732</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="E22" s="11" t="n">
+        <v>-22670</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>20527</v>
+      <c r="G22" s="11" t="n">
+        <v>48957</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J22" s="14" t="n">
+        <v>-4327597</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-4376554</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="14" t="n">
         <v>-4397081</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="14" t="n">
         <v>-4435039</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="14" t="n">
         <v>-4368184</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4356639</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
+      <c r="Q22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>-142433</v>
+      <c r="S22" s="11" t="n">
+        <v>-62984</v>
       </c>
     </row>
     <row r="23">
@@ -2013,56 +2013,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n">
-        <v>12856</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="n">
-        <v>-29719</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="n">
-        <v>42575</v>
+      <c r="C23" s="11" t="n">
+        <v>9346</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>19243</v>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="n">
+        <v>-9897</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="J23" s="14" t="n">
+        <v>776664</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>786561</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <v>743986</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="14" t="n">
         <v>774020</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="14" t="n">
         <v>685578</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>675468</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
+      <c r="Q23" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>-20097</v>
+      <c r="S23" s="13" t="n">
+        <v>-18776</v>
       </c>
     </row>
     <row r="24">
@@ -2082,58 +2082,58 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C24" s="14" t="n">
-        <v>9022</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="C24" s="11" t="n">
+        <v>21955</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>29119</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="E24" s="13" t="n">
+        <v>40731</v>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>-20097</v>
+      <c r="G24" s="13" t="n">
+        <v>-18776</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J24" s="14" t="n">
+        <v>392147</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>410923</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="14" t="n">
         <v>431020</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="14" t="n">
         <v>448410</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="14" t="n">
         <v>449902</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>463600</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q24" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>63635</v>
+      <c r="S24" s="13" t="n">
+        <v>-60906</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>24451</v>
+        <v>80511</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>24451</v>
+        <v>80511</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,7 +2178,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
+      <c r="Q25" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>-28813</v>
+      <c r="S25" s="11" t="n">
+        <v>-38333</v>
       </c>
     </row>
     <row r="26">
@@ -2251,47 +2251,47 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>-39331</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+        <v>130579</v>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>4593</v>
+      <c r="E27" s="13" t="n">
+        <v>42679</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>-43924</v>
+        <v>87900</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>1031589</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>943689</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>987613</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="14" t="n">
         <v>863596</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>1019337</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>898561</v>
       </c>
     </row>
     <row r="28">
@@ -2302,47 +2302,47 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>-7195</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+        <v>100</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>28913</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="13" t="n">
+        <v>19024</v>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>-36108</v>
+      <c r="G28" s="13" t="n">
+        <v>-18924</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-423028</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-404104</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-367996</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="14" t="n">
         <v>-354012</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>-343568</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-337557</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,53 +2359,53 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>34243</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>17279</v>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
-        <v>17846</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G29" s="14" t="n">
-        <v>16397</v>
+      <c r="E29" s="13" t="n">
+        <v>25349</v>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>-8070</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-157660</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-149590</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-165987</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="14" t="n">
         <v>-152484</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>-169150</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-150201</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 15-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 16-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,57 +2418,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
-        <v>66328</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="C30" s="11" t="n">
+        <v>23023</v>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n">
-        <v>2693</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G30" s="14" t="n">
-        <v>63635</v>
+      <c r="E30" s="13" t="n">
+        <v>83929</v>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>-60906</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-450901</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-389995</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-453630</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="14" t="n">
         <v>-357100</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="14" t="n">
         <v>-506619</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-410803</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22671.3</v>
+        <v>23065.1</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23056.4</v>
+        <v>23149.85</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>54045</v>
+        <v>170981</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>54045</v>
+        <v>170981</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22637.4</v>
+        <v>22913.8</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22997.35</v>
+        <v>23146.15</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23575.7</v>
+        <v>23462.11666666666</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22947.2</v>
+        <v>23108.04166666666</v>
       </c>
     </row>
     <row r="33">
@@ -2597,57 +2597,57 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>54952</v>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="C33" s="13" t="n">
+        <v>83125</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="14" t="n">
-        <v>11871</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="E33" s="11" t="n">
+        <v>49067</v>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G33" s="11" t="n">
-        <v>43081</v>
+      <c r="G33" s="13" t="n">
+        <v>34058</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-141259</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-175317</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-218398</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="14" t="n">
         <v>-202004</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="14" t="n">
         <v>-282546</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-259122</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23316.05</v>
+        <v>23305.98333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22897.05</v>
+        <v>23069.93333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2664,57 +2664,57 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>90</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="C34" s="13" t="n">
+        <v>1070</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>663</v>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
+      <c r="E34" s="11" t="n">
+        <v>1634</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>-573</v>
+      <c r="G34" s="11" t="n">
+        <v>-564</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>3183</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>3747</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>4320</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="14" t="n">
         <v>7596</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="14" t="n">
         <v>8709</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>9473</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23156.7</v>
+        <v>23226.06666666666</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22846.9</v>
+        <v>23031.825</v>
       </c>
     </row>
     <row r="35">
@@ -2731,57 +2731,57 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>16767</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="13" t="n">
+        <v>25819</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>30462</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="n">
-        <v>-13695</v>
+      <c r="E35" s="11" t="n">
+        <v>20980</v>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="n">
+        <v>4839</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>124210</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>119371</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>133066</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="14" t="n">
         <v>124293</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="14" t="n">
         <v>137224</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>129653</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22897.05</v>
+        <v>23069.93333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,57 +2792,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>10521</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="13" t="n">
+        <v>15199</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>39334</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
+      <c r="E36" s="11" t="n">
+        <v>53532</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>-28813</v>
+      <c r="G36" s="11" t="n">
+        <v>-38333</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>13866</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>52199</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>81012</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="14" t="n">
         <v>70115</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="14" t="n">
         <v>136613</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>119996</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22737.7</v>
+        <v>22990.01666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>82330</v>
+        <v>125213</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>82330</v>
+        <v>125213</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22478.05</v>
+        <v>22833.88333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22318.7</v>
+        <v>22753.96666666666</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>14.06</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>14.03</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>14.63</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>14.12</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>15.25</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>14.38</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9729851533215025</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9663308743049036</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9501517111819584</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9538116838234366</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9382791147640293</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9443977202311479</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,997    PCR(OI) 1.66    Max Pain 22,900</t>
+          <t>Spot 23,146    PCR(OI) 1.32    Max Pain 23,050</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23788.80080645161</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23798.62903225806</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23809.56612903226</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23822.26008064516</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23834.43225806452</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23846.36209677419</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23146.15</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22997.35</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22622.7</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22721.95</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22363.35</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22520.45</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23000</v>
-      </c>
-      <c r="Q45" s="12" t="n">
-        <v>126323</v>
+        <v>23500</v>
+      </c>
+      <c r="Q45" s="14" t="n">
+        <v>208554</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>-47517</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>4888084</v>
+        <v>63909</v>
+      </c>
+      <c r="S45" s="14" t="n">
+        <v>3484002</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9435136467083808</v>
+        <v>0.9495717233987274</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9240905192059701</v>
@@ -3173,16 +3173,16 @@
         <v>0.9581623376424576</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>23500</v>
-      </c>
-      <c r="Q46" s="12" t="n">
-        <v>144645</v>
+        <v>24000</v>
+      </c>
+      <c r="Q46" s="14" t="n">
+        <v>217028</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>-6238</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>1838543</v>
+        <v>63421</v>
+      </c>
+      <c r="S46" s="14" t="n">
+        <v>1530921</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24374.15725806452</v>
+        <v>24375.35725806452</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24370.3939516129</v>
@@ -3212,16 +3212,16 @@
         <v>24365.80846774194</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>24000</v>
-      </c>
-      <c r="Q47" s="12" t="n">
-        <v>153607</v>
-      </c>
-      <c r="R47" s="14" t="n">
-        <v>14618</v>
-      </c>
-      <c r="S47" s="12" t="n">
-        <v>981119</v>
+        <v>24500</v>
+      </c>
+      <c r="Q47" s="14" t="n">
+        <v>144716</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>110299</v>
+      </c>
+      <c r="S47" s="14" t="n">
+        <v>467380</v>
       </c>
       <c r="T47" s="31" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22997.35</v>
+        <v>23146.15</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>22520.45</v>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="K49" s="30" t="inlineStr">
@@ -3321,18 +3321,18 @@
       <c r="P50" s="33" t="n">
         <v>22700</v>
       </c>
-      <c r="Q50" s="12" t="n">
-        <v>170492</v>
-      </c>
-      <c r="R50" s="14" t="n">
-        <v>106948</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>2167043</v>
-      </c>
-      <c r="T50" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="Q50" s="14" t="n">
+        <v>183052</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>12560</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>3030287</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3340,18 +3340,18 @@
       <c r="P51" s="33" t="n">
         <v>22500</v>
       </c>
-      <c r="Q51" s="12" t="n">
-        <v>199031</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>93378</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>1636842</v>
-      </c>
-      <c r="T51" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="Q51" s="14" t="n">
+        <v>200627</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>1596</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>2463494</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3359,25 +3359,25 @@
       <c r="P52" s="33" t="n">
         <v>22000</v>
       </c>
-      <c r="Q52" s="12" t="n">
-        <v>188301</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>72921</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>1180605</v>
-      </c>
-      <c r="T52" s="31" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="Q52" s="14" t="n">
+        <v>281076</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>92775</v>
+      </c>
+      <c r="S52" s="14" t="n">
+        <v>1961569</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 15-Oct-2026    1 DAY AGO = 14-Oct-2026    2 DAYS AGO = 13-Oct-2026    3 DAYS AGO = 12-Oct-2026    4 DAYS AGO = 09-Oct-2026    (generated 15-Oct-2026 20:32 IST)</t>
+          <t>TODAY = 16-Oct-2026    1 DAY AGO = 15-Oct-2026    2 DAYS AGO = 14-Oct-2026    3 DAYS AGO = 13-Oct-2026    4 DAYS AGO = 12-Oct-2026    (generated 16-Oct-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-19
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -190,17 +190,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>602</v>
+        <v>10877</v>
       </c>
     </row>
     <row r="3">
@@ -705,15 +705,15 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>2253</v>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>1651</v>
+        <v>4779</v>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>-6098</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,36 +721,36 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>602</v>
+        <v>10877</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>230791</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>219914</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>219312</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>245358</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="12" t="n">
         <v>229857</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>242929</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="13" t="n">
-        <v>-1388</v>
+      <c r="S3" s="11" t="n">
+        <v>135953</v>
       </c>
     </row>
     <row r="4">
@@ -774,44 +774,44 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>752</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
+        <v>82</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>752</v>
+      <c r="E4" s="14" t="n">
+        <v>421</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>-339</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="12" t="n">
+        <v>36854</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>37193</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="12" t="n">
         <v>36441</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="12" t="n">
         <v>30022</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="12" t="n">
         <v>34531</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>34161</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-19445</v>
+        <v>-235937</v>
       </c>
     </row>
     <row r="5">
@@ -837,67 +837,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>1417</v>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>-5411</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>-3305</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>3626</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>-6931</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-279930</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-272999</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-279827</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-296697</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-289495</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="11" t="n">
-        <v>6828</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="n">
-        <v>-272999</v>
-      </c>
-      <c r="K5" s="14" t="n">
-        <v>-279827</v>
-      </c>
-      <c r="L5" s="14" t="n">
-        <v>-296697</v>
-      </c>
-      <c r="M5" s="14" t="n">
-        <v>-289495</v>
-      </c>
-      <c r="N5" s="14" t="n">
-        <v>-295860</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="13" t="n">
-        <v>-20284</v>
+      <c r="S5" s="11" t="n">
+        <v>34518</v>
       </c>
     </row>
     <row r="6">
@@ -906,50 +906,50 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
-        <v>-5127</v>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="C6" s="14" t="n">
+        <v>-1781</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E6" s="13" t="n">
-        <v>3055</v>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="E6" s="14" t="n">
+        <v>1826</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="13" t="n">
-        <v>-8182</v>
+      <c r="G6" s="14" t="n">
+        <v>-3607</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="12" t="n">
+        <v>12285</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>15892</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="12" t="n">
         <v>24074</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>21317</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="12" t="n">
         <v>25107</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>18770</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>87900</v>
+        <v>128392</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-705</v>
+        <v>-225</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-705</v>
+        <v>-225</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="13" t="n">
-        <v>34058</v>
+      <c r="S7" s="11" t="n">
+        <v>-64731</v>
       </c>
     </row>
     <row r="8">
@@ -1071,9 +1071,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>752</v>
+      <c r="S8" s="14" t="n">
+        <v>-339</v>
       </c>
     </row>
     <row r="9">
@@ -1091,67 +1091,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>900722</v>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>902110</v>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>-1217512</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>-1353465</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>135953</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>192478</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>56525</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>57913</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>187421</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>111452</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="13" t="n">
-        <v>-1388</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>56525</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>57913</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>187421</v>
-      </c>
-      <c r="M9" s="14" t="n">
-        <v>111452</v>
-      </c>
-      <c r="N9" s="14" t="n">
-        <v>388031</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="13" t="n">
-        <v>-10430</v>
+      <c r="S9" s="14" t="n">
+        <v>-1062</v>
       </c>
     </row>
     <row r="10">
@@ -1160,56 +1160,56 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
-        <v>-10430</v>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="C10" s="14" t="n">
+        <v>-907</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
+      <c r="E10" s="14" t="n">
+        <v>155</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="13" t="n">
-        <v>-10430</v>
+      <c r="G10" s="14" t="n">
+        <v>-1062</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="12" t="n">
+        <v>7613</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>8675</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="12" t="n">
         <v>19105</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="12" t="n">
         <v>98383</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="12" t="n">
         <v>94848</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>87643</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="12" t="inlineStr">
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="13" t="n">
-        <v>8220</v>
+      <c r="S10" s="14" t="n">
+        <v>7470</v>
       </c>
     </row>
     <row r="11">
@@ -1229,50 +1229,50 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="n">
-        <v>23506</v>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>89300</v>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="n">
-        <v>-65794</v>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>-150166</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>-171180</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>21014</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="14" t="n">
+      <c r="J11" s="12" t="n">
+        <v>-252661</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-273675</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="12" t="n">
         <v>-207881</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="M11" s="12" t="n">
         <v>-332906</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="12" t="n">
         <v>-288995</v>
       </c>
-      <c r="N11" s="14" t="n">
-        <v>-361786</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="S11" s="11" t="n">
-        <v>48957</v>
+        <v>9829</v>
       </c>
     </row>
     <row r="12">
@@ -1298,56 +1298,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>171587</v>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>93975</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>77612</v>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>-367104</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>-211198</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>-155906</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="14" t="n">
+      <c r="J12" s="12" t="n">
+        <v>52569</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>208475</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="12" t="n">
         <v>130863</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="M12" s="12" t="n">
         <v>47101</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="12" t="n">
         <v>82695</v>
       </c>
-      <c r="N12" s="14" t="n">
-        <v>-113888</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="12" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="13" t="n">
-        <v>-18924</v>
+      <c r="S12" s="14" t="n">
+        <v>-15602</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1085385</v>
+        <v>-1735689</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1085385</v>
+        <v>-1735688</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-564</v>
+        <v>-2771</v>
       </c>
     </row>
     <row r="14">
@@ -1463,9 +1463,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q14" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="11" t="n">
-        <v>6828</v>
+      <c r="S14" s="14" t="n">
+        <v>-6931</v>
       </c>
     </row>
     <row r="15">
@@ -1483,21 +1483,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="n">
-        <v>625270</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="n">
-        <v>644715</v>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>-2251398</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>-2015461</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1505,36 +1505,36 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-19445</v>
+        <v>-235937</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="12" t="n">
+        <v>-727423</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-491486</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="12" t="n">
         <v>-472041</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="12" t="n">
         <v>-706501</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="12" t="n">
         <v>-586835</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-733157</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="13" t="n">
-        <v>-65794</v>
+      <c r="S15" s="11" t="n">
+        <v>21014</v>
       </c>
     </row>
     <row r="16">
@@ -1552,13 +1552,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
-        <v>8220</v>
+      <c r="C16" s="14" t="n">
+        <v>7925</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1566,42 +1566,42 @@
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
+        <v>455</v>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="13" t="n">
-        <v>8220</v>
+      <c r="G16" s="14" t="n">
+        <v>7470</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="14" t="n">
+      <c r="J16" s="12" t="n">
+        <v>97351</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>89881</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="12" t="n">
         <v>81661</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="12" t="n">
         <v>75950</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="12" t="n">
         <v>74365</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>67284</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="12" t="inlineStr">
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="13" t="n">
-        <v>74210</v>
+      <c r="S16" s="14" t="n">
+        <v>52260</v>
       </c>
     </row>
     <row r="17">
@@ -1621,56 +1621,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>61927</v>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>-306805</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E17" s="13" t="n">
-        <v>-12283</v>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="E17" s="14" t="n">
+        <v>-359065</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
-        <v>74210</v>
+      <c r="G17" s="14" t="n">
+        <v>52260</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="14" t="n">
+      <c r="J17" s="12" t="n">
+        <v>573497</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>521237</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="L17" s="12" t="n">
         <v>447027</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="M17" s="12" t="n">
         <v>544765</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="N17" s="12" t="n">
         <v>565338</v>
       </c>
-      <c r="N17" s="14" t="n">
-        <v>586423</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="12" t="inlineStr">
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1680,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="13" t="n">
-        <v>-9897</v>
+      <c r="S17" s="14" t="n">
+        <v>-39183</v>
       </c>
     </row>
     <row r="18">
@@ -1696,61 +1696,61 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>-14153</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>48831</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+        <v>-551692</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>-727899</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>176207</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>56576</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>-119631</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>-56647</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>85786</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>-52868</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>-62984</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="14" t="n">
-        <v>-119631</v>
-      </c>
-      <c r="K18" s="14" t="n">
-        <v>-56647</v>
-      </c>
-      <c r="L18" s="14" t="n">
-        <v>85786</v>
-      </c>
-      <c r="M18" s="14" t="n">
-        <v>-52868</v>
-      </c>
-      <c r="N18" s="14" t="n">
-        <v>79450</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="13" t="n">
-        <v>-8070</v>
+      <c r="S18" s="14" t="n">
+        <v>-51830</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>681264</v>
+        <v>-3101970</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>681263</v>
+        <v>-3101970</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="12" t="inlineStr">
+      <c r="Q19" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="13" t="n">
-        <v>4839</v>
+      <c r="S19" s="14" t="n">
+        <v>19214</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="12" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="13" t="n">
-        <v>-8182</v>
+      <c r="S20" s="14" t="n">
+        <v>-3607</v>
       </c>
     </row>
     <row r="21">
@@ -1881,61 +1881,61 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>22923</v>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
+        <v>41616</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="13" t="n">
-        <v>43207</v>
-      </c>
-      <c r="F21" s="12" t="inlineStr">
+      <c r="E21" s="14" t="n">
+        <v>7098</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>34518</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3193304</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3158786</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3179070</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3222075</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3212609</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="13" t="n">
-        <v>-20284</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="14" t="n">
-        <v>3158786</v>
-      </c>
-      <c r="K21" s="14" t="n">
-        <v>3179070</v>
-      </c>
-      <c r="L21" s="14" t="n">
-        <v>3222075</v>
-      </c>
-      <c r="M21" s="14" t="n">
-        <v>3212609</v>
-      </c>
-      <c r="N21" s="14" t="n">
-        <v>3232704</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>77612</v>
+      <c r="S21" s="14" t="n">
+        <v>-155906</v>
       </c>
     </row>
     <row r="22">
@@ -1950,15 +1950,15 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>26287</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>-22670</v>
+        <v>18266</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>8437</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
@@ -1966,36 +1966,36 @@
         </is>
       </c>
       <c r="G22" s="11" t="n">
-        <v>48957</v>
+        <v>9829</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="14" t="n">
+      <c r="J22" s="12" t="n">
+        <v>-4317768</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4327597</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4376554</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4397081</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4435039</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-4368184</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>-62984</v>
+      <c r="S22" s="14" t="n">
+        <v>176207</v>
       </c>
     </row>
     <row r="23">
@@ -2013,56 +2013,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="n">
-        <v>9346</v>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>-3319</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="13" t="n">
-        <v>19243</v>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="E23" s="14" t="n">
+        <v>35864</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="13" t="n">
-        <v>-9897</v>
+      <c r="G23" s="14" t="n">
+        <v>-39183</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="14" t="n">
+      <c r="J23" s="12" t="n">
+        <v>737481</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>776664</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="L23" s="12" t="n">
         <v>786561</v>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="M23" s="12" t="n">
         <v>743986</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="N23" s="12" t="n">
         <v>774020</v>
       </c>
-      <c r="N23" s="14" t="n">
-        <v>685578</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="12" t="inlineStr">
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="13" t="n">
-        <v>-18776</v>
+      <c r="S23" s="14" t="n">
+        <v>-5164</v>
       </c>
     </row>
     <row r="24">
@@ -2088,50 +2088,50 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>21955</v>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
+        <v>29079</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="13" t="n">
-        <v>40731</v>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
+      <c r="E24" s="14" t="n">
+        <v>34243</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="13" t="n">
-        <v>-18776</v>
+      <c r="G24" s="14" t="n">
+        <v>-5164</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="14" t="n">
+      <c r="J24" s="12" t="n">
+        <v>386983</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>392147</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="12" t="n">
         <v>410923</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="12" t="n">
         <v>431020</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="12" t="n">
         <v>448410</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>449902</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="12" t="inlineStr">
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="13" t="n">
-        <v>-60906</v>
+      <c r="S24" s="14" t="n">
+        <v>-60960</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>80511</v>
+        <v>85642</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>80511</v>
+        <v>85642</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="11" t="n">
-        <v>-38333</v>
+      <c r="S25" s="14" t="n">
+        <v>48288</v>
       </c>
     </row>
     <row r="26">
@@ -2255,15 +2255,15 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>130579</v>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
+        <v>142557</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="13" t="n">
-        <v>42679</v>
+      <c r="E27" s="14" t="n">
+        <v>14165</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,27 +2271,27 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>87900</v>
+        <v>128392</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>1159981</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1031589</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>943689</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>987613</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="12" t="n">
         <v>863596</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>1019337</v>
       </c>
     </row>
     <row r="28">
@@ -2306,43 +2306,43 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="13" t="n">
-        <v>19024</v>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>15802</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="13" t="n">
-        <v>-18924</v>
+      <c r="G28" s="14" t="n">
+        <v>-15602</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-438630</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-423028</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-404104</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-367996</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="12" t="n">
         <v>-354012</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-343568</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,53 +2359,53 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="n">
-        <v>17279</v>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>-7080</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="13" t="n">
-        <v>25349</v>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
+      <c r="E29" s="14" t="n">
+        <v>44750</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="13" t="n">
-        <v>-8070</v>
+      <c r="G29" s="14" t="n">
+        <v>-51830</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-209490</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-157660</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-149590</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-165987</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="12" t="n">
         <v>-152484</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-169150</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 16-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 19-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,51 +2424,51 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>23023</v>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
+        <v>11913</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="13" t="n">
-        <v>83929</v>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
+      <c r="E30" s="14" t="n">
+        <v>72873</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G30" s="13" t="n">
-        <v>-60906</v>
+      <c r="G30" s="14" t="n">
+        <v>-60960</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-511861</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-450901</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-389995</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-453630</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="12" t="n">
         <v>-357100</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-506619</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23065.1</v>
+        <v>23150.85</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23149.85</v>
+        <v>23175.25</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>170981</v>
+        <v>147590</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>170981</v>
+        <v>147590</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22913.8</v>
+        <v>22845</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23146.15</v>
+        <v>22888.95</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23462.11666666666</v>
+        <v>23424.71666666667</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23108.04166666666</v>
+        <v>22929.34166666667</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2597,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v>83125</v>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>-55662</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,43 +2611,43 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>49067</v>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G33" s="13" t="n">
-        <v>34058</v>
+        <v>9069</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>-64731</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="14" t="n">
+      <c r="J33" s="12" t="n">
+        <v>-205990</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-141259</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="12" t="n">
         <v>-175317</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="12" t="n">
         <v>-218398</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="12" t="n">
         <v>-202004</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-282546</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23305.98333333333</v>
+        <v>23299.98333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23069.93333333333</v>
+        <v>22969.73333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2664,13 +2664,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="13" t="n">
-        <v>1070</v>
+      <c r="C34" s="14" t="n">
+        <v>328</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>1634</v>
+        <v>3099</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,35 +2686,35 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-564</v>
+        <v>-2771</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="14" t="n">
+      <c r="J34" s="12" t="n">
+        <v>412</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>3183</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="12" t="n">
         <v>3747</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="12" t="n">
         <v>4320</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="12" t="n">
         <v>7596</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>8709</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23226.06666666666</v>
+        <v>23094.46666666667</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23031.825</v>
+        <v>23010.125</v>
       </c>
     </row>
     <row r="35">
@@ -2731,57 +2731,57 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="13" t="n">
-        <v>25819</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E35" s="11" t="n">
-        <v>20980</v>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
+      <c r="C35" s="14" t="n">
+        <v>17183</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="n">
+        <v>-2031</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G35" s="13" t="n">
-        <v>4839</v>
+      <c r="G35" s="14" t="n">
+        <v>19214</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="14" t="n">
+      <c r="J35" s="12" t="n">
+        <v>143424</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>124210</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="12" t="n">
         <v>119371</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="12" t="n">
         <v>133066</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="12" t="n">
         <v>124293</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>137224</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23069.93333333333</v>
+        <v>22969.73333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,57 +2792,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="13" t="n">
-        <v>15199</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E36" s="11" t="n">
-        <v>53532</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="n">
-        <v>-38333</v>
+      <c r="C36" s="14" t="n">
+        <v>36216</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>-12072</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>48288</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="14" t="n">
+      <c r="J36" s="12" t="n">
+        <v>62154</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>13866</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="12" t="n">
         <v>52199</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="12" t="n">
         <v>81012</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="12" t="n">
         <v>70115</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>136613</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22990.01666666666</v>
+        <v>22764.21666666667</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>125213</v>
+        <v>-1935</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>125213</v>
+        <v>-1935</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22833.88333333333</v>
+        <v>22639.48333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22753.96666666666</v>
+        <v>22433.96666666667</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>14.77</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>14.06</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>14.03</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>14.63</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>14.12</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>15.25</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.962724138114085</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9729851533215025</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9663308743049036</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9501517111819584</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9538116838234366</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9382791147640293</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,146    PCR(OI) 1.32    Max Pain 23,050</t>
+          <t>Spot 22,889    PCR(OI) 0.80    Max Pain 22,900</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23775.19072580645</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23788.80080645161</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23798.62903225806</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23809.56612903226</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23822.26008064516</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23834.43225806452</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22888.95</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23146.15</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22997.35</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22622.7</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22721.95</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22363.35</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>23500</v>
-      </c>
-      <c r="Q45" s="14" t="n">
-        <v>208554</v>
+        <v>22900</v>
+      </c>
+      <c r="Q45" s="12" t="n">
+        <v>363408</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>63909</v>
-      </c>
-      <c r="S45" s="14" t="n">
-        <v>3484002</v>
+        <v>321581</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>21355500</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,35 +3158,35 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
+        <v>0.939144741359203</v>
+      </c>
+      <c r="K46" s="25" t="n">
         <v>0.9495717233987274</v>
       </c>
-      <c r="K46" s="25" t="n">
+      <c r="L46" s="25" t="n">
         <v>0.9240905192059701</v>
       </c>
-      <c r="L46" s="25" t="n">
+      <c r="M46" s="25" t="n">
         <v>0.9199158076678682</v>
       </c>
-      <c r="M46" s="25" t="n">
+      <c r="N46" s="25" t="n">
         <v>0.9493709489654826</v>
       </c>
-      <c r="N46" s="25" t="n">
-        <v>0.9581623376424576</v>
-      </c>
       <c r="P46" s="28" t="n">
-        <v>24000</v>
-      </c>
-      <c r="Q46" s="14" t="n">
-        <v>217028</v>
+        <v>22950</v>
+      </c>
+      <c r="Q46" s="12" t="n">
+        <v>226788</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>63421</v>
-      </c>
-      <c r="S46" s="14" t="n">
-        <v>1530921</v>
-      </c>
-      <c r="T46" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>210018</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>19141660</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3197,35 +3197,35 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
+        <v>24372.12177419355</v>
+      </c>
+      <c r="K47" s="18" t="n">
         <v>24375.35725806452</v>
       </c>
-      <c r="K47" s="18" t="n">
+      <c r="L47" s="18" t="n">
         <v>24370.3939516129</v>
       </c>
-      <c r="L47" s="18" t="n">
+      <c r="M47" s="18" t="n">
         <v>24373.91532258064</v>
       </c>
-      <c r="M47" s="18" t="n">
+      <c r="N47" s="18" t="n">
         <v>24374.56088709677</v>
       </c>
-      <c r="N47" s="18" t="n">
-        <v>24365.80846774194</v>
-      </c>
       <c r="P47" s="28" t="n">
-        <v>24500</v>
-      </c>
-      <c r="Q47" s="14" t="n">
-        <v>144716</v>
+        <v>23000</v>
+      </c>
+      <c r="Q47" s="12" t="n">
+        <v>252235</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>110299</v>
-      </c>
-      <c r="S47" s="14" t="n">
-        <v>467380</v>
-      </c>
-      <c r="T47" s="31" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>150703</v>
+      </c>
+      <c r="S47" s="12" t="n">
+        <v>23111861</v>
+      </c>
+      <c r="T47" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3236,21 +3236,21 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
+        <v>22888.95</v>
+      </c>
+      <c r="K48" s="18" t="n">
         <v>23146.15</v>
       </c>
-      <c r="K48" s="18" t="n">
+      <c r="L48" s="18" t="n">
         <v>22520.45</v>
       </c>
-      <c r="L48" s="18" t="n">
+      <c r="M48" s="18" t="n">
         <v>22421.95</v>
       </c>
-      <c r="M48" s="18" t="n">
+      <c r="N48" s="18" t="n">
         <v>23140.5</v>
       </c>
-      <c r="N48" s="18" t="n">
-        <v>23346.4</v>
-      </c>
-      <c r="P48" s="32" t="inlineStr">
+      <c r="P48" s="30" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3266,31 +3266,31 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="30" t="inlineStr">
+      <c r="J49" s="31" t="inlineStr">
+        <is>
+          <t>19-Oct-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="31" t="inlineStr">
         <is>
           <t>16-Oct-2026</t>
         </is>
       </c>
-      <c r="K49" s="30" t="inlineStr">
+      <c r="L49" s="31" t="inlineStr">
         <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="L49" s="30" t="inlineStr">
+      <c r="M49" s="31" t="inlineStr">
         <is>
           <t>01-Oct-2026</t>
         </is>
       </c>
-      <c r="M49" s="30" t="inlineStr">
+      <c r="N49" s="31" t="inlineStr">
         <is>
           <t>25-Sep-2026</t>
         </is>
       </c>
-      <c r="N49" s="30" t="inlineStr">
-        <is>
-          <t>18-Sep-2026</t>
-        </is>
-      </c>
       <c r="P49" s="27" t="inlineStr">
         <is>
           <t>Strike</t>
@@ -3318,17 +3318,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
-        <v>22700</v>
-      </c>
-      <c r="Q50" s="14" t="n">
-        <v>183052</v>
+      <c r="P50" s="32" t="n">
+        <v>22900</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>202833</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>12560</v>
-      </c>
-      <c r="S50" s="14" t="n">
-        <v>3030287</v>
+        <v>34131</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>28744190</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3337,47 +3337,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="33" t="n">
+      <c r="P51" s="32" t="n">
+        <v>22850</v>
+      </c>
+      <c r="Q51" s="12" t="n">
+        <v>242715</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>157290</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>25809034</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="P52" s="32" t="n">
         <v>22500</v>
       </c>
-      <c r="Q51" s="14" t="n">
-        <v>200627</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>1596</v>
-      </c>
-      <c r="S51" s="14" t="n">
-        <v>2463494</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="P52" s="33" t="n">
-        <v>22000</v>
-      </c>
-      <c r="Q52" s="14" t="n">
-        <v>281076</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>92775</v>
-      </c>
-      <c r="S52" s="14" t="n">
-        <v>1961569</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="Q52" s="12" t="n">
+        <v>163830</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>-36797</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>4265927</v>
+      </c>
+      <c r="T52" s="33" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 16-Oct-2026    1 DAY AGO = 15-Oct-2026    2 DAYS AGO = 14-Oct-2026    3 DAYS AGO = 13-Oct-2026    4 DAYS AGO = 12-Oct-2026    (generated 16-Oct-2026 20:32 IST)</t>
+          <t>TODAY = 19-Oct-2026    1 DAY AGO = 16-Oct-2026    2 DAYS AGO = 15-Oct-2026    3 DAYS AGO = 14-Oct-2026    4 DAYS AGO = 13-Oct-2026    (generated 19-Oct-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-21
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -190,17 +190,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>10877</v>
+        <v>-6860</v>
       </c>
     </row>
     <row r="3">
@@ -701,65 +701,65 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>4779</v>
+        <v>-4819</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-6098</v>
+        <v>2041</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>-6860</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J3" s="12" t="n">
+        <v>223931</v>
+      </c>
+      <c r="K3" s="12" t="n">
+        <v>230791</v>
+      </c>
+      <c r="L3" s="12" t="n">
+        <v>219914</v>
+      </c>
+      <c r="M3" s="12" t="n">
+        <v>219312</v>
+      </c>
+      <c r="N3" s="12" t="n">
+        <v>245358</v>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G3" s="11" t="n">
-        <v>10877</v>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n">
-        <v>230791</v>
-      </c>
-      <c r="K3" s="12" t="n">
-        <v>219914</v>
-      </c>
-      <c r="L3" s="12" t="n">
-        <v>219312</v>
-      </c>
-      <c r="M3" s="12" t="n">
-        <v>245358</v>
-      </c>
-      <c r="N3" s="12" t="n">
-        <v>229857</v>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>135953</v>
+      <c r="S3" s="14" t="n">
+        <v>197440</v>
       </c>
     </row>
     <row r="4">
@@ -770,65 +770,65 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>82</v>
+        <v>-77</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>421</v>
+        <v>-1194</v>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>1117</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>37971</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>36854</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>37193</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>36441</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>30022</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>-339</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>36854</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>37193</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>36441</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>30022</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>34531</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>-235937</v>
+      <c r="S4" s="14" t="n">
+        <v>-99008</v>
       </c>
     </row>
     <row r="5">
@@ -837,67 +837,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
-        <v>-3305</v>
+      <c r="C5" s="11" t="n">
+        <v>-4063</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>3626</v>
+        <v>-6365</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>2302</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-277628</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-279930</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-272999</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-279827</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-296697</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-6931</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-279930</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-272999</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-279827</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-296697</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-289495</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>34518</v>
+        <v>-38656</v>
       </c>
     </row>
     <row r="6">
@@ -908,27 +908,27 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>-1781</v>
+        <v>1273</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>1826</v>
+        <v>-2168</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-3607</v>
+        <v>3441</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,26 +936,26 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>15726</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>12285</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>15892</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>24074</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>21317</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>25107</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="9" t="inlineStr">
+      <c r="Q6" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -965,8 +965,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="11" t="n">
-        <v>128392</v>
+      <c r="S6" s="14" t="n">
+        <v>57869</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-225</v>
+        <v>-7686</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-225</v>
+        <v>-7686</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,7 +1002,7 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
+      <c r="Q7" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>-64731</v>
+      <c r="S7" s="14" t="n">
+        <v>-14943</v>
       </c>
     </row>
     <row r="8">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="14" t="n">
-        <v>-339</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="9">
@@ -1093,27 +1093,27 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>-1217512</v>
+        <v>1141372</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>-1353465</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
+        <v>943932</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>135953</v>
+      <c r="G9" s="14" t="n">
+        <v>197440</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,26 +1121,26 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>389918</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>192478</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>56525</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>57913</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>187421</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>111452</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>-1062</v>
+      <c r="S9" s="11" t="n">
+        <v>-165</v>
       </c>
     </row>
     <row r="10">
@@ -1160,29 +1160,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>-907</v>
+      <c r="C10" s="11" t="n">
+        <v>-350</v>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E10" s="14" t="n">
-        <v>155</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+        <v>-185</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>-1062</v>
+      <c r="G10" s="11" t="n">
+        <v>-165</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,26 +1190,26 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>7448</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>7613</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>8675</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>19105</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>98383</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>94848</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
+      <c r="Q10" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>7470</v>
+      <c r="S10" s="11" t="n">
+        <v>15910</v>
       </c>
     </row>
     <row r="11">
@@ -1231,65 +1231,65 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>-150166</v>
+        <v>209550</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>-171180</v>
+        <v>298416</v>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>-88866</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-341527</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-252661</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-273675</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-207881</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-332906</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>21014</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-252661</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-273675</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-207881</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-332906</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-288995</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>9829</v>
+      <c r="S11" s="14" t="n">
+        <v>13571</v>
       </c>
     </row>
     <row r="12">
@@ -1300,27 +1300,27 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>-367104</v>
+        <v>374391</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>-211198</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+        <v>482799</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-155906</v>
+      <c r="G12" s="11" t="n">
+        <v>-108408</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,20 +1328,20 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>-55839</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>52569</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>208475</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>130863</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>47101</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>82695</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R12" s="10" t="inlineStr">
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-15602</v>
+        <v>2039</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-1735689</v>
+        <v>1724963</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-1735688</v>
+        <v>1724962</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="Q13" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-2771</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-6931</v>
+        <v>2302</v>
       </c>
     </row>
     <row r="15">
@@ -1485,27 +1485,27 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>-2251398</v>
+        <v>406790</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E15" s="14" t="n">
-        <v>-2015461</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+        <v>505798</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>-235937</v>
+      <c r="G15" s="14" t="n">
+        <v>-99008</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-826431</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-727423</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-491486</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-472041</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-706501</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-586835</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="Q15" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="11" t="n">
-        <v>21014</v>
+        <v>-88866</v>
       </c>
     </row>
     <row r="16">
@@ -1552,29 +1552,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
-        <v>7925</v>
+      <c r="C16" s="11" t="n">
+        <v>15735</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>455</v>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
+        <v>-175</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>7470</v>
+      <c r="G16" s="11" t="n">
+        <v>15910</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,26 +1582,26 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>113261</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>97351</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>89881</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>81661</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>75950</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>74365</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
+      <c r="Q16" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>52260</v>
+      <c r="S16" s="11" t="n">
+        <v>23723</v>
       </c>
     </row>
     <row r="17">
@@ -1623,27 +1623,27 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>-306805</v>
+        <v>148216</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E17" s="14" t="n">
-        <v>-359065</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+        <v>124493</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>52260</v>
+      <c r="G17" s="11" t="n">
+        <v>23723</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,20 +1651,20 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>597220</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>573497</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>521237</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>447027</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>544765</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>565338</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="Q17" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="14" t="n">
-        <v>-39183</v>
+        <v>44069</v>
       </c>
     </row>
     <row r="18">
@@ -1692,27 +1692,27 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>-551692</v>
+        <v>238049</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>-727899</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
+        <v>178676</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>176207</v>
+      <c r="G18" s="11" t="n">
+        <v>59373</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1720,26 +1720,26 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>115949</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>56576</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>-119631</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>-56647</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>85786</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>-52868</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="13" t="inlineStr">
+      <c r="Q18" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>-51830</v>
+      <c r="S18" s="11" t="n">
+        <v>-13604</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-3101970</v>
+        <v>808790</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-3101970</v>
+        <v>808792</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
+      <c r="Q19" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>19214</v>
+      <c r="S19" s="11" t="n">
+        <v>16818</v>
       </c>
     </row>
     <row r="20">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="14" t="n">
-        <v>-3607</v>
+        <v>3441</v>
       </c>
     </row>
     <row r="21">
@@ -1877,27 +1877,27 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>41616</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+        <v>-19204</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
-        <v>7098</v>
+      <c r="E21" s="11" t="n">
+        <v>19452</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>34518</v>
+        <v>-38656</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,26 +1905,26 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3154648</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3193304</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3158786</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3179070</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>3222075</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3212609</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
+      <c r="Q21" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-155906</v>
+      <c r="S21" s="11" t="n">
+        <v>-108408</v>
       </c>
     </row>
     <row r="22">
@@ -1944,29 +1944,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
-        <v>18266</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="n">
+        <v>14231</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
-        <v>8437</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="E22" s="11" t="n">
+        <v>660</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>9829</v>
+      <c r="G22" s="14" t="n">
+        <v>13571</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,26 +1974,26 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4304197</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4317768</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4327597</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4376554</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4397081</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4435039</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
+      <c r="Q22" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>176207</v>
+      <c r="S22" s="11" t="n">
+        <v>59373</v>
       </c>
     </row>
     <row r="23">
@@ -2015,65 +2015,65 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>-3319</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+        <v>46842</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n">
-        <v>35864</v>
+      <c r="E23" s="11" t="n">
+        <v>2773</v>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>44069</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>781550</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>737481</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>776664</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>786561</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>743986</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>-39183</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>737481</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>776664</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>786561</v>
-      </c>
-      <c r="M23" s="12" t="n">
-        <v>743986</v>
-      </c>
-      <c r="N23" s="12" t="n">
-        <v>774020</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-5164</v>
+      <c r="S23" s="11" t="n">
+        <v>-18984</v>
       </c>
     </row>
     <row r="24">
@@ -2082,29 +2082,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C24" s="11" t="n">
-        <v>29079</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="C24" s="14" t="n">
+        <v>43489</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>34243</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+      <c r="E24" s="11" t="n">
+        <v>62473</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-5164</v>
+      <c r="G24" s="11" t="n">
+        <v>-18984</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,26 +2112,26 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>367999</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>386983</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>392147</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>410923</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>431020</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>448410</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
+      <c r="Q24" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>-60960</v>
+      <c r="S24" s="11" t="n">
+        <v>-46304</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>85642</v>
+        <v>85358</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>85642</v>
+        <v>85358</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>48288</v>
+        <v>-1982</v>
       </c>
     </row>
     <row r="26">
@@ -2249,29 +2249,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C27" s="11" t="n">
-        <v>142557</v>
+      <c r="C27" s="14" t="n">
+        <v>43176</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>14165</v>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
+        <v>-14693</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G27" s="11" t="n">
-        <v>128392</v>
+      <c r="G27" s="14" t="n">
+        <v>57869</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1217850</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1159981</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1031589</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>943689</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>987613</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>863596</v>
       </c>
     </row>
     <row r="28">
@@ -2300,29 +2300,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="11" t="n">
-        <v>200</v>
+      <c r="C28" s="14" t="n">
+        <v>153</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>15802</v>
+        <v>-1886</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-15602</v>
+        <v>2039</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-436591</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-438630</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-423028</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-404104</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-367996</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-354012</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>-7080</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>-5541</v>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>44750</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
+      <c r="E29" s="11" t="n">
+        <v>8063</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>-51830</v>
+      <c r="G29" s="11" t="n">
+        <v>-13604</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-223094</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-209490</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-157660</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-149590</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-165987</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-152484</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 19-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 21-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,29 +2418,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
-        <v>11913</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="C30" s="14" t="n">
+        <v>19095</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>72873</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
+      <c r="E30" s="11" t="n">
+        <v>65399</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>-60960</v>
+      <c r="G30" s="11" t="n">
+        <v>-46304</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-558165</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-511861</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-450901</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-389995</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-453630</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-357100</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23150.85</v>
+        <v>23016</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23175.25</v>
+        <v>23120.9</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>147590</v>
+        <v>56883</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>147590</v>
+        <v>56883</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22845</v>
+        <v>22649.9</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22888.95</v>
+        <v>22811.35</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23424.71666666667</v>
+        <v>23542.53333333333</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22929.34166666667</v>
+        <v>22836.03333333333</v>
       </c>
     </row>
     <row r="33">
@@ -2597,29 +2597,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>-55662</v>
+      <c r="C33" s="14" t="n">
+        <v>-46393</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>9069</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
+        <v>-31450</v>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G33" s="11" t="n">
-        <v>-64731</v>
+      <c r="G33" s="14" t="n">
+        <v>-14943</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-220933</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-205990</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-141259</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-175317</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-218398</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-202004</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23299.98333333333</v>
+        <v>23331.71666666666</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22969.73333333333</v>
+        <v>22860.71666666666</v>
       </c>
     </row>
     <row r="34">
@@ -2666,27 +2666,27 @@
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>328</v>
+        <v>-144</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>3099</v>
+        <v>-251</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-2771</v>
+        <v>107</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>519</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>412</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>3183</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>3747</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>4320</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>7596</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23094.46666666667</v>
+        <v>23071.53333333333</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23010.125</v>
+        <v>22885.4</v>
       </c>
     </row>
     <row r="35">
@@ -2731,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>17183</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="11" t="n">
+        <v>12929</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>-2031</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
+      <c r="E35" s="11" t="n">
+        <v>-3889</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>19214</v>
+      <c r="G35" s="11" t="n">
+        <v>16818</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>160242</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>143424</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>124210</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>119371</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>133066</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>124293</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22969.73333333333</v>
+        <v>22860.71666666666</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,29 +2792,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>36216</v>
+      <c r="C36" s="11" t="n">
+        <v>31028</v>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E36" s="14" t="n">
-        <v>-12072</v>
+        <v>33010</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>48288</v>
+        <v>-1982</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>60172</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>62154</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>13866</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>52199</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>81012</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>70115</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22764.21666666667</v>
+        <v>22600.53333333333</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-1935</v>
+        <v>-2580</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-1935</v>
+        <v>-2580</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22639.48333333333</v>
+        <v>22389.71666666666</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22433.96666666667</v>
+        <v>22129.53333333333</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>15.68</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>14.77</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>14.06</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>14.03</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>14.63</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>14.12</v>
       </c>
     </row>
     <row r="41">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 19-Oct-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 27-Oct-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9599703979923143</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.962724138114085</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9729851533215025</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9663308743049036</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9501517111819584</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9538116838234366</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,889    PCR(OI) 0.80    Max Pain 22,900</t>
+          <t>Spot 22,811    PCR(OI) 0.70    Max Pain 22,900</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23762.55564516129</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23775.19072580645</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23788.80080645161</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23798.62903225806</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23809.56612903226</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23822.26008064516</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22811.35</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22888.95</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23146.15</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>22997.35</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22622.7</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22721.95</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>22900</v>
+        <v>23000</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>363408</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>321581</v>
+        <v>250604</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>101653</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>21355500</v>
+        <v>3137681</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.939144741359203</v>
+        <v>0.9359848090651907</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9495717233987274</v>
@@ -3173,20 +3173,20 @@
         <v>0.9493709489654826</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>22950</v>
+        <v>23500</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>226788</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>210018</v>
+        <v>233700</v>
+      </c>
+      <c r="R46" s="14" t="n">
+        <v>36920</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>19141660</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>1711123</v>
+      </c>
+      <c r="T46" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24372.12177419355</v>
+        <v>24371.49596774194</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24375.35725806452</v>
@@ -3212,20 +3212,20 @@
         <v>24374.56088709677</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>23000</v>
+        <v>24000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>252235</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>150703</v>
+        <v>216371</v>
+      </c>
+      <c r="R47" s="14" t="n">
+        <v>3087</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>23111861</v>
-      </c>
-      <c r="T47" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>917549</v>
+      </c>
+      <c r="T47" s="31" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22888.95</v>
+        <v>22811.35</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23146.15</v>
@@ -3250,7 +3250,7 @@
       <c r="N48" s="18" t="n">
         <v>23140.5</v>
       </c>
-      <c r="P48" s="30" t="inlineStr">
+      <c r="P48" s="32" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="31" t="inlineStr">
-        <is>
-          <t>19-Oct-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="31" t="inlineStr">
+      <c r="J49" s="30" t="inlineStr">
+        <is>
+          <t>21-Oct-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="30" t="inlineStr">
         <is>
           <t>16-Oct-2026</t>
         </is>
       </c>
-      <c r="L49" s="31" t="inlineStr">
+      <c r="L49" s="30" t="inlineStr">
         <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="M49" s="31" t="inlineStr">
+      <c r="M49" s="30" t="inlineStr">
         <is>
           <t>01-Oct-2026</t>
         </is>
       </c>
-      <c r="N49" s="31" t="inlineStr">
+      <c r="N49" s="30" t="inlineStr">
         <is>
           <t>25-Sep-2026</t>
         </is>
@@ -3318,17 +3318,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
-        <v>22900</v>
+      <c r="P50" s="33" t="n">
+        <v>22500</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>202833</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>34131</v>
+        <v>130765</v>
+      </c>
+      <c r="R50" s="14" t="n">
+        <v>7967</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>28744190</v>
+        <v>2189704</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3337,38 +3337,38 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="32" t="n">
-        <v>22850</v>
+      <c r="P51" s="33" t="n">
+        <v>22000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>242715</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>157290</v>
+        <v>148913</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>26609</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>25809034</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>1217994</v>
+      </c>
+      <c r="T51" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>22500</v>
+      <c r="P52" s="33" t="n">
+        <v>21000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>163830</v>
+        <v>125579</v>
       </c>
       <c r="R52" s="14" t="n">
-        <v>-36797</v>
+        <v>20795</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>4265927</v>
-      </c>
-      <c r="T52" s="33" t="inlineStr">
+        <v>292368</v>
+      </c>
+      <c r="T52" s="31" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 19-Oct-2026    1 DAY AGO = 16-Oct-2026    2 DAYS AGO = 15-Oct-2026    3 DAYS AGO = 14-Oct-2026    4 DAYS AGO = 13-Oct-2026    (generated 19-Oct-2026 20:32 IST)</t>
+          <t>TODAY = 21-Oct-2026    1 DAY AGO = 19-Oct-2026    2 DAYS AGO = 16-Oct-2026    3 DAYS AGO = 15-Oct-2026    4 DAYS AGO = 14-Oct-2026    (generated 21-Oct-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-22
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -129,22 +129,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-6860</v>
+        <v>-5646</v>
       </c>
     </row>
     <row r="3">
@@ -699,13 +699,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="n">
-        <v>-4819</v>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>1469</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>2041</v>
+        <v>7115</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,36 +721,36 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-6860</v>
+        <v>-5646</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="14" t="n">
+        <v>218285</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>223931</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="14" t="n">
         <v>230791</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="14" t="n">
         <v>219914</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>219312</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>245358</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="14" t="n">
-        <v>197440</v>
+      <c r="S3" s="11" t="n">
+        <v>-107615</v>
       </c>
     </row>
     <row r="4">
@@ -774,61 +774,61 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>-77</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+        <v>-211</v>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E4" s="14" t="n">
-        <v>-1194</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="E4" s="13" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>-201</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>37770</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>37971</v>
+      </c>
+      <c r="L4" s="14" t="n">
+        <v>36854</v>
+      </c>
+      <c r="M4" s="14" t="n">
+        <v>37193</v>
+      </c>
+      <c r="N4" s="14" t="n">
+        <v>36441</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>1117</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>37971</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>36854</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>37193</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>36441</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>30022</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>-99008</v>
+      <c r="S4" s="11" t="n">
+        <v>81549</v>
       </c>
     </row>
     <row r="5">
@@ -837,67 +837,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>-4063</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>-6365</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>2105</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>4777</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>-2672</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>-280300</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>-277628</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>-279930</v>
+      </c>
+      <c r="M5" s="14" t="n">
+        <v>-272999</v>
+      </c>
+      <c r="N5" s="14" t="n">
+        <v>-279827</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>2302</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-277628</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-279930</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-272999</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-279827</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-296697</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>-38656</v>
+      <c r="S5" s="13" t="n">
+        <v>7842</v>
       </c>
     </row>
     <row r="6">
@@ -906,58 +906,58 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
-        <v>1273</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>-2168</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="C6" s="13" t="n">
+        <v>16105</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>7586</v>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>3441</v>
+      <c r="G6" s="13" t="n">
+        <v>8519</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
+        <v>24245</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>15726</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>12285</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="14" t="n">
         <v>15892</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="14" t="n">
         <v>24074</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>21317</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R6" s="10" t="inlineStr">
@@ -965,8 +965,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="14" t="n">
-        <v>57869</v>
+      <c r="S6" s="11" t="n">
+        <v>-50104</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-7686</v>
+        <v>19468</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-7686</v>
+        <v>19468</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="14" t="n">
-        <v>-14943</v>
+      <c r="S7" s="11" t="n">
+        <v>18892</v>
       </c>
     </row>
     <row r="8">
@@ -1071,9 +1071,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>1117</v>
+      <c r="S8" s="11" t="n">
+        <v>-201</v>
       </c>
     </row>
     <row r="9">
@@ -1091,13 +1091,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
-        <v>1141372</v>
+      <c r="C9" s="13" t="n">
+        <v>173317</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
@@ -1105,53 +1105,53 @@
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>943932</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+        <v>280932</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>-107615</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>282303</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>389918</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>192478</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <v>56525</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <v>57913</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>197440</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>389918</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>192478</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>56525</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>57913</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>187421</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>-165</v>
+      <c r="S9" s="13" t="n">
+        <v>630</v>
       </c>
     </row>
     <row r="10">
@@ -1160,67 +1160,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>-350</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>-185</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>630</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>630</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="n">
+        <v>8078</v>
+      </c>
+      <c r="K10" s="14" t="n">
+        <v>7448</v>
+      </c>
+      <c r="L10" s="14" t="n">
+        <v>7613</v>
+      </c>
+      <c r="M10" s="14" t="n">
+        <v>8675</v>
+      </c>
+      <c r="N10" s="14" t="n">
+        <v>19105</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q10" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>-165</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>7448</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>7613</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>8675</v>
-      </c>
-      <c r="M10" s="12" t="n">
-        <v>19105</v>
-      </c>
-      <c r="N10" s="12" t="n">
-        <v>98383</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q10" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>15910</v>
+      <c r="S10" s="13" t="n">
+        <v>-21171</v>
       </c>
     </row>
     <row r="11">
@@ -1229,67 +1229,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
-        <v>209550</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>298416</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="C11" s="13" t="n">
+        <v>41685</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>-9493</v>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>51178</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="n">
+        <v>-290349</v>
+      </c>
+      <c r="K11" s="14" t="n">
+        <v>-341527</v>
+      </c>
+      <c r="L11" s="14" t="n">
+        <v>-252661</v>
+      </c>
+      <c r="M11" s="14" t="n">
+        <v>-273675</v>
+      </c>
+      <c r="N11" s="14" t="n">
+        <v>-207881</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>-88866</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-341527</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-252661</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-273675</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-207881</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-332906</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>13571</v>
+      <c r="S11" s="11" t="n">
+        <v>-30681</v>
       </c>
     </row>
     <row r="12">
@@ -1298,56 +1298,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>374391</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>482799</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>-108408</v>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>-66485</v>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>-122292</v>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="n">
+        <v>55807</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="14" t="n">
+        <v>-32</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>-55839</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <v>52569</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="14" t="n">
         <v>208475</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="14" t="n">
         <v>130863</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>47101</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="13" t="inlineStr">
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>2039</v>
+      <c r="S12" s="13" t="n">
+        <v>1835</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1724963</v>
+        <v>149147</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1724962</v>
+        <v>149147</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>107</v>
+        <v>7394</v>
       </c>
     </row>
     <row r="14">
@@ -1463,9 +1463,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q14" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>2302</v>
+      <c r="S14" s="11" t="n">
+        <v>-2672</v>
       </c>
     </row>
     <row r="15">
@@ -1489,52 +1489,52 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>406790</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
+        <v>496011</v>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="14" t="n">
-        <v>505798</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G15" s="14" t="n">
-        <v>-99008</v>
+      <c r="E15" s="13" t="n">
+        <v>414462</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>81549</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-744882</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-826431</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-727423</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>-491486</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>-472041</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-706501</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q15" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="11" t="n">
-        <v>-88866</v>
+      <c r="S15" s="13" t="n">
+        <v>51178</v>
       </c>
     </row>
     <row r="16">
@@ -1552,13 +1552,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>15735</v>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>-21371</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1566,44 +1566,44 @@
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>-175</v>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="n">
-        <v>15910</v>
+        <v>-200</v>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>-21171</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="14" t="n">
+        <v>92090</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>113261</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <v>97351</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="14" t="n">
         <v>89881</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="14" t="n">
         <v>81661</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>75950</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q16" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>23723</v>
+      <c r="S16" s="13" t="n">
+        <v>-95060</v>
       </c>
     </row>
     <row r="17">
@@ -1627,61 +1627,61 @@
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>148216</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
+        <v>11980</v>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="14" t="n">
-        <v>124493</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="E17" s="13" t="n">
+        <v>107040</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>-95060</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>502160</v>
+      </c>
+      <c r="K17" s="14" t="n">
+        <v>597220</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <v>573497</v>
+      </c>
+      <c r="M17" s="14" t="n">
+        <v>521237</v>
+      </c>
+      <c r="N17" s="14" t="n">
+        <v>447027</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>23723</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>597220</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>573497</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>521237</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>447027</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>544765</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>44069</v>
+      <c r="S17" s="13" t="n">
+        <v>19963</v>
       </c>
     </row>
     <row r="18">
@@ -1696,15 +1696,15 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>238049</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+        <v>164453</v>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="14" t="n">
-        <v>178676</v>
+      <c r="E18" s="13" t="n">
+        <v>129771</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
@@ -1712,36 +1712,36 @@
         </is>
       </c>
       <c r="G18" s="11" t="n">
-        <v>59373</v>
+        <v>34682</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="12" t="n">
+      <c r="J18" s="14" t="n">
+        <v>150631</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>115949</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="14" t="n">
         <v>56576</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="14" t="n">
         <v>-119631</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="14" t="n">
         <v>-56647</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>85786</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q18" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R18" s="10" t="inlineStr">
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="11" t="n">
-        <v>-13604</v>
+      <c r="S18" s="13" t="n">
+        <v>20447</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>808790</v>
+        <v>651073</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>808792</v>
+        <v>651073</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q19" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="11" t="n">
-        <v>16818</v>
+      <c r="S19" s="13" t="n">
+        <v>-21919</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
+      <c r="Q20" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>3441</v>
+      <c r="S20" s="13" t="n">
+        <v>8519</v>
       </c>
     </row>
     <row r="21">
@@ -1881,52 +1881,52 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-19204</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="11" t="n">
-        <v>19452</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G21" s="11" t="n">
-        <v>-38656</v>
+        <v>-19468</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>-27310</v>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>7842</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="14" t="n">
+        <v>3162490</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3154648</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <v>3193304</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="14" t="n">
         <v>3158786</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="14" t="n">
         <v>3179070</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3222075</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>-108408</v>
+      <c r="S21" s="13" t="n">
+        <v>55807</v>
       </c>
     </row>
     <row r="22">
@@ -1944,13 +1944,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="n">
-        <v>14231</v>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>-902</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
@@ -1958,53 +1958,53 @@
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>660</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+        <v>29779</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="n">
+        <v>-30681</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>-4334878</v>
+      </c>
+      <c r="K22" s="14" t="n">
+        <v>-4304197</v>
+      </c>
+      <c r="L22" s="14" t="n">
+        <v>-4317768</v>
+      </c>
+      <c r="M22" s="14" t="n">
+        <v>-4327597</v>
+      </c>
+      <c r="N22" s="14" t="n">
+        <v>-4376554</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q22" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>13571</v>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J22" s="12" t="n">
-        <v>-4304197</v>
-      </c>
-      <c r="K22" s="12" t="n">
-        <v>-4317768</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>-4327597</v>
-      </c>
-      <c r="M22" s="12" t="n">
-        <v>-4376554</v>
-      </c>
-      <c r="N22" s="12" t="n">
-        <v>-4397081</v>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
       <c r="S22" s="11" t="n">
-        <v>59373</v>
+        <v>34682</v>
       </c>
     </row>
     <row r="23">
@@ -2013,58 +2013,58 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n">
-        <v>46842</v>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E23" s="11" t="n">
-        <v>2773</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
+      <c r="C23" s="13" t="n">
+        <v>9975</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>-9988</v>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>44069</v>
+      <c r="G23" s="13" t="n">
+        <v>19963</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="J23" s="14" t="n">
+        <v>801513</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>781550</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <v>737481</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="14" t="n">
         <v>776664</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="14" t="n">
         <v>786561</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>743986</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q23" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>-18984</v>
+      <c r="S23" s="13" t="n">
+        <v>2876</v>
       </c>
     </row>
     <row r="24">
@@ -2082,58 +2082,58 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="n">
-        <v>43489</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="n">
-        <v>62473</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="n">
-        <v>-18984</v>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>-39905</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>-42781</v>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>2876</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J24" s="14" t="n">
+        <v>370875</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>367999</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="14" t="n">
         <v>386983</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="14" t="n">
         <v>392147</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="14" t="n">
         <v>410923</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>431020</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q24" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="11" t="n">
-        <v>-46304</v>
+      <c r="S24" s="13" t="n">
+        <v>27822</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>85358</v>
+        <v>-50300</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>85358</v>
+        <v>-50300</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,7 +2178,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
+      <c r="Q25" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>-1982</v>
+      <c r="S25" s="13" t="n">
+        <v>-4367</v>
       </c>
     </row>
     <row r="26">
@@ -2249,49 +2249,49 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="n">
-        <v>43176</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>-61610</v>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
-        <v>-14693</v>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G27" s="14" t="n">
-        <v>57869</v>
+      <c r="E27" s="13" t="n">
+        <v>-11506</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="n">
+        <v>-50104</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>1167746</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>1217850</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>1159981</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="14" t="n">
         <v>1031589</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>943689</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>987613</v>
       </c>
     </row>
     <row r="28">
@@ -2300,49 +2300,49 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="14" t="n">
-        <v>153</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>-201</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E28" s="14" t="n">
-        <v>-1886</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="E28" s="13" t="n">
+        <v>-2036</v>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>2039</v>
+      <c r="G28" s="13" t="n">
+        <v>1835</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-434756</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-436591</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-438630</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="14" t="n">
         <v>-423028</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>-404104</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-367996</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,53 +2359,53 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="n">
-        <v>-5541</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E29" s="11" t="n">
-        <v>8063</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G29" s="11" t="n">
-        <v>-13604</v>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="n">
+        <v>8933</v>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>-11514</v>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>20447</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-202647</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-223094</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-209490</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="14" t="n">
         <v>-157660</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>-149590</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-165987</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 21-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 22-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,57 +2418,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
-        <v>19095</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E30" s="11" t="n">
-        <v>65399</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G30" s="11" t="n">
-        <v>-46304</v>
+      <c r="C30" s="13" t="n">
+        <v>19596</v>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>-8226</v>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>27822</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-530343</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-558165</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-511861</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="14" t="n">
         <v>-450901</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="14" t="n">
         <v>-389995</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-453630</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23016</v>
+        <v>22687.75</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23120.9</v>
+        <v>22785</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>56883</v>
+        <v>-33282</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>56883</v>
+        <v>-33282</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>22649.9</v>
+        <v>22554.85</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>22811.35</v>
+        <v>22687.65</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>23542.53333333333</v>
+        <v>23026.96666666667</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>22836.03333333333</v>
+        <v>22681.74166666666</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2597,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
-        <v>-46393</v>
+      <c r="C33" s="13" t="n">
+        <v>-3360</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,43 +2611,43 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>-31450</v>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="n">
-        <v>-14943</v>
+        <v>-22252</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>18892</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-202041</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-220933</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-205990</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="14" t="n">
         <v>-141259</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="14" t="n">
         <v>-175317</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-218398</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23331.71666666666</v>
+        <v>22905.98333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>22860.71666666666</v>
+        <v>22675.83333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2664,21 +2664,21 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="n">
-        <v>-144</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E34" s="11" t="n">
-        <v>-251</v>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>7812</v>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="n">
+        <v>418</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,35 +2686,35 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>107</v>
+        <v>7394</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>7913</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>519</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>412</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="14" t="n">
         <v>3183</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="14" t="n">
         <v>3747</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>4320</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23071.53333333333</v>
+        <v>22796.81666666667</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>22885.4</v>
+        <v>22669.925</v>
       </c>
     </row>
     <row r="35">
@@ -2731,57 +2731,57 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C35" s="11" t="n">
-        <v>12929</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E35" s="11" t="n">
-        <v>-3889</v>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G35" s="11" t="n">
-        <v>16818</v>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="n">
+        <v>-7574</v>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="n">
+        <v>14345</v>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="n">
+        <v>-21919</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>138323</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>160242</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>143424</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="14" t="n">
         <v>124210</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="14" t="n">
         <v>119371</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>133066</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>22860.71666666666</v>
+        <v>22675.83333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2798,51 +2798,51 @@
         </is>
       </c>
       <c r="C36" s="11" t="n">
-        <v>31028</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+        <v>21473</v>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>33010</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
+      <c r="E36" s="13" t="n">
+        <v>25840</v>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G36" s="14" t="n">
-        <v>-1982</v>
+      <c r="G36" s="13" t="n">
+        <v>-4367</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>55805</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>60172</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>62154</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="14" t="n">
         <v>13866</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="14" t="n">
         <v>52199</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>81012</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>22600.53333333333</v>
+        <v>22566.66666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-2580</v>
+        <v>18351</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-2580</v>
+        <v>18351</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>22389.71666666666</v>
+        <v>22445.68333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>22129.53333333333</v>
+        <v>22336.51666666666</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>15.76</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>15.68</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>14.77</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>14.06</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>14.03</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>14.63</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.955246281796554</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9599703979923143</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.962724138114085</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>0.9729851533215025</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.9663308743049036</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>0.9501517111819584</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 22,811    PCR(OI) 0.70    Max Pain 22,900</t>
+          <t>Spot 22,688    PCR(OI) 0.82    Max Pain 22,850</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23750.57661290323</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23762.55564516129</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23775.19072580645</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23788.80080645161</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23798.62903225806</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23809.56612903226</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>22687.65</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>22811.35</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>22888.95</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>23146.15</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>22997.35</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>22622.7</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3136,14 +3136,14 @@
       <c r="P45" s="28" t="n">
         <v>23000</v>
       </c>
-      <c r="Q45" s="12" t="n">
-        <v>250604</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>101653</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>3137681</v>
+      <c r="Q45" s="14" t="n">
+        <v>239754</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>-10850</v>
+      </c>
+      <c r="S45" s="14" t="n">
+        <v>2294613</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9359848090651907</v>
+        <v>0.9309473134128528</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9495717233987274</v>
@@ -3175,14 +3175,14 @@
       <c r="P46" s="28" t="n">
         <v>23500</v>
       </c>
-      <c r="Q46" s="12" t="n">
-        <v>233700</v>
-      </c>
-      <c r="R46" s="14" t="n">
-        <v>36920</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>1711123</v>
+      <c r="Q46" s="14" t="n">
+        <v>227799</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>-5901</v>
+      </c>
+      <c r="S46" s="14" t="n">
+        <v>1065946</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24371.49596774194</v>
+        <v>24370.49838709677</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24375.35725806452</v>
@@ -3214,14 +3214,14 @@
       <c r="P47" s="28" t="n">
         <v>24000</v>
       </c>
-      <c r="Q47" s="12" t="n">
-        <v>216371</v>
-      </c>
-      <c r="R47" s="14" t="n">
-        <v>3087</v>
-      </c>
-      <c r="S47" s="12" t="n">
-        <v>917549</v>
+      <c r="Q47" s="14" t="n">
+        <v>282795</v>
+      </c>
+      <c r="R47" s="13" t="n">
+        <v>66424</v>
+      </c>
+      <c r="S47" s="14" t="n">
+        <v>803581</v>
       </c>
       <c r="T47" s="31" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>22811.35</v>
+        <v>22687.65</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>23146.15</v>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
-          <t>21-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="K49" s="30" t="inlineStr">
@@ -3321,14 +3321,14 @@
       <c r="P50" s="33" t="n">
         <v>22500</v>
       </c>
-      <c r="Q50" s="12" t="n">
-        <v>130765</v>
-      </c>
-      <c r="R50" s="14" t="n">
-        <v>7967</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>2189704</v>
+      <c r="Q50" s="14" t="n">
+        <v>142386</v>
+      </c>
+      <c r="R50" s="13" t="n">
+        <v>11621</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>2819587</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3340,14 +3340,14 @@
       <c r="P51" s="33" t="n">
         <v>22000</v>
       </c>
-      <c r="Q51" s="12" t="n">
-        <v>148913</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>26609</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>1217994</v>
+      <c r="Q51" s="14" t="n">
+        <v>188564</v>
+      </c>
+      <c r="R51" s="13" t="n">
+        <v>39651</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>1253033</v>
       </c>
       <c r="T51" s="30" t="inlineStr">
         <is>
@@ -3357,16 +3357,16 @@
     </row>
     <row r="52">
       <c r="P52" s="33" t="n">
-        <v>21000</v>
-      </c>
-      <c r="Q52" s="12" t="n">
-        <v>125579</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>20795</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>292368</v>
+        <v>21500</v>
+      </c>
+      <c r="Q52" s="14" t="n">
+        <v>174850</v>
+      </c>
+      <c r="R52" s="13" t="n">
+        <v>62459</v>
+      </c>
+      <c r="S52" s="14" t="n">
+        <v>587876</v>
       </c>
       <c r="T52" s="31" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 21-Oct-2026    1 DAY AGO = 19-Oct-2026    2 DAYS AGO = 16-Oct-2026    3 DAYS AGO = 15-Oct-2026    4 DAYS AGO = 14-Oct-2026    (generated 21-Oct-2026 20:31 IST)</t>
+          <t>TODAY = 22-Oct-2026    1 DAY AGO = 21-Oct-2026    2 DAYS AGO = 19-Oct-2026    3 DAYS AGO = 16-Oct-2026    4 DAYS AGO = 15-Oct-2026    (generated 22-Oct-2026 20:32 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-10-23
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -129,22 +129,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,9 +187,6 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -201,6 +198,9 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-5646</v>
+        <v>-2977</v>
       </c>
     </row>
     <row r="3">
@@ -699,13 +699,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="n">
-        <v>1469</v>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>-56</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>7115</v>
+        <v>2921</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,28 +721,28 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-5646</v>
+        <v>-2977</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>215308</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>218285</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>223931</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>230791</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="12" t="n">
         <v>219914</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>219312</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>-107615</v>
+        <v>-56344</v>
       </c>
     </row>
     <row r="4">
@@ -774,61 +774,61 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>-211</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
+        <v>-663</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E4" s="13" t="n">
-        <v>-10</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="E4" s="14" t="n">
+        <v>-2273</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>1610</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>39380</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>37770</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>37971</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>36854</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>37193</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>-201</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="14" t="n">
-        <v>37770</v>
-      </c>
-      <c r="K4" s="14" t="n">
-        <v>37971</v>
-      </c>
-      <c r="L4" s="14" t="n">
-        <v>36854</v>
-      </c>
-      <c r="M4" s="14" t="n">
-        <v>37193</v>
-      </c>
-      <c r="N4" s="14" t="n">
-        <v>36441</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>81549</v>
+      <c r="S4" s="14" t="n">
+        <v>-144179</v>
       </c>
     </row>
     <row r="5">
@@ -837,13 +837,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
-        <v>2105</v>
+      <c r="C5" s="14" t="n">
+        <v>2283</v>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
@@ -851,53 +851,53 @@
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>4777</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
+        <v>2166</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>117</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-280183</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-280300</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-277628</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-279930</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-272999</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="11" t="n">
-        <v>-2672</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="n">
-        <v>-280300</v>
-      </c>
-      <c r="K5" s="14" t="n">
-        <v>-277628</v>
-      </c>
-      <c r="L5" s="14" t="n">
-        <v>-279930</v>
-      </c>
-      <c r="M5" s="14" t="n">
-        <v>-272999</v>
-      </c>
-      <c r="N5" s="14" t="n">
-        <v>-279827</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="13" t="n">
-        <v>7842</v>
+      <c r="S5" s="11" t="n">
+        <v>-38490</v>
       </c>
     </row>
     <row r="6">
@@ -906,13 +906,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
-        <v>16105</v>
+      <c r="C6" s="14" t="n">
+        <v>8833</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -920,36 +920,36 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>7586</v>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
+        <v>7583</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="13" t="n">
-        <v>8519</v>
+      <c r="G6" s="14" t="n">
+        <v>1250</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="12" t="n">
+        <v>25495</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>24245</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="12" t="n">
         <v>15726</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>12285</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="12" t="n">
         <v>15892</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>24074</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>-50104</v>
+        <v>-21867</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>19468</v>
+        <v>10397</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>19468</v>
+        <v>10397</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>18892</v>
+      <c r="S7" s="14" t="n">
+        <v>-9827</v>
       </c>
     </row>
     <row r="8">
@@ -1071,9 +1071,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>-201</v>
+      <c r="S8" s="14" t="n">
+        <v>1610</v>
       </c>
     </row>
     <row r="9">
@@ -1091,13 +1091,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
-        <v>173317</v>
+      <c r="C9" s="14" t="n">
+        <v>468886</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>280932</v>
+        <v>525230</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -1113,34 +1113,34 @@
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>-107615</v>
+        <v>-56344</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="14" t="n">
+      <c r="J9" s="12" t="n">
+        <v>225959</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>282303</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="L9" s="12" t="n">
         <v>389918</v>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="M9" s="12" t="n">
         <v>192478</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="N9" s="12" t="n">
         <v>56525</v>
       </c>
-      <c r="N9" s="14" t="n">
-        <v>57913</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="12" t="inlineStr">
+      <c r="Q9" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="13" t="n">
-        <v>630</v>
+      <c r="S9" s="14" t="n">
+        <v>1077</v>
       </c>
     </row>
     <row r="10">
@@ -1160,13 +1160,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
-        <v>630</v>
+      <c r="C10" s="14" t="n">
+        <v>1143</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
@@ -1174,44 +1174,44 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
+        <v>66</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="13" t="n">
-        <v>630</v>
+      <c r="G10" s="14" t="n">
+        <v>1077</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="12" t="n">
+        <v>9155</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>8078</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="12" t="n">
         <v>7448</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="12" t="n">
         <v>7613</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="12" t="n">
         <v>8675</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>19105</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="13" t="n">
-        <v>-21171</v>
+      <c r="S10" s="11" t="n">
+        <v>917</v>
       </c>
     </row>
     <row r="11">
@@ -1229,58 +1229,58 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
-        <v>41685</v>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>-9493</v>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="C11" s="14" t="n">
+        <v>153409</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>143003</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="13" t="n">
-        <v>51178</v>
+      <c r="G11" s="14" t="n">
+        <v>10406</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="14" t="n">
+      <c r="J11" s="12" t="n">
+        <v>-279943</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-290349</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="12" t="n">
         <v>-341527</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="M11" s="12" t="n">
         <v>-252661</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="12" t="n">
         <v>-273675</v>
       </c>
-      <c r="N11" s="14" t="n">
-        <v>-207881</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q11" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>-30681</v>
+      <c r="S11" s="14" t="n">
+        <v>16965</v>
       </c>
     </row>
     <row r="12">
@@ -1298,56 +1298,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>-66485</v>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>-122292</v>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>293650</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>248788</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G12" s="13" t="n">
-        <v>55807</v>
+      <c r="G12" s="14" t="n">
+        <v>44862</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="14" t="n">
+      <c r="J12" s="12" t="n">
+        <v>44830</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>-32</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="12" t="n">
         <v>-55839</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="M12" s="12" t="n">
         <v>52569</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="12" t="n">
         <v>208475</v>
       </c>
-      <c r="N12" s="14" t="n">
-        <v>130863</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="12" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="13" t="n">
-        <v>1835</v>
+      <c r="S12" s="14" t="n">
+        <v>2140</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>149147</v>
+        <v>917088</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>149147</v>
+        <v>917087</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>7394</v>
+        <v>9049</v>
       </c>
     </row>
     <row r="14">
@@ -1463,9 +1463,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q14" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="11" t="n">
-        <v>-2672</v>
+      <c r="S14" s="14" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="15">
@@ -1489,61 +1489,61 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>496011</v>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
+        <v>102621</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="13" t="n">
-        <v>414462</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="E15" s="14" t="n">
+        <v>246800</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>-144179</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>-889061</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>-744882</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>-826431</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>-727423</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>-491486</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>81549</v>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J15" s="14" t="n">
-        <v>-744882</v>
-      </c>
-      <c r="K15" s="14" t="n">
-        <v>-826431</v>
-      </c>
-      <c r="L15" s="14" t="n">
-        <v>-727423</v>
-      </c>
-      <c r="M15" s="14" t="n">
-        <v>-491486</v>
-      </c>
-      <c r="N15" s="14" t="n">
-        <v>-472041</v>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q15" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="13" t="n">
-        <v>51178</v>
+      <c r="S15" s="14" t="n">
+        <v>10406</v>
       </c>
     </row>
     <row r="16">
@@ -1552,58 +1552,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>-21371</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="n">
-        <v>-200</v>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="n">
-        <v>-21171</v>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>1083</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>166</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>917</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="14" t="n">
+      <c r="J16" s="12" t="n">
+        <v>93007</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>92090</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="12" t="n">
         <v>113261</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="12" t="n">
         <v>97351</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="12" t="n">
         <v>89881</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>81661</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="13" t="n">
-        <v>-95060</v>
+      <c r="S16" s="11" t="n">
+        <v>70771</v>
       </c>
     </row>
     <row r="17">
@@ -1627,61 +1627,61 @@
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>11980</v>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
+        <v>115545</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="13" t="n">
-        <v>107040</v>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="E17" s="14" t="n">
+        <v>44774</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>70771</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>572931</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>502160</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>597220</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>573497</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>521237</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
-        <v>-95060</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="14" t="n">
-        <v>502160</v>
-      </c>
-      <c r="K17" s="14" t="n">
-        <v>597220</v>
-      </c>
-      <c r="L17" s="14" t="n">
-        <v>573497</v>
-      </c>
-      <c r="M17" s="14" t="n">
-        <v>521237</v>
-      </c>
-      <c r="N17" s="14" t="n">
-        <v>447027</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="13" t="n">
-        <v>19963</v>
+      <c r="S17" s="11" t="n">
+        <v>-423</v>
       </c>
     </row>
     <row r="18">
@@ -1696,15 +1696,15 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>164453</v>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
+        <v>167352</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="13" t="n">
-        <v>129771</v>
+      <c r="E18" s="14" t="n">
+        <v>94860</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
@@ -1712,34 +1712,34 @@
         </is>
       </c>
       <c r="G18" s="11" t="n">
-        <v>34682</v>
+        <v>72492</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="14" t="n">
+      <c r="J18" s="12" t="n">
+        <v>223123</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>150631</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="12" t="n">
         <v>115949</v>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="M18" s="12" t="n">
         <v>56576</v>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="N18" s="12" t="n">
         <v>-119631</v>
       </c>
-      <c r="N18" s="14" t="n">
-        <v>-56647</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="12" t="inlineStr">
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="13" t="n">
-        <v>20447</v>
+      <c r="S18" s="14" t="n">
+        <v>21130</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>651073</v>
+        <v>386601</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>651073</v>
+        <v>386600</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q19" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="13" t="n">
-        <v>-21919</v>
+      <c r="S19" s="11" t="n">
+        <v>18396</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="12" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="13" t="n">
-        <v>8519</v>
+      <c r="S20" s="14" t="n">
+        <v>1250</v>
       </c>
     </row>
     <row r="21">
@@ -1881,61 +1881,61 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-19468</v>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
+        <v>-64685</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E21" s="13" t="n">
-        <v>-27310</v>
-      </c>
-      <c r="F21" s="12" t="inlineStr">
+      <c r="E21" s="14" t="n">
+        <v>-26195</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>-38490</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3124000</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3162490</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3154648</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3193304</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3158786</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="13" t="n">
-        <v>7842</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="14" t="n">
-        <v>3162490</v>
-      </c>
-      <c r="K21" s="14" t="n">
-        <v>3154648</v>
-      </c>
-      <c r="L21" s="14" t="n">
-        <v>3193304</v>
-      </c>
-      <c r="M21" s="14" t="n">
-        <v>3158786</v>
-      </c>
-      <c r="N21" s="14" t="n">
-        <v>3179070</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="13" t="n">
-        <v>55807</v>
+      <c r="S21" s="14" t="n">
+        <v>44862</v>
       </c>
     </row>
     <row r="22">
@@ -1944,50 +1944,50 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="n">
-        <v>-902</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>29779</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G22" s="11" t="n">
-        <v>-30681</v>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>12197</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>-4768</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>16965</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="14" t="n">
+      <c r="J22" s="12" t="n">
+        <v>-4317913</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4334878</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4304197</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4317768</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4327597</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-4376554</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="11" t="n">
-        <v>34682</v>
+        <v>72492</v>
       </c>
     </row>
     <row r="23">
@@ -2013,67 +2013,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="13" t="n">
-        <v>9975</v>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>-26040</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E23" s="13" t="n">
-        <v>-9988</v>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="E23" s="14" t="n">
+        <v>-25617</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>-423</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>801090</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>801513</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>781550</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>737481</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>776664</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="13" t="n">
-        <v>19963</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="14" t="n">
-        <v>801513</v>
-      </c>
-      <c r="K23" s="14" t="n">
-        <v>781550</v>
-      </c>
-      <c r="L23" s="14" t="n">
-        <v>737481</v>
-      </c>
-      <c r="M23" s="14" t="n">
-        <v>776664</v>
-      </c>
-      <c r="N23" s="14" t="n">
-        <v>786561</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="13" t="n">
-        <v>2876</v>
+      <c r="S23" s="14" t="n">
+        <v>21948</v>
       </c>
     </row>
     <row r="24">
@@ -2088,52 +2088,52 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>-39905</v>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
+        <v>-4560</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E24" s="13" t="n">
-        <v>-42781</v>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
+      <c r="E24" s="14" t="n">
+        <v>-26508</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G24" s="13" t="n">
-        <v>2876</v>
+      <c r="G24" s="14" t="n">
+        <v>21948</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="14" t="n">
+      <c r="J24" s="12" t="n">
+        <v>392823</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>370875</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="12" t="n">
         <v>367999</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="12" t="n">
         <v>386983</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="12" t="n">
         <v>392147</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>410923</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q24" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="13" t="n">
-        <v>27822</v>
+      <c r="S24" s="11" t="n">
+        <v>-1403</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-50300</v>
+        <v>-83088</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-50300</v>
+        <v>-83088</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,7 +2178,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="12" t="inlineStr">
+      <c r="Q25" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="13" t="n">
-        <v>-4367</v>
+      <c r="S25" s="14" t="n">
+        <v>-17618</v>
       </c>
     </row>
     <row r="26">
@@ -2255,15 +2255,15 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>-61610</v>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
+        <v>-62719</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E27" s="13" t="n">
-        <v>-11506</v>
+      <c r="E27" s="14" t="n">
+        <v>-40852</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,27 +2271,27 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>-50104</v>
+        <v>-21867</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>1145879</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1167746</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>1217850</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>1159981</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="12" t="n">
         <v>1031589</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>943689</v>
       </c>
     </row>
     <row r="28">
@@ -2306,43 +2306,43 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>-201</v>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
+        <v>-225</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E28" s="13" t="n">
-        <v>-2036</v>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>-2365</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G28" s="13" t="n">
-        <v>1835</v>
+      <c r="G28" s="14" t="n">
+        <v>2140</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-432616</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-434756</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-436591</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-438630</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="12" t="n">
         <v>-423028</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-404104</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,53 +2359,53 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="13" t="n">
-        <v>8933</v>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="C29" s="14" t="n">
+        <v>2076</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E29" s="13" t="n">
-        <v>-11514</v>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
+      <c r="E29" s="14" t="n">
+        <v>-19054</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G29" s="13" t="n">
-        <v>20447</v>
+      <c r="G29" s="14" t="n">
+        <v>21130</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-181517</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-202647</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-223094</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-209490</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="12" t="n">
         <v>-157660</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-149590</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 22-Oct-2026 OHLC</t>
+          <t>Next session  -  based on 23-Oct-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,57 +2418,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="n">
-        <v>19596</v>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>-1528</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E30" s="13" t="n">
-        <v>-8226</v>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="n">
-        <v>27822</v>
+      <c r="E30" s="14" t="n">
+        <v>-125</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="n">
+        <v>-1403</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-531746</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-530343</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-558165</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-511861</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="12" t="n">
         <v>-450901</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-389995</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>22687.75